<commit_message>
comit code sau khi code xong kpi gen
</commit_message>
<xml_diff>
--- a/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
+++ b/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonzai/dev/odoo 19/odoo/my_custom_addons/dl_salary_kpi/static/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95443975-FFCE-AA43-BF24-9AE56EB1AB53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA8ACBB7-B4DC-0145-8532-EB1074419478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kangatang" sheetId="43" state="veryHidden" r:id="rId1"/>
@@ -2476,37 +2476,70 @@
     <xf numFmtId="14" fontId="59" fillId="0" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="59" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="14" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="55" fillId="14" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2551,22 +2584,10 @@
     <xf numFmtId="0" fontId="66" fillId="25" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2575,72 +2596,35 @@
     <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="14" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="14" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="7" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2655,6 +2639,22 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="32">
@@ -3484,11 +3484,11 @@
       <c r="AL1" s="213"/>
       <c r="AM1" s="213"/>
       <c r="AN1" s="213"/>
-      <c r="AO1" s="276"/>
-      <c r="AP1" s="276"/>
-      <c r="AQ1" s="276"/>
-      <c r="AR1" s="276"/>
-      <c r="AS1" s="276"/>
+      <c r="AO1" s="325"/>
+      <c r="AP1" s="325"/>
+      <c r="AQ1" s="325"/>
+      <c r="AR1" s="325"/>
+      <c r="AS1" s="325"/>
       <c r="AT1" s="120"/>
       <c r="AU1" s="120"/>
       <c r="AV1" s="120"/>
@@ -3902,40 +3902,40 @@
       <c r="G4" s="238"/>
       <c r="H4" s="108"/>
       <c r="I4" s="275"/>
-      <c r="J4" s="277" t="s">
+      <c r="J4" s="316" t="s">
         <v>68</v>
       </c>
-      <c r="K4" s="277"/>
-      <c r="L4" s="278">
+      <c r="K4" s="316"/>
+      <c r="L4" s="319">
         <v>3</v>
       </c>
-      <c r="M4" s="278"/>
-      <c r="N4" s="277" t="s">
+      <c r="M4" s="319"/>
+      <c r="N4" s="316" t="s">
         <v>69</v>
       </c>
-      <c r="O4" s="277"/>
-      <c r="P4" s="277">
+      <c r="O4" s="316"/>
+      <c r="P4" s="316">
         <v>2026</v>
       </c>
-      <c r="Q4" s="277"/>
+      <c r="Q4" s="316"/>
       <c r="R4" s="109"/>
-      <c r="S4" s="277"/>
-      <c r="T4" s="277"/>
-      <c r="U4" s="277"/>
+      <c r="S4" s="316"/>
+      <c r="T4" s="316"/>
+      <c r="U4" s="316"/>
       <c r="V4" s="109"/>
-      <c r="W4" s="277"/>
-      <c r="X4" s="277"/>
-      <c r="Y4" s="277"/>
-      <c r="Z4" s="277"/>
-      <c r="AA4" s="277"/>
-      <c r="AB4" s="277"/>
-      <c r="AC4" s="277"/>
-      <c r="AD4" s="277"/>
+      <c r="W4" s="316"/>
+      <c r="X4" s="316"/>
+      <c r="Y4" s="316"/>
+      <c r="Z4" s="316"/>
+      <c r="AA4" s="316"/>
+      <c r="AB4" s="316"/>
+      <c r="AC4" s="316"/>
+      <c r="AD4" s="316"/>
       <c r="AE4" s="109"/>
       <c r="AF4" s="110"/>
-      <c r="AG4" s="277"/>
-      <c r="AH4" s="277"/>
-      <c r="AI4" s="277"/>
+      <c r="AG4" s="316"/>
+      <c r="AH4" s="316"/>
+      <c r="AI4" s="316"/>
       <c r="AJ4" s="109"/>
       <c r="AK4" s="109"/>
       <c r="AL4" s="109"/>
@@ -3946,41 +3946,41 @@
       <c r="AQ4" s="113"/>
       <c r="AR4" s="224"/>
       <c r="AS4" s="233"/>
-      <c r="AT4" s="277" t="s">
+      <c r="AT4" s="316" t="s">
         <v>68</v>
       </c>
-      <c r="AU4" s="277"/>
-      <c r="AV4" s="278">
+      <c r="AU4" s="316"/>
+      <c r="AV4" s="319">
         <f>L4</f>
         <v>3</v>
       </c>
-      <c r="AW4" s="278"/>
-      <c r="AX4" s="277" t="s">
+      <c r="AW4" s="319"/>
+      <c r="AX4" s="316" t="s">
         <v>69</v>
       </c>
-      <c r="AY4" s="277"/>
-      <c r="AZ4" s="277">
+      <c r="AY4" s="316"/>
+      <c r="AZ4" s="316">
         <v>2025</v>
       </c>
-      <c r="BA4" s="277"/>
+      <c r="BA4" s="316"/>
       <c r="BB4" s="109"/>
-      <c r="BC4" s="277"/>
-      <c r="BD4" s="277"/>
-      <c r="BE4" s="277"/>
+      <c r="BC4" s="316"/>
+      <c r="BD4" s="316"/>
+      <c r="BE4" s="316"/>
       <c r="BF4" s="109"/>
-      <c r="BG4" s="277"/>
-      <c r="BH4" s="277"/>
-      <c r="BI4" s="277"/>
-      <c r="BJ4" s="277"/>
-      <c r="BK4" s="277"/>
-      <c r="BL4" s="277"/>
-      <c r="BM4" s="277"/>
-      <c r="BN4" s="277"/>
+      <c r="BG4" s="316"/>
+      <c r="BH4" s="316"/>
+      <c r="BI4" s="316"/>
+      <c r="BJ4" s="316"/>
+      <c r="BK4" s="316"/>
+      <c r="BL4" s="316"/>
+      <c r="BM4" s="316"/>
+      <c r="BN4" s="316"/>
       <c r="BO4" s="109"/>
       <c r="BP4" s="110"/>
-      <c r="BQ4" s="277"/>
-      <c r="BR4" s="277"/>
-      <c r="BS4" s="277"/>
+      <c r="BQ4" s="316"/>
+      <c r="BR4" s="316"/>
+      <c r="BS4" s="316"/>
       <c r="BT4" s="114"/>
       <c r="BU4" s="114" t="str">
         <f>IF(WEEKDAY(BU5,1)=1,"CN","")</f>
@@ -4097,31 +4097,31 @@
       <c r="EV4" s="247"/>
     </row>
     <row r="5" spans="1:154" s="184" customFormat="1" ht="92.25" customHeight="1">
-      <c r="A5" s="279" t="s">
+      <c r="A5" s="317" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="280" t="s">
+      <c r="B5" s="277" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="279" t="s">
+      <c r="C5" s="317" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="281" t="s">
+      <c r="D5" s="322" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="282" t="s">
+      <c r="E5" s="323" t="s">
         <v>122</v>
       </c>
-      <c r="F5" s="279" t="s">
+      <c r="F5" s="317" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="279" t="s">
+      <c r="G5" s="317" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="279" t="s">
+      <c r="H5" s="317" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="284" t="s">
+      <c r="I5" s="318" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="175">
@@ -4248,19 +4248,19 @@
         <f t="shared" si="0"/>
         <v>46112</v>
       </c>
-      <c r="AO5" s="285" t="s">
+      <c r="AO5" s="320" t="s">
         <v>82</v>
       </c>
-      <c r="AP5" s="285" t="s">
+      <c r="AP5" s="320" t="s">
         <v>83</v>
       </c>
-      <c r="AQ5" s="285" t="s">
+      <c r="AQ5" s="320" t="s">
         <v>84</v>
       </c>
-      <c r="AR5" s="286" t="s">
+      <c r="AR5" s="321" t="s">
         <v>5</v>
       </c>
-      <c r="AS5" s="286" t="s">
+      <c r="AS5" s="321" t="s">
         <v>6</v>
       </c>
       <c r="AT5" s="179">
@@ -4387,46 +4387,46 @@
         <f t="shared" si="1"/>
         <v>46112</v>
       </c>
-      <c r="BY5" s="309" t="s">
+      <c r="BY5" s="294" t="s">
         <v>86</v>
       </c>
-      <c r="BZ5" s="309" t="s">
+      <c r="BZ5" s="294" t="s">
         <v>87</v>
       </c>
-      <c r="CA5" s="309" t="s">
+      <c r="CA5" s="294" t="s">
         <v>88</v>
       </c>
-      <c r="CB5" s="309" t="s">
+      <c r="CB5" s="294" t="s">
         <v>89</v>
       </c>
-      <c r="CC5" s="309" t="s">
+      <c r="CC5" s="294" t="s">
         <v>90</v>
       </c>
-      <c r="CD5" s="309" t="s">
+      <c r="CD5" s="294" t="s">
         <v>91</v>
       </c>
-      <c r="CE5" s="309" t="s">
+      <c r="CE5" s="294" t="s">
         <v>92</v>
       </c>
-      <c r="CF5" s="311" t="s">
+      <c r="CF5" s="296" t="s">
         <v>19</v>
       </c>
-      <c r="CG5" s="311"/>
-      <c r="CH5" s="311"/>
-      <c r="CI5" s="311"/>
-      <c r="CJ5" s="311"/>
-      <c r="CK5" s="311"/>
-      <c r="CL5" s="311"/>
-      <c r="CM5" s="311"/>
-      <c r="CN5" s="311"/>
-      <c r="CO5" s="311"/>
-      <c r="CP5" s="311"/>
-      <c r="CQ5" s="315" t="s">
+      <c r="CG5" s="296"/>
+      <c r="CH5" s="296"/>
+      <c r="CI5" s="296"/>
+      <c r="CJ5" s="296"/>
+      <c r="CK5" s="296"/>
+      <c r="CL5" s="296"/>
+      <c r="CM5" s="296"/>
+      <c r="CN5" s="296"/>
+      <c r="CO5" s="296"/>
+      <c r="CP5" s="296"/>
+      <c r="CQ5" s="280" t="s">
         <v>59</v>
       </c>
-      <c r="CR5" s="316"/>
-      <c r="CS5" s="317"/>
-      <c r="CT5" s="322" t="s">
+      <c r="CR5" s="281"/>
+      <c r="CS5" s="282"/>
+      <c r="CT5" s="287" t="s">
         <v>60</v>
       </c>
       <c r="CU5" s="261" t="s">
@@ -4449,117 +4449,117 @@
       <c r="DF5" s="259" t="s">
         <v>130</v>
       </c>
-      <c r="DG5" s="318" t="s">
+      <c r="DG5" s="283" t="s">
         <v>119</v>
       </c>
-      <c r="DH5" s="323" t="s">
+      <c r="DH5" s="288" t="s">
         <v>113</v>
       </c>
-      <c r="DI5" s="320" t="s">
+      <c r="DI5" s="285" t="s">
         <v>81</v>
       </c>
-      <c r="DJ5" s="321"/>
-      <c r="DK5" s="304" t="s">
+      <c r="DJ5" s="286"/>
+      <c r="DK5" s="289" t="s">
         <v>61</v>
       </c>
-      <c r="DL5" s="312" t="s">
+      <c r="DL5" s="297" t="s">
         <v>8</v>
       </c>
-      <c r="DM5" s="305" t="s">
+      <c r="DM5" s="290" t="s">
         <v>71</v>
       </c>
-      <c r="DN5" s="305"/>
-      <c r="DO5" s="305"/>
-      <c r="DP5" s="305"/>
-      <c r="DQ5" s="305"/>
-      <c r="DR5" s="305"/>
-      <c r="DS5" s="324" t="s">
+      <c r="DN5" s="290"/>
+      <c r="DO5" s="290"/>
+      <c r="DP5" s="290"/>
+      <c r="DQ5" s="290"/>
+      <c r="DR5" s="290"/>
+      <c r="DS5" s="291" t="s">
         <v>12</v>
       </c>
-      <c r="DT5" s="305" t="s">
+      <c r="DT5" s="290" t="s">
         <v>128</v>
       </c>
-      <c r="DU5" s="280" t="s">
+      <c r="DU5" s="277" t="s">
         <v>13</v>
       </c>
-      <c r="DV5" s="313" t="s">
+      <c r="DV5" s="278" t="s">
         <v>64</v>
       </c>
-      <c r="DW5" s="314"/>
-      <c r="DX5" s="313"/>
-      <c r="DY5" s="302" t="s">
+      <c r="DW5" s="279"/>
+      <c r="DX5" s="278"/>
+      <c r="DY5" s="312" t="s">
         <v>63</v>
       </c>
-      <c r="DZ5" s="302"/>
-      <c r="EA5" s="302"/>
-      <c r="EB5" s="302"/>
-      <c r="EC5" s="303" t="s">
+      <c r="DZ5" s="312"/>
+      <c r="EA5" s="312"/>
+      <c r="EB5" s="312"/>
+      <c r="EC5" s="313" t="s">
         <v>131</v>
       </c>
-      <c r="ED5" s="305" t="s">
+      <c r="ED5" s="290" t="s">
         <v>7</v>
       </c>
-      <c r="EE5" s="306" t="s">
+      <c r="EE5" s="292" t="s">
         <v>65</v>
       </c>
-      <c r="EF5" s="306"/>
-      <c r="EG5" s="306" t="s">
+      <c r="EF5" s="292"/>
+      <c r="EG5" s="292" t="s">
         <v>66</v>
       </c>
-      <c r="EH5" s="306" t="s">
+      <c r="EH5" s="292" t="s">
         <v>67</v>
       </c>
-      <c r="EI5" s="306" t="s">
+      <c r="EI5" s="292" t="s">
         <v>72</v>
       </c>
-      <c r="EJ5" s="325" t="s">
+      <c r="EJ5" s="293" t="s">
         <v>78</v>
       </c>
-      <c r="EK5" s="325" t="s">
+      <c r="EK5" s="293" t="s">
         <v>80</v>
       </c>
-      <c r="EL5" s="325" t="s">
+      <c r="EL5" s="293" t="s">
         <v>79</v>
       </c>
-      <c r="EM5" s="291" t="s">
+      <c r="EM5" s="302" t="s">
         <v>127</v>
       </c>
-      <c r="EN5" s="293"/>
-      <c r="EO5" s="295" t="s">
+      <c r="EN5" s="304"/>
+      <c r="EO5" s="306" t="s">
         <v>132</v>
       </c>
-      <c r="EP5" s="297" t="s">
+      <c r="EP5" s="308" t="s">
         <v>118</v>
       </c>
-      <c r="EQ5" s="299" t="s">
+      <c r="EQ5" s="310" t="s">
         <v>133</v>
       </c>
-      <c r="ER5" s="301" t="s">
+      <c r="ER5" s="276" t="s">
         <v>125</v>
       </c>
-      <c r="ES5" s="301" t="s">
+      <c r="ES5" s="276" t="s">
         <v>124</v>
       </c>
-      <c r="ET5" s="307" t="s">
+      <c r="ET5" s="314" t="s">
         <v>120</v>
       </c>
-      <c r="EU5" s="287" t="s">
+      <c r="EU5" s="298" t="s">
         <v>123</v>
       </c>
-      <c r="EV5" s="289" t="s">
+      <c r="EV5" s="300" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:154" s="206" customFormat="1" ht="148.5" customHeight="1">
-      <c r="A6" s="279"/>
-      <c r="B6" s="280"/>
-      <c r="C6" s="279"/>
-      <c r="D6" s="281"/>
-      <c r="E6" s="283"/>
-      <c r="F6" s="279"/>
-      <c r="G6" s="279"/>
-      <c r="H6" s="279"/>
-      <c r="I6" s="284"/>
+      <c r="A6" s="317"/>
+      <c r="B6" s="277"/>
+      <c r="C6" s="317"/>
+      <c r="D6" s="322"/>
+      <c r="E6" s="324"/>
+      <c r="F6" s="317"/>
+      <c r="G6" s="317"/>
+      <c r="H6" s="317"/>
+      <c r="I6" s="318"/>
       <c r="J6" s="185" t="str">
         <f t="shared" ref="J6:AN6" si="2">IF(WEEKDAY(J5)=1,"CN",WEEKDAY(J5))</f>
         <v>CN</v>
@@ -4684,11 +4684,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AO6" s="285"/>
-      <c r="AP6" s="285"/>
-      <c r="AQ6" s="285"/>
-      <c r="AR6" s="286"/>
-      <c r="AS6" s="286"/>
+      <c r="AO6" s="320"/>
+      <c r="AP6" s="320"/>
+      <c r="AQ6" s="320"/>
+      <c r="AR6" s="321"/>
+      <c r="AS6" s="321"/>
       <c r="AT6" s="187" t="str">
         <f>+J6</f>
         <v>CN</v>
@@ -4813,13 +4813,13 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="BY6" s="310"/>
-      <c r="BZ6" s="310"/>
-      <c r="CA6" s="310"/>
-      <c r="CB6" s="310"/>
-      <c r="CC6" s="310"/>
-      <c r="CD6" s="310"/>
-      <c r="CE6" s="310"/>
+      <c r="BY6" s="295"/>
+      <c r="BZ6" s="295"/>
+      <c r="CA6" s="295"/>
+      <c r="CB6" s="295"/>
+      <c r="CC6" s="295"/>
+      <c r="CD6" s="295"/>
+      <c r="CE6" s="295"/>
       <c r="CF6" s="189" t="s">
         <v>93</v>
       </c>
@@ -4862,7 +4862,7 @@
       <c r="CS6" s="181" t="s">
         <v>58</v>
       </c>
-      <c r="CT6" s="322"/>
+      <c r="CT6" s="287"/>
       <c r="CU6" s="189" t="s">
         <v>104</v>
       </c>
@@ -4899,16 +4899,16 @@
       <c r="DF6" s="260" t="s">
         <v>134</v>
       </c>
-      <c r="DG6" s="319"/>
-      <c r="DH6" s="323"/>
+      <c r="DG6" s="284"/>
+      <c r="DH6" s="288"/>
       <c r="DI6" s="152" t="s">
         <v>14</v>
       </c>
       <c r="DJ6" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="DK6" s="304"/>
-      <c r="DL6" s="312"/>
+      <c r="DK6" s="289"/>
+      <c r="DL6" s="297"/>
       <c r="DM6" s="181" t="s">
         <v>9</v>
       </c>
@@ -4927,9 +4927,9 @@
       <c r="DR6" s="181" t="s">
         <v>116</v>
       </c>
-      <c r="DS6" s="324"/>
-      <c r="DT6" s="305"/>
-      <c r="DU6" s="280"/>
+      <c r="DS6" s="291"/>
+      <c r="DT6" s="290"/>
+      <c r="DU6" s="277"/>
       <c r="DV6" s="204">
         <v>0.17499999999999999</v>
       </c>
@@ -4951,176 +4951,176 @@
       <c r="EB6" s="152" t="s">
         <v>62</v>
       </c>
-      <c r="EC6" s="304"/>
-      <c r="ED6" s="305"/>
+      <c r="EC6" s="289"/>
+      <c r="ED6" s="290"/>
       <c r="EE6" s="183" t="s">
         <v>73</v>
       </c>
       <c r="EF6" s="183" t="s">
         <v>74</v>
       </c>
-      <c r="EG6" s="306"/>
-      <c r="EH6" s="306"/>
-      <c r="EI6" s="306"/>
-      <c r="EJ6" s="325"/>
-      <c r="EK6" s="325"/>
-      <c r="EL6" s="325"/>
-      <c r="EM6" s="292"/>
-      <c r="EN6" s="294"/>
-      <c r="EO6" s="296"/>
-      <c r="EP6" s="298"/>
-      <c r="EQ6" s="300"/>
-      <c r="ER6" s="301"/>
-      <c r="ES6" s="301"/>
-      <c r="ET6" s="308"/>
-      <c r="EU6" s="288"/>
-      <c r="EV6" s="289"/>
+      <c r="EG6" s="292"/>
+      <c r="EH6" s="292"/>
+      <c r="EI6" s="292"/>
+      <c r="EJ6" s="293"/>
+      <c r="EK6" s="293"/>
+      <c r="EL6" s="293"/>
+      <c r="EM6" s="303"/>
+      <c r="EN6" s="305"/>
+      <c r="EO6" s="307"/>
+      <c r="EP6" s="309"/>
+      <c r="EQ6" s="311"/>
+      <c r="ER6" s="276"/>
+      <c r="ES6" s="276"/>
+      <c r="ET6" s="315"/>
+      <c r="EU6" s="299"/>
+      <c r="EV6" s="300"/>
     </row>
     <row r="7" spans="1:154" s="106" customFormat="1" ht="87.75" customHeight="1">
-      <c r="A7" s="290" t="s">
+      <c r="A7" s="301" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="290"/>
-      <c r="C7" s="290"/>
-      <c r="D7" s="290"/>
-      <c r="E7" s="290"/>
-      <c r="F7" s="290"/>
-      <c r="G7" s="290"/>
-      <c r="H7" s="290"/>
-      <c r="I7" s="290"/>
-      <c r="J7" s="290"/>
-      <c r="K7" s="290"/>
-      <c r="L7" s="290"/>
-      <c r="M7" s="290"/>
-      <c r="N7" s="290"/>
-      <c r="O7" s="290"/>
-      <c r="P7" s="290"/>
-      <c r="Q7" s="290"/>
-      <c r="R7" s="290"/>
-      <c r="S7" s="290"/>
-      <c r="T7" s="290"/>
-      <c r="U7" s="290"/>
-      <c r="V7" s="290"/>
-      <c r="W7" s="290"/>
-      <c r="X7" s="290"/>
-      <c r="Y7" s="290"/>
-      <c r="Z7" s="290"/>
-      <c r="AA7" s="290"/>
-      <c r="AB7" s="290"/>
-      <c r="AC7" s="290"/>
-      <c r="AD7" s="290"/>
-      <c r="AE7" s="290"/>
-      <c r="AF7" s="290"/>
-      <c r="AG7" s="290"/>
-      <c r="AH7" s="290"/>
-      <c r="AI7" s="290"/>
-      <c r="AJ7" s="290"/>
-      <c r="AK7" s="290"/>
-      <c r="AL7" s="290"/>
-      <c r="AM7" s="290"/>
-      <c r="AN7" s="290"/>
-      <c r="AO7" s="290"/>
-      <c r="AP7" s="290"/>
-      <c r="AQ7" s="290"/>
-      <c r="AR7" s="290"/>
-      <c r="AS7" s="290"/>
-      <c r="AT7" s="290"/>
-      <c r="AU7" s="290"/>
-      <c r="AV7" s="290"/>
-      <c r="AW7" s="290"/>
-      <c r="AX7" s="290"/>
-      <c r="AY7" s="290"/>
-      <c r="AZ7" s="290"/>
-      <c r="BA7" s="290"/>
-      <c r="BB7" s="290"/>
-      <c r="BC7" s="290"/>
-      <c r="BD7" s="290"/>
-      <c r="BE7" s="290"/>
-      <c r="BF7" s="290"/>
-      <c r="BG7" s="290"/>
-      <c r="BH7" s="290"/>
-      <c r="BI7" s="290"/>
-      <c r="BJ7" s="290"/>
-      <c r="BK7" s="290"/>
-      <c r="BL7" s="290"/>
-      <c r="BM7" s="290"/>
-      <c r="BN7" s="290"/>
-      <c r="BO7" s="290"/>
-      <c r="BP7" s="290"/>
-      <c r="BQ7" s="290"/>
-      <c r="BR7" s="290"/>
-      <c r="BS7" s="290"/>
-      <c r="BT7" s="290"/>
-      <c r="BU7" s="290"/>
-      <c r="BV7" s="290"/>
-      <c r="BW7" s="290"/>
-      <c r="BX7" s="290"/>
-      <c r="BY7" s="290"/>
-      <c r="BZ7" s="290"/>
-      <c r="CA7" s="290"/>
-      <c r="CB7" s="290"/>
-      <c r="CC7" s="290"/>
-      <c r="CD7" s="290"/>
-      <c r="CE7" s="290"/>
-      <c r="CF7" s="290"/>
-      <c r="CG7" s="290"/>
-      <c r="CH7" s="290"/>
-      <c r="CI7" s="290"/>
-      <c r="CJ7" s="290"/>
-      <c r="CK7" s="290"/>
-      <c r="CL7" s="290"/>
-      <c r="CM7" s="290"/>
-      <c r="CN7" s="290"/>
-      <c r="CO7" s="290"/>
-      <c r="CP7" s="290"/>
-      <c r="CQ7" s="290"/>
-      <c r="CR7" s="290"/>
-      <c r="CS7" s="290"/>
-      <c r="CT7" s="290"/>
-      <c r="CU7" s="290"/>
-      <c r="CV7" s="290"/>
-      <c r="CW7" s="290"/>
-      <c r="CX7" s="290"/>
-      <c r="CY7" s="290"/>
-      <c r="CZ7" s="290"/>
-      <c r="DA7" s="290"/>
-      <c r="DB7" s="290"/>
-      <c r="DC7" s="290"/>
-      <c r="DD7" s="290"/>
-      <c r="DE7" s="290"/>
-      <c r="DF7" s="290"/>
-      <c r="DG7" s="290"/>
-      <c r="DH7" s="290"/>
-      <c r="DI7" s="290"/>
-      <c r="DJ7" s="290"/>
-      <c r="DK7" s="290"/>
-      <c r="DL7" s="290"/>
-      <c r="DM7" s="290"/>
-      <c r="DN7" s="290"/>
-      <c r="DO7" s="290"/>
-      <c r="DP7" s="290"/>
-      <c r="DQ7" s="290"/>
-      <c r="DR7" s="290"/>
-      <c r="DS7" s="290"/>
-      <c r="DT7" s="290"/>
-      <c r="DU7" s="290"/>
-      <c r="DV7" s="290"/>
-      <c r="DW7" s="290"/>
-      <c r="DX7" s="290"/>
-      <c r="DY7" s="290"/>
-      <c r="DZ7" s="290"/>
-      <c r="EA7" s="290"/>
-      <c r="EB7" s="290"/>
-      <c r="EC7" s="290"/>
-      <c r="ED7" s="290"/>
-      <c r="EE7" s="290"/>
-      <c r="EF7" s="290"/>
-      <c r="EG7" s="290"/>
-      <c r="EH7" s="290"/>
-      <c r="EI7" s="290"/>
-      <c r="EJ7" s="290"/>
-      <c r="EK7" s="290"/>
-      <c r="EL7" s="290"/>
+      <c r="B7" s="301"/>
+      <c r="C7" s="301"/>
+      <c r="D7" s="301"/>
+      <c r="E7" s="301"/>
+      <c r="F7" s="301"/>
+      <c r="G7" s="301"/>
+      <c r="H7" s="301"/>
+      <c r="I7" s="301"/>
+      <c r="J7" s="301"/>
+      <c r="K7" s="301"/>
+      <c r="L7" s="301"/>
+      <c r="M7" s="301"/>
+      <c r="N7" s="301"/>
+      <c r="O7" s="301"/>
+      <c r="P7" s="301"/>
+      <c r="Q7" s="301"/>
+      <c r="R7" s="301"/>
+      <c r="S7" s="301"/>
+      <c r="T7" s="301"/>
+      <c r="U7" s="301"/>
+      <c r="V7" s="301"/>
+      <c r="W7" s="301"/>
+      <c r="X7" s="301"/>
+      <c r="Y7" s="301"/>
+      <c r="Z7" s="301"/>
+      <c r="AA7" s="301"/>
+      <c r="AB7" s="301"/>
+      <c r="AC7" s="301"/>
+      <c r="AD7" s="301"/>
+      <c r="AE7" s="301"/>
+      <c r="AF7" s="301"/>
+      <c r="AG7" s="301"/>
+      <c r="AH7" s="301"/>
+      <c r="AI7" s="301"/>
+      <c r="AJ7" s="301"/>
+      <c r="AK7" s="301"/>
+      <c r="AL7" s="301"/>
+      <c r="AM7" s="301"/>
+      <c r="AN7" s="301"/>
+      <c r="AO7" s="301"/>
+      <c r="AP7" s="301"/>
+      <c r="AQ7" s="301"/>
+      <c r="AR7" s="301"/>
+      <c r="AS7" s="301"/>
+      <c r="AT7" s="301"/>
+      <c r="AU7" s="301"/>
+      <c r="AV7" s="301"/>
+      <c r="AW7" s="301"/>
+      <c r="AX7" s="301"/>
+      <c r="AY7" s="301"/>
+      <c r="AZ7" s="301"/>
+      <c r="BA7" s="301"/>
+      <c r="BB7" s="301"/>
+      <c r="BC7" s="301"/>
+      <c r="BD7" s="301"/>
+      <c r="BE7" s="301"/>
+      <c r="BF7" s="301"/>
+      <c r="BG7" s="301"/>
+      <c r="BH7" s="301"/>
+      <c r="BI7" s="301"/>
+      <c r="BJ7" s="301"/>
+      <c r="BK7" s="301"/>
+      <c r="BL7" s="301"/>
+      <c r="BM7" s="301"/>
+      <c r="BN7" s="301"/>
+      <c r="BO7" s="301"/>
+      <c r="BP7" s="301"/>
+      <c r="BQ7" s="301"/>
+      <c r="BR7" s="301"/>
+      <c r="BS7" s="301"/>
+      <c r="BT7" s="301"/>
+      <c r="BU7" s="301"/>
+      <c r="BV7" s="301"/>
+      <c r="BW7" s="301"/>
+      <c r="BX7" s="301"/>
+      <c r="BY7" s="301"/>
+      <c r="BZ7" s="301"/>
+      <c r="CA7" s="301"/>
+      <c r="CB7" s="301"/>
+      <c r="CC7" s="301"/>
+      <c r="CD7" s="301"/>
+      <c r="CE7" s="301"/>
+      <c r="CF7" s="301"/>
+      <c r="CG7" s="301"/>
+      <c r="CH7" s="301"/>
+      <c r="CI7" s="301"/>
+      <c r="CJ7" s="301"/>
+      <c r="CK7" s="301"/>
+      <c r="CL7" s="301"/>
+      <c r="CM7" s="301"/>
+      <c r="CN7" s="301"/>
+      <c r="CO7" s="301"/>
+      <c r="CP7" s="301"/>
+      <c r="CQ7" s="301"/>
+      <c r="CR7" s="301"/>
+      <c r="CS7" s="301"/>
+      <c r="CT7" s="301"/>
+      <c r="CU7" s="301"/>
+      <c r="CV7" s="301"/>
+      <c r="CW7" s="301"/>
+      <c r="CX7" s="301"/>
+      <c r="CY7" s="301"/>
+      <c r="CZ7" s="301"/>
+      <c r="DA7" s="301"/>
+      <c r="DB7" s="301"/>
+      <c r="DC7" s="301"/>
+      <c r="DD7" s="301"/>
+      <c r="DE7" s="301"/>
+      <c r="DF7" s="301"/>
+      <c r="DG7" s="301"/>
+      <c r="DH7" s="301"/>
+      <c r="DI7" s="301"/>
+      <c r="DJ7" s="301"/>
+      <c r="DK7" s="301"/>
+      <c r="DL7" s="301"/>
+      <c r="DM7" s="301"/>
+      <c r="DN7" s="301"/>
+      <c r="DO7" s="301"/>
+      <c r="DP7" s="301"/>
+      <c r="DQ7" s="301"/>
+      <c r="DR7" s="301"/>
+      <c r="DS7" s="301"/>
+      <c r="DT7" s="301"/>
+      <c r="DU7" s="301"/>
+      <c r="DV7" s="301"/>
+      <c r="DW7" s="301"/>
+      <c r="DX7" s="301"/>
+      <c r="DY7" s="301"/>
+      <c r="DZ7" s="301"/>
+      <c r="EA7" s="301"/>
+      <c r="EB7" s="301"/>
+      <c r="EC7" s="301"/>
+      <c r="ED7" s="301"/>
+      <c r="EE7" s="301"/>
+      <c r="EF7" s="301"/>
+      <c r="EG7" s="301"/>
+      <c r="EH7" s="301"/>
+      <c r="EI7" s="301"/>
+      <c r="EJ7" s="301"/>
+      <c r="EK7" s="301"/>
+      <c r="EL7" s="301"/>
       <c r="EM7" s="248"/>
       <c r="EN7" s="248"/>
       <c r="EO7" s="248"/>
@@ -27901,6 +27901,64 @@
   </sheetData>
   <autoFilter ref="A6:EX8" xr:uid="{00000000-0001-0000-0900-000000000000}"/>
   <mergeCells count="74">
+    <mergeCell ref="AO1:AS1"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:U4"/>
+    <mergeCell ref="W4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="AG4:AI4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="BG4:BI4"/>
+    <mergeCell ref="AT4:AU4"/>
+    <mergeCell ref="AV4:AW4"/>
+    <mergeCell ref="AX4:AY4"/>
+    <mergeCell ref="AO5:AO6"/>
+    <mergeCell ref="AP5:AP6"/>
+    <mergeCell ref="AQ5:AQ6"/>
+    <mergeCell ref="AR5:AR6"/>
+    <mergeCell ref="AS5:AS6"/>
+    <mergeCell ref="BJ4:BK4"/>
+    <mergeCell ref="BL4:BN4"/>
+    <mergeCell ref="BQ4:BS4"/>
+    <mergeCell ref="AZ4:BA4"/>
+    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="EU5:EU6"/>
+    <mergeCell ref="EV5:EV6"/>
+    <mergeCell ref="A7:EL7"/>
+    <mergeCell ref="EM5:EM6"/>
+    <mergeCell ref="EN5:EN6"/>
+    <mergeCell ref="EO5:EO6"/>
+    <mergeCell ref="EP5:EP6"/>
+    <mergeCell ref="EQ5:EQ6"/>
+    <mergeCell ref="ER5:ER6"/>
+    <mergeCell ref="DY5:EB5"/>
+    <mergeCell ref="EC5:EC6"/>
+    <mergeCell ref="ED5:ED6"/>
+    <mergeCell ref="EE5:EF5"/>
+    <mergeCell ref="DT5:DT6"/>
+    <mergeCell ref="ET5:ET6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="CF5:CP5"/>
+    <mergeCell ref="CD5:CD6"/>
+    <mergeCell ref="CE5:CE6"/>
+    <mergeCell ref="DL5:DL6"/>
+    <mergeCell ref="EG5:EG6"/>
+    <mergeCell ref="BY5:BY6"/>
+    <mergeCell ref="BZ5:BZ6"/>
+    <mergeCell ref="CA5:CA6"/>
+    <mergeCell ref="CB5:CB6"/>
+    <mergeCell ref="CC5:CC6"/>
     <mergeCell ref="ES5:ES6"/>
     <mergeCell ref="DU5:DU6"/>
     <mergeCell ref="DV5:DX5"/>
@@ -27917,64 +27975,6 @@
     <mergeCell ref="EK5:EK6"/>
     <mergeCell ref="EL5:EL6"/>
     <mergeCell ref="EH5:EH6"/>
-    <mergeCell ref="BY5:BY6"/>
-    <mergeCell ref="BZ5:BZ6"/>
-    <mergeCell ref="CA5:CA6"/>
-    <mergeCell ref="CB5:CB6"/>
-    <mergeCell ref="CC5:CC6"/>
-    <mergeCell ref="CF5:CP5"/>
-    <mergeCell ref="CD5:CD6"/>
-    <mergeCell ref="CE5:CE6"/>
-    <mergeCell ref="DL5:DL6"/>
-    <mergeCell ref="EG5:EG6"/>
-    <mergeCell ref="EU5:EU6"/>
-    <mergeCell ref="EV5:EV6"/>
-    <mergeCell ref="A7:EL7"/>
-    <mergeCell ref="EM5:EM6"/>
-    <mergeCell ref="EN5:EN6"/>
-    <mergeCell ref="EO5:EO6"/>
-    <mergeCell ref="EP5:EP6"/>
-    <mergeCell ref="EQ5:EQ6"/>
-    <mergeCell ref="ER5:ER6"/>
-    <mergeCell ref="DY5:EB5"/>
-    <mergeCell ref="EC5:EC6"/>
-    <mergeCell ref="ED5:ED6"/>
-    <mergeCell ref="EE5:EF5"/>
-    <mergeCell ref="DT5:DT6"/>
-    <mergeCell ref="ET5:ET6"/>
-    <mergeCell ref="BJ4:BK4"/>
-    <mergeCell ref="BL4:BN4"/>
-    <mergeCell ref="BQ4:BS4"/>
-    <mergeCell ref="AZ4:BA4"/>
-    <mergeCell ref="BC4:BE4"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="BG4:BI4"/>
-    <mergeCell ref="AT4:AU4"/>
-    <mergeCell ref="AV4:AW4"/>
-    <mergeCell ref="AX4:AY4"/>
-    <mergeCell ref="AO5:AO6"/>
-    <mergeCell ref="AP5:AP6"/>
-    <mergeCell ref="AQ5:AQ6"/>
-    <mergeCell ref="AR5:AR6"/>
-    <mergeCell ref="AS5:AS6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="AO1:AS1"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:U4"/>
-    <mergeCell ref="W4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AD4"/>
-    <mergeCell ref="AG4:AI4"/>
   </mergeCells>
   <conditionalFormatting sqref="A5 A8:B8">
     <cfRule type="duplicateValues" dxfId="20" priority="20879"/>
@@ -28631,11 +28631,11 @@
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
       <c r="H8" s="20"/>
-      <c r="I8" s="332">
+      <c r="I8" s="326">
         <v>2026</v>
       </c>
-      <c r="J8" s="333"/>
-      <c r="K8" s="333"/>
+      <c r="J8" s="327"/>
+      <c r="K8" s="327"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="21" t="s">
@@ -28660,13 +28660,13 @@
     <row r="9" spans="1:29" ht="15.75" customHeight="1" thickBot="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="334" t="s">
+      <c r="C9" s="328" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="335"/>
-      <c r="E9" s="335"/>
-      <c r="F9" s="335"/>
-      <c r="G9" s="335"/>
+      <c r="D9" s="329"/>
+      <c r="E9" s="329"/>
+      <c r="F9" s="329"/>
+      <c r="G9" s="329"/>
       <c r="H9" s="20"/>
       <c r="I9" s="24"/>
       <c r="J9" s="24"/>
@@ -28762,19 +28762,19 @@
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
-      <c r="J12" s="336" t="s">
+      <c r="J12" s="330" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="335"/>
-      <c r="L12" s="335"/>
-      <c r="M12" s="335"/>
-      <c r="N12" s="335"/>
-      <c r="O12" s="335"/>
-      <c r="P12" s="337">
+      <c r="K12" s="329"/>
+      <c r="L12" s="329"/>
+      <c r="M12" s="329"/>
+      <c r="N12" s="329"/>
+      <c r="O12" s="329"/>
+      <c r="P12" s="331">
         <f>I8</f>
         <v>2026</v>
       </c>
-      <c r="Q12" s="335"/>
+      <c r="Q12" s="329"/>
       <c r="R12" s="33"/>
       <c r="S12" s="34"/>
       <c r="T12" s="34"/>
@@ -29038,38 +29038,38 @@
     </row>
     <row r="21" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A21" s="39"/>
-      <c r="B21" s="331" t="s">
+      <c r="B21" s="332" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="327"/>
-      <c r="D21" s="327"/>
-      <c r="E21" s="327"/>
-      <c r="F21" s="327"/>
-      <c r="G21" s="327"/>
-      <c r="H21" s="327"/>
-      <c r="I21" s="327"/>
+      <c r="C21" s="333"/>
+      <c r="D21" s="333"/>
+      <c r="E21" s="333"/>
+      <c r="F21" s="333"/>
+      <c r="G21" s="333"/>
+      <c r="H21" s="333"/>
+      <c r="I21" s="333"/>
       <c r="J21" s="40"/>
-      <c r="K21" s="328" t="s">
+      <c r="K21" s="334" t="s">
         <v>37</v>
       </c>
-      <c r="L21" s="327"/>
-      <c r="M21" s="327"/>
-      <c r="N21" s="327"/>
-      <c r="O21" s="327"/>
-      <c r="P21" s="327"/>
-      <c r="Q21" s="327"/>
-      <c r="R21" s="327"/>
+      <c r="L21" s="333"/>
+      <c r="M21" s="333"/>
+      <c r="N21" s="333"/>
+      <c r="O21" s="333"/>
+      <c r="P21" s="333"/>
+      <c r="Q21" s="333"/>
+      <c r="R21" s="333"/>
       <c r="S21" s="40"/>
-      <c r="T21" s="326" t="s">
+      <c r="T21" s="335" t="s">
         <v>38</v>
       </c>
-      <c r="U21" s="327"/>
-      <c r="V21" s="327"/>
-      <c r="W21" s="327"/>
-      <c r="X21" s="327"/>
-      <c r="Y21" s="327"/>
-      <c r="Z21" s="327"/>
-      <c r="AA21" s="327"/>
+      <c r="U21" s="333"/>
+      <c r="V21" s="333"/>
+      <c r="W21" s="333"/>
+      <c r="X21" s="333"/>
+      <c r="Y21" s="333"/>
+      <c r="Z21" s="333"/>
+      <c r="AA21" s="333"/>
       <c r="AB21" s="41"/>
       <c r="AC21" s="42"/>
     </row>
@@ -29969,38 +29969,38 @@
     </row>
     <row r="35" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="329" t="s">
+      <c r="B35" s="336" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="327"/>
-      <c r="D35" s="327"/>
-      <c r="E35" s="327"/>
-      <c r="F35" s="327"/>
-      <c r="G35" s="327"/>
-      <c r="H35" s="327"/>
-      <c r="I35" s="327"/>
+      <c r="C35" s="333"/>
+      <c r="D35" s="333"/>
+      <c r="E35" s="333"/>
+      <c r="F35" s="333"/>
+      <c r="G35" s="333"/>
+      <c r="H35" s="333"/>
+      <c r="I35" s="333"/>
       <c r="J35" s="40"/>
-      <c r="K35" s="330" t="s">
+      <c r="K35" s="337" t="s">
         <v>48</v>
       </c>
-      <c r="L35" s="327"/>
-      <c r="M35" s="327"/>
-      <c r="N35" s="327"/>
-      <c r="O35" s="327"/>
-      <c r="P35" s="327"/>
-      <c r="Q35" s="327"/>
-      <c r="R35" s="327"/>
+      <c r="L35" s="333"/>
+      <c r="M35" s="333"/>
+      <c r="N35" s="333"/>
+      <c r="O35" s="333"/>
+      <c r="P35" s="333"/>
+      <c r="Q35" s="333"/>
+      <c r="R35" s="333"/>
       <c r="S35" s="40"/>
-      <c r="T35" s="328" t="s">
+      <c r="T35" s="334" t="s">
         <v>49</v>
       </c>
-      <c r="U35" s="327"/>
-      <c r="V35" s="327"/>
-      <c r="W35" s="327"/>
-      <c r="X35" s="327"/>
-      <c r="Y35" s="327"/>
-      <c r="Z35" s="327"/>
-      <c r="AA35" s="327"/>
+      <c r="U35" s="333"/>
+      <c r="V35" s="333"/>
+      <c r="W35" s="333"/>
+      <c r="X35" s="333"/>
+      <c r="Y35" s="333"/>
+      <c r="Z35" s="333"/>
+      <c r="AA35" s="333"/>
       <c r="AB35" s="70"/>
       <c r="AC35" s="40"/>
     </row>
@@ -30889,38 +30889,38 @@
     </row>
     <row r="49" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A49" s="69"/>
-      <c r="B49" s="328" t="s">
+      <c r="B49" s="334" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="327"/>
-      <c r="D49" s="327"/>
-      <c r="E49" s="327"/>
-      <c r="F49" s="327"/>
-      <c r="G49" s="327"/>
-      <c r="H49" s="327"/>
-      <c r="I49" s="327"/>
+      <c r="C49" s="333"/>
+      <c r="D49" s="333"/>
+      <c r="E49" s="333"/>
+      <c r="F49" s="333"/>
+      <c r="G49" s="333"/>
+      <c r="H49" s="333"/>
+      <c r="I49" s="333"/>
       <c r="J49" s="40"/>
-      <c r="K49" s="329" t="s">
+      <c r="K49" s="336" t="s">
         <v>51</v>
       </c>
-      <c r="L49" s="327"/>
-      <c r="M49" s="327"/>
-      <c r="N49" s="327"/>
-      <c r="O49" s="327"/>
-      <c r="P49" s="327"/>
-      <c r="Q49" s="327"/>
-      <c r="R49" s="327"/>
+      <c r="L49" s="333"/>
+      <c r="M49" s="333"/>
+      <c r="N49" s="333"/>
+      <c r="O49" s="333"/>
+      <c r="P49" s="333"/>
+      <c r="Q49" s="333"/>
+      <c r="R49" s="333"/>
       <c r="S49" s="40"/>
-      <c r="T49" s="331" t="s">
+      <c r="T49" s="332" t="s">
         <v>52</v>
       </c>
-      <c r="U49" s="327"/>
-      <c r="V49" s="327"/>
-      <c r="W49" s="327"/>
-      <c r="X49" s="327"/>
-      <c r="Y49" s="327"/>
-      <c r="Z49" s="327"/>
-      <c r="AA49" s="327"/>
+      <c r="U49" s="333"/>
+      <c r="V49" s="333"/>
+      <c r="W49" s="333"/>
+      <c r="X49" s="333"/>
+      <c r="Y49" s="333"/>
+      <c r="Z49" s="333"/>
+      <c r="AA49" s="333"/>
       <c r="AB49" s="70"/>
       <c r="AC49" s="40"/>
     </row>
@@ -31809,38 +31809,38 @@
     </row>
     <row r="63" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A63" s="69"/>
-      <c r="B63" s="326" t="s">
+      <c r="B63" s="335" t="s">
         <v>53</v>
       </c>
-      <c r="C63" s="327"/>
-      <c r="D63" s="327"/>
-      <c r="E63" s="327"/>
-      <c r="F63" s="327"/>
-      <c r="G63" s="327"/>
-      <c r="H63" s="327"/>
-      <c r="I63" s="327"/>
+      <c r="C63" s="333"/>
+      <c r="D63" s="333"/>
+      <c r="E63" s="333"/>
+      <c r="F63" s="333"/>
+      <c r="G63" s="333"/>
+      <c r="H63" s="333"/>
+      <c r="I63" s="333"/>
       <c r="J63" s="40"/>
-      <c r="K63" s="328" t="s">
+      <c r="K63" s="334" t="s">
         <v>54</v>
       </c>
-      <c r="L63" s="327"/>
-      <c r="M63" s="327"/>
-      <c r="N63" s="327"/>
-      <c r="O63" s="327"/>
-      <c r="P63" s="327"/>
-      <c r="Q63" s="327"/>
-      <c r="R63" s="327"/>
+      <c r="L63" s="333"/>
+      <c r="M63" s="333"/>
+      <c r="N63" s="333"/>
+      <c r="O63" s="333"/>
+      <c r="P63" s="333"/>
+      <c r="Q63" s="333"/>
+      <c r="R63" s="333"/>
       <c r="S63" s="40"/>
-      <c r="T63" s="329" t="s">
+      <c r="T63" s="336" t="s">
         <v>55</v>
       </c>
-      <c r="U63" s="327"/>
-      <c r="V63" s="327"/>
-      <c r="W63" s="327"/>
-      <c r="X63" s="327"/>
-      <c r="Y63" s="327"/>
-      <c r="Z63" s="327"/>
-      <c r="AA63" s="327"/>
+      <c r="U63" s="333"/>
+      <c r="V63" s="333"/>
+      <c r="W63" s="333"/>
+      <c r="X63" s="333"/>
+      <c r="Y63" s="333"/>
+      <c r="Z63" s="333"/>
+      <c r="AA63" s="333"/>
       <c r="AB63" s="70"/>
       <c r="AC63" s="40"/>
     </row>
@@ -61375,12 +61375,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="J12:O12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="K21:R21"/>
     <mergeCell ref="B63:I63"/>
     <mergeCell ref="K63:R63"/>
     <mergeCell ref="T63:AA63"/>
@@ -61391,6 +61385,12 @@
     <mergeCell ref="B49:I49"/>
     <mergeCell ref="K49:R49"/>
     <mergeCell ref="T49:AA49"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="J12:O12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="K21:R21"/>
   </mergeCells>
   <conditionalFormatting sqref="C51:I55">
     <cfRule type="expression" dxfId="2" priority="3">

</xml_diff>

<commit_message>
đã code xong chức năng cân đối với những dữ liệu bất thường
</commit_message>
<xml_diff>
--- a/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
+++ b/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonzai/dev/odoo 19/odoo/my_custom_addons/dl_salary_kpi/static/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA8ACBB7-B4DC-0145-8532-EB1074419478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD56066D-31D9-0647-A5A0-9C0B4AE71F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="17760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kangatang" sheetId="43" state="veryHidden" r:id="rId1"/>
@@ -2476,70 +2476,37 @@
     <xf numFmtId="14" fontId="59" fillId="0" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="14" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="55" fillId="14" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2584,10 +2551,22 @@
     <xf numFmtId="0" fontId="66" fillId="25" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2596,35 +2575,72 @@
     <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="14" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="55" fillId="14" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="7" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2639,22 +2655,6 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="32">
@@ -3484,11 +3484,11 @@
       <c r="AL1" s="213"/>
       <c r="AM1" s="213"/>
       <c r="AN1" s="213"/>
-      <c r="AO1" s="325"/>
-      <c r="AP1" s="325"/>
-      <c r="AQ1" s="325"/>
-      <c r="AR1" s="325"/>
-      <c r="AS1" s="325"/>
+      <c r="AO1" s="276"/>
+      <c r="AP1" s="276"/>
+      <c r="AQ1" s="276"/>
+      <c r="AR1" s="276"/>
+      <c r="AS1" s="276"/>
       <c r="AT1" s="120"/>
       <c r="AU1" s="120"/>
       <c r="AV1" s="120"/>
@@ -3902,40 +3902,40 @@
       <c r="G4" s="238"/>
       <c r="H4" s="108"/>
       <c r="I4" s="275"/>
-      <c r="J4" s="316" t="s">
+      <c r="J4" s="277" t="s">
         <v>68</v>
       </c>
-      <c r="K4" s="316"/>
-      <c r="L4" s="319">
+      <c r="K4" s="277"/>
+      <c r="L4" s="278">
         <v>3</v>
       </c>
-      <c r="M4" s="319"/>
-      <c r="N4" s="316" t="s">
+      <c r="M4" s="278"/>
+      <c r="N4" s="277" t="s">
         <v>69</v>
       </c>
-      <c r="O4" s="316"/>
-      <c r="P4" s="316">
+      <c r="O4" s="277"/>
+      <c r="P4" s="277">
         <v>2026</v>
       </c>
-      <c r="Q4" s="316"/>
+      <c r="Q4" s="277"/>
       <c r="R4" s="109"/>
-      <c r="S4" s="316"/>
-      <c r="T4" s="316"/>
-      <c r="U4" s="316"/>
+      <c r="S4" s="277"/>
+      <c r="T4" s="277"/>
+      <c r="U4" s="277"/>
       <c r="V4" s="109"/>
-      <c r="W4" s="316"/>
-      <c r="X4" s="316"/>
-      <c r="Y4" s="316"/>
-      <c r="Z4" s="316"/>
-      <c r="AA4" s="316"/>
-      <c r="AB4" s="316"/>
-      <c r="AC4" s="316"/>
-      <c r="AD4" s="316"/>
+      <c r="W4" s="277"/>
+      <c r="X4" s="277"/>
+      <c r="Y4" s="277"/>
+      <c r="Z4" s="277"/>
+      <c r="AA4" s="277"/>
+      <c r="AB4" s="277"/>
+      <c r="AC4" s="277"/>
+      <c r="AD4" s="277"/>
       <c r="AE4" s="109"/>
       <c r="AF4" s="110"/>
-      <c r="AG4" s="316"/>
-      <c r="AH4" s="316"/>
-      <c r="AI4" s="316"/>
+      <c r="AG4" s="277"/>
+      <c r="AH4" s="277"/>
+      <c r="AI4" s="277"/>
       <c r="AJ4" s="109"/>
       <c r="AK4" s="109"/>
       <c r="AL4" s="109"/>
@@ -3946,41 +3946,41 @@
       <c r="AQ4" s="113"/>
       <c r="AR4" s="224"/>
       <c r="AS4" s="233"/>
-      <c r="AT4" s="316" t="s">
+      <c r="AT4" s="277" t="s">
         <v>68</v>
       </c>
-      <c r="AU4" s="316"/>
-      <c r="AV4" s="319">
+      <c r="AU4" s="277"/>
+      <c r="AV4" s="278">
         <f>L4</f>
         <v>3</v>
       </c>
-      <c r="AW4" s="319"/>
-      <c r="AX4" s="316" t="s">
+      <c r="AW4" s="278"/>
+      <c r="AX4" s="277" t="s">
         <v>69</v>
       </c>
-      <c r="AY4" s="316"/>
-      <c r="AZ4" s="316">
+      <c r="AY4" s="277"/>
+      <c r="AZ4" s="277">
         <v>2025</v>
       </c>
-      <c r="BA4" s="316"/>
+      <c r="BA4" s="277"/>
       <c r="BB4" s="109"/>
-      <c r="BC4" s="316"/>
-      <c r="BD4" s="316"/>
-      <c r="BE4" s="316"/>
+      <c r="BC4" s="277"/>
+      <c r="BD4" s="277"/>
+      <c r="BE4" s="277"/>
       <c r="BF4" s="109"/>
-      <c r="BG4" s="316"/>
-      <c r="BH4" s="316"/>
-      <c r="BI4" s="316"/>
-      <c r="BJ4" s="316"/>
-      <c r="BK4" s="316"/>
-      <c r="BL4" s="316"/>
-      <c r="BM4" s="316"/>
-      <c r="BN4" s="316"/>
+      <c r="BG4" s="277"/>
+      <c r="BH4" s="277"/>
+      <c r="BI4" s="277"/>
+      <c r="BJ4" s="277"/>
+      <c r="BK4" s="277"/>
+      <c r="BL4" s="277"/>
+      <c r="BM4" s="277"/>
+      <c r="BN4" s="277"/>
       <c r="BO4" s="109"/>
       <c r="BP4" s="110"/>
-      <c r="BQ4" s="316"/>
-      <c r="BR4" s="316"/>
-      <c r="BS4" s="316"/>
+      <c r="BQ4" s="277"/>
+      <c r="BR4" s="277"/>
+      <c r="BS4" s="277"/>
       <c r="BT4" s="114"/>
       <c r="BU4" s="114" t="str">
         <f>IF(WEEKDAY(BU5,1)=1,"CN","")</f>
@@ -4046,34 +4046,16 @@
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="DO4" s="149" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="DO4" s="149"/>
       <c r="DP4" s="216"/>
       <c r="DQ4" s="216"/>
       <c r="DR4" s="216"/>
-      <c r="DS4" s="218" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="DS4" s="218"/>
       <c r="DT4" s="115"/>
-      <c r="DU4" s="115" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="DV4" s="115" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="DW4" s="115" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="DX4" s="115" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="DU4" s="115"/>
+      <c r="DV4" s="115"/>
+      <c r="DW4" s="115"/>
+      <c r="DX4" s="115"/>
       <c r="DY4" s="116"/>
       <c r="DZ4" s="117"/>
       <c r="EA4" s="103"/>
@@ -4097,31 +4079,31 @@
       <c r="EV4" s="247"/>
     </row>
     <row r="5" spans="1:154" s="184" customFormat="1" ht="92.25" customHeight="1">
-      <c r="A5" s="317" t="s">
+      <c r="A5" s="279" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="277" t="s">
+      <c r="B5" s="280" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="317" t="s">
+      <c r="C5" s="279" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="322" t="s">
+      <c r="D5" s="281" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="323" t="s">
+      <c r="E5" s="282" t="s">
         <v>122</v>
       </c>
-      <c r="F5" s="317" t="s">
+      <c r="F5" s="279" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="317" t="s">
+      <c r="G5" s="279" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="317" t="s">
+      <c r="H5" s="279" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="318" t="s">
+      <c r="I5" s="284" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="175">
@@ -4248,19 +4230,19 @@
         <f t="shared" si="0"/>
         <v>46112</v>
       </c>
-      <c r="AO5" s="320" t="s">
+      <c r="AO5" s="285" t="s">
         <v>82</v>
       </c>
-      <c r="AP5" s="320" t="s">
+      <c r="AP5" s="285" t="s">
         <v>83</v>
       </c>
-      <c r="AQ5" s="320" t="s">
+      <c r="AQ5" s="285" t="s">
         <v>84</v>
       </c>
-      <c r="AR5" s="321" t="s">
+      <c r="AR5" s="286" t="s">
         <v>5</v>
       </c>
-      <c r="AS5" s="321" t="s">
+      <c r="AS5" s="286" t="s">
         <v>6</v>
       </c>
       <c r="AT5" s="179">
@@ -4387,46 +4369,46 @@
         <f t="shared" si="1"/>
         <v>46112</v>
       </c>
-      <c r="BY5" s="294" t="s">
+      <c r="BY5" s="310" t="s">
         <v>86</v>
       </c>
-      <c r="BZ5" s="294" t="s">
+      <c r="BZ5" s="310" t="s">
         <v>87</v>
       </c>
-      <c r="CA5" s="294" t="s">
+      <c r="CA5" s="310" t="s">
         <v>88</v>
       </c>
-      <c r="CB5" s="294" t="s">
+      <c r="CB5" s="310" t="s">
         <v>89</v>
       </c>
-      <c r="CC5" s="294" t="s">
+      <c r="CC5" s="310" t="s">
         <v>90</v>
       </c>
-      <c r="CD5" s="294" t="s">
+      <c r="CD5" s="310" t="s">
         <v>91</v>
       </c>
-      <c r="CE5" s="294" t="s">
+      <c r="CE5" s="310" t="s">
         <v>92</v>
       </c>
-      <c r="CF5" s="296" t="s">
+      <c r="CF5" s="309" t="s">
         <v>19</v>
       </c>
-      <c r="CG5" s="296"/>
-      <c r="CH5" s="296"/>
-      <c r="CI5" s="296"/>
-      <c r="CJ5" s="296"/>
-      <c r="CK5" s="296"/>
-      <c r="CL5" s="296"/>
-      <c r="CM5" s="296"/>
-      <c r="CN5" s="296"/>
-      <c r="CO5" s="296"/>
-      <c r="CP5" s="296"/>
-      <c r="CQ5" s="280" t="s">
+      <c r="CG5" s="309"/>
+      <c r="CH5" s="309"/>
+      <c r="CI5" s="309"/>
+      <c r="CJ5" s="309"/>
+      <c r="CK5" s="309"/>
+      <c r="CL5" s="309"/>
+      <c r="CM5" s="309"/>
+      <c r="CN5" s="309"/>
+      <c r="CO5" s="309"/>
+      <c r="CP5" s="309"/>
+      <c r="CQ5" s="315" t="s">
         <v>59</v>
       </c>
-      <c r="CR5" s="281"/>
-      <c r="CS5" s="282"/>
-      <c r="CT5" s="287" t="s">
+      <c r="CR5" s="316"/>
+      <c r="CS5" s="317"/>
+      <c r="CT5" s="322" t="s">
         <v>60</v>
       </c>
       <c r="CU5" s="261" t="s">
@@ -4449,117 +4431,117 @@
       <c r="DF5" s="259" t="s">
         <v>130</v>
       </c>
-      <c r="DG5" s="283" t="s">
+      <c r="DG5" s="318" t="s">
         <v>119</v>
       </c>
-      <c r="DH5" s="288" t="s">
+      <c r="DH5" s="323" t="s">
         <v>113</v>
       </c>
-      <c r="DI5" s="285" t="s">
+      <c r="DI5" s="320" t="s">
         <v>81</v>
       </c>
-      <c r="DJ5" s="286"/>
-      <c r="DK5" s="289" t="s">
+      <c r="DJ5" s="321"/>
+      <c r="DK5" s="304" t="s">
         <v>61</v>
       </c>
-      <c r="DL5" s="297" t="s">
+      <c r="DL5" s="312" t="s">
         <v>8</v>
       </c>
-      <c r="DM5" s="290" t="s">
+      <c r="DM5" s="305" t="s">
         <v>71</v>
       </c>
-      <c r="DN5" s="290"/>
-      <c r="DO5" s="290"/>
-      <c r="DP5" s="290"/>
-      <c r="DQ5" s="290"/>
-      <c r="DR5" s="290"/>
-      <c r="DS5" s="291" t="s">
+      <c r="DN5" s="305"/>
+      <c r="DO5" s="305"/>
+      <c r="DP5" s="305"/>
+      <c r="DQ5" s="305"/>
+      <c r="DR5" s="305"/>
+      <c r="DS5" s="324" t="s">
         <v>12</v>
       </c>
-      <c r="DT5" s="290" t="s">
+      <c r="DT5" s="305" t="s">
         <v>128</v>
       </c>
-      <c r="DU5" s="277" t="s">
+      <c r="DU5" s="280" t="s">
         <v>13</v>
       </c>
-      <c r="DV5" s="278" t="s">
+      <c r="DV5" s="313" t="s">
         <v>64</v>
       </c>
-      <c r="DW5" s="279"/>
-      <c r="DX5" s="278"/>
-      <c r="DY5" s="312" t="s">
+      <c r="DW5" s="314"/>
+      <c r="DX5" s="313"/>
+      <c r="DY5" s="302" t="s">
         <v>63</v>
       </c>
-      <c r="DZ5" s="312"/>
-      <c r="EA5" s="312"/>
-      <c r="EB5" s="312"/>
-      <c r="EC5" s="313" t="s">
+      <c r="DZ5" s="302"/>
+      <c r="EA5" s="302"/>
+      <c r="EB5" s="302"/>
+      <c r="EC5" s="303" t="s">
         <v>131</v>
       </c>
-      <c r="ED5" s="290" t="s">
+      <c r="ED5" s="305" t="s">
         <v>7</v>
       </c>
-      <c r="EE5" s="292" t="s">
+      <c r="EE5" s="306" t="s">
         <v>65</v>
       </c>
-      <c r="EF5" s="292"/>
-      <c r="EG5" s="292" t="s">
+      <c r="EF5" s="306"/>
+      <c r="EG5" s="306" t="s">
         <v>66</v>
       </c>
-      <c r="EH5" s="292" t="s">
+      <c r="EH5" s="306" t="s">
         <v>67</v>
       </c>
-      <c r="EI5" s="292" t="s">
+      <c r="EI5" s="306" t="s">
         <v>72</v>
       </c>
-      <c r="EJ5" s="293" t="s">
+      <c r="EJ5" s="325" t="s">
         <v>78</v>
       </c>
-      <c r="EK5" s="293" t="s">
+      <c r="EK5" s="325" t="s">
         <v>80</v>
       </c>
-      <c r="EL5" s="293" t="s">
+      <c r="EL5" s="325" t="s">
         <v>79</v>
       </c>
-      <c r="EM5" s="302" t="s">
+      <c r="EM5" s="291" t="s">
         <v>127</v>
       </c>
-      <c r="EN5" s="304"/>
-      <c r="EO5" s="306" t="s">
+      <c r="EN5" s="293"/>
+      <c r="EO5" s="295" t="s">
         <v>132</v>
       </c>
-      <c r="EP5" s="308" t="s">
+      <c r="EP5" s="297" t="s">
         <v>118</v>
       </c>
-      <c r="EQ5" s="310" t="s">
+      <c r="EQ5" s="299" t="s">
         <v>133</v>
       </c>
-      <c r="ER5" s="276" t="s">
+      <c r="ER5" s="301" t="s">
         <v>125</v>
       </c>
-      <c r="ES5" s="276" t="s">
+      <c r="ES5" s="301" t="s">
         <v>124</v>
       </c>
-      <c r="ET5" s="314" t="s">
+      <c r="ET5" s="307" t="s">
         <v>120</v>
       </c>
-      <c r="EU5" s="298" t="s">
+      <c r="EU5" s="287" t="s">
         <v>123</v>
       </c>
-      <c r="EV5" s="300" t="s">
+      <c r="EV5" s="289" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:154" s="206" customFormat="1" ht="148.5" customHeight="1">
-      <c r="A6" s="317"/>
-      <c r="B6" s="277"/>
-      <c r="C6" s="317"/>
-      <c r="D6" s="322"/>
-      <c r="E6" s="324"/>
-      <c r="F6" s="317"/>
-      <c r="G6" s="317"/>
-      <c r="H6" s="317"/>
-      <c r="I6" s="318"/>
+      <c r="A6" s="279"/>
+      <c r="B6" s="280"/>
+      <c r="C6" s="279"/>
+      <c r="D6" s="281"/>
+      <c r="E6" s="283"/>
+      <c r="F6" s="279"/>
+      <c r="G6" s="279"/>
+      <c r="H6" s="279"/>
+      <c r="I6" s="284"/>
       <c r="J6" s="185" t="str">
         <f t="shared" ref="J6:AN6" si="2">IF(WEEKDAY(J5)=1,"CN",WEEKDAY(J5))</f>
         <v>CN</v>
@@ -4684,11 +4666,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AO6" s="320"/>
-      <c r="AP6" s="320"/>
-      <c r="AQ6" s="320"/>
-      <c r="AR6" s="321"/>
-      <c r="AS6" s="321"/>
+      <c r="AO6" s="285"/>
+      <c r="AP6" s="285"/>
+      <c r="AQ6" s="285"/>
+      <c r="AR6" s="286"/>
+      <c r="AS6" s="286"/>
       <c r="AT6" s="187" t="str">
         <f>+J6</f>
         <v>CN</v>
@@ -4813,13 +4795,13 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="BY6" s="295"/>
-      <c r="BZ6" s="295"/>
-      <c r="CA6" s="295"/>
-      <c r="CB6" s="295"/>
-      <c r="CC6" s="295"/>
-      <c r="CD6" s="295"/>
-      <c r="CE6" s="295"/>
+      <c r="BY6" s="311"/>
+      <c r="BZ6" s="311"/>
+      <c r="CA6" s="311"/>
+      <c r="CB6" s="311"/>
+      <c r="CC6" s="311"/>
+      <c r="CD6" s="311"/>
+      <c r="CE6" s="311"/>
       <c r="CF6" s="189" t="s">
         <v>93</v>
       </c>
@@ -4862,7 +4844,7 @@
       <c r="CS6" s="181" t="s">
         <v>58</v>
       </c>
-      <c r="CT6" s="287"/>
+      <c r="CT6" s="322"/>
       <c r="CU6" s="189" t="s">
         <v>104</v>
       </c>
@@ -4899,16 +4881,16 @@
       <c r="DF6" s="260" t="s">
         <v>134</v>
       </c>
-      <c r="DG6" s="284"/>
-      <c r="DH6" s="288"/>
+      <c r="DG6" s="319"/>
+      <c r="DH6" s="323"/>
       <c r="DI6" s="152" t="s">
         <v>14</v>
       </c>
       <c r="DJ6" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="DK6" s="289"/>
-      <c r="DL6" s="297"/>
+      <c r="DK6" s="304"/>
+      <c r="DL6" s="312"/>
       <c r="DM6" s="181" t="s">
         <v>9</v>
       </c>
@@ -4927,9 +4909,9 @@
       <c r="DR6" s="181" t="s">
         <v>116</v>
       </c>
-      <c r="DS6" s="291"/>
-      <c r="DT6" s="290"/>
-      <c r="DU6" s="277"/>
+      <c r="DS6" s="324"/>
+      <c r="DT6" s="305"/>
+      <c r="DU6" s="280"/>
       <c r="DV6" s="204">
         <v>0.17499999999999999</v>
       </c>
@@ -4951,176 +4933,176 @@
       <c r="EB6" s="152" t="s">
         <v>62</v>
       </c>
-      <c r="EC6" s="289"/>
-      <c r="ED6" s="290"/>
+      <c r="EC6" s="304"/>
+      <c r="ED6" s="305"/>
       <c r="EE6" s="183" t="s">
         <v>73</v>
       </c>
       <c r="EF6" s="183" t="s">
         <v>74</v>
       </c>
-      <c r="EG6" s="292"/>
-      <c r="EH6" s="292"/>
-      <c r="EI6" s="292"/>
-      <c r="EJ6" s="293"/>
-      <c r="EK6" s="293"/>
-      <c r="EL6" s="293"/>
-      <c r="EM6" s="303"/>
-      <c r="EN6" s="305"/>
-      <c r="EO6" s="307"/>
-      <c r="EP6" s="309"/>
-      <c r="EQ6" s="311"/>
-      <c r="ER6" s="276"/>
-      <c r="ES6" s="276"/>
-      <c r="ET6" s="315"/>
-      <c r="EU6" s="299"/>
-      <c r="EV6" s="300"/>
+      <c r="EG6" s="306"/>
+      <c r="EH6" s="306"/>
+      <c r="EI6" s="306"/>
+      <c r="EJ6" s="325"/>
+      <c r="EK6" s="325"/>
+      <c r="EL6" s="325"/>
+      <c r="EM6" s="292"/>
+      <c r="EN6" s="294"/>
+      <c r="EO6" s="296"/>
+      <c r="EP6" s="298"/>
+      <c r="EQ6" s="300"/>
+      <c r="ER6" s="301"/>
+      <c r="ES6" s="301"/>
+      <c r="ET6" s="308"/>
+      <c r="EU6" s="288"/>
+      <c r="EV6" s="289"/>
     </row>
     <row r="7" spans="1:154" s="106" customFormat="1" ht="87.75" customHeight="1">
-      <c r="A7" s="301" t="s">
+      <c r="A7" s="290" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="301"/>
-      <c r="C7" s="301"/>
-      <c r="D7" s="301"/>
-      <c r="E7" s="301"/>
-      <c r="F7" s="301"/>
-      <c r="G7" s="301"/>
-      <c r="H7" s="301"/>
-      <c r="I7" s="301"/>
-      <c r="J7" s="301"/>
-      <c r="K7" s="301"/>
-      <c r="L7" s="301"/>
-      <c r="M7" s="301"/>
-      <c r="N7" s="301"/>
-      <c r="O7" s="301"/>
-      <c r="P7" s="301"/>
-      <c r="Q7" s="301"/>
-      <c r="R7" s="301"/>
-      <c r="S7" s="301"/>
-      <c r="T7" s="301"/>
-      <c r="U7" s="301"/>
-      <c r="V7" s="301"/>
-      <c r="W7" s="301"/>
-      <c r="X7" s="301"/>
-      <c r="Y7" s="301"/>
-      <c r="Z7" s="301"/>
-      <c r="AA7" s="301"/>
-      <c r="AB7" s="301"/>
-      <c r="AC7" s="301"/>
-      <c r="AD7" s="301"/>
-      <c r="AE7" s="301"/>
-      <c r="AF7" s="301"/>
-      <c r="AG7" s="301"/>
-      <c r="AH7" s="301"/>
-      <c r="AI7" s="301"/>
-      <c r="AJ7" s="301"/>
-      <c r="AK7" s="301"/>
-      <c r="AL7" s="301"/>
-      <c r="AM7" s="301"/>
-      <c r="AN7" s="301"/>
-      <c r="AO7" s="301"/>
-      <c r="AP7" s="301"/>
-      <c r="AQ7" s="301"/>
-      <c r="AR7" s="301"/>
-      <c r="AS7" s="301"/>
-      <c r="AT7" s="301"/>
-      <c r="AU7" s="301"/>
-      <c r="AV7" s="301"/>
-      <c r="AW7" s="301"/>
-      <c r="AX7" s="301"/>
-      <c r="AY7" s="301"/>
-      <c r="AZ7" s="301"/>
-      <c r="BA7" s="301"/>
-      <c r="BB7" s="301"/>
-      <c r="BC7" s="301"/>
-      <c r="BD7" s="301"/>
-      <c r="BE7" s="301"/>
-      <c r="BF7" s="301"/>
-      <c r="BG7" s="301"/>
-      <c r="BH7" s="301"/>
-      <c r="BI7" s="301"/>
-      <c r="BJ7" s="301"/>
-      <c r="BK7" s="301"/>
-      <c r="BL7" s="301"/>
-      <c r="BM7" s="301"/>
-      <c r="BN7" s="301"/>
-      <c r="BO7" s="301"/>
-      <c r="BP7" s="301"/>
-      <c r="BQ7" s="301"/>
-      <c r="BR7" s="301"/>
-      <c r="BS7" s="301"/>
-      <c r="BT7" s="301"/>
-      <c r="BU7" s="301"/>
-      <c r="BV7" s="301"/>
-      <c r="BW7" s="301"/>
-      <c r="BX7" s="301"/>
-      <c r="BY7" s="301"/>
-      <c r="BZ7" s="301"/>
-      <c r="CA7" s="301"/>
-      <c r="CB7" s="301"/>
-      <c r="CC7" s="301"/>
-      <c r="CD7" s="301"/>
-      <c r="CE7" s="301"/>
-      <c r="CF7" s="301"/>
-      <c r="CG7" s="301"/>
-      <c r="CH7" s="301"/>
-      <c r="CI7" s="301"/>
-      <c r="CJ7" s="301"/>
-      <c r="CK7" s="301"/>
-      <c r="CL7" s="301"/>
-      <c r="CM7" s="301"/>
-      <c r="CN7" s="301"/>
-      <c r="CO7" s="301"/>
-      <c r="CP7" s="301"/>
-      <c r="CQ7" s="301"/>
-      <c r="CR7" s="301"/>
-      <c r="CS7" s="301"/>
-      <c r="CT7" s="301"/>
-      <c r="CU7" s="301"/>
-      <c r="CV7" s="301"/>
-      <c r="CW7" s="301"/>
-      <c r="CX7" s="301"/>
-      <c r="CY7" s="301"/>
-      <c r="CZ7" s="301"/>
-      <c r="DA7" s="301"/>
-      <c r="DB7" s="301"/>
-      <c r="DC7" s="301"/>
-      <c r="DD7" s="301"/>
-      <c r="DE7" s="301"/>
-      <c r="DF7" s="301"/>
-      <c r="DG7" s="301"/>
-      <c r="DH7" s="301"/>
-      <c r="DI7" s="301"/>
-      <c r="DJ7" s="301"/>
-      <c r="DK7" s="301"/>
-      <c r="DL7" s="301"/>
-      <c r="DM7" s="301"/>
-      <c r="DN7" s="301"/>
-      <c r="DO7" s="301"/>
-      <c r="DP7" s="301"/>
-      <c r="DQ7" s="301"/>
-      <c r="DR7" s="301"/>
-      <c r="DS7" s="301"/>
-      <c r="DT7" s="301"/>
-      <c r="DU7" s="301"/>
-      <c r="DV7" s="301"/>
-      <c r="DW7" s="301"/>
-      <c r="DX7" s="301"/>
-      <c r="DY7" s="301"/>
-      <c r="DZ7" s="301"/>
-      <c r="EA7" s="301"/>
-      <c r="EB7" s="301"/>
-      <c r="EC7" s="301"/>
-      <c r="ED7" s="301"/>
-      <c r="EE7" s="301"/>
-      <c r="EF7" s="301"/>
-      <c r="EG7" s="301"/>
-      <c r="EH7" s="301"/>
-      <c r="EI7" s="301"/>
-      <c r="EJ7" s="301"/>
-      <c r="EK7" s="301"/>
-      <c r="EL7" s="301"/>
+      <c r="B7" s="290"/>
+      <c r="C7" s="290"/>
+      <c r="D7" s="290"/>
+      <c r="E7" s="290"/>
+      <c r="F7" s="290"/>
+      <c r="G7" s="290"/>
+      <c r="H7" s="290"/>
+      <c r="I7" s="290"/>
+      <c r="J7" s="290"/>
+      <c r="K7" s="290"/>
+      <c r="L7" s="290"/>
+      <c r="M7" s="290"/>
+      <c r="N7" s="290"/>
+      <c r="O7" s="290"/>
+      <c r="P7" s="290"/>
+      <c r="Q7" s="290"/>
+      <c r="R7" s="290"/>
+      <c r="S7" s="290"/>
+      <c r="T7" s="290"/>
+      <c r="U7" s="290"/>
+      <c r="V7" s="290"/>
+      <c r="W7" s="290"/>
+      <c r="X7" s="290"/>
+      <c r="Y7" s="290"/>
+      <c r="Z7" s="290"/>
+      <c r="AA7" s="290"/>
+      <c r="AB7" s="290"/>
+      <c r="AC7" s="290"/>
+      <c r="AD7" s="290"/>
+      <c r="AE7" s="290"/>
+      <c r="AF7" s="290"/>
+      <c r="AG7" s="290"/>
+      <c r="AH7" s="290"/>
+      <c r="AI7" s="290"/>
+      <c r="AJ7" s="290"/>
+      <c r="AK7" s="290"/>
+      <c r="AL7" s="290"/>
+      <c r="AM7" s="290"/>
+      <c r="AN7" s="290"/>
+      <c r="AO7" s="290"/>
+      <c r="AP7" s="290"/>
+      <c r="AQ7" s="290"/>
+      <c r="AR7" s="290"/>
+      <c r="AS7" s="290"/>
+      <c r="AT7" s="290"/>
+      <c r="AU7" s="290"/>
+      <c r="AV7" s="290"/>
+      <c r="AW7" s="290"/>
+      <c r="AX7" s="290"/>
+      <c r="AY7" s="290"/>
+      <c r="AZ7" s="290"/>
+      <c r="BA7" s="290"/>
+      <c r="BB7" s="290"/>
+      <c r="BC7" s="290"/>
+      <c r="BD7" s="290"/>
+      <c r="BE7" s="290"/>
+      <c r="BF7" s="290"/>
+      <c r="BG7" s="290"/>
+      <c r="BH7" s="290"/>
+      <c r="BI7" s="290"/>
+      <c r="BJ7" s="290"/>
+      <c r="BK7" s="290"/>
+      <c r="BL7" s="290"/>
+      <c r="BM7" s="290"/>
+      <c r="BN7" s="290"/>
+      <c r="BO7" s="290"/>
+      <c r="BP7" s="290"/>
+      <c r="BQ7" s="290"/>
+      <c r="BR7" s="290"/>
+      <c r="BS7" s="290"/>
+      <c r="BT7" s="290"/>
+      <c r="BU7" s="290"/>
+      <c r="BV7" s="290"/>
+      <c r="BW7" s="290"/>
+      <c r="BX7" s="290"/>
+      <c r="BY7" s="290"/>
+      <c r="BZ7" s="290"/>
+      <c r="CA7" s="290"/>
+      <c r="CB7" s="290"/>
+      <c r="CC7" s="290"/>
+      <c r="CD7" s="290"/>
+      <c r="CE7" s="290"/>
+      <c r="CF7" s="290"/>
+      <c r="CG7" s="290"/>
+      <c r="CH7" s="290"/>
+      <c r="CI7" s="290"/>
+      <c r="CJ7" s="290"/>
+      <c r="CK7" s="290"/>
+      <c r="CL7" s="290"/>
+      <c r="CM7" s="290"/>
+      <c r="CN7" s="290"/>
+      <c r="CO7" s="290"/>
+      <c r="CP7" s="290"/>
+      <c r="CQ7" s="290"/>
+      <c r="CR7" s="290"/>
+      <c r="CS7" s="290"/>
+      <c r="CT7" s="290"/>
+      <c r="CU7" s="290"/>
+      <c r="CV7" s="290"/>
+      <c r="CW7" s="290"/>
+      <c r="CX7" s="290"/>
+      <c r="CY7" s="290"/>
+      <c r="CZ7" s="290"/>
+      <c r="DA7" s="290"/>
+      <c r="DB7" s="290"/>
+      <c r="DC7" s="290"/>
+      <c r="DD7" s="290"/>
+      <c r="DE7" s="290"/>
+      <c r="DF7" s="290"/>
+      <c r="DG7" s="290"/>
+      <c r="DH7" s="290"/>
+      <c r="DI7" s="290"/>
+      <c r="DJ7" s="290"/>
+      <c r="DK7" s="290"/>
+      <c r="DL7" s="290"/>
+      <c r="DM7" s="290"/>
+      <c r="DN7" s="290"/>
+      <c r="DO7" s="290"/>
+      <c r="DP7" s="290"/>
+      <c r="DQ7" s="290"/>
+      <c r="DR7" s="290"/>
+      <c r="DS7" s="290"/>
+      <c r="DT7" s="290"/>
+      <c r="DU7" s="290"/>
+      <c r="DV7" s="290"/>
+      <c r="DW7" s="290"/>
+      <c r="DX7" s="290"/>
+      <c r="DY7" s="290"/>
+      <c r="DZ7" s="290"/>
+      <c r="EA7" s="290"/>
+      <c r="EB7" s="290"/>
+      <c r="EC7" s="290"/>
+      <c r="ED7" s="290"/>
+      <c r="EE7" s="290"/>
+      <c r="EF7" s="290"/>
+      <c r="EG7" s="290"/>
+      <c r="EH7" s="290"/>
+      <c r="EI7" s="290"/>
+      <c r="EJ7" s="290"/>
+      <c r="EK7" s="290"/>
+      <c r="EL7" s="290"/>
       <c r="EM7" s="248"/>
       <c r="EN7" s="248"/>
       <c r="EO7" s="248"/>
@@ -5496,10 +5478,7 @@
         <f t="shared" ref="DS8" ca="1" si="80">ROUNDDOWN(DK8-DQ8,-3)</f>
         <v>#REF!</v>
       </c>
-      <c r="DT8" s="157" t="e">
-        <f ca="1">+DS8-#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="DT8" s="157"/>
       <c r="DU8" s="159">
         <f>+DL8*2%</f>
         <v>0</v>
@@ -27901,38 +27880,32 @@
   </sheetData>
   <autoFilter ref="A6:EX8" xr:uid="{00000000-0001-0000-0900-000000000000}"/>
   <mergeCells count="74">
-    <mergeCell ref="AO1:AS1"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:U4"/>
-    <mergeCell ref="W4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AD4"/>
-    <mergeCell ref="AG4:AI4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="BG4:BI4"/>
-    <mergeCell ref="AT4:AU4"/>
-    <mergeCell ref="AV4:AW4"/>
-    <mergeCell ref="AX4:AY4"/>
-    <mergeCell ref="AO5:AO6"/>
-    <mergeCell ref="AP5:AP6"/>
-    <mergeCell ref="AQ5:AQ6"/>
-    <mergeCell ref="AR5:AR6"/>
-    <mergeCell ref="AS5:AS6"/>
-    <mergeCell ref="BJ4:BK4"/>
-    <mergeCell ref="BL4:BN4"/>
-    <mergeCell ref="BQ4:BS4"/>
-    <mergeCell ref="AZ4:BA4"/>
-    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="ES5:ES6"/>
+    <mergeCell ref="DU5:DU6"/>
+    <mergeCell ref="DV5:DX5"/>
+    <mergeCell ref="CQ5:CS5"/>
+    <mergeCell ref="DG5:DG6"/>
+    <mergeCell ref="DI5:DJ5"/>
+    <mergeCell ref="CT5:CT6"/>
+    <mergeCell ref="DH5:DH6"/>
+    <mergeCell ref="DK5:DK6"/>
+    <mergeCell ref="DM5:DR5"/>
+    <mergeCell ref="DS5:DS6"/>
+    <mergeCell ref="EI5:EI6"/>
+    <mergeCell ref="EJ5:EJ6"/>
+    <mergeCell ref="EK5:EK6"/>
+    <mergeCell ref="EL5:EL6"/>
+    <mergeCell ref="EH5:EH6"/>
+    <mergeCell ref="BY5:BY6"/>
+    <mergeCell ref="BZ5:BZ6"/>
+    <mergeCell ref="CA5:CA6"/>
+    <mergeCell ref="CB5:CB6"/>
+    <mergeCell ref="CC5:CC6"/>
+    <mergeCell ref="CF5:CP5"/>
+    <mergeCell ref="CD5:CD6"/>
+    <mergeCell ref="CE5:CE6"/>
+    <mergeCell ref="DL5:DL6"/>
+    <mergeCell ref="EG5:EG6"/>
     <mergeCell ref="EU5:EU6"/>
     <mergeCell ref="EV5:EV6"/>
     <mergeCell ref="A7:EL7"/>
@@ -27949,32 +27922,38 @@
     <mergeCell ref="DT5:DT6"/>
     <mergeCell ref="ET5:ET6"/>
     <mergeCell ref="F5:F6"/>
-    <mergeCell ref="CF5:CP5"/>
-    <mergeCell ref="CD5:CD6"/>
-    <mergeCell ref="CE5:CE6"/>
-    <mergeCell ref="DL5:DL6"/>
-    <mergeCell ref="EG5:EG6"/>
-    <mergeCell ref="BY5:BY6"/>
-    <mergeCell ref="BZ5:BZ6"/>
-    <mergeCell ref="CA5:CA6"/>
-    <mergeCell ref="CB5:CB6"/>
-    <mergeCell ref="CC5:CC6"/>
-    <mergeCell ref="ES5:ES6"/>
-    <mergeCell ref="DU5:DU6"/>
-    <mergeCell ref="DV5:DX5"/>
-    <mergeCell ref="CQ5:CS5"/>
-    <mergeCell ref="DG5:DG6"/>
-    <mergeCell ref="DI5:DJ5"/>
-    <mergeCell ref="CT5:CT6"/>
-    <mergeCell ref="DH5:DH6"/>
-    <mergeCell ref="DK5:DK6"/>
-    <mergeCell ref="DM5:DR5"/>
-    <mergeCell ref="DS5:DS6"/>
-    <mergeCell ref="EI5:EI6"/>
-    <mergeCell ref="EJ5:EJ6"/>
-    <mergeCell ref="EK5:EK6"/>
-    <mergeCell ref="EL5:EL6"/>
-    <mergeCell ref="EH5:EH6"/>
+    <mergeCell ref="BJ4:BK4"/>
+    <mergeCell ref="BL4:BN4"/>
+    <mergeCell ref="BQ4:BS4"/>
+    <mergeCell ref="AZ4:BA4"/>
+    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="BG4:BI4"/>
+    <mergeCell ref="AT4:AU4"/>
+    <mergeCell ref="AV4:AW4"/>
+    <mergeCell ref="AX4:AY4"/>
+    <mergeCell ref="AO5:AO6"/>
+    <mergeCell ref="AP5:AP6"/>
+    <mergeCell ref="AQ5:AQ6"/>
+    <mergeCell ref="AR5:AR6"/>
+    <mergeCell ref="AS5:AS6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="AO1:AS1"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:U4"/>
+    <mergeCell ref="W4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="AG4:AI4"/>
   </mergeCells>
   <conditionalFormatting sqref="A5 A8:B8">
     <cfRule type="duplicateValues" dxfId="20" priority="20879"/>
@@ -28631,11 +28610,11 @@
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
       <c r="H8" s="20"/>
-      <c r="I8" s="326">
+      <c r="I8" s="332">
         <v>2026</v>
       </c>
-      <c r="J8" s="327"/>
-      <c r="K8" s="327"/>
+      <c r="J8" s="333"/>
+      <c r="K8" s="333"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="21" t="s">
@@ -28660,13 +28639,13 @@
     <row r="9" spans="1:29" ht="15.75" customHeight="1" thickBot="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="328" t="s">
+      <c r="C9" s="334" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="329"/>
-      <c r="E9" s="329"/>
-      <c r="F9" s="329"/>
-      <c r="G9" s="329"/>
+      <c r="D9" s="335"/>
+      <c r="E9" s="335"/>
+      <c r="F9" s="335"/>
+      <c r="G9" s="335"/>
       <c r="H9" s="20"/>
       <c r="I9" s="24"/>
       <c r="J9" s="24"/>
@@ -28762,19 +28741,19 @@
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
-      <c r="J12" s="330" t="s">
+      <c r="J12" s="336" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="329"/>
-      <c r="L12" s="329"/>
-      <c r="M12" s="329"/>
-      <c r="N12" s="329"/>
-      <c r="O12" s="329"/>
-      <c r="P12" s="331">
+      <c r="K12" s="335"/>
+      <c r="L12" s="335"/>
+      <c r="M12" s="335"/>
+      <c r="N12" s="335"/>
+      <c r="O12" s="335"/>
+      <c r="P12" s="337">
         <f>I8</f>
         <v>2026</v>
       </c>
-      <c r="Q12" s="329"/>
+      <c r="Q12" s="335"/>
       <c r="R12" s="33"/>
       <c r="S12" s="34"/>
       <c r="T12" s="34"/>
@@ -29038,38 +29017,38 @@
     </row>
     <row r="21" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A21" s="39"/>
-      <c r="B21" s="332" t="s">
+      <c r="B21" s="331" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="333"/>
-      <c r="D21" s="333"/>
-      <c r="E21" s="333"/>
-      <c r="F21" s="333"/>
-      <c r="G21" s="333"/>
-      <c r="H21" s="333"/>
-      <c r="I21" s="333"/>
+      <c r="C21" s="327"/>
+      <c r="D21" s="327"/>
+      <c r="E21" s="327"/>
+      <c r="F21" s="327"/>
+      <c r="G21" s="327"/>
+      <c r="H21" s="327"/>
+      <c r="I21" s="327"/>
       <c r="J21" s="40"/>
-      <c r="K21" s="334" t="s">
+      <c r="K21" s="328" t="s">
         <v>37</v>
       </c>
-      <c r="L21" s="333"/>
-      <c r="M21" s="333"/>
-      <c r="N21" s="333"/>
-      <c r="O21" s="333"/>
-      <c r="P21" s="333"/>
-      <c r="Q21" s="333"/>
-      <c r="R21" s="333"/>
+      <c r="L21" s="327"/>
+      <c r="M21" s="327"/>
+      <c r="N21" s="327"/>
+      <c r="O21" s="327"/>
+      <c r="P21" s="327"/>
+      <c r="Q21" s="327"/>
+      <c r="R21" s="327"/>
       <c r="S21" s="40"/>
-      <c r="T21" s="335" t="s">
+      <c r="T21" s="326" t="s">
         <v>38</v>
       </c>
-      <c r="U21" s="333"/>
-      <c r="V21" s="333"/>
-      <c r="W21" s="333"/>
-      <c r="X21" s="333"/>
-      <c r="Y21" s="333"/>
-      <c r="Z21" s="333"/>
-      <c r="AA21" s="333"/>
+      <c r="U21" s="327"/>
+      <c r="V21" s="327"/>
+      <c r="W21" s="327"/>
+      <c r="X21" s="327"/>
+      <c r="Y21" s="327"/>
+      <c r="Z21" s="327"/>
+      <c r="AA21" s="327"/>
       <c r="AB21" s="41"/>
       <c r="AC21" s="42"/>
     </row>
@@ -29969,38 +29948,38 @@
     </row>
     <row r="35" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="336" t="s">
+      <c r="B35" s="329" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="333"/>
-      <c r="D35" s="333"/>
-      <c r="E35" s="333"/>
-      <c r="F35" s="333"/>
-      <c r="G35" s="333"/>
-      <c r="H35" s="333"/>
-      <c r="I35" s="333"/>
+      <c r="C35" s="327"/>
+      <c r="D35" s="327"/>
+      <c r="E35" s="327"/>
+      <c r="F35" s="327"/>
+      <c r="G35" s="327"/>
+      <c r="H35" s="327"/>
+      <c r="I35" s="327"/>
       <c r="J35" s="40"/>
-      <c r="K35" s="337" t="s">
+      <c r="K35" s="330" t="s">
         <v>48</v>
       </c>
-      <c r="L35" s="333"/>
-      <c r="M35" s="333"/>
-      <c r="N35" s="333"/>
-      <c r="O35" s="333"/>
-      <c r="P35" s="333"/>
-      <c r="Q35" s="333"/>
-      <c r="R35" s="333"/>
+      <c r="L35" s="327"/>
+      <c r="M35" s="327"/>
+      <c r="N35" s="327"/>
+      <c r="O35" s="327"/>
+      <c r="P35" s="327"/>
+      <c r="Q35" s="327"/>
+      <c r="R35" s="327"/>
       <c r="S35" s="40"/>
-      <c r="T35" s="334" t="s">
+      <c r="T35" s="328" t="s">
         <v>49</v>
       </c>
-      <c r="U35" s="333"/>
-      <c r="V35" s="333"/>
-      <c r="W35" s="333"/>
-      <c r="X35" s="333"/>
-      <c r="Y35" s="333"/>
-      <c r="Z35" s="333"/>
-      <c r="AA35" s="333"/>
+      <c r="U35" s="327"/>
+      <c r="V35" s="327"/>
+      <c r="W35" s="327"/>
+      <c r="X35" s="327"/>
+      <c r="Y35" s="327"/>
+      <c r="Z35" s="327"/>
+      <c r="AA35" s="327"/>
       <c r="AB35" s="70"/>
       <c r="AC35" s="40"/>
     </row>
@@ -30889,38 +30868,38 @@
     </row>
     <row r="49" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A49" s="69"/>
-      <c r="B49" s="334" t="s">
+      <c r="B49" s="328" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="333"/>
-      <c r="D49" s="333"/>
-      <c r="E49" s="333"/>
-      <c r="F49" s="333"/>
-      <c r="G49" s="333"/>
-      <c r="H49" s="333"/>
-      <c r="I49" s="333"/>
+      <c r="C49" s="327"/>
+      <c r="D49" s="327"/>
+      <c r="E49" s="327"/>
+      <c r="F49" s="327"/>
+      <c r="G49" s="327"/>
+      <c r="H49" s="327"/>
+      <c r="I49" s="327"/>
       <c r="J49" s="40"/>
-      <c r="K49" s="336" t="s">
+      <c r="K49" s="329" t="s">
         <v>51</v>
       </c>
-      <c r="L49" s="333"/>
-      <c r="M49" s="333"/>
-      <c r="N49" s="333"/>
-      <c r="O49" s="333"/>
-      <c r="P49" s="333"/>
-      <c r="Q49" s="333"/>
-      <c r="R49" s="333"/>
+      <c r="L49" s="327"/>
+      <c r="M49" s="327"/>
+      <c r="N49" s="327"/>
+      <c r="O49" s="327"/>
+      <c r="P49" s="327"/>
+      <c r="Q49" s="327"/>
+      <c r="R49" s="327"/>
       <c r="S49" s="40"/>
-      <c r="T49" s="332" t="s">
+      <c r="T49" s="331" t="s">
         <v>52</v>
       </c>
-      <c r="U49" s="333"/>
-      <c r="V49" s="333"/>
-      <c r="W49" s="333"/>
-      <c r="X49" s="333"/>
-      <c r="Y49" s="333"/>
-      <c r="Z49" s="333"/>
-      <c r="AA49" s="333"/>
+      <c r="U49" s="327"/>
+      <c r="V49" s="327"/>
+      <c r="W49" s="327"/>
+      <c r="X49" s="327"/>
+      <c r="Y49" s="327"/>
+      <c r="Z49" s="327"/>
+      <c r="AA49" s="327"/>
       <c r="AB49" s="70"/>
       <c r="AC49" s="40"/>
     </row>
@@ -31809,38 +31788,38 @@
     </row>
     <row r="63" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A63" s="69"/>
-      <c r="B63" s="335" t="s">
+      <c r="B63" s="326" t="s">
         <v>53</v>
       </c>
-      <c r="C63" s="333"/>
-      <c r="D63" s="333"/>
-      <c r="E63" s="333"/>
-      <c r="F63" s="333"/>
-      <c r="G63" s="333"/>
-      <c r="H63" s="333"/>
-      <c r="I63" s="333"/>
+      <c r="C63" s="327"/>
+      <c r="D63" s="327"/>
+      <c r="E63" s="327"/>
+      <c r="F63" s="327"/>
+      <c r="G63" s="327"/>
+      <c r="H63" s="327"/>
+      <c r="I63" s="327"/>
       <c r="J63" s="40"/>
-      <c r="K63" s="334" t="s">
+      <c r="K63" s="328" t="s">
         <v>54</v>
       </c>
-      <c r="L63" s="333"/>
-      <c r="M63" s="333"/>
-      <c r="N63" s="333"/>
-      <c r="O63" s="333"/>
-      <c r="P63" s="333"/>
-      <c r="Q63" s="333"/>
-      <c r="R63" s="333"/>
+      <c r="L63" s="327"/>
+      <c r="M63" s="327"/>
+      <c r="N63" s="327"/>
+      <c r="O63" s="327"/>
+      <c r="P63" s="327"/>
+      <c r="Q63" s="327"/>
+      <c r="R63" s="327"/>
       <c r="S63" s="40"/>
-      <c r="T63" s="336" t="s">
+      <c r="T63" s="329" t="s">
         <v>55</v>
       </c>
-      <c r="U63" s="333"/>
-      <c r="V63" s="333"/>
-      <c r="W63" s="333"/>
-      <c r="X63" s="333"/>
-      <c r="Y63" s="333"/>
-      <c r="Z63" s="333"/>
-      <c r="AA63" s="333"/>
+      <c r="U63" s="327"/>
+      <c r="V63" s="327"/>
+      <c r="W63" s="327"/>
+      <c r="X63" s="327"/>
+      <c r="Y63" s="327"/>
+      <c r="Z63" s="327"/>
+      <c r="AA63" s="327"/>
       <c r="AB63" s="70"/>
       <c r="AC63" s="40"/>
     </row>
@@ -61375,6 +61354,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="J12:O12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="K21:R21"/>
     <mergeCell ref="B63:I63"/>
     <mergeCell ref="K63:R63"/>
     <mergeCell ref="T63:AA63"/>
@@ -61385,12 +61370,6 @@
     <mergeCell ref="B49:I49"/>
     <mergeCell ref="K49:R49"/>
     <mergeCell ref="T49:AA49"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="J12:O12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="K21:R21"/>
   </mergeCells>
   <conditionalFormatting sqref="C51:I55">
     <cfRule type="expression" dxfId="2" priority="3">

</xml_diff>

<commit_message>
ghi thêm kpi vào file báo cáo
</commit_message>
<xml_diff>
--- a/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
+++ b/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonzai/dev/odoo 19/odoo/my_custom_addons/dl_salary_kpi/static/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD56066D-31D9-0647-A5A0-9C0B4AE71F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A42865AC-1BC7-FB40-BBA3-68F680C5895E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="17760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2476,37 +2476,70 @@
     <xf numFmtId="14" fontId="59" fillId="0" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="59" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="14" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="55" fillId="14" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2551,22 +2584,10 @@
     <xf numFmtId="0" fontId="66" fillId="25" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2575,72 +2596,35 @@
     <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="14" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="14" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="7" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2655,6 +2639,22 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="32">
@@ -3484,11 +3484,11 @@
       <c r="AL1" s="213"/>
       <c r="AM1" s="213"/>
       <c r="AN1" s="213"/>
-      <c r="AO1" s="276"/>
-      <c r="AP1" s="276"/>
-      <c r="AQ1" s="276"/>
-      <c r="AR1" s="276"/>
-      <c r="AS1" s="276"/>
+      <c r="AO1" s="325"/>
+      <c r="AP1" s="325"/>
+      <c r="AQ1" s="325"/>
+      <c r="AR1" s="325"/>
+      <c r="AS1" s="325"/>
       <c r="AT1" s="120"/>
       <c r="AU1" s="120"/>
       <c r="AV1" s="120"/>
@@ -3902,40 +3902,40 @@
       <c r="G4" s="238"/>
       <c r="H4" s="108"/>
       <c r="I4" s="275"/>
-      <c r="J4" s="277" t="s">
+      <c r="J4" s="317" t="s">
         <v>68</v>
       </c>
-      <c r="K4" s="277"/>
-      <c r="L4" s="278">
+      <c r="K4" s="317"/>
+      <c r="L4" s="319">
         <v>3</v>
       </c>
-      <c r="M4" s="278"/>
-      <c r="N4" s="277" t="s">
+      <c r="M4" s="319"/>
+      <c r="N4" s="317" t="s">
         <v>69</v>
       </c>
-      <c r="O4" s="277"/>
-      <c r="P4" s="277">
+      <c r="O4" s="317"/>
+      <c r="P4" s="317">
         <v>2026</v>
       </c>
-      <c r="Q4" s="277"/>
+      <c r="Q4" s="317"/>
       <c r="R4" s="109"/>
-      <c r="S4" s="277"/>
-      <c r="T4" s="277"/>
-      <c r="U4" s="277"/>
+      <c r="S4" s="317"/>
+      <c r="T4" s="317"/>
+      <c r="U4" s="317"/>
       <c r="V4" s="109"/>
-      <c r="W4" s="277"/>
-      <c r="X4" s="277"/>
-      <c r="Y4" s="277"/>
-      <c r="Z4" s="277"/>
-      <c r="AA4" s="277"/>
-      <c r="AB4" s="277"/>
-      <c r="AC4" s="277"/>
-      <c r="AD4" s="277"/>
+      <c r="W4" s="317"/>
+      <c r="X4" s="317"/>
+      <c r="Y4" s="317"/>
+      <c r="Z4" s="317"/>
+      <c r="AA4" s="317"/>
+      <c r="AB4" s="317"/>
+      <c r="AC4" s="317"/>
+      <c r="AD4" s="317"/>
       <c r="AE4" s="109"/>
       <c r="AF4" s="110"/>
-      <c r="AG4" s="277"/>
-      <c r="AH4" s="277"/>
-      <c r="AI4" s="277"/>
+      <c r="AG4" s="317"/>
+      <c r="AH4" s="317"/>
+      <c r="AI4" s="317"/>
       <c r="AJ4" s="109"/>
       <c r="AK4" s="109"/>
       <c r="AL4" s="109"/>
@@ -3946,50 +3946,47 @@
       <c r="AQ4" s="113"/>
       <c r="AR4" s="224"/>
       <c r="AS4" s="233"/>
-      <c r="AT4" s="277" t="s">
+      <c r="AT4" s="317" t="s">
         <v>68</v>
       </c>
-      <c r="AU4" s="277"/>
-      <c r="AV4" s="278">
+      <c r="AU4" s="317"/>
+      <c r="AV4" s="319">
         <f>L4</f>
         <v>3</v>
       </c>
-      <c r="AW4" s="278"/>
-      <c r="AX4" s="277" t="s">
+      <c r="AW4" s="319"/>
+      <c r="AX4" s="317" t="s">
         <v>69</v>
       </c>
-      <c r="AY4" s="277"/>
-      <c r="AZ4" s="277">
+      <c r="AY4" s="317"/>
+      <c r="AZ4" s="317">
         <v>2025</v>
       </c>
-      <c r="BA4" s="277"/>
+      <c r="BA4" s="317"/>
       <c r="BB4" s="109"/>
-      <c r="BC4" s="277"/>
-      <c r="BD4" s="277"/>
-      <c r="BE4" s="277"/>
+      <c r="BC4" s="317"/>
+      <c r="BD4" s="317"/>
+      <c r="BE4" s="317"/>
       <c r="BF4" s="109"/>
-      <c r="BG4" s="277"/>
-      <c r="BH4" s="277"/>
-      <c r="BI4" s="277"/>
-      <c r="BJ4" s="277"/>
-      <c r="BK4" s="277"/>
-      <c r="BL4" s="277"/>
-      <c r="BM4" s="277"/>
-      <c r="BN4" s="277"/>
+      <c r="BG4" s="317"/>
+      <c r="BH4" s="317"/>
+      <c r="BI4" s="317"/>
+      <c r="BJ4" s="317"/>
+      <c r="BK4" s="317"/>
+      <c r="BL4" s="317"/>
+      <c r="BM4" s="317"/>
+      <c r="BN4" s="317"/>
       <c r="BO4" s="109"/>
       <c r="BP4" s="110"/>
-      <c r="BQ4" s="277"/>
-      <c r="BR4" s="277"/>
-      <c r="BS4" s="277"/>
+      <c r="BQ4" s="317"/>
+      <c r="BR4" s="317"/>
+      <c r="BS4" s="317"/>
       <c r="BT4" s="114"/>
       <c r="BU4" s="114" t="str">
         <f>IF(WEEKDAY(BU5,1)=1,"CN","")</f>
         <v/>
       </c>
-      <c r="BV4" s="114" t="str">
-        <f>IF(WEEKDAY(BV5,1)=1,"CN","")</f>
-        <v>CN</v>
-      </c>
+      <c r="BV4" s="114"/>
       <c r="BW4" s="114"/>
       <c r="BX4" s="114" t="str">
         <f>IF(WEEKDAY(BX5,1)=1,"CN","")</f>
@@ -4033,19 +4030,10 @@
       <c r="DH4" s="141"/>
       <c r="DI4" s="115"/>
       <c r="DJ4" s="115"/>
-      <c r="DK4" s="149" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="DL4" s="149" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="DK4" s="149"/>
+      <c r="DL4" s="149"/>
       <c r="DM4" s="149"/>
-      <c r="DN4" s="149" t="e">
-        <f>#REF!</f>
-        <v>#REF!</v>
-      </c>
+      <c r="DN4" s="149"/>
       <c r="DO4" s="149"/>
       <c r="DP4" s="216"/>
       <c r="DQ4" s="216"/>
@@ -4079,31 +4067,31 @@
       <c r="EV4" s="247"/>
     </row>
     <row r="5" spans="1:154" s="184" customFormat="1" ht="92.25" customHeight="1">
-      <c r="A5" s="279" t="s">
+      <c r="A5" s="316" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="280" t="s">
+      <c r="B5" s="277" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="279" t="s">
+      <c r="C5" s="316" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="281" t="s">
+      <c r="D5" s="322" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="282" t="s">
+      <c r="E5" s="323" t="s">
         <v>122</v>
       </c>
-      <c r="F5" s="279" t="s">
+      <c r="F5" s="316" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="279" t="s">
+      <c r="G5" s="316" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="279" t="s">
+      <c r="H5" s="316" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="284" t="s">
+      <c r="I5" s="318" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="175">
@@ -4230,19 +4218,19 @@
         <f t="shared" si="0"/>
         <v>46112</v>
       </c>
-      <c r="AO5" s="285" t="s">
+      <c r="AO5" s="320" t="s">
         <v>82</v>
       </c>
-      <c r="AP5" s="285" t="s">
+      <c r="AP5" s="320" t="s">
         <v>83</v>
       </c>
-      <c r="AQ5" s="285" t="s">
+      <c r="AQ5" s="320" t="s">
         <v>84</v>
       </c>
-      <c r="AR5" s="286" t="s">
+      <c r="AR5" s="321" t="s">
         <v>5</v>
       </c>
-      <c r="AS5" s="286" t="s">
+      <c r="AS5" s="321" t="s">
         <v>6</v>
       </c>
       <c r="AT5" s="179">
@@ -4369,46 +4357,46 @@
         <f t="shared" si="1"/>
         <v>46112</v>
       </c>
-      <c r="BY5" s="310" t="s">
+      <c r="BY5" s="294" t="s">
         <v>86</v>
       </c>
-      <c r="BZ5" s="310" t="s">
+      <c r="BZ5" s="294" t="s">
         <v>87</v>
       </c>
-      <c r="CA5" s="310" t="s">
+      <c r="CA5" s="294" t="s">
         <v>88</v>
       </c>
-      <c r="CB5" s="310" t="s">
+      <c r="CB5" s="294" t="s">
         <v>89</v>
       </c>
-      <c r="CC5" s="310" t="s">
+      <c r="CC5" s="294" t="s">
         <v>90</v>
       </c>
-      <c r="CD5" s="310" t="s">
+      <c r="CD5" s="294" t="s">
         <v>91</v>
       </c>
-      <c r="CE5" s="310" t="s">
+      <c r="CE5" s="294" t="s">
         <v>92</v>
       </c>
-      <c r="CF5" s="309" t="s">
+      <c r="CF5" s="296" t="s">
         <v>19</v>
       </c>
-      <c r="CG5" s="309"/>
-      <c r="CH5" s="309"/>
-      <c r="CI5" s="309"/>
-      <c r="CJ5" s="309"/>
-      <c r="CK5" s="309"/>
-      <c r="CL5" s="309"/>
-      <c r="CM5" s="309"/>
-      <c r="CN5" s="309"/>
-      <c r="CO5" s="309"/>
-      <c r="CP5" s="309"/>
-      <c r="CQ5" s="315" t="s">
+      <c r="CG5" s="296"/>
+      <c r="CH5" s="296"/>
+      <c r="CI5" s="296"/>
+      <c r="CJ5" s="296"/>
+      <c r="CK5" s="296"/>
+      <c r="CL5" s="296"/>
+      <c r="CM5" s="296"/>
+      <c r="CN5" s="296"/>
+      <c r="CO5" s="296"/>
+      <c r="CP5" s="296"/>
+      <c r="CQ5" s="280" t="s">
         <v>59</v>
       </c>
-      <c r="CR5" s="316"/>
-      <c r="CS5" s="317"/>
-      <c r="CT5" s="322" t="s">
+      <c r="CR5" s="281"/>
+      <c r="CS5" s="282"/>
+      <c r="CT5" s="287" t="s">
         <v>60</v>
       </c>
       <c r="CU5" s="261" t="s">
@@ -4431,117 +4419,117 @@
       <c r="DF5" s="259" t="s">
         <v>130</v>
       </c>
-      <c r="DG5" s="318" t="s">
+      <c r="DG5" s="283" t="s">
         <v>119</v>
       </c>
-      <c r="DH5" s="323" t="s">
+      <c r="DH5" s="288" t="s">
         <v>113</v>
       </c>
-      <c r="DI5" s="320" t="s">
+      <c r="DI5" s="285" t="s">
         <v>81</v>
       </c>
-      <c r="DJ5" s="321"/>
-      <c r="DK5" s="304" t="s">
+      <c r="DJ5" s="286"/>
+      <c r="DK5" s="289" t="s">
         <v>61</v>
       </c>
-      <c r="DL5" s="312" t="s">
+      <c r="DL5" s="297" t="s">
         <v>8</v>
       </c>
-      <c r="DM5" s="305" t="s">
+      <c r="DM5" s="290" t="s">
         <v>71</v>
       </c>
-      <c r="DN5" s="305"/>
-      <c r="DO5" s="305"/>
-      <c r="DP5" s="305"/>
-      <c r="DQ5" s="305"/>
-      <c r="DR5" s="305"/>
-      <c r="DS5" s="324" t="s">
+      <c r="DN5" s="290"/>
+      <c r="DO5" s="290"/>
+      <c r="DP5" s="290"/>
+      <c r="DQ5" s="290"/>
+      <c r="DR5" s="290"/>
+      <c r="DS5" s="291" t="s">
         <v>12</v>
       </c>
-      <c r="DT5" s="305" t="s">
+      <c r="DT5" s="290" t="s">
         <v>128</v>
       </c>
-      <c r="DU5" s="280" t="s">
+      <c r="DU5" s="277" t="s">
         <v>13</v>
       </c>
-      <c r="DV5" s="313" t="s">
+      <c r="DV5" s="278" t="s">
         <v>64</v>
       </c>
-      <c r="DW5" s="314"/>
-      <c r="DX5" s="313"/>
-      <c r="DY5" s="302" t="s">
+      <c r="DW5" s="279"/>
+      <c r="DX5" s="278"/>
+      <c r="DY5" s="312" t="s">
         <v>63</v>
       </c>
-      <c r="DZ5" s="302"/>
-      <c r="EA5" s="302"/>
-      <c r="EB5" s="302"/>
-      <c r="EC5" s="303" t="s">
+      <c r="DZ5" s="312"/>
+      <c r="EA5" s="312"/>
+      <c r="EB5" s="312"/>
+      <c r="EC5" s="313" t="s">
         <v>131</v>
       </c>
-      <c r="ED5" s="305" t="s">
+      <c r="ED5" s="290" t="s">
         <v>7</v>
       </c>
-      <c r="EE5" s="306" t="s">
+      <c r="EE5" s="292" t="s">
         <v>65</v>
       </c>
-      <c r="EF5" s="306"/>
-      <c r="EG5" s="306" t="s">
+      <c r="EF5" s="292"/>
+      <c r="EG5" s="292" t="s">
         <v>66</v>
       </c>
-      <c r="EH5" s="306" t="s">
+      <c r="EH5" s="292" t="s">
         <v>67</v>
       </c>
-      <c r="EI5" s="306" t="s">
+      <c r="EI5" s="292" t="s">
         <v>72</v>
       </c>
-      <c r="EJ5" s="325" t="s">
+      <c r="EJ5" s="293" t="s">
         <v>78</v>
       </c>
-      <c r="EK5" s="325" t="s">
+      <c r="EK5" s="293" t="s">
         <v>80</v>
       </c>
-      <c r="EL5" s="325" t="s">
+      <c r="EL5" s="293" t="s">
         <v>79</v>
       </c>
-      <c r="EM5" s="291" t="s">
+      <c r="EM5" s="302" t="s">
         <v>127</v>
       </c>
-      <c r="EN5" s="293"/>
-      <c r="EO5" s="295" t="s">
+      <c r="EN5" s="304"/>
+      <c r="EO5" s="306" t="s">
         <v>132</v>
       </c>
-      <c r="EP5" s="297" t="s">
+      <c r="EP5" s="308" t="s">
         <v>118</v>
       </c>
-      <c r="EQ5" s="299" t="s">
+      <c r="EQ5" s="310" t="s">
         <v>133</v>
       </c>
-      <c r="ER5" s="301" t="s">
+      <c r="ER5" s="276" t="s">
         <v>125</v>
       </c>
-      <c r="ES5" s="301" t="s">
+      <c r="ES5" s="276" t="s">
         <v>124</v>
       </c>
-      <c r="ET5" s="307" t="s">
+      <c r="ET5" s="314" t="s">
         <v>120</v>
       </c>
-      <c r="EU5" s="287" t="s">
+      <c r="EU5" s="298" t="s">
         <v>123</v>
       </c>
-      <c r="EV5" s="289" t="s">
+      <c r="EV5" s="300" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:154" s="206" customFormat="1" ht="148.5" customHeight="1">
-      <c r="A6" s="279"/>
-      <c r="B6" s="280"/>
-      <c r="C6" s="279"/>
-      <c r="D6" s="281"/>
-      <c r="E6" s="283"/>
-      <c r="F6" s="279"/>
-      <c r="G6" s="279"/>
-      <c r="H6" s="279"/>
-      <c r="I6" s="284"/>
+      <c r="A6" s="316"/>
+      <c r="B6" s="277"/>
+      <c r="C6" s="316"/>
+      <c r="D6" s="322"/>
+      <c r="E6" s="324"/>
+      <c r="F6" s="316"/>
+      <c r="G6" s="316"/>
+      <c r="H6" s="316"/>
+      <c r="I6" s="318"/>
       <c r="J6" s="185" t="str">
         <f t="shared" ref="J6:AN6" si="2">IF(WEEKDAY(J5)=1,"CN",WEEKDAY(J5))</f>
         <v>CN</v>
@@ -4666,11 +4654,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AO6" s="285"/>
-      <c r="AP6" s="285"/>
-      <c r="AQ6" s="285"/>
-      <c r="AR6" s="286"/>
-      <c r="AS6" s="286"/>
+      <c r="AO6" s="320"/>
+      <c r="AP6" s="320"/>
+      <c r="AQ6" s="320"/>
+      <c r="AR6" s="321"/>
+      <c r="AS6" s="321"/>
       <c r="AT6" s="187" t="str">
         <f>+J6</f>
         <v>CN</v>
@@ -4795,13 +4783,13 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="BY6" s="311"/>
-      <c r="BZ6" s="311"/>
-      <c r="CA6" s="311"/>
-      <c r="CB6" s="311"/>
-      <c r="CC6" s="311"/>
-      <c r="CD6" s="311"/>
-      <c r="CE6" s="311"/>
+      <c r="BY6" s="295"/>
+      <c r="BZ6" s="295"/>
+      <c r="CA6" s="295"/>
+      <c r="CB6" s="295"/>
+      <c r="CC6" s="295"/>
+      <c r="CD6" s="295"/>
+      <c r="CE6" s="295"/>
       <c r="CF6" s="189" t="s">
         <v>93</v>
       </c>
@@ -4844,7 +4832,7 @@
       <c r="CS6" s="181" t="s">
         <v>58</v>
       </c>
-      <c r="CT6" s="322"/>
+      <c r="CT6" s="287"/>
       <c r="CU6" s="189" t="s">
         <v>104</v>
       </c>
@@ -4881,16 +4869,16 @@
       <c r="DF6" s="260" t="s">
         <v>134</v>
       </c>
-      <c r="DG6" s="319"/>
-      <c r="DH6" s="323"/>
+      <c r="DG6" s="284"/>
+      <c r="DH6" s="288"/>
       <c r="DI6" s="152" t="s">
         <v>14</v>
       </c>
       <c r="DJ6" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="DK6" s="304"/>
-      <c r="DL6" s="312"/>
+      <c r="DK6" s="289"/>
+      <c r="DL6" s="297"/>
       <c r="DM6" s="181" t="s">
         <v>9</v>
       </c>
@@ -4909,9 +4897,9 @@
       <c r="DR6" s="181" t="s">
         <v>116</v>
       </c>
-      <c r="DS6" s="324"/>
-      <c r="DT6" s="305"/>
-      <c r="DU6" s="280"/>
+      <c r="DS6" s="291"/>
+      <c r="DT6" s="290"/>
+      <c r="DU6" s="277"/>
       <c r="DV6" s="204">
         <v>0.17499999999999999</v>
       </c>
@@ -4933,176 +4921,176 @@
       <c r="EB6" s="152" t="s">
         <v>62</v>
       </c>
-      <c r="EC6" s="304"/>
-      <c r="ED6" s="305"/>
+      <c r="EC6" s="289"/>
+      <c r="ED6" s="290"/>
       <c r="EE6" s="183" t="s">
         <v>73</v>
       </c>
       <c r="EF6" s="183" t="s">
         <v>74</v>
       </c>
-      <c r="EG6" s="306"/>
-      <c r="EH6" s="306"/>
-      <c r="EI6" s="306"/>
-      <c r="EJ6" s="325"/>
-      <c r="EK6" s="325"/>
-      <c r="EL6" s="325"/>
-      <c r="EM6" s="292"/>
-      <c r="EN6" s="294"/>
-      <c r="EO6" s="296"/>
-      <c r="EP6" s="298"/>
-      <c r="EQ6" s="300"/>
-      <c r="ER6" s="301"/>
-      <c r="ES6" s="301"/>
-      <c r="ET6" s="308"/>
-      <c r="EU6" s="288"/>
-      <c r="EV6" s="289"/>
+      <c r="EG6" s="292"/>
+      <c r="EH6" s="292"/>
+      <c r="EI6" s="292"/>
+      <c r="EJ6" s="293"/>
+      <c r="EK6" s="293"/>
+      <c r="EL6" s="293"/>
+      <c r="EM6" s="303"/>
+      <c r="EN6" s="305"/>
+      <c r="EO6" s="307"/>
+      <c r="EP6" s="309"/>
+      <c r="EQ6" s="311"/>
+      <c r="ER6" s="276"/>
+      <c r="ES6" s="276"/>
+      <c r="ET6" s="315"/>
+      <c r="EU6" s="299"/>
+      <c r="EV6" s="300"/>
     </row>
     <row r="7" spans="1:154" s="106" customFormat="1" ht="87.75" customHeight="1">
-      <c r="A7" s="290" t="s">
+      <c r="A7" s="301" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="290"/>
-      <c r="C7" s="290"/>
-      <c r="D7" s="290"/>
-      <c r="E7" s="290"/>
-      <c r="F7" s="290"/>
-      <c r="G7" s="290"/>
-      <c r="H7" s="290"/>
-      <c r="I7" s="290"/>
-      <c r="J7" s="290"/>
-      <c r="K7" s="290"/>
-      <c r="L7" s="290"/>
-      <c r="M7" s="290"/>
-      <c r="N7" s="290"/>
-      <c r="O7" s="290"/>
-      <c r="P7" s="290"/>
-      <c r="Q7" s="290"/>
-      <c r="R7" s="290"/>
-      <c r="S7" s="290"/>
-      <c r="T7" s="290"/>
-      <c r="U7" s="290"/>
-      <c r="V7" s="290"/>
-      <c r="W7" s="290"/>
-      <c r="X7" s="290"/>
-      <c r="Y7" s="290"/>
-      <c r="Z7" s="290"/>
-      <c r="AA7" s="290"/>
-      <c r="AB7" s="290"/>
-      <c r="AC7" s="290"/>
-      <c r="AD7" s="290"/>
-      <c r="AE7" s="290"/>
-      <c r="AF7" s="290"/>
-      <c r="AG7" s="290"/>
-      <c r="AH7" s="290"/>
-      <c r="AI7" s="290"/>
-      <c r="AJ7" s="290"/>
-      <c r="AK7" s="290"/>
-      <c r="AL7" s="290"/>
-      <c r="AM7" s="290"/>
-      <c r="AN7" s="290"/>
-      <c r="AO7" s="290"/>
-      <c r="AP7" s="290"/>
-      <c r="AQ7" s="290"/>
-      <c r="AR7" s="290"/>
-      <c r="AS7" s="290"/>
-      <c r="AT7" s="290"/>
-      <c r="AU7" s="290"/>
-      <c r="AV7" s="290"/>
-      <c r="AW7" s="290"/>
-      <c r="AX7" s="290"/>
-      <c r="AY7" s="290"/>
-      <c r="AZ7" s="290"/>
-      <c r="BA7" s="290"/>
-      <c r="BB7" s="290"/>
-      <c r="BC7" s="290"/>
-      <c r="BD7" s="290"/>
-      <c r="BE7" s="290"/>
-      <c r="BF7" s="290"/>
-      <c r="BG7" s="290"/>
-      <c r="BH7" s="290"/>
-      <c r="BI7" s="290"/>
-      <c r="BJ7" s="290"/>
-      <c r="BK7" s="290"/>
-      <c r="BL7" s="290"/>
-      <c r="BM7" s="290"/>
-      <c r="BN7" s="290"/>
-      <c r="BO7" s="290"/>
-      <c r="BP7" s="290"/>
-      <c r="BQ7" s="290"/>
-      <c r="BR7" s="290"/>
-      <c r="BS7" s="290"/>
-      <c r="BT7" s="290"/>
-      <c r="BU7" s="290"/>
-      <c r="BV7" s="290"/>
-      <c r="BW7" s="290"/>
-      <c r="BX7" s="290"/>
-      <c r="BY7" s="290"/>
-      <c r="BZ7" s="290"/>
-      <c r="CA7" s="290"/>
-      <c r="CB7" s="290"/>
-      <c r="CC7" s="290"/>
-      <c r="CD7" s="290"/>
-      <c r="CE7" s="290"/>
-      <c r="CF7" s="290"/>
-      <c r="CG7" s="290"/>
-      <c r="CH7" s="290"/>
-      <c r="CI7" s="290"/>
-      <c r="CJ7" s="290"/>
-      <c r="CK7" s="290"/>
-      <c r="CL7" s="290"/>
-      <c r="CM7" s="290"/>
-      <c r="CN7" s="290"/>
-      <c r="CO7" s="290"/>
-      <c r="CP7" s="290"/>
-      <c r="CQ7" s="290"/>
-      <c r="CR7" s="290"/>
-      <c r="CS7" s="290"/>
-      <c r="CT7" s="290"/>
-      <c r="CU7" s="290"/>
-      <c r="CV7" s="290"/>
-      <c r="CW7" s="290"/>
-      <c r="CX7" s="290"/>
-      <c r="CY7" s="290"/>
-      <c r="CZ7" s="290"/>
-      <c r="DA7" s="290"/>
-      <c r="DB7" s="290"/>
-      <c r="DC7" s="290"/>
-      <c r="DD7" s="290"/>
-      <c r="DE7" s="290"/>
-      <c r="DF7" s="290"/>
-      <c r="DG7" s="290"/>
-      <c r="DH7" s="290"/>
-      <c r="DI7" s="290"/>
-      <c r="DJ7" s="290"/>
-      <c r="DK7" s="290"/>
-      <c r="DL7" s="290"/>
-      <c r="DM7" s="290"/>
-      <c r="DN7" s="290"/>
-      <c r="DO7" s="290"/>
-      <c r="DP7" s="290"/>
-      <c r="DQ7" s="290"/>
-      <c r="DR7" s="290"/>
-      <c r="DS7" s="290"/>
-      <c r="DT7" s="290"/>
-      <c r="DU7" s="290"/>
-      <c r="DV7" s="290"/>
-      <c r="DW7" s="290"/>
-      <c r="DX7" s="290"/>
-      <c r="DY7" s="290"/>
-      <c r="DZ7" s="290"/>
-      <c r="EA7" s="290"/>
-      <c r="EB7" s="290"/>
-      <c r="EC7" s="290"/>
-      <c r="ED7" s="290"/>
-      <c r="EE7" s="290"/>
-      <c r="EF7" s="290"/>
-      <c r="EG7" s="290"/>
-      <c r="EH7" s="290"/>
-      <c r="EI7" s="290"/>
-      <c r="EJ7" s="290"/>
-      <c r="EK7" s="290"/>
-      <c r="EL7" s="290"/>
+      <c r="B7" s="301"/>
+      <c r="C7" s="301"/>
+      <c r="D7" s="301"/>
+      <c r="E7" s="301"/>
+      <c r="F7" s="301"/>
+      <c r="G7" s="301"/>
+      <c r="H7" s="301"/>
+      <c r="I7" s="301"/>
+      <c r="J7" s="301"/>
+      <c r="K7" s="301"/>
+      <c r="L7" s="301"/>
+      <c r="M7" s="301"/>
+      <c r="N7" s="301"/>
+      <c r="O7" s="301"/>
+      <c r="P7" s="301"/>
+      <c r="Q7" s="301"/>
+      <c r="R7" s="301"/>
+      <c r="S7" s="301"/>
+      <c r="T7" s="301"/>
+      <c r="U7" s="301"/>
+      <c r="V7" s="301"/>
+      <c r="W7" s="301"/>
+      <c r="X7" s="301"/>
+      <c r="Y7" s="301"/>
+      <c r="Z7" s="301"/>
+      <c r="AA7" s="301"/>
+      <c r="AB7" s="301"/>
+      <c r="AC7" s="301"/>
+      <c r="AD7" s="301"/>
+      <c r="AE7" s="301"/>
+      <c r="AF7" s="301"/>
+      <c r="AG7" s="301"/>
+      <c r="AH7" s="301"/>
+      <c r="AI7" s="301"/>
+      <c r="AJ7" s="301"/>
+      <c r="AK7" s="301"/>
+      <c r="AL7" s="301"/>
+      <c r="AM7" s="301"/>
+      <c r="AN7" s="301"/>
+      <c r="AO7" s="301"/>
+      <c r="AP7" s="301"/>
+      <c r="AQ7" s="301"/>
+      <c r="AR7" s="301"/>
+      <c r="AS7" s="301"/>
+      <c r="AT7" s="301"/>
+      <c r="AU7" s="301"/>
+      <c r="AV7" s="301"/>
+      <c r="AW7" s="301"/>
+      <c r="AX7" s="301"/>
+      <c r="AY7" s="301"/>
+      <c r="AZ7" s="301"/>
+      <c r="BA7" s="301"/>
+      <c r="BB7" s="301"/>
+      <c r="BC7" s="301"/>
+      <c r="BD7" s="301"/>
+      <c r="BE7" s="301"/>
+      <c r="BF7" s="301"/>
+      <c r="BG7" s="301"/>
+      <c r="BH7" s="301"/>
+      <c r="BI7" s="301"/>
+      <c r="BJ7" s="301"/>
+      <c r="BK7" s="301"/>
+      <c r="BL7" s="301"/>
+      <c r="BM7" s="301"/>
+      <c r="BN7" s="301"/>
+      <c r="BO7" s="301"/>
+      <c r="BP7" s="301"/>
+      <c r="BQ7" s="301"/>
+      <c r="BR7" s="301"/>
+      <c r="BS7" s="301"/>
+      <c r="BT7" s="301"/>
+      <c r="BU7" s="301"/>
+      <c r="BV7" s="301"/>
+      <c r="BW7" s="301"/>
+      <c r="BX7" s="301"/>
+      <c r="BY7" s="301"/>
+      <c r="BZ7" s="301"/>
+      <c r="CA7" s="301"/>
+      <c r="CB7" s="301"/>
+      <c r="CC7" s="301"/>
+      <c r="CD7" s="301"/>
+      <c r="CE7" s="301"/>
+      <c r="CF7" s="301"/>
+      <c r="CG7" s="301"/>
+      <c r="CH7" s="301"/>
+      <c r="CI7" s="301"/>
+      <c r="CJ7" s="301"/>
+      <c r="CK7" s="301"/>
+      <c r="CL7" s="301"/>
+      <c r="CM7" s="301"/>
+      <c r="CN7" s="301"/>
+      <c r="CO7" s="301"/>
+      <c r="CP7" s="301"/>
+      <c r="CQ7" s="301"/>
+      <c r="CR7" s="301"/>
+      <c r="CS7" s="301"/>
+      <c r="CT7" s="301"/>
+      <c r="CU7" s="301"/>
+      <c r="CV7" s="301"/>
+      <c r="CW7" s="301"/>
+      <c r="CX7" s="301"/>
+      <c r="CY7" s="301"/>
+      <c r="CZ7" s="301"/>
+      <c r="DA7" s="301"/>
+      <c r="DB7" s="301"/>
+      <c r="DC7" s="301"/>
+      <c r="DD7" s="301"/>
+      <c r="DE7" s="301"/>
+      <c r="DF7" s="301"/>
+      <c r="DG7" s="301"/>
+      <c r="DH7" s="301"/>
+      <c r="DI7" s="301"/>
+      <c r="DJ7" s="301"/>
+      <c r="DK7" s="301"/>
+      <c r="DL7" s="301"/>
+      <c r="DM7" s="301"/>
+      <c r="DN7" s="301"/>
+      <c r="DO7" s="301"/>
+      <c r="DP7" s="301"/>
+      <c r="DQ7" s="301"/>
+      <c r="DR7" s="301"/>
+      <c r="DS7" s="301"/>
+      <c r="DT7" s="301"/>
+      <c r="DU7" s="301"/>
+      <c r="DV7" s="301"/>
+      <c r="DW7" s="301"/>
+      <c r="DX7" s="301"/>
+      <c r="DY7" s="301"/>
+      <c r="DZ7" s="301"/>
+      <c r="EA7" s="301"/>
+      <c r="EB7" s="301"/>
+      <c r="EC7" s="301"/>
+      <c r="ED7" s="301"/>
+      <c r="EE7" s="301"/>
+      <c r="EF7" s="301"/>
+      <c r="EG7" s="301"/>
+      <c r="EH7" s="301"/>
+      <c r="EI7" s="301"/>
+      <c r="EJ7" s="301"/>
+      <c r="EK7" s="301"/>
+      <c r="EL7" s="301"/>
       <c r="EM7" s="248"/>
       <c r="EN7" s="248"/>
       <c r="EO7" s="248"/>
@@ -27880,6 +27868,64 @@
   </sheetData>
   <autoFilter ref="A6:EX8" xr:uid="{00000000-0001-0000-0900-000000000000}"/>
   <mergeCells count="74">
+    <mergeCell ref="AO1:AS1"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:U4"/>
+    <mergeCell ref="W4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="AG4:AI4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="BG4:BI4"/>
+    <mergeCell ref="AT4:AU4"/>
+    <mergeCell ref="AV4:AW4"/>
+    <mergeCell ref="AX4:AY4"/>
+    <mergeCell ref="AO5:AO6"/>
+    <mergeCell ref="AP5:AP6"/>
+    <mergeCell ref="AQ5:AQ6"/>
+    <mergeCell ref="AR5:AR6"/>
+    <mergeCell ref="AS5:AS6"/>
+    <mergeCell ref="BJ4:BK4"/>
+    <mergeCell ref="BL4:BN4"/>
+    <mergeCell ref="BQ4:BS4"/>
+    <mergeCell ref="AZ4:BA4"/>
+    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="EU5:EU6"/>
+    <mergeCell ref="EV5:EV6"/>
+    <mergeCell ref="A7:EL7"/>
+    <mergeCell ref="EM5:EM6"/>
+    <mergeCell ref="EN5:EN6"/>
+    <mergeCell ref="EO5:EO6"/>
+    <mergeCell ref="EP5:EP6"/>
+    <mergeCell ref="EQ5:EQ6"/>
+    <mergeCell ref="ER5:ER6"/>
+    <mergeCell ref="DY5:EB5"/>
+    <mergeCell ref="EC5:EC6"/>
+    <mergeCell ref="ED5:ED6"/>
+    <mergeCell ref="EE5:EF5"/>
+    <mergeCell ref="DT5:DT6"/>
+    <mergeCell ref="ET5:ET6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="CF5:CP5"/>
+    <mergeCell ref="CD5:CD6"/>
+    <mergeCell ref="CE5:CE6"/>
+    <mergeCell ref="DL5:DL6"/>
+    <mergeCell ref="EG5:EG6"/>
+    <mergeCell ref="BY5:BY6"/>
+    <mergeCell ref="BZ5:BZ6"/>
+    <mergeCell ref="CA5:CA6"/>
+    <mergeCell ref="CB5:CB6"/>
+    <mergeCell ref="CC5:CC6"/>
     <mergeCell ref="ES5:ES6"/>
     <mergeCell ref="DU5:DU6"/>
     <mergeCell ref="DV5:DX5"/>
@@ -27896,64 +27942,6 @@
     <mergeCell ref="EK5:EK6"/>
     <mergeCell ref="EL5:EL6"/>
     <mergeCell ref="EH5:EH6"/>
-    <mergeCell ref="BY5:BY6"/>
-    <mergeCell ref="BZ5:BZ6"/>
-    <mergeCell ref="CA5:CA6"/>
-    <mergeCell ref="CB5:CB6"/>
-    <mergeCell ref="CC5:CC6"/>
-    <mergeCell ref="CF5:CP5"/>
-    <mergeCell ref="CD5:CD6"/>
-    <mergeCell ref="CE5:CE6"/>
-    <mergeCell ref="DL5:DL6"/>
-    <mergeCell ref="EG5:EG6"/>
-    <mergeCell ref="EU5:EU6"/>
-    <mergeCell ref="EV5:EV6"/>
-    <mergeCell ref="A7:EL7"/>
-    <mergeCell ref="EM5:EM6"/>
-    <mergeCell ref="EN5:EN6"/>
-    <mergeCell ref="EO5:EO6"/>
-    <mergeCell ref="EP5:EP6"/>
-    <mergeCell ref="EQ5:EQ6"/>
-    <mergeCell ref="ER5:ER6"/>
-    <mergeCell ref="DY5:EB5"/>
-    <mergeCell ref="EC5:EC6"/>
-    <mergeCell ref="ED5:ED6"/>
-    <mergeCell ref="EE5:EF5"/>
-    <mergeCell ref="DT5:DT6"/>
-    <mergeCell ref="ET5:ET6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="BJ4:BK4"/>
-    <mergeCell ref="BL4:BN4"/>
-    <mergeCell ref="BQ4:BS4"/>
-    <mergeCell ref="AZ4:BA4"/>
-    <mergeCell ref="BC4:BE4"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="BG4:BI4"/>
-    <mergeCell ref="AT4:AU4"/>
-    <mergeCell ref="AV4:AW4"/>
-    <mergeCell ref="AX4:AY4"/>
-    <mergeCell ref="AO5:AO6"/>
-    <mergeCell ref="AP5:AP6"/>
-    <mergeCell ref="AQ5:AQ6"/>
-    <mergeCell ref="AR5:AR6"/>
-    <mergeCell ref="AS5:AS6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="AO1:AS1"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:U4"/>
-    <mergeCell ref="W4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AD4"/>
-    <mergeCell ref="AG4:AI4"/>
   </mergeCells>
   <conditionalFormatting sqref="A5 A8:B8">
     <cfRule type="duplicateValues" dxfId="20" priority="20879"/>
@@ -28610,11 +28598,11 @@
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
       <c r="H8" s="20"/>
-      <c r="I8" s="332">
+      <c r="I8" s="326">
         <v>2026</v>
       </c>
-      <c r="J8" s="333"/>
-      <c r="K8" s="333"/>
+      <c r="J8" s="327"/>
+      <c r="K8" s="327"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="21" t="s">
@@ -28639,13 +28627,13 @@
     <row r="9" spans="1:29" ht="15.75" customHeight="1" thickBot="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="334" t="s">
+      <c r="C9" s="328" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="335"/>
-      <c r="E9" s="335"/>
-      <c r="F9" s="335"/>
-      <c r="G9" s="335"/>
+      <c r="D9" s="329"/>
+      <c r="E9" s="329"/>
+      <c r="F9" s="329"/>
+      <c r="G9" s="329"/>
       <c r="H9" s="20"/>
       <c r="I9" s="24"/>
       <c r="J9" s="24"/>
@@ -28741,19 +28729,19 @@
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
-      <c r="J12" s="336" t="s">
+      <c r="J12" s="330" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="335"/>
-      <c r="L12" s="335"/>
-      <c r="M12" s="335"/>
-      <c r="N12" s="335"/>
-      <c r="O12" s="335"/>
-      <c r="P12" s="337">
+      <c r="K12" s="329"/>
+      <c r="L12" s="329"/>
+      <c r="M12" s="329"/>
+      <c r="N12" s="329"/>
+      <c r="O12" s="329"/>
+      <c r="P12" s="331">
         <f>I8</f>
         <v>2026</v>
       </c>
-      <c r="Q12" s="335"/>
+      <c r="Q12" s="329"/>
       <c r="R12" s="33"/>
       <c r="S12" s="34"/>
       <c r="T12" s="34"/>
@@ -29017,38 +29005,38 @@
     </row>
     <row r="21" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A21" s="39"/>
-      <c r="B21" s="331" t="s">
+      <c r="B21" s="332" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="327"/>
-      <c r="D21" s="327"/>
-      <c r="E21" s="327"/>
-      <c r="F21" s="327"/>
-      <c r="G21" s="327"/>
-      <c r="H21" s="327"/>
-      <c r="I21" s="327"/>
+      <c r="C21" s="333"/>
+      <c r="D21" s="333"/>
+      <c r="E21" s="333"/>
+      <c r="F21" s="333"/>
+      <c r="G21" s="333"/>
+      <c r="H21" s="333"/>
+      <c r="I21" s="333"/>
       <c r="J21" s="40"/>
-      <c r="K21" s="328" t="s">
+      <c r="K21" s="334" t="s">
         <v>37</v>
       </c>
-      <c r="L21" s="327"/>
-      <c r="M21" s="327"/>
-      <c r="N21" s="327"/>
-      <c r="O21" s="327"/>
-      <c r="P21" s="327"/>
-      <c r="Q21" s="327"/>
-      <c r="R21" s="327"/>
+      <c r="L21" s="333"/>
+      <c r="M21" s="333"/>
+      <c r="N21" s="333"/>
+      <c r="O21" s="333"/>
+      <c r="P21" s="333"/>
+      <c r="Q21" s="333"/>
+      <c r="R21" s="333"/>
       <c r="S21" s="40"/>
-      <c r="T21" s="326" t="s">
+      <c r="T21" s="335" t="s">
         <v>38</v>
       </c>
-      <c r="U21" s="327"/>
-      <c r="V21" s="327"/>
-      <c r="W21" s="327"/>
-      <c r="X21" s="327"/>
-      <c r="Y21" s="327"/>
-      <c r="Z21" s="327"/>
-      <c r="AA21" s="327"/>
+      <c r="U21" s="333"/>
+      <c r="V21" s="333"/>
+      <c r="W21" s="333"/>
+      <c r="X21" s="333"/>
+      <c r="Y21" s="333"/>
+      <c r="Z21" s="333"/>
+      <c r="AA21" s="333"/>
       <c r="AB21" s="41"/>
       <c r="AC21" s="42"/>
     </row>
@@ -29948,38 +29936,38 @@
     </row>
     <row r="35" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="329" t="s">
+      <c r="B35" s="336" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="327"/>
-      <c r="D35" s="327"/>
-      <c r="E35" s="327"/>
-      <c r="F35" s="327"/>
-      <c r="G35" s="327"/>
-      <c r="H35" s="327"/>
-      <c r="I35" s="327"/>
+      <c r="C35" s="333"/>
+      <c r="D35" s="333"/>
+      <c r="E35" s="333"/>
+      <c r="F35" s="333"/>
+      <c r="G35" s="333"/>
+      <c r="H35" s="333"/>
+      <c r="I35" s="333"/>
       <c r="J35" s="40"/>
-      <c r="K35" s="330" t="s">
+      <c r="K35" s="337" t="s">
         <v>48</v>
       </c>
-      <c r="L35" s="327"/>
-      <c r="M35" s="327"/>
-      <c r="N35" s="327"/>
-      <c r="O35" s="327"/>
-      <c r="P35" s="327"/>
-      <c r="Q35" s="327"/>
-      <c r="R35" s="327"/>
+      <c r="L35" s="333"/>
+      <c r="M35" s="333"/>
+      <c r="N35" s="333"/>
+      <c r="O35" s="333"/>
+      <c r="P35" s="333"/>
+      <c r="Q35" s="333"/>
+      <c r="R35" s="333"/>
       <c r="S35" s="40"/>
-      <c r="T35" s="328" t="s">
+      <c r="T35" s="334" t="s">
         <v>49</v>
       </c>
-      <c r="U35" s="327"/>
-      <c r="V35" s="327"/>
-      <c r="W35" s="327"/>
-      <c r="X35" s="327"/>
-      <c r="Y35" s="327"/>
-      <c r="Z35" s="327"/>
-      <c r="AA35" s="327"/>
+      <c r="U35" s="333"/>
+      <c r="V35" s="333"/>
+      <c r="W35" s="333"/>
+      <c r="X35" s="333"/>
+      <c r="Y35" s="333"/>
+      <c r="Z35" s="333"/>
+      <c r="AA35" s="333"/>
       <c r="AB35" s="70"/>
       <c r="AC35" s="40"/>
     </row>
@@ -30868,38 +30856,38 @@
     </row>
     <row r="49" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A49" s="69"/>
-      <c r="B49" s="328" t="s">
+      <c r="B49" s="334" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="327"/>
-      <c r="D49" s="327"/>
-      <c r="E49" s="327"/>
-      <c r="F49" s="327"/>
-      <c r="G49" s="327"/>
-      <c r="H49" s="327"/>
-      <c r="I49" s="327"/>
+      <c r="C49" s="333"/>
+      <c r="D49" s="333"/>
+      <c r="E49" s="333"/>
+      <c r="F49" s="333"/>
+      <c r="G49" s="333"/>
+      <c r="H49" s="333"/>
+      <c r="I49" s="333"/>
       <c r="J49" s="40"/>
-      <c r="K49" s="329" t="s">
+      <c r="K49" s="336" t="s">
         <v>51</v>
       </c>
-      <c r="L49" s="327"/>
-      <c r="M49" s="327"/>
-      <c r="N49" s="327"/>
-      <c r="O49" s="327"/>
-      <c r="P49" s="327"/>
-      <c r="Q49" s="327"/>
-      <c r="R49" s="327"/>
+      <c r="L49" s="333"/>
+      <c r="M49" s="333"/>
+      <c r="N49" s="333"/>
+      <c r="O49" s="333"/>
+      <c r="P49" s="333"/>
+      <c r="Q49" s="333"/>
+      <c r="R49" s="333"/>
       <c r="S49" s="40"/>
-      <c r="T49" s="331" t="s">
+      <c r="T49" s="332" t="s">
         <v>52</v>
       </c>
-      <c r="U49" s="327"/>
-      <c r="V49" s="327"/>
-      <c r="W49" s="327"/>
-      <c r="X49" s="327"/>
-      <c r="Y49" s="327"/>
-      <c r="Z49" s="327"/>
-      <c r="AA49" s="327"/>
+      <c r="U49" s="333"/>
+      <c r="V49" s="333"/>
+      <c r="W49" s="333"/>
+      <c r="X49" s="333"/>
+      <c r="Y49" s="333"/>
+      <c r="Z49" s="333"/>
+      <c r="AA49" s="333"/>
       <c r="AB49" s="70"/>
       <c r="AC49" s="40"/>
     </row>
@@ -31788,38 +31776,38 @@
     </row>
     <row r="63" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A63" s="69"/>
-      <c r="B63" s="326" t="s">
+      <c r="B63" s="335" t="s">
         <v>53</v>
       </c>
-      <c r="C63" s="327"/>
-      <c r="D63" s="327"/>
-      <c r="E63" s="327"/>
-      <c r="F63" s="327"/>
-      <c r="G63" s="327"/>
-      <c r="H63" s="327"/>
-      <c r="I63" s="327"/>
+      <c r="C63" s="333"/>
+      <c r="D63" s="333"/>
+      <c r="E63" s="333"/>
+      <c r="F63" s="333"/>
+      <c r="G63" s="333"/>
+      <c r="H63" s="333"/>
+      <c r="I63" s="333"/>
       <c r="J63" s="40"/>
-      <c r="K63" s="328" t="s">
+      <c r="K63" s="334" t="s">
         <v>54</v>
       </c>
-      <c r="L63" s="327"/>
-      <c r="M63" s="327"/>
-      <c r="N63" s="327"/>
-      <c r="O63" s="327"/>
-      <c r="P63" s="327"/>
-      <c r="Q63" s="327"/>
-      <c r="R63" s="327"/>
+      <c r="L63" s="333"/>
+      <c r="M63" s="333"/>
+      <c r="N63" s="333"/>
+      <c r="O63" s="333"/>
+      <c r="P63" s="333"/>
+      <c r="Q63" s="333"/>
+      <c r="R63" s="333"/>
       <c r="S63" s="40"/>
-      <c r="T63" s="329" t="s">
+      <c r="T63" s="336" t="s">
         <v>55</v>
       </c>
-      <c r="U63" s="327"/>
-      <c r="V63" s="327"/>
-      <c r="W63" s="327"/>
-      <c r="X63" s="327"/>
-      <c r="Y63" s="327"/>
-      <c r="Z63" s="327"/>
-      <c r="AA63" s="327"/>
+      <c r="U63" s="333"/>
+      <c r="V63" s="333"/>
+      <c r="W63" s="333"/>
+      <c r="X63" s="333"/>
+      <c r="Y63" s="333"/>
+      <c r="Z63" s="333"/>
+      <c r="AA63" s="333"/>
       <c r="AB63" s="70"/>
       <c r="AC63" s="40"/>
     </row>
@@ -61354,12 +61342,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="J12:O12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="K21:R21"/>
     <mergeCell ref="B63:I63"/>
     <mergeCell ref="K63:R63"/>
     <mergeCell ref="T63:AA63"/>
@@ -61370,6 +61352,12 @@
     <mergeCell ref="B49:I49"/>
     <mergeCell ref="K49:R49"/>
     <mergeCell ref="T49:AA49"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="J12:O12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="K21:R21"/>
   </mergeCells>
   <conditionalFormatting sqref="C51:I55">
     <cfRule type="expression" dxfId="2" priority="3">

</xml_diff>

<commit_message>
thêm người phụ thuộc
</commit_message>
<xml_diff>
--- a/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
+++ b/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonzai/dev/odoo 19/odoo/my_custom_addons/dl_salary_kpi/static/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59E82727-6651-2D45-969D-DB19574CB68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3BEA9F-AB2F-1348-8C43-650487FA27F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="17760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2473,70 +2473,41 @@
     <xf numFmtId="14" fontId="59" fillId="0" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="61" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="59" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="14" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="55" fillId="14" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2581,10 +2552,22 @@
     <xf numFmtId="0" fontId="66" fillId="25" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2593,32 +2576,72 @@
     <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="14" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="55" fillId="14" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="7" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2633,29 +2656,6 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="61" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="59" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="32">
@@ -3488,11 +3488,11 @@
       <c r="AL1" s="213"/>
       <c r="AM1" s="213"/>
       <c r="AN1" s="213"/>
-      <c r="AO1" s="323"/>
-      <c r="AP1" s="323"/>
-      <c r="AQ1" s="323"/>
-      <c r="AR1" s="323"/>
-      <c r="AS1" s="323"/>
+      <c r="AO1" s="278"/>
+      <c r="AP1" s="278"/>
+      <c r="AQ1" s="278"/>
+      <c r="AR1" s="278"/>
+      <c r="AS1" s="278"/>
       <c r="AT1" s="120"/>
       <c r="AU1" s="120"/>
       <c r="AV1" s="120"/>
@@ -3902,44 +3902,44 @@
       <c r="E4" s="234" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="336"/>
+      <c r="F4" s="275"/>
       <c r="G4" s="237"/>
       <c r="H4" s="108"/>
       <c r="I4" s="274"/>
-      <c r="J4" s="316" t="s">
+      <c r="J4" s="279" t="s">
         <v>68</v>
       </c>
-      <c r="K4" s="316"/>
-      <c r="L4" s="337">
+      <c r="K4" s="279"/>
+      <c r="L4" s="276">
         <v>3</v>
       </c>
-      <c r="M4" s="337"/>
-      <c r="N4" s="338" t="s">
+      <c r="M4" s="276"/>
+      <c r="N4" s="277" t="s">
         <v>69</v>
       </c>
-      <c r="O4" s="338"/>
-      <c r="P4" s="338">
+      <c r="O4" s="277"/>
+      <c r="P4" s="277">
         <v>2026</v>
       </c>
-      <c r="Q4" s="338"/>
+      <c r="Q4" s="277"/>
       <c r="R4" s="109"/>
-      <c r="S4" s="316"/>
-      <c r="T4" s="316"/>
-      <c r="U4" s="316"/>
+      <c r="S4" s="279"/>
+      <c r="T4" s="279"/>
+      <c r="U4" s="279"/>
       <c r="V4" s="109"/>
-      <c r="W4" s="316"/>
-      <c r="X4" s="316"/>
-      <c r="Y4" s="316"/>
-      <c r="Z4" s="316"/>
-      <c r="AA4" s="316"/>
-      <c r="AB4" s="316"/>
-      <c r="AC4" s="316"/>
-      <c r="AD4" s="316"/>
+      <c r="W4" s="279"/>
+      <c r="X4" s="279"/>
+      <c r="Y4" s="279"/>
+      <c r="Z4" s="279"/>
+      <c r="AA4" s="279"/>
+      <c r="AB4" s="279"/>
+      <c r="AC4" s="279"/>
+      <c r="AD4" s="279"/>
       <c r="AE4" s="109"/>
       <c r="AF4" s="110"/>
-      <c r="AG4" s="316"/>
-      <c r="AH4" s="316"/>
-      <c r="AI4" s="316"/>
+      <c r="AG4" s="279"/>
+      <c r="AH4" s="279"/>
+      <c r="AI4" s="279"/>
       <c r="AJ4" s="109"/>
       <c r="AK4" s="109"/>
       <c r="AL4" s="109"/>
@@ -3950,42 +3950,42 @@
       <c r="AQ4" s="113"/>
       <c r="AR4" s="223"/>
       <c r="AS4" s="232"/>
-      <c r="AT4" s="316" t="s">
+      <c r="AT4" s="279" t="s">
         <v>68</v>
       </c>
-      <c r="AU4" s="316"/>
-      <c r="AV4" s="337">
+      <c r="AU4" s="279"/>
+      <c r="AV4" s="276">
         <f>L4</f>
         <v>3</v>
       </c>
-      <c r="AW4" s="337"/>
-      <c r="AX4" s="338" t="s">
+      <c r="AW4" s="276"/>
+      <c r="AX4" s="277" t="s">
         <v>69</v>
       </c>
-      <c r="AY4" s="338"/>
-      <c r="AZ4" s="338">
+      <c r="AY4" s="277"/>
+      <c r="AZ4" s="277">
         <f>P4</f>
         <v>2026</v>
       </c>
-      <c r="BA4" s="338"/>
+      <c r="BA4" s="277"/>
       <c r="BB4" s="109"/>
-      <c r="BC4" s="316"/>
-      <c r="BD4" s="316"/>
-      <c r="BE4" s="316"/>
+      <c r="BC4" s="279"/>
+      <c r="BD4" s="279"/>
+      <c r="BE4" s="279"/>
       <c r="BF4" s="109"/>
-      <c r="BG4" s="316"/>
-      <c r="BH4" s="316"/>
-      <c r="BI4" s="316"/>
-      <c r="BJ4" s="316"/>
-      <c r="BK4" s="316"/>
-      <c r="BL4" s="316"/>
-      <c r="BM4" s="316"/>
-      <c r="BN4" s="316"/>
+      <c r="BG4" s="279"/>
+      <c r="BH4" s="279"/>
+      <c r="BI4" s="279"/>
+      <c r="BJ4" s="279"/>
+      <c r="BK4" s="279"/>
+      <c r="BL4" s="279"/>
+      <c r="BM4" s="279"/>
+      <c r="BN4" s="279"/>
       <c r="BO4" s="109"/>
       <c r="BP4" s="110"/>
-      <c r="BQ4" s="316"/>
-      <c r="BR4" s="316"/>
-      <c r="BS4" s="316"/>
+      <c r="BQ4" s="279"/>
+      <c r="BR4" s="279"/>
+      <c r="BS4" s="279"/>
       <c r="BT4" s="114"/>
       <c r="BU4" s="114" t="str">
         <f>IF(WEEKDAY(BU5,1)=1,"CN","")</f>
@@ -4069,31 +4069,31 @@
       <c r="EV4" s="246"/>
     </row>
     <row r="5" spans="1:154" s="184" customFormat="1" ht="92.25" customHeight="1">
-      <c r="A5" s="315" t="s">
+      <c r="A5" s="280" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="276" t="s">
+      <c r="B5" s="281" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="315" t="s">
+      <c r="C5" s="280" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="320" t="s">
+      <c r="D5" s="282" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="321" t="s">
+      <c r="E5" s="283" t="s">
         <v>122</v>
       </c>
-      <c r="F5" s="315" t="s">
+      <c r="F5" s="280" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="315" t="s">
+      <c r="G5" s="280" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="315" t="s">
+      <c r="H5" s="280" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="317" t="s">
+      <c r="I5" s="285" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="175">
@@ -4220,19 +4220,19 @@
         <f t="shared" si="0"/>
         <v>46112</v>
       </c>
-      <c r="AO5" s="318" t="s">
+      <c r="AO5" s="286" t="s">
         <v>82</v>
       </c>
-      <c r="AP5" s="318" t="s">
+      <c r="AP5" s="286" t="s">
         <v>83</v>
       </c>
-      <c r="AQ5" s="318" t="s">
+      <c r="AQ5" s="286" t="s">
         <v>84</v>
       </c>
-      <c r="AR5" s="319" t="s">
+      <c r="AR5" s="287" t="s">
         <v>5</v>
       </c>
-      <c r="AS5" s="319" t="s">
+      <c r="AS5" s="287" t="s">
         <v>6</v>
       </c>
       <c r="AT5" s="179">
@@ -4359,46 +4359,46 @@
         <f t="shared" si="1"/>
         <v>46112</v>
       </c>
-      <c r="BY5" s="293" t="s">
+      <c r="BY5" s="311" t="s">
         <v>86</v>
       </c>
-      <c r="BZ5" s="293" t="s">
+      <c r="BZ5" s="311" t="s">
         <v>87</v>
       </c>
-      <c r="CA5" s="293" t="s">
+      <c r="CA5" s="311" t="s">
         <v>88</v>
       </c>
-      <c r="CB5" s="293" t="s">
+      <c r="CB5" s="311" t="s">
         <v>89</v>
       </c>
-      <c r="CC5" s="293" t="s">
+      <c r="CC5" s="311" t="s">
         <v>90</v>
       </c>
-      <c r="CD5" s="293" t="s">
+      <c r="CD5" s="311" t="s">
         <v>91</v>
       </c>
-      <c r="CE5" s="293" t="s">
+      <c r="CE5" s="311" t="s">
         <v>92</v>
       </c>
-      <c r="CF5" s="295" t="s">
+      <c r="CF5" s="310" t="s">
         <v>19</v>
       </c>
-      <c r="CG5" s="295"/>
-      <c r="CH5" s="295"/>
-      <c r="CI5" s="295"/>
-      <c r="CJ5" s="295"/>
-      <c r="CK5" s="295"/>
-      <c r="CL5" s="295"/>
-      <c r="CM5" s="295"/>
-      <c r="CN5" s="295"/>
-      <c r="CO5" s="295"/>
-      <c r="CP5" s="295"/>
-      <c r="CQ5" s="279" t="s">
+      <c r="CG5" s="310"/>
+      <c r="CH5" s="310"/>
+      <c r="CI5" s="310"/>
+      <c r="CJ5" s="310"/>
+      <c r="CK5" s="310"/>
+      <c r="CL5" s="310"/>
+      <c r="CM5" s="310"/>
+      <c r="CN5" s="310"/>
+      <c r="CO5" s="310"/>
+      <c r="CP5" s="310"/>
+      <c r="CQ5" s="316" t="s">
         <v>59</v>
       </c>
-      <c r="CR5" s="280"/>
-      <c r="CS5" s="281"/>
-      <c r="CT5" s="286" t="s">
+      <c r="CR5" s="317"/>
+      <c r="CS5" s="318"/>
+      <c r="CT5" s="323" t="s">
         <v>60</v>
       </c>
       <c r="CU5" s="260" t="s">
@@ -4421,117 +4421,117 @@
       <c r="DF5" s="258" t="s">
         <v>130</v>
       </c>
-      <c r="DG5" s="282" t="s">
+      <c r="DG5" s="319" t="s">
         <v>119</v>
       </c>
-      <c r="DH5" s="287" t="s">
+      <c r="DH5" s="324" t="s">
         <v>113</v>
       </c>
-      <c r="DI5" s="284" t="s">
+      <c r="DI5" s="321" t="s">
         <v>81</v>
       </c>
-      <c r="DJ5" s="285"/>
-      <c r="DK5" s="288" t="s">
+      <c r="DJ5" s="322"/>
+      <c r="DK5" s="305" t="s">
         <v>61</v>
       </c>
-      <c r="DL5" s="296" t="s">
+      <c r="DL5" s="313" t="s">
         <v>8</v>
       </c>
-      <c r="DM5" s="289" t="s">
+      <c r="DM5" s="306" t="s">
         <v>71</v>
       </c>
-      <c r="DN5" s="289"/>
-      <c r="DO5" s="289"/>
-      <c r="DP5" s="289"/>
-      <c r="DQ5" s="289"/>
-      <c r="DR5" s="289"/>
-      <c r="DS5" s="290" t="s">
+      <c r="DN5" s="306"/>
+      <c r="DO5" s="306"/>
+      <c r="DP5" s="306"/>
+      <c r="DQ5" s="306"/>
+      <c r="DR5" s="306"/>
+      <c r="DS5" s="325" t="s">
         <v>12</v>
       </c>
-      <c r="DT5" s="289" t="s">
+      <c r="DT5" s="306" t="s">
         <v>128</v>
       </c>
-      <c r="DU5" s="276" t="s">
+      <c r="DU5" s="281" t="s">
         <v>13</v>
       </c>
-      <c r="DV5" s="277" t="s">
+      <c r="DV5" s="314" t="s">
         <v>64</v>
       </c>
-      <c r="DW5" s="278"/>
-      <c r="DX5" s="277"/>
-      <c r="DY5" s="311" t="s">
+      <c r="DW5" s="315"/>
+      <c r="DX5" s="314"/>
+      <c r="DY5" s="303" t="s">
         <v>63</v>
       </c>
-      <c r="DZ5" s="311"/>
-      <c r="EA5" s="311"/>
-      <c r="EB5" s="311"/>
-      <c r="EC5" s="312" t="s">
+      <c r="DZ5" s="303"/>
+      <c r="EA5" s="303"/>
+      <c r="EB5" s="303"/>
+      <c r="EC5" s="304" t="s">
         <v>131</v>
       </c>
-      <c r="ED5" s="289" t="s">
+      <c r="ED5" s="306" t="s">
         <v>7</v>
       </c>
-      <c r="EE5" s="291" t="s">
+      <c r="EE5" s="307" t="s">
         <v>65</v>
       </c>
-      <c r="EF5" s="291"/>
-      <c r="EG5" s="291" t="s">
+      <c r="EF5" s="307"/>
+      <c r="EG5" s="307" t="s">
         <v>66</v>
       </c>
-      <c r="EH5" s="291" t="s">
+      <c r="EH5" s="307" t="s">
         <v>67</v>
       </c>
-      <c r="EI5" s="291" t="s">
+      <c r="EI5" s="307" t="s">
         <v>72</v>
       </c>
-      <c r="EJ5" s="292" t="s">
+      <c r="EJ5" s="326" t="s">
         <v>78</v>
       </c>
-      <c r="EK5" s="292" t="s">
+      <c r="EK5" s="326" t="s">
         <v>80</v>
       </c>
-      <c r="EL5" s="292" t="s">
+      <c r="EL5" s="326" t="s">
         <v>79</v>
       </c>
-      <c r="EM5" s="301" t="s">
+      <c r="EM5" s="292" t="s">
         <v>127</v>
       </c>
-      <c r="EN5" s="303"/>
-      <c r="EO5" s="305" t="s">
+      <c r="EN5" s="294"/>
+      <c r="EO5" s="296" t="s">
         <v>132</v>
       </c>
-      <c r="EP5" s="307" t="s">
+      <c r="EP5" s="298" t="s">
         <v>118</v>
       </c>
-      <c r="EQ5" s="309" t="s">
+      <c r="EQ5" s="300" t="s">
         <v>133</v>
       </c>
-      <c r="ER5" s="275" t="s">
+      <c r="ER5" s="302" t="s">
         <v>125</v>
       </c>
-      <c r="ES5" s="275" t="s">
+      <c r="ES5" s="302" t="s">
         <v>124</v>
       </c>
-      <c r="ET5" s="313" t="s">
+      <c r="ET5" s="308" t="s">
         <v>120</v>
       </c>
-      <c r="EU5" s="297" t="s">
+      <c r="EU5" s="288" t="s">
         <v>123</v>
       </c>
-      <c r="EV5" s="299" t="s">
+      <c r="EV5" s="290" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:154" s="206" customFormat="1" ht="148.5" customHeight="1">
-      <c r="A6" s="315"/>
-      <c r="B6" s="276"/>
-      <c r="C6" s="315"/>
-      <c r="D6" s="320"/>
-      <c r="E6" s="322"/>
-      <c r="F6" s="315"/>
-      <c r="G6" s="315"/>
-      <c r="H6" s="315"/>
-      <c r="I6" s="317"/>
+      <c r="A6" s="280"/>
+      <c r="B6" s="281"/>
+      <c r="C6" s="280"/>
+      <c r="D6" s="282"/>
+      <c r="E6" s="284"/>
+      <c r="F6" s="280"/>
+      <c r="G6" s="280"/>
+      <c r="H6" s="280"/>
+      <c r="I6" s="285"/>
       <c r="J6" s="185" t="str">
         <f t="shared" ref="J6:AN6" si="2">IF(WEEKDAY(J5)=1,"CN",WEEKDAY(J5))</f>
         <v>CN</v>
@@ -4656,11 +4656,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AO6" s="318"/>
-      <c r="AP6" s="318"/>
-      <c r="AQ6" s="318"/>
-      <c r="AR6" s="319"/>
-      <c r="AS6" s="319"/>
+      <c r="AO6" s="286"/>
+      <c r="AP6" s="286"/>
+      <c r="AQ6" s="286"/>
+      <c r="AR6" s="287"/>
+      <c r="AS6" s="287"/>
       <c r="AT6" s="187" t="str">
         <f>+J6</f>
         <v>CN</v>
@@ -4785,13 +4785,13 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="BY6" s="294"/>
-      <c r="BZ6" s="294"/>
-      <c r="CA6" s="294"/>
-      <c r="CB6" s="294"/>
-      <c r="CC6" s="294"/>
-      <c r="CD6" s="294"/>
-      <c r="CE6" s="294"/>
+      <c r="BY6" s="312"/>
+      <c r="BZ6" s="312"/>
+      <c r="CA6" s="312"/>
+      <c r="CB6" s="312"/>
+      <c r="CC6" s="312"/>
+      <c r="CD6" s="312"/>
+      <c r="CE6" s="312"/>
       <c r="CF6" s="189" t="s">
         <v>93</v>
       </c>
@@ -4834,7 +4834,7 @@
       <c r="CS6" s="181" t="s">
         <v>58</v>
       </c>
-      <c r="CT6" s="286"/>
+      <c r="CT6" s="323"/>
       <c r="CU6" s="189" t="s">
         <v>104</v>
       </c>
@@ -4871,16 +4871,16 @@
       <c r="DF6" s="259" t="s">
         <v>134</v>
       </c>
-      <c r="DG6" s="283"/>
-      <c r="DH6" s="287"/>
+      <c r="DG6" s="320"/>
+      <c r="DH6" s="324"/>
       <c r="DI6" s="152" t="s">
         <v>14</v>
       </c>
       <c r="DJ6" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="DK6" s="288"/>
-      <c r="DL6" s="296"/>
+      <c r="DK6" s="305"/>
+      <c r="DL6" s="313"/>
       <c r="DM6" s="181" t="s">
         <v>9</v>
       </c>
@@ -4899,9 +4899,9 @@
       <c r="DR6" s="181" t="s">
         <v>116</v>
       </c>
-      <c r="DS6" s="290"/>
-      <c r="DT6" s="289"/>
-      <c r="DU6" s="276"/>
+      <c r="DS6" s="325"/>
+      <c r="DT6" s="306"/>
+      <c r="DU6" s="281"/>
       <c r="DV6" s="204">
         <v>0.17499999999999999</v>
       </c>
@@ -4923,176 +4923,176 @@
       <c r="EB6" s="152" t="s">
         <v>62</v>
       </c>
-      <c r="EC6" s="288"/>
-      <c r="ED6" s="289"/>
+      <c r="EC6" s="305"/>
+      <c r="ED6" s="306"/>
       <c r="EE6" s="183" t="s">
         <v>73</v>
       </c>
       <c r="EF6" s="183" t="s">
         <v>74</v>
       </c>
-      <c r="EG6" s="291"/>
-      <c r="EH6" s="291"/>
-      <c r="EI6" s="291"/>
-      <c r="EJ6" s="292"/>
-      <c r="EK6" s="292"/>
-      <c r="EL6" s="292"/>
-      <c r="EM6" s="302"/>
-      <c r="EN6" s="304"/>
-      <c r="EO6" s="306"/>
-      <c r="EP6" s="308"/>
-      <c r="EQ6" s="310"/>
-      <c r="ER6" s="275"/>
-      <c r="ES6" s="275"/>
-      <c r="ET6" s="314"/>
-      <c r="EU6" s="298"/>
-      <c r="EV6" s="299"/>
+      <c r="EG6" s="307"/>
+      <c r="EH6" s="307"/>
+      <c r="EI6" s="307"/>
+      <c r="EJ6" s="326"/>
+      <c r="EK6" s="326"/>
+      <c r="EL6" s="326"/>
+      <c r="EM6" s="293"/>
+      <c r="EN6" s="295"/>
+      <c r="EO6" s="297"/>
+      <c r="EP6" s="299"/>
+      <c r="EQ6" s="301"/>
+      <c r="ER6" s="302"/>
+      <c r="ES6" s="302"/>
+      <c r="ET6" s="309"/>
+      <c r="EU6" s="289"/>
+      <c r="EV6" s="290"/>
     </row>
     <row r="7" spans="1:154" s="106" customFormat="1" ht="87.75" customHeight="1">
-      <c r="A7" s="300" t="s">
+      <c r="A7" s="291" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="300"/>
-      <c r="C7" s="300"/>
-      <c r="D7" s="300"/>
-      <c r="E7" s="300"/>
-      <c r="F7" s="300"/>
-      <c r="G7" s="300"/>
-      <c r="H7" s="300"/>
-      <c r="I7" s="300"/>
-      <c r="J7" s="300"/>
-      <c r="K7" s="300"/>
-      <c r="L7" s="300"/>
-      <c r="M7" s="300"/>
-      <c r="N7" s="300"/>
-      <c r="O7" s="300"/>
-      <c r="P7" s="300"/>
-      <c r="Q7" s="300"/>
-      <c r="R7" s="300"/>
-      <c r="S7" s="300"/>
-      <c r="T7" s="300"/>
-      <c r="U7" s="300"/>
-      <c r="V7" s="300"/>
-      <c r="W7" s="300"/>
-      <c r="X7" s="300"/>
-      <c r="Y7" s="300"/>
-      <c r="Z7" s="300"/>
-      <c r="AA7" s="300"/>
-      <c r="AB7" s="300"/>
-      <c r="AC7" s="300"/>
-      <c r="AD7" s="300"/>
-      <c r="AE7" s="300"/>
-      <c r="AF7" s="300"/>
-      <c r="AG7" s="300"/>
-      <c r="AH7" s="300"/>
-      <c r="AI7" s="300"/>
-      <c r="AJ7" s="300"/>
-      <c r="AK7" s="300"/>
-      <c r="AL7" s="300"/>
-      <c r="AM7" s="300"/>
-      <c r="AN7" s="300"/>
-      <c r="AO7" s="300"/>
-      <c r="AP7" s="300"/>
-      <c r="AQ7" s="300"/>
-      <c r="AR7" s="300"/>
-      <c r="AS7" s="300"/>
-      <c r="AT7" s="300"/>
-      <c r="AU7" s="300"/>
-      <c r="AV7" s="300"/>
-      <c r="AW7" s="300"/>
-      <c r="AX7" s="300"/>
-      <c r="AY7" s="300"/>
-      <c r="AZ7" s="300"/>
-      <c r="BA7" s="300"/>
-      <c r="BB7" s="300"/>
-      <c r="BC7" s="300"/>
-      <c r="BD7" s="300"/>
-      <c r="BE7" s="300"/>
-      <c r="BF7" s="300"/>
-      <c r="BG7" s="300"/>
-      <c r="BH7" s="300"/>
-      <c r="BI7" s="300"/>
-      <c r="BJ7" s="300"/>
-      <c r="BK7" s="300"/>
-      <c r="BL7" s="300"/>
-      <c r="BM7" s="300"/>
-      <c r="BN7" s="300"/>
-      <c r="BO7" s="300"/>
-      <c r="BP7" s="300"/>
-      <c r="BQ7" s="300"/>
-      <c r="BR7" s="300"/>
-      <c r="BS7" s="300"/>
-      <c r="BT7" s="300"/>
-      <c r="BU7" s="300"/>
-      <c r="BV7" s="300"/>
-      <c r="BW7" s="300"/>
-      <c r="BX7" s="300"/>
-      <c r="BY7" s="300"/>
-      <c r="BZ7" s="300"/>
-      <c r="CA7" s="300"/>
-      <c r="CB7" s="300"/>
-      <c r="CC7" s="300"/>
-      <c r="CD7" s="300"/>
-      <c r="CE7" s="300"/>
-      <c r="CF7" s="300"/>
-      <c r="CG7" s="300"/>
-      <c r="CH7" s="300"/>
-      <c r="CI7" s="300"/>
-      <c r="CJ7" s="300"/>
-      <c r="CK7" s="300"/>
-      <c r="CL7" s="300"/>
-      <c r="CM7" s="300"/>
-      <c r="CN7" s="300"/>
-      <c r="CO7" s="300"/>
-      <c r="CP7" s="300"/>
-      <c r="CQ7" s="300"/>
-      <c r="CR7" s="300"/>
-      <c r="CS7" s="300"/>
-      <c r="CT7" s="300"/>
-      <c r="CU7" s="300"/>
-      <c r="CV7" s="300"/>
-      <c r="CW7" s="300"/>
-      <c r="CX7" s="300"/>
-      <c r="CY7" s="300"/>
-      <c r="CZ7" s="300"/>
-      <c r="DA7" s="300"/>
-      <c r="DB7" s="300"/>
-      <c r="DC7" s="300"/>
-      <c r="DD7" s="300"/>
-      <c r="DE7" s="300"/>
-      <c r="DF7" s="300"/>
-      <c r="DG7" s="300"/>
-      <c r="DH7" s="300"/>
-      <c r="DI7" s="300"/>
-      <c r="DJ7" s="300"/>
-      <c r="DK7" s="300"/>
-      <c r="DL7" s="300"/>
-      <c r="DM7" s="300"/>
-      <c r="DN7" s="300"/>
-      <c r="DO7" s="300"/>
-      <c r="DP7" s="300"/>
-      <c r="DQ7" s="300"/>
-      <c r="DR7" s="300"/>
-      <c r="DS7" s="300"/>
-      <c r="DT7" s="300"/>
-      <c r="DU7" s="300"/>
-      <c r="DV7" s="300"/>
-      <c r="DW7" s="300"/>
-      <c r="DX7" s="300"/>
-      <c r="DY7" s="300"/>
-      <c r="DZ7" s="300"/>
-      <c r="EA7" s="300"/>
-      <c r="EB7" s="300"/>
-      <c r="EC7" s="300"/>
-      <c r="ED7" s="300"/>
-      <c r="EE7" s="300"/>
-      <c r="EF7" s="300"/>
-      <c r="EG7" s="300"/>
-      <c r="EH7" s="300"/>
-      <c r="EI7" s="300"/>
-      <c r="EJ7" s="300"/>
-      <c r="EK7" s="300"/>
-      <c r="EL7" s="300"/>
+      <c r="B7" s="291"/>
+      <c r="C7" s="291"/>
+      <c r="D7" s="291"/>
+      <c r="E7" s="291"/>
+      <c r="F7" s="291"/>
+      <c r="G7" s="291"/>
+      <c r="H7" s="291"/>
+      <c r="I7" s="291"/>
+      <c r="J7" s="291"/>
+      <c r="K7" s="291"/>
+      <c r="L7" s="291"/>
+      <c r="M7" s="291"/>
+      <c r="N7" s="291"/>
+      <c r="O7" s="291"/>
+      <c r="P7" s="291"/>
+      <c r="Q7" s="291"/>
+      <c r="R7" s="291"/>
+      <c r="S7" s="291"/>
+      <c r="T7" s="291"/>
+      <c r="U7" s="291"/>
+      <c r="V7" s="291"/>
+      <c r="W7" s="291"/>
+      <c r="X7" s="291"/>
+      <c r="Y7" s="291"/>
+      <c r="Z7" s="291"/>
+      <c r="AA7" s="291"/>
+      <c r="AB7" s="291"/>
+      <c r="AC7" s="291"/>
+      <c r="AD7" s="291"/>
+      <c r="AE7" s="291"/>
+      <c r="AF7" s="291"/>
+      <c r="AG7" s="291"/>
+      <c r="AH7" s="291"/>
+      <c r="AI7" s="291"/>
+      <c r="AJ7" s="291"/>
+      <c r="AK7" s="291"/>
+      <c r="AL7" s="291"/>
+      <c r="AM7" s="291"/>
+      <c r="AN7" s="291"/>
+      <c r="AO7" s="291"/>
+      <c r="AP7" s="291"/>
+      <c r="AQ7" s="291"/>
+      <c r="AR7" s="291"/>
+      <c r="AS7" s="291"/>
+      <c r="AT7" s="291"/>
+      <c r="AU7" s="291"/>
+      <c r="AV7" s="291"/>
+      <c r="AW7" s="291"/>
+      <c r="AX7" s="291"/>
+      <c r="AY7" s="291"/>
+      <c r="AZ7" s="291"/>
+      <c r="BA7" s="291"/>
+      <c r="BB7" s="291"/>
+      <c r="BC7" s="291"/>
+      <c r="BD7" s="291"/>
+      <c r="BE7" s="291"/>
+      <c r="BF7" s="291"/>
+      <c r="BG7" s="291"/>
+      <c r="BH7" s="291"/>
+      <c r="BI7" s="291"/>
+      <c r="BJ7" s="291"/>
+      <c r="BK7" s="291"/>
+      <c r="BL7" s="291"/>
+      <c r="BM7" s="291"/>
+      <c r="BN7" s="291"/>
+      <c r="BO7" s="291"/>
+      <c r="BP7" s="291"/>
+      <c r="BQ7" s="291"/>
+      <c r="BR7" s="291"/>
+      <c r="BS7" s="291"/>
+      <c r="BT7" s="291"/>
+      <c r="BU7" s="291"/>
+      <c r="BV7" s="291"/>
+      <c r="BW7" s="291"/>
+      <c r="BX7" s="291"/>
+      <c r="BY7" s="291"/>
+      <c r="BZ7" s="291"/>
+      <c r="CA7" s="291"/>
+      <c r="CB7" s="291"/>
+      <c r="CC7" s="291"/>
+      <c r="CD7" s="291"/>
+      <c r="CE7" s="291"/>
+      <c r="CF7" s="291"/>
+      <c r="CG7" s="291"/>
+      <c r="CH7" s="291"/>
+      <c r="CI7" s="291"/>
+      <c r="CJ7" s="291"/>
+      <c r="CK7" s="291"/>
+      <c r="CL7" s="291"/>
+      <c r="CM7" s="291"/>
+      <c r="CN7" s="291"/>
+      <c r="CO7" s="291"/>
+      <c r="CP7" s="291"/>
+      <c r="CQ7" s="291"/>
+      <c r="CR7" s="291"/>
+      <c r="CS7" s="291"/>
+      <c r="CT7" s="291"/>
+      <c r="CU7" s="291"/>
+      <c r="CV7" s="291"/>
+      <c r="CW7" s="291"/>
+      <c r="CX7" s="291"/>
+      <c r="CY7" s="291"/>
+      <c r="CZ7" s="291"/>
+      <c r="DA7" s="291"/>
+      <c r="DB7" s="291"/>
+      <c r="DC7" s="291"/>
+      <c r="DD7" s="291"/>
+      <c r="DE7" s="291"/>
+      <c r="DF7" s="291"/>
+      <c r="DG7" s="291"/>
+      <c r="DH7" s="291"/>
+      <c r="DI7" s="291"/>
+      <c r="DJ7" s="291"/>
+      <c r="DK7" s="291"/>
+      <c r="DL7" s="291"/>
+      <c r="DM7" s="291"/>
+      <c r="DN7" s="291"/>
+      <c r="DO7" s="291"/>
+      <c r="DP7" s="291"/>
+      <c r="DQ7" s="291"/>
+      <c r="DR7" s="291"/>
+      <c r="DS7" s="291"/>
+      <c r="DT7" s="291"/>
+      <c r="DU7" s="291"/>
+      <c r="DV7" s="291"/>
+      <c r="DW7" s="291"/>
+      <c r="DX7" s="291"/>
+      <c r="DY7" s="291"/>
+      <c r="DZ7" s="291"/>
+      <c r="EA7" s="291"/>
+      <c r="EB7" s="291"/>
+      <c r="EC7" s="291"/>
+      <c r="ED7" s="291"/>
+      <c r="EE7" s="291"/>
+      <c r="EF7" s="291"/>
+      <c r="EG7" s="291"/>
+      <c r="EH7" s="291"/>
+      <c r="EI7" s="291"/>
+      <c r="EJ7" s="291"/>
+      <c r="EK7" s="291"/>
+      <c r="EL7" s="291"/>
       <c r="EM7" s="247"/>
       <c r="EN7" s="247"/>
       <c r="EO7" s="247"/>
@@ -5452,21 +5452,21 @@
         <f t="shared" ref="DO8" si="76">DL8*1%</f>
         <v>0</v>
       </c>
-      <c r="DP8" s="159" t="e">
-        <f t="shared" ref="DP8" ca="1" si="77">EI8</f>
-        <v>#REF!</v>
-      </c>
-      <c r="DQ8" s="159" t="e">
-        <f t="shared" ref="DQ8" ca="1" si="78">+SUM(DM8:DP8)</f>
-        <v>#REF!</v>
+      <c r="DP8" s="159">
+        <f t="shared" ref="DP8" si="77">EI8</f>
+        <v>0</v>
+      </c>
+      <c r="DQ8" s="159">
+        <f t="shared" ref="DQ8" si="78">+SUM(DM8:DP8)</f>
+        <v>0</v>
       </c>
       <c r="DR8" s="159">
         <f t="shared" ref="DR8" si="79">SUM(DM8:DO8)</f>
         <v>0</v>
       </c>
-      <c r="DS8" s="160" t="e">
-        <f t="shared" ref="DS8" ca="1" si="80">ROUNDDOWN(DK8-DQ8,-3)</f>
-        <v>#REF!</v>
+      <c r="DS8" s="160">
+        <f t="shared" ref="DS8" si="80">ROUNDDOWN(DK8-DQ8,-3)</f>
+        <v>0</v>
       </c>
       <c r="DT8" s="157"/>
       <c r="DU8" s="159">
@@ -5509,25 +5509,24 @@
         <f>+DK8-DJ8+EC8</f>
         <v>0</v>
       </c>
-      <c r="EE8" s="166" t="e">
-        <f ca="1">15500000+DR8+EF8*6200000</f>
-        <v>#REF!</v>
-      </c>
-      <c r="EF8" s="161" t="e">
-        <f ca="1">SUMIF(INDIRECT("'QTTTNCN'!$D$7:$D$500"),B8,INDIRECT("'QTTTNCN'!$S$7:$S$500"))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="EG8" s="173" t="e">
-        <f t="shared" ref="EG8" ca="1" si="82">+ED8-EE8</f>
-        <v>#REF!</v>
-      </c>
-      <c r="EH8" s="173" t="e">
-        <f t="shared" ref="EH8" ca="1" si="83">IF(EG8&lt;=5000000,EG8*5/100,IF(EG8&lt;=10000000,EG8*10/100-250000,IF(EG8&lt;=18000000,EG8*15/100-750000,IF(EG8&lt;=32000000,EG8*20/100-1650000,IF(EG8&lt;=52000000,EG8*25/100-3250000,IF(EG8&lt;=80000000,EG8*30%-5850000,EG8*35%-9850000))))))</f>
-        <v>#REF!</v>
-      </c>
-      <c r="EI8" s="173" t="e">
-        <f t="shared" ref="EI8" ca="1" si="84">+IF(EH8&lt;0,0,EH8)</f>
-        <v>#REF!</v>
+      <c r="EE8" s="166">
+        <f>15500000+DR8+EF8*6200000</f>
+        <v>15500000</v>
+      </c>
+      <c r="EF8" s="161">
+        <v>0</v>
+      </c>
+      <c r="EG8" s="173">
+        <f t="shared" ref="EG8" si="82">+ED8-EE8</f>
+        <v>-15500000</v>
+      </c>
+      <c r="EH8" s="173">
+        <f t="shared" ref="EH8" si="83">IF(EG8&lt;=5000000,EG8*5/100,IF(EG8&lt;=10000000,EG8*10/100-250000,IF(EG8&lt;=18000000,EG8*15/100-750000,IF(EG8&lt;=32000000,EG8*20/100-1650000,IF(EG8&lt;=52000000,EG8*25/100-3250000,IF(EG8&lt;=80000000,EG8*30%-5850000,EG8*35%-9850000))))))</f>
+        <v>-775000</v>
+      </c>
+      <c r="EI8" s="173">
+        <f t="shared" ref="EI8" si="84">+IF(EH8&lt;0,0,EH8)</f>
+        <v>0</v>
       </c>
       <c r="EJ8" s="166" t="b">
         <f>+IF(AQ8&gt;0,I8/26)</f>
@@ -5543,13 +5542,13 @@
       </c>
       <c r="EM8" s="166"/>
       <c r="EN8" s="166"/>
-      <c r="EO8" s="166" t="e">
-        <f ca="1">DS8+EC8+EN8</f>
-        <v>#REF!</v>
-      </c>
-      <c r="EP8" s="224" t="e">
-        <f t="shared" ref="EP8" ca="1" si="86">EM8-EO8</f>
-        <v>#REF!</v>
+      <c r="EO8" s="166">
+        <f>DS8+EC8+EN8</f>
+        <v>0</v>
+      </c>
+      <c r="EP8" s="224">
+        <f t="shared" ref="EP8" si="86">EM8-EO8</f>
+        <v>0</v>
       </c>
       <c r="EQ8" s="225">
         <f t="shared" ref="EQ8" si="87">EM8</f>
@@ -27870,33 +27869,20 @@
   </sheetData>
   <autoFilter ref="A6:EX8" xr:uid="{00000000-0001-0000-0900-000000000000}"/>
   <mergeCells count="68">
-    <mergeCell ref="AO1:AS1"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="S4:U4"/>
-    <mergeCell ref="W4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AD4"/>
-    <mergeCell ref="AG4:AI4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="BG4:BI4"/>
-    <mergeCell ref="AT4:AU4"/>
-    <mergeCell ref="AO5:AO6"/>
-    <mergeCell ref="AP5:AP6"/>
-    <mergeCell ref="AQ5:AQ6"/>
-    <mergeCell ref="AR5:AR6"/>
-    <mergeCell ref="AS5:AS6"/>
-    <mergeCell ref="BJ4:BK4"/>
-    <mergeCell ref="BL4:BN4"/>
-    <mergeCell ref="BQ4:BS4"/>
-    <mergeCell ref="BC4:BE4"/>
-    <mergeCell ref="EU5:EU6"/>
+    <mergeCell ref="EI5:EI6"/>
+    <mergeCell ref="EJ5:EJ6"/>
+    <mergeCell ref="EK5:EK6"/>
+    <mergeCell ref="EL5:EL6"/>
+    <mergeCell ref="EH5:EH6"/>
+    <mergeCell ref="DV5:DX5"/>
+    <mergeCell ref="CQ5:CS5"/>
+    <mergeCell ref="DG5:DG6"/>
+    <mergeCell ref="DI5:DJ5"/>
+    <mergeCell ref="CT5:CT6"/>
+    <mergeCell ref="DH5:DH6"/>
+    <mergeCell ref="DK5:DK6"/>
+    <mergeCell ref="DM5:DR5"/>
+    <mergeCell ref="DS5:DS6"/>
     <mergeCell ref="EV5:EV6"/>
     <mergeCell ref="A7:EL7"/>
     <mergeCell ref="EM5:EM6"/>
@@ -27913,6 +27899,11 @@
     <mergeCell ref="ET5:ET6"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="CF5:CP5"/>
+    <mergeCell ref="BJ4:BK4"/>
+    <mergeCell ref="BL4:BN4"/>
+    <mergeCell ref="BQ4:BS4"/>
+    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="EU5:EU6"/>
     <mergeCell ref="CD5:CD6"/>
     <mergeCell ref="CE5:CE6"/>
     <mergeCell ref="DL5:DL6"/>
@@ -27924,20 +27915,28 @@
     <mergeCell ref="CC5:CC6"/>
     <mergeCell ref="ES5:ES6"/>
     <mergeCell ref="DU5:DU6"/>
-    <mergeCell ref="DV5:DX5"/>
-    <mergeCell ref="CQ5:CS5"/>
-    <mergeCell ref="DG5:DG6"/>
-    <mergeCell ref="DI5:DJ5"/>
-    <mergeCell ref="CT5:CT6"/>
-    <mergeCell ref="DH5:DH6"/>
-    <mergeCell ref="DK5:DK6"/>
-    <mergeCell ref="DM5:DR5"/>
-    <mergeCell ref="DS5:DS6"/>
-    <mergeCell ref="EI5:EI6"/>
-    <mergeCell ref="EJ5:EJ6"/>
-    <mergeCell ref="EK5:EK6"/>
-    <mergeCell ref="EL5:EL6"/>
-    <mergeCell ref="EH5:EH6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="BG4:BI4"/>
+    <mergeCell ref="AT4:AU4"/>
+    <mergeCell ref="AO5:AO6"/>
+    <mergeCell ref="AP5:AP6"/>
+    <mergeCell ref="AQ5:AQ6"/>
+    <mergeCell ref="AR5:AR6"/>
+    <mergeCell ref="AS5:AS6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="AO1:AS1"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="S4:U4"/>
+    <mergeCell ref="W4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="AG4:AI4"/>
   </mergeCells>
   <conditionalFormatting sqref="A5 A8:B8">
     <cfRule type="duplicateValues" dxfId="20" priority="20879"/>
@@ -28594,11 +28593,11 @@
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
       <c r="H8" s="20"/>
-      <c r="I8" s="324">
+      <c r="I8" s="333">
         <v>2026</v>
       </c>
-      <c r="J8" s="325"/>
-      <c r="K8" s="325"/>
+      <c r="J8" s="334"/>
+      <c r="K8" s="334"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="21" t="s">
@@ -28623,13 +28622,13 @@
     <row r="9" spans="1:29" ht="15.75" customHeight="1" thickBot="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="326" t="s">
+      <c r="C9" s="335" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="327"/>
-      <c r="E9" s="327"/>
-      <c r="F9" s="327"/>
-      <c r="G9" s="327"/>
+      <c r="D9" s="336"/>
+      <c r="E9" s="336"/>
+      <c r="F9" s="336"/>
+      <c r="G9" s="336"/>
       <c r="H9" s="20"/>
       <c r="I9" s="24"/>
       <c r="J9" s="24"/>
@@ -28725,19 +28724,19 @@
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
-      <c r="J12" s="328" t="s">
+      <c r="J12" s="337" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="327"/>
-      <c r="L12" s="327"/>
-      <c r="M12" s="327"/>
-      <c r="N12" s="327"/>
-      <c r="O12" s="327"/>
-      <c r="P12" s="329">
+      <c r="K12" s="336"/>
+      <c r="L12" s="336"/>
+      <c r="M12" s="336"/>
+      <c r="N12" s="336"/>
+      <c r="O12" s="336"/>
+      <c r="P12" s="338">
         <f>I8</f>
         <v>2026</v>
       </c>
-      <c r="Q12" s="327"/>
+      <c r="Q12" s="336"/>
       <c r="R12" s="33"/>
       <c r="S12" s="34"/>
       <c r="T12" s="34"/>
@@ -29001,38 +29000,38 @@
     </row>
     <row r="21" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A21" s="39"/>
-      <c r="B21" s="330" t="s">
+      <c r="B21" s="332" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="331"/>
-      <c r="D21" s="331"/>
-      <c r="E21" s="331"/>
-      <c r="F21" s="331"/>
-      <c r="G21" s="331"/>
-      <c r="H21" s="331"/>
-      <c r="I21" s="331"/>
+      <c r="C21" s="328"/>
+      <c r="D21" s="328"/>
+      <c r="E21" s="328"/>
+      <c r="F21" s="328"/>
+      <c r="G21" s="328"/>
+      <c r="H21" s="328"/>
+      <c r="I21" s="328"/>
       <c r="J21" s="40"/>
-      <c r="K21" s="332" t="s">
+      <c r="K21" s="329" t="s">
         <v>37</v>
       </c>
-      <c r="L21" s="331"/>
-      <c r="M21" s="331"/>
-      <c r="N21" s="331"/>
-      <c r="O21" s="331"/>
-      <c r="P21" s="331"/>
-      <c r="Q21" s="331"/>
-      <c r="R21" s="331"/>
+      <c r="L21" s="328"/>
+      <c r="M21" s="328"/>
+      <c r="N21" s="328"/>
+      <c r="O21" s="328"/>
+      <c r="P21" s="328"/>
+      <c r="Q21" s="328"/>
+      <c r="R21" s="328"/>
       <c r="S21" s="40"/>
-      <c r="T21" s="333" t="s">
+      <c r="T21" s="327" t="s">
         <v>38</v>
       </c>
-      <c r="U21" s="331"/>
-      <c r="V21" s="331"/>
-      <c r="W21" s="331"/>
-      <c r="X21" s="331"/>
-      <c r="Y21" s="331"/>
-      <c r="Z21" s="331"/>
-      <c r="AA21" s="331"/>
+      <c r="U21" s="328"/>
+      <c r="V21" s="328"/>
+      <c r="W21" s="328"/>
+      <c r="X21" s="328"/>
+      <c r="Y21" s="328"/>
+      <c r="Z21" s="328"/>
+      <c r="AA21" s="328"/>
       <c r="AB21" s="41"/>
       <c r="AC21" s="42"/>
     </row>
@@ -29932,38 +29931,38 @@
     </row>
     <row r="35" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="334" t="s">
+      <c r="B35" s="330" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="331"/>
-      <c r="D35" s="331"/>
-      <c r="E35" s="331"/>
-      <c r="F35" s="331"/>
-      <c r="G35" s="331"/>
-      <c r="H35" s="331"/>
-      <c r="I35" s="331"/>
+      <c r="C35" s="328"/>
+      <c r="D35" s="328"/>
+      <c r="E35" s="328"/>
+      <c r="F35" s="328"/>
+      <c r="G35" s="328"/>
+      <c r="H35" s="328"/>
+      <c r="I35" s="328"/>
       <c r="J35" s="40"/>
-      <c r="K35" s="335" t="s">
+      <c r="K35" s="331" t="s">
         <v>48</v>
       </c>
-      <c r="L35" s="331"/>
-      <c r="M35" s="331"/>
-      <c r="N35" s="331"/>
-      <c r="O35" s="331"/>
-      <c r="P35" s="331"/>
-      <c r="Q35" s="331"/>
-      <c r="R35" s="331"/>
+      <c r="L35" s="328"/>
+      <c r="M35" s="328"/>
+      <c r="N35" s="328"/>
+      <c r="O35" s="328"/>
+      <c r="P35" s="328"/>
+      <c r="Q35" s="328"/>
+      <c r="R35" s="328"/>
       <c r="S35" s="40"/>
-      <c r="T35" s="332" t="s">
+      <c r="T35" s="329" t="s">
         <v>49</v>
       </c>
-      <c r="U35" s="331"/>
-      <c r="V35" s="331"/>
-      <c r="W35" s="331"/>
-      <c r="X35" s="331"/>
-      <c r="Y35" s="331"/>
-      <c r="Z35" s="331"/>
-      <c r="AA35" s="331"/>
+      <c r="U35" s="328"/>
+      <c r="V35" s="328"/>
+      <c r="W35" s="328"/>
+      <c r="X35" s="328"/>
+      <c r="Y35" s="328"/>
+      <c r="Z35" s="328"/>
+      <c r="AA35" s="328"/>
       <c r="AB35" s="70"/>
       <c r="AC35" s="40"/>
     </row>
@@ -30852,38 +30851,38 @@
     </row>
     <row r="49" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A49" s="69"/>
-      <c r="B49" s="332" t="s">
+      <c r="B49" s="329" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="331"/>
-      <c r="D49" s="331"/>
-      <c r="E49" s="331"/>
-      <c r="F49" s="331"/>
-      <c r="G49" s="331"/>
-      <c r="H49" s="331"/>
-      <c r="I49" s="331"/>
+      <c r="C49" s="328"/>
+      <c r="D49" s="328"/>
+      <c r="E49" s="328"/>
+      <c r="F49" s="328"/>
+      <c r="G49" s="328"/>
+      <c r="H49" s="328"/>
+      <c r="I49" s="328"/>
       <c r="J49" s="40"/>
-      <c r="K49" s="334" t="s">
+      <c r="K49" s="330" t="s">
         <v>51</v>
       </c>
-      <c r="L49" s="331"/>
-      <c r="M49" s="331"/>
-      <c r="N49" s="331"/>
-      <c r="O49" s="331"/>
-      <c r="P49" s="331"/>
-      <c r="Q49" s="331"/>
-      <c r="R49" s="331"/>
+      <c r="L49" s="328"/>
+      <c r="M49" s="328"/>
+      <c r="N49" s="328"/>
+      <c r="O49" s="328"/>
+      <c r="P49" s="328"/>
+      <c r="Q49" s="328"/>
+      <c r="R49" s="328"/>
       <c r="S49" s="40"/>
-      <c r="T49" s="330" t="s">
+      <c r="T49" s="332" t="s">
         <v>52</v>
       </c>
-      <c r="U49" s="331"/>
-      <c r="V49" s="331"/>
-      <c r="W49" s="331"/>
-      <c r="X49" s="331"/>
-      <c r="Y49" s="331"/>
-      <c r="Z49" s="331"/>
-      <c r="AA49" s="331"/>
+      <c r="U49" s="328"/>
+      <c r="V49" s="328"/>
+      <c r="W49" s="328"/>
+      <c r="X49" s="328"/>
+      <c r="Y49" s="328"/>
+      <c r="Z49" s="328"/>
+      <c r="AA49" s="328"/>
       <c r="AB49" s="70"/>
       <c r="AC49" s="40"/>
     </row>
@@ -31772,38 +31771,38 @@
     </row>
     <row r="63" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A63" s="69"/>
-      <c r="B63" s="333" t="s">
+      <c r="B63" s="327" t="s">
         <v>53</v>
       </c>
-      <c r="C63" s="331"/>
-      <c r="D63" s="331"/>
-      <c r="E63" s="331"/>
-      <c r="F63" s="331"/>
-      <c r="G63" s="331"/>
-      <c r="H63" s="331"/>
-      <c r="I63" s="331"/>
+      <c r="C63" s="328"/>
+      <c r="D63" s="328"/>
+      <c r="E63" s="328"/>
+      <c r="F63" s="328"/>
+      <c r="G63" s="328"/>
+      <c r="H63" s="328"/>
+      <c r="I63" s="328"/>
       <c r="J63" s="40"/>
-      <c r="K63" s="332" t="s">
+      <c r="K63" s="329" t="s">
         <v>54</v>
       </c>
-      <c r="L63" s="331"/>
-      <c r="M63" s="331"/>
-      <c r="N63" s="331"/>
-      <c r="O63" s="331"/>
-      <c r="P63" s="331"/>
-      <c r="Q63" s="331"/>
-      <c r="R63" s="331"/>
+      <c r="L63" s="328"/>
+      <c r="M63" s="328"/>
+      <c r="N63" s="328"/>
+      <c r="O63" s="328"/>
+      <c r="P63" s="328"/>
+      <c r="Q63" s="328"/>
+      <c r="R63" s="328"/>
       <c r="S63" s="40"/>
-      <c r="T63" s="334" t="s">
+      <c r="T63" s="330" t="s">
         <v>55</v>
       </c>
-      <c r="U63" s="331"/>
-      <c r="V63" s="331"/>
-      <c r="W63" s="331"/>
-      <c r="X63" s="331"/>
-      <c r="Y63" s="331"/>
-      <c r="Z63" s="331"/>
-      <c r="AA63" s="331"/>
+      <c r="U63" s="328"/>
+      <c r="V63" s="328"/>
+      <c r="W63" s="328"/>
+      <c r="X63" s="328"/>
+      <c r="Y63" s="328"/>
+      <c r="Z63" s="328"/>
+      <c r="AA63" s="328"/>
       <c r="AB63" s="70"/>
       <c r="AC63" s="40"/>
     </row>
@@ -61338,6 +61337,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="J12:O12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="K21:R21"/>
     <mergeCell ref="B63:I63"/>
     <mergeCell ref="K63:R63"/>
     <mergeCell ref="T63:AA63"/>
@@ -61348,12 +61353,6 @@
     <mergeCell ref="B49:I49"/>
     <mergeCell ref="K49:R49"/>
     <mergeCell ref="T49:AA49"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="J12:O12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="K21:R21"/>
   </mergeCells>
   <conditionalFormatting sqref="C51:I55">
     <cfRule type="expression" dxfId="2" priority="3">

</xml_diff>

<commit_message>
đã tính được lương ngoài để chuyển sang tính KPI
</commit_message>
<xml_diff>
--- a/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
+++ b/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonzai/dev/odoo 19/odoo/my_custom_addons/dl_salary_kpi/static/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3BEA9F-AB2F-1348-8C43-650487FA27F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D7C67FC-5C33-254E-9970-BAC1D7DCC46E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="17760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2516,6 +2516,21 @@
     <xf numFmtId="171" fontId="55" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2552,9 +2567,6 @@
     <xf numFmtId="0" fontId="66" fillId="25" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2567,9 +2579,6 @@
     <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2578,15 +2587,6 @@
     </xf>
     <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3362,11 +3362,11 @@
     <col min="1" max="1" width="17.796875" style="95" customWidth="1"/>
     <col min="2" max="2" width="30.19921875" style="95" customWidth="1"/>
     <col min="3" max="3" width="45.796875" style="94" customWidth="1"/>
-    <col min="4" max="4" width="24.3984375" style="100" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="5" width="29.19921875" style="100" customWidth="1" outlineLevel="1"/>
-    <col min="6" max="6" width="15.3984375" style="100" customWidth="1" outlineLevel="1"/>
-    <col min="7" max="7" width="31.796875" style="221" customWidth="1" outlineLevel="1"/>
-    <col min="8" max="8" width="13.796875" style="95" customWidth="1"/>
+    <col min="4" max="4" width="24.3984375" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="29.19921875" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="15.3984375" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="31.796875" style="221" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="13.796875" style="95" customWidth="1" collapsed="1"/>
     <col min="9" max="9" width="25.19921875" style="101" customWidth="1"/>
     <col min="10" max="40" width="11.796875" style="1" customWidth="1" outlineLevel="1"/>
     <col min="41" max="43" width="15.796875" style="92" customWidth="1" outlineLevel="1"/>
@@ -3443,7 +3443,7 @@
     <col min="152" max="152" width="41.796875" style="255" hidden="1" customWidth="1"/>
     <col min="153" max="153" width="34.796875" style="94" hidden="1" customWidth="1"/>
     <col min="154" max="154" width="28.59765625" style="94" hidden="1" customWidth="1"/>
-    <col min="155" max="156" width="0" style="94" hidden="1" customWidth="1"/>
+    <col min="155" max="156" width="9.19921875" style="94" customWidth="1"/>
     <col min="157" max="16384" width="9.19921875" style="94"/>
   </cols>
   <sheetData>
@@ -4359,40 +4359,40 @@
         <f t="shared" si="1"/>
         <v>46112</v>
       </c>
-      <c r="BY5" s="311" t="s">
+      <c r="BY5" s="290" t="s">
         <v>86</v>
       </c>
-      <c r="BZ5" s="311" t="s">
+      <c r="BZ5" s="290" t="s">
         <v>87</v>
       </c>
-      <c r="CA5" s="311" t="s">
+      <c r="CA5" s="290" t="s">
         <v>88</v>
       </c>
-      <c r="CB5" s="311" t="s">
+      <c r="CB5" s="290" t="s">
         <v>89</v>
       </c>
-      <c r="CC5" s="311" t="s">
+      <c r="CC5" s="290" t="s">
         <v>90</v>
       </c>
-      <c r="CD5" s="311" t="s">
+      <c r="CD5" s="290" t="s">
         <v>91</v>
       </c>
-      <c r="CE5" s="311" t="s">
+      <c r="CE5" s="290" t="s">
         <v>92</v>
       </c>
-      <c r="CF5" s="310" t="s">
+      <c r="CF5" s="313" t="s">
         <v>19</v>
       </c>
-      <c r="CG5" s="310"/>
-      <c r="CH5" s="310"/>
-      <c r="CI5" s="310"/>
-      <c r="CJ5" s="310"/>
-      <c r="CK5" s="310"/>
-      <c r="CL5" s="310"/>
-      <c r="CM5" s="310"/>
-      <c r="CN5" s="310"/>
-      <c r="CO5" s="310"/>
-      <c r="CP5" s="310"/>
+      <c r="CG5" s="313"/>
+      <c r="CH5" s="313"/>
+      <c r="CI5" s="313"/>
+      <c r="CJ5" s="313"/>
+      <c r="CK5" s="313"/>
+      <c r="CL5" s="313"/>
+      <c r="CM5" s="313"/>
+      <c r="CN5" s="313"/>
+      <c r="CO5" s="313"/>
+      <c r="CP5" s="313"/>
       <c r="CQ5" s="316" t="s">
         <v>59</v>
       </c>
@@ -4431,24 +4431,24 @@
         <v>81</v>
       </c>
       <c r="DJ5" s="322"/>
-      <c r="DK5" s="305" t="s">
+      <c r="DK5" s="309" t="s">
         <v>61</v>
       </c>
-      <c r="DL5" s="313" t="s">
+      <c r="DL5" s="292" t="s">
         <v>8</v>
       </c>
-      <c r="DM5" s="306" t="s">
+      <c r="DM5" s="310" t="s">
         <v>71</v>
       </c>
-      <c r="DN5" s="306"/>
-      <c r="DO5" s="306"/>
-      <c r="DP5" s="306"/>
-      <c r="DQ5" s="306"/>
-      <c r="DR5" s="306"/>
+      <c r="DN5" s="310"/>
+      <c r="DO5" s="310"/>
+      <c r="DP5" s="310"/>
+      <c r="DQ5" s="310"/>
+      <c r="DR5" s="310"/>
       <c r="DS5" s="325" t="s">
         <v>12</v>
       </c>
-      <c r="DT5" s="306" t="s">
+      <c r="DT5" s="310" t="s">
         <v>128</v>
       </c>
       <c r="DU5" s="281" t="s">
@@ -4459,29 +4459,29 @@
       </c>
       <c r="DW5" s="315"/>
       <c r="DX5" s="314"/>
-      <c r="DY5" s="303" t="s">
+      <c r="DY5" s="307" t="s">
         <v>63</v>
       </c>
-      <c r="DZ5" s="303"/>
-      <c r="EA5" s="303"/>
-      <c r="EB5" s="303"/>
-      <c r="EC5" s="304" t="s">
+      <c r="DZ5" s="307"/>
+      <c r="EA5" s="307"/>
+      <c r="EB5" s="307"/>
+      <c r="EC5" s="308" t="s">
         <v>131</v>
       </c>
-      <c r="ED5" s="306" t="s">
+      <c r="ED5" s="310" t="s">
         <v>7</v>
       </c>
-      <c r="EE5" s="307" t="s">
+      <c r="EE5" s="293" t="s">
         <v>65</v>
       </c>
-      <c r="EF5" s="307"/>
-      <c r="EG5" s="307" t="s">
+      <c r="EF5" s="293"/>
+      <c r="EG5" s="293" t="s">
         <v>66</v>
       </c>
-      <c r="EH5" s="307" t="s">
+      <c r="EH5" s="293" t="s">
         <v>67</v>
       </c>
-      <c r="EI5" s="307" t="s">
+      <c r="EI5" s="293" t="s">
         <v>72</v>
       </c>
       <c r="EJ5" s="326" t="s">
@@ -4493,32 +4493,32 @@
       <c r="EL5" s="326" t="s">
         <v>79</v>
       </c>
-      <c r="EM5" s="292" t="s">
+      <c r="EM5" s="297" t="s">
         <v>127</v>
       </c>
-      <c r="EN5" s="294"/>
-      <c r="EO5" s="296" t="s">
+      <c r="EN5" s="299"/>
+      <c r="EO5" s="301" t="s">
         <v>132</v>
       </c>
-      <c r="EP5" s="298" t="s">
+      <c r="EP5" s="303" t="s">
         <v>118</v>
       </c>
-      <c r="EQ5" s="300" t="s">
+      <c r="EQ5" s="305" t="s">
         <v>133</v>
       </c>
-      <c r="ER5" s="302" t="s">
+      <c r="ER5" s="294" t="s">
         <v>125</v>
       </c>
-      <c r="ES5" s="302" t="s">
+      <c r="ES5" s="294" t="s">
         <v>124</v>
       </c>
-      <c r="ET5" s="308" t="s">
+      <c r="ET5" s="311" t="s">
         <v>120</v>
       </c>
       <c r="EU5" s="288" t="s">
         <v>123</v>
       </c>
-      <c r="EV5" s="290" t="s">
+      <c r="EV5" s="295" t="s">
         <v>121</v>
       </c>
     </row>
@@ -4785,13 +4785,13 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="BY6" s="312"/>
-      <c r="BZ6" s="312"/>
-      <c r="CA6" s="312"/>
-      <c r="CB6" s="312"/>
-      <c r="CC6" s="312"/>
-      <c r="CD6" s="312"/>
-      <c r="CE6" s="312"/>
+      <c r="BY6" s="291"/>
+      <c r="BZ6" s="291"/>
+      <c r="CA6" s="291"/>
+      <c r="CB6" s="291"/>
+      <c r="CC6" s="291"/>
+      <c r="CD6" s="291"/>
+      <c r="CE6" s="291"/>
       <c r="CF6" s="189" t="s">
         <v>93</v>
       </c>
@@ -4879,8 +4879,8 @@
       <c r="DJ6" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="DK6" s="305"/>
-      <c r="DL6" s="313"/>
+      <c r="DK6" s="309"/>
+      <c r="DL6" s="292"/>
       <c r="DM6" s="181" t="s">
         <v>9</v>
       </c>
@@ -4900,7 +4900,7 @@
         <v>116</v>
       </c>
       <c r="DS6" s="325"/>
-      <c r="DT6" s="306"/>
+      <c r="DT6" s="310"/>
       <c r="DU6" s="281"/>
       <c r="DV6" s="204">
         <v>0.17499999999999999</v>
@@ -4923,176 +4923,176 @@
       <c r="EB6" s="152" t="s">
         <v>62</v>
       </c>
-      <c r="EC6" s="305"/>
-      <c r="ED6" s="306"/>
+      <c r="EC6" s="309"/>
+      <c r="ED6" s="310"/>
       <c r="EE6" s="183" t="s">
         <v>73</v>
       </c>
       <c r="EF6" s="183" t="s">
         <v>74</v>
       </c>
-      <c r="EG6" s="307"/>
-      <c r="EH6" s="307"/>
-      <c r="EI6" s="307"/>
+      <c r="EG6" s="293"/>
+      <c r="EH6" s="293"/>
+      <c r="EI6" s="293"/>
       <c r="EJ6" s="326"/>
       <c r="EK6" s="326"/>
       <c r="EL6" s="326"/>
-      <c r="EM6" s="293"/>
-      <c r="EN6" s="295"/>
-      <c r="EO6" s="297"/>
-      <c r="EP6" s="299"/>
-      <c r="EQ6" s="301"/>
-      <c r="ER6" s="302"/>
-      <c r="ES6" s="302"/>
-      <c r="ET6" s="309"/>
+      <c r="EM6" s="298"/>
+      <c r="EN6" s="300"/>
+      <c r="EO6" s="302"/>
+      <c r="EP6" s="304"/>
+      <c r="EQ6" s="306"/>
+      <c r="ER6" s="294"/>
+      <c r="ES6" s="294"/>
+      <c r="ET6" s="312"/>
       <c r="EU6" s="289"/>
-      <c r="EV6" s="290"/>
+      <c r="EV6" s="295"/>
     </row>
     <row r="7" spans="1:154" s="106" customFormat="1" ht="87.75" customHeight="1">
-      <c r="A7" s="291" t="s">
+      <c r="A7" s="296" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="291"/>
-      <c r="C7" s="291"/>
-      <c r="D7" s="291"/>
-      <c r="E7" s="291"/>
-      <c r="F7" s="291"/>
-      <c r="G7" s="291"/>
-      <c r="H7" s="291"/>
-      <c r="I7" s="291"/>
-      <c r="J7" s="291"/>
-      <c r="K7" s="291"/>
-      <c r="L7" s="291"/>
-      <c r="M7" s="291"/>
-      <c r="N7" s="291"/>
-      <c r="O7" s="291"/>
-      <c r="P7" s="291"/>
-      <c r="Q7" s="291"/>
-      <c r="R7" s="291"/>
-      <c r="S7" s="291"/>
-      <c r="T7" s="291"/>
-      <c r="U7" s="291"/>
-      <c r="V7" s="291"/>
-      <c r="W7" s="291"/>
-      <c r="X7" s="291"/>
-      <c r="Y7" s="291"/>
-      <c r="Z7" s="291"/>
-      <c r="AA7" s="291"/>
-      <c r="AB7" s="291"/>
-      <c r="AC7" s="291"/>
-      <c r="AD7" s="291"/>
-      <c r="AE7" s="291"/>
-      <c r="AF7" s="291"/>
-      <c r="AG7" s="291"/>
-      <c r="AH7" s="291"/>
-      <c r="AI7" s="291"/>
-      <c r="AJ7" s="291"/>
-      <c r="AK7" s="291"/>
-      <c r="AL7" s="291"/>
-      <c r="AM7" s="291"/>
-      <c r="AN7" s="291"/>
-      <c r="AO7" s="291"/>
-      <c r="AP7" s="291"/>
-      <c r="AQ7" s="291"/>
-      <c r="AR7" s="291"/>
-      <c r="AS7" s="291"/>
-      <c r="AT7" s="291"/>
-      <c r="AU7" s="291"/>
-      <c r="AV7" s="291"/>
-      <c r="AW7" s="291"/>
-      <c r="AX7" s="291"/>
-      <c r="AY7" s="291"/>
-      <c r="AZ7" s="291"/>
-      <c r="BA7" s="291"/>
-      <c r="BB7" s="291"/>
-      <c r="BC7" s="291"/>
-      <c r="BD7" s="291"/>
-      <c r="BE7" s="291"/>
-      <c r="BF7" s="291"/>
-      <c r="BG7" s="291"/>
-      <c r="BH7" s="291"/>
-      <c r="BI7" s="291"/>
-      <c r="BJ7" s="291"/>
-      <c r="BK7" s="291"/>
-      <c r="BL7" s="291"/>
-      <c r="BM7" s="291"/>
-      <c r="BN7" s="291"/>
-      <c r="BO7" s="291"/>
-      <c r="BP7" s="291"/>
-      <c r="BQ7" s="291"/>
-      <c r="BR7" s="291"/>
-      <c r="BS7" s="291"/>
-      <c r="BT7" s="291"/>
-      <c r="BU7" s="291"/>
-      <c r="BV7" s="291"/>
-      <c r="BW7" s="291"/>
-      <c r="BX7" s="291"/>
-      <c r="BY7" s="291"/>
-      <c r="BZ7" s="291"/>
-      <c r="CA7" s="291"/>
-      <c r="CB7" s="291"/>
-      <c r="CC7" s="291"/>
-      <c r="CD7" s="291"/>
-      <c r="CE7" s="291"/>
-      <c r="CF7" s="291"/>
-      <c r="CG7" s="291"/>
-      <c r="CH7" s="291"/>
-      <c r="CI7" s="291"/>
-      <c r="CJ7" s="291"/>
-      <c r="CK7" s="291"/>
-      <c r="CL7" s="291"/>
-      <c r="CM7" s="291"/>
-      <c r="CN7" s="291"/>
-      <c r="CO7" s="291"/>
-      <c r="CP7" s="291"/>
-      <c r="CQ7" s="291"/>
-      <c r="CR7" s="291"/>
-      <c r="CS7" s="291"/>
-      <c r="CT7" s="291"/>
-      <c r="CU7" s="291"/>
-      <c r="CV7" s="291"/>
-      <c r="CW7" s="291"/>
-      <c r="CX7" s="291"/>
-      <c r="CY7" s="291"/>
-      <c r="CZ7" s="291"/>
-      <c r="DA7" s="291"/>
-      <c r="DB7" s="291"/>
-      <c r="DC7" s="291"/>
-      <c r="DD7" s="291"/>
-      <c r="DE7" s="291"/>
-      <c r="DF7" s="291"/>
-      <c r="DG7" s="291"/>
-      <c r="DH7" s="291"/>
-      <c r="DI7" s="291"/>
-      <c r="DJ7" s="291"/>
-      <c r="DK7" s="291"/>
-      <c r="DL7" s="291"/>
-      <c r="DM7" s="291"/>
-      <c r="DN7" s="291"/>
-      <c r="DO7" s="291"/>
-      <c r="DP7" s="291"/>
-      <c r="DQ7" s="291"/>
-      <c r="DR7" s="291"/>
-      <c r="DS7" s="291"/>
-      <c r="DT7" s="291"/>
-      <c r="DU7" s="291"/>
-      <c r="DV7" s="291"/>
-      <c r="DW7" s="291"/>
-      <c r="DX7" s="291"/>
-      <c r="DY7" s="291"/>
-      <c r="DZ7" s="291"/>
-      <c r="EA7" s="291"/>
-      <c r="EB7" s="291"/>
-      <c r="EC7" s="291"/>
-      <c r="ED7" s="291"/>
-      <c r="EE7" s="291"/>
-      <c r="EF7" s="291"/>
-      <c r="EG7" s="291"/>
-      <c r="EH7" s="291"/>
-      <c r="EI7" s="291"/>
-      <c r="EJ7" s="291"/>
-      <c r="EK7" s="291"/>
-      <c r="EL7" s="291"/>
+      <c r="B7" s="296"/>
+      <c r="C7" s="296"/>
+      <c r="D7" s="296"/>
+      <c r="E7" s="296"/>
+      <c r="F7" s="296"/>
+      <c r="G7" s="296"/>
+      <c r="H7" s="296"/>
+      <c r="I7" s="296"/>
+      <c r="J7" s="296"/>
+      <c r="K7" s="296"/>
+      <c r="L7" s="296"/>
+      <c r="M7" s="296"/>
+      <c r="N7" s="296"/>
+      <c r="O7" s="296"/>
+      <c r="P7" s="296"/>
+      <c r="Q7" s="296"/>
+      <c r="R7" s="296"/>
+      <c r="S7" s="296"/>
+      <c r="T7" s="296"/>
+      <c r="U7" s="296"/>
+      <c r="V7" s="296"/>
+      <c r="W7" s="296"/>
+      <c r="X7" s="296"/>
+      <c r="Y7" s="296"/>
+      <c r="Z7" s="296"/>
+      <c r="AA7" s="296"/>
+      <c r="AB7" s="296"/>
+      <c r="AC7" s="296"/>
+      <c r="AD7" s="296"/>
+      <c r="AE7" s="296"/>
+      <c r="AF7" s="296"/>
+      <c r="AG7" s="296"/>
+      <c r="AH7" s="296"/>
+      <c r="AI7" s="296"/>
+      <c r="AJ7" s="296"/>
+      <c r="AK7" s="296"/>
+      <c r="AL7" s="296"/>
+      <c r="AM7" s="296"/>
+      <c r="AN7" s="296"/>
+      <c r="AO7" s="296"/>
+      <c r="AP7" s="296"/>
+      <c r="AQ7" s="296"/>
+      <c r="AR7" s="296"/>
+      <c r="AS7" s="296"/>
+      <c r="AT7" s="296"/>
+      <c r="AU7" s="296"/>
+      <c r="AV7" s="296"/>
+      <c r="AW7" s="296"/>
+      <c r="AX7" s="296"/>
+      <c r="AY7" s="296"/>
+      <c r="AZ7" s="296"/>
+      <c r="BA7" s="296"/>
+      <c r="BB7" s="296"/>
+      <c r="BC7" s="296"/>
+      <c r="BD7" s="296"/>
+      <c r="BE7" s="296"/>
+      <c r="BF7" s="296"/>
+      <c r="BG7" s="296"/>
+      <c r="BH7" s="296"/>
+      <c r="BI7" s="296"/>
+      <c r="BJ7" s="296"/>
+      <c r="BK7" s="296"/>
+      <c r="BL7" s="296"/>
+      <c r="BM7" s="296"/>
+      <c r="BN7" s="296"/>
+      <c r="BO7" s="296"/>
+      <c r="BP7" s="296"/>
+      <c r="BQ7" s="296"/>
+      <c r="BR7" s="296"/>
+      <c r="BS7" s="296"/>
+      <c r="BT7" s="296"/>
+      <c r="BU7" s="296"/>
+      <c r="BV7" s="296"/>
+      <c r="BW7" s="296"/>
+      <c r="BX7" s="296"/>
+      <c r="BY7" s="296"/>
+      <c r="BZ7" s="296"/>
+      <c r="CA7" s="296"/>
+      <c r="CB7" s="296"/>
+      <c r="CC7" s="296"/>
+      <c r="CD7" s="296"/>
+      <c r="CE7" s="296"/>
+      <c r="CF7" s="296"/>
+      <c r="CG7" s="296"/>
+      <c r="CH7" s="296"/>
+      <c r="CI7" s="296"/>
+      <c r="CJ7" s="296"/>
+      <c r="CK7" s="296"/>
+      <c r="CL7" s="296"/>
+      <c r="CM7" s="296"/>
+      <c r="CN7" s="296"/>
+      <c r="CO7" s="296"/>
+      <c r="CP7" s="296"/>
+      <c r="CQ7" s="296"/>
+      <c r="CR7" s="296"/>
+      <c r="CS7" s="296"/>
+      <c r="CT7" s="296"/>
+      <c r="CU7" s="296"/>
+      <c r="CV7" s="296"/>
+      <c r="CW7" s="296"/>
+      <c r="CX7" s="296"/>
+      <c r="CY7" s="296"/>
+      <c r="CZ7" s="296"/>
+      <c r="DA7" s="296"/>
+      <c r="DB7" s="296"/>
+      <c r="DC7" s="296"/>
+      <c r="DD7" s="296"/>
+      <c r="DE7" s="296"/>
+      <c r="DF7" s="296"/>
+      <c r="DG7" s="296"/>
+      <c r="DH7" s="296"/>
+      <c r="DI7" s="296"/>
+      <c r="DJ7" s="296"/>
+      <c r="DK7" s="296"/>
+      <c r="DL7" s="296"/>
+      <c r="DM7" s="296"/>
+      <c r="DN7" s="296"/>
+      <c r="DO7" s="296"/>
+      <c r="DP7" s="296"/>
+      <c r="DQ7" s="296"/>
+      <c r="DR7" s="296"/>
+      <c r="DS7" s="296"/>
+      <c r="DT7" s="296"/>
+      <c r="DU7" s="296"/>
+      <c r="DV7" s="296"/>
+      <c r="DW7" s="296"/>
+      <c r="DX7" s="296"/>
+      <c r="DY7" s="296"/>
+      <c r="DZ7" s="296"/>
+      <c r="EA7" s="296"/>
+      <c r="EB7" s="296"/>
+      <c r="EC7" s="296"/>
+      <c r="ED7" s="296"/>
+      <c r="EE7" s="296"/>
+      <c r="EF7" s="296"/>
+      <c r="EG7" s="296"/>
+      <c r="EH7" s="296"/>
+      <c r="EI7" s="296"/>
+      <c r="EJ7" s="296"/>
+      <c r="EK7" s="296"/>
+      <c r="EL7" s="296"/>
       <c r="EM7" s="247"/>
       <c r="EN7" s="247"/>
       <c r="EO7" s="247"/>
@@ -5465,7 +5465,7 @@
         <v>0</v>
       </c>
       <c r="DS8" s="160">
-        <f t="shared" ref="DS8" si="80">ROUNDDOWN(DK8-DQ8,-3)</f>
+        <f>IF(ROUNDDOWN(DK8-DQ8,-3) &lt;0, 0,ROUNDDOWN(DK8-DQ8,-3) )</f>
         <v>0</v>
       </c>
       <c r="DT8" s="157"/>
@@ -5498,7 +5498,7 @@
         <v>0</v>
       </c>
       <c r="EB8" s="174">
-        <f t="shared" ref="EB8" si="81">DY8+DZ8+EA8</f>
+        <f t="shared" ref="EB8" si="80">DY8+DZ8+EA8</f>
         <v>0</v>
       </c>
       <c r="EC8" s="165">
@@ -5510,22 +5510,22 @@
         <v>0</v>
       </c>
       <c r="EE8" s="166">
-        <f>15500000+DR8+EF8*6200000</f>
+        <f>15500000+EF8*6200000</f>
         <v>15500000</v>
       </c>
       <c r="EF8" s="161">
         <v>0</v>
       </c>
       <c r="EG8" s="173">
-        <f t="shared" ref="EG8" si="82">+ED8-EE8</f>
+        <f>+ED8-EE8-DR8</f>
         <v>-15500000</v>
       </c>
       <c r="EH8" s="173">
-        <f t="shared" ref="EH8" si="83">IF(EG8&lt;=5000000,EG8*5/100,IF(EG8&lt;=10000000,EG8*10/100-250000,IF(EG8&lt;=18000000,EG8*15/100-750000,IF(EG8&lt;=32000000,EG8*20/100-1650000,IF(EG8&lt;=52000000,EG8*25/100-3250000,IF(EG8&lt;=80000000,EG8*30%-5850000,EG8*35%-9850000))))))</f>
+        <f>IF(EG8&lt;=10000000,EG8*5/100,IF(EG8&lt;=30000000,EG8*10/100-500000,IF(EG8&lt;=60000000,EG8*20/100-3500000,IF(EG8&lt;=100000000,EG8*30/100-9500000,EG8*35%-14500000))))</f>
         <v>-775000</v>
       </c>
       <c r="EI8" s="173">
-        <f t="shared" ref="EI8" si="84">+IF(EH8&lt;0,0,EH8)</f>
+        <f t="shared" ref="EI8" si="81">+IF(EH8&lt;0,0,EH8)</f>
         <v>0</v>
       </c>
       <c r="EJ8" s="166" t="b">
@@ -5537,7 +5537,7 @@
         <v>0</v>
       </c>
       <c r="EL8" s="166">
-        <f t="shared" ref="EL8" si="85">+EJ8+EK8</f>
+        <f>+EJ8+EK8</f>
         <v>0</v>
       </c>
       <c r="EM8" s="166"/>
@@ -5547,27 +5547,27 @@
         <v>0</v>
       </c>
       <c r="EP8" s="224">
-        <f t="shared" ref="EP8" si="86">EM8-EO8</f>
+        <f>EM8-EO8</f>
         <v>0</v>
       </c>
       <c r="EQ8" s="225">
-        <f t="shared" ref="EQ8" si="87">EM8</f>
+        <f>EM8</f>
         <v>0</v>
       </c>
       <c r="ER8" s="150"/>
       <c r="ES8" s="150"/>
       <c r="ET8" s="266">
-        <f t="shared" ref="ET8" si="88">EQ8-EU8</f>
+        <f t="shared" ref="ET8" si="82">EQ8-EU8</f>
         <v>0</v>
       </c>
       <c r="EU8" s="163"/>
       <c r="EV8" s="252"/>
       <c r="EW8" s="222">
-        <f t="shared" ref="EW8" si="89">EQ8-ET8-EU8</f>
+        <f t="shared" ref="EW8" si="83">EQ8-ET8-EU8</f>
         <v>0</v>
       </c>
       <c r="EX8" s="226">
-        <f t="shared" ref="EX8" si="90">+EM8-ET8-EU8</f>
+        <f>+EM8-ET8-EU8</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sửa lại cách cân đối ở tab dữ liệu bất thường , sửa khi nào ưng ý thì thôi. thêm phân quyền giữa các công ty - chỉnh sửa template suất ra báo cáo , hiển thị thêm dữ liệu ở màn hình danh sách , thêm 2 loại công làm thêm ngày lễ
</commit_message>
<xml_diff>
--- a/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
+++ b/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonzai/dev/odoo 19/odoo/my_custom_addons/dl_salary_kpi/static/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D82EA6C-7A19-1B4E-8C4D-B8FE2355EA74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F823649D-7A95-C24F-896C-7B74BD7D0E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="17760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kangatang" sheetId="43" state="veryHidden" r:id="rId1"/>
@@ -2408,16 +2408,82 @@
     <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2453,83 +2519,33 @@
     <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="66" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="67" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="67" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="7" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2544,22 +2560,6 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="32">
@@ -3384,11 +3384,11 @@
       <c r="AL1" s="212"/>
       <c r="AM1" s="212"/>
       <c r="AN1" s="212"/>
-      <c r="AO1" s="300"/>
-      <c r="AP1" s="300"/>
-      <c r="AQ1" s="300"/>
-      <c r="AR1" s="300"/>
-      <c r="AS1" s="300"/>
+      <c r="AO1" s="260"/>
+      <c r="AP1" s="260"/>
+      <c r="AQ1" s="260"/>
+      <c r="AR1" s="260"/>
+      <c r="AS1" s="260"/>
       <c r="AT1" s="120"/>
       <c r="AU1" s="120"/>
       <c r="AV1" s="120"/>
@@ -3790,10 +3790,10 @@
       <c r="G4" s="232"/>
       <c r="H4" s="108"/>
       <c r="I4" s="256"/>
-      <c r="J4" s="289" t="s">
+      <c r="J4" s="261" t="s">
         <v>68</v>
       </c>
-      <c r="K4" s="289"/>
+      <c r="K4" s="261"/>
       <c r="L4" s="258">
         <v>3</v>
       </c>
@@ -3807,23 +3807,23 @@
       </c>
       <c r="Q4" s="259"/>
       <c r="R4" s="109"/>
-      <c r="S4" s="289"/>
-      <c r="T4" s="289"/>
-      <c r="U4" s="289"/>
+      <c r="S4" s="261"/>
+      <c r="T4" s="261"/>
+      <c r="U4" s="261"/>
       <c r="V4" s="109"/>
-      <c r="W4" s="289"/>
-      <c r="X4" s="289"/>
-      <c r="Y4" s="289"/>
-      <c r="Z4" s="289"/>
-      <c r="AA4" s="289"/>
-      <c r="AB4" s="289"/>
-      <c r="AC4" s="289"/>
-      <c r="AD4" s="289"/>
+      <c r="W4" s="261"/>
+      <c r="X4" s="261"/>
+      <c r="Y4" s="261"/>
+      <c r="Z4" s="261"/>
+      <c r="AA4" s="261"/>
+      <c r="AB4" s="261"/>
+      <c r="AC4" s="261"/>
+      <c r="AD4" s="261"/>
       <c r="AE4" s="109"/>
       <c r="AF4" s="110"/>
-      <c r="AG4" s="289"/>
-      <c r="AH4" s="289"/>
-      <c r="AI4" s="289"/>
+      <c r="AG4" s="261"/>
+      <c r="AH4" s="261"/>
+      <c r="AI4" s="261"/>
       <c r="AJ4" s="109"/>
       <c r="AK4" s="109"/>
       <c r="AL4" s="109"/>
@@ -3834,10 +3834,10 @@
       <c r="AQ4" s="113"/>
       <c r="AR4" s="221"/>
       <c r="AS4" s="227"/>
-      <c r="AT4" s="289" t="s">
+      <c r="AT4" s="261" t="s">
         <v>68</v>
       </c>
-      <c r="AU4" s="289"/>
+      <c r="AU4" s="261"/>
       <c r="AV4" s="258">
         <f>L4</f>
         <v>3</v>
@@ -3853,23 +3853,23 @@
       </c>
       <c r="BA4" s="259"/>
       <c r="BB4" s="109"/>
-      <c r="BC4" s="289"/>
-      <c r="BD4" s="289"/>
-      <c r="BE4" s="289"/>
+      <c r="BC4" s="261"/>
+      <c r="BD4" s="261"/>
+      <c r="BE4" s="261"/>
       <c r="BF4" s="109"/>
-      <c r="BG4" s="289"/>
-      <c r="BH4" s="289"/>
-      <c r="BI4" s="289"/>
-      <c r="BJ4" s="289"/>
-      <c r="BK4" s="289"/>
-      <c r="BL4" s="289"/>
-      <c r="BM4" s="289"/>
-      <c r="BN4" s="289"/>
+      <c r="BG4" s="261"/>
+      <c r="BH4" s="261"/>
+      <c r="BI4" s="261"/>
+      <c r="BJ4" s="261"/>
+      <c r="BK4" s="261"/>
+      <c r="BL4" s="261"/>
+      <c r="BM4" s="261"/>
+      <c r="BN4" s="261"/>
       <c r="BO4" s="109"/>
       <c r="BP4" s="110"/>
-      <c r="BQ4" s="289"/>
-      <c r="BR4" s="289"/>
-      <c r="BS4" s="289"/>
+      <c r="BQ4" s="261"/>
+      <c r="BR4" s="261"/>
+      <c r="BS4" s="261"/>
       <c r="BT4" s="114"/>
       <c r="BU4" s="114" t="str">
         <f>IF(WEEKDAY(BU5,1)=1,"CN","")</f>
@@ -3949,31 +3949,31 @@
       <c r="ER4" s="237"/>
     </row>
     <row r="5" spans="1:148" s="183" customFormat="1" ht="92.25" customHeight="1">
-      <c r="A5" s="287" t="s">
+      <c r="A5" s="262" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="293" t="s">
+      <c r="B5" s="263" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="287" t="s">
+      <c r="C5" s="262" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="297" t="s">
+      <c r="D5" s="264" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="298" t="s">
+      <c r="E5" s="265" t="s">
         <v>120</v>
       </c>
-      <c r="F5" s="287" t="s">
+      <c r="F5" s="262" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="287" t="s">
+      <c r="G5" s="262" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="287" t="s">
+      <c r="H5" s="262" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="294" t="s">
+      <c r="I5" s="267" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="174">
@@ -4100,19 +4100,19 @@
         <f t="shared" si="0"/>
         <v>46112</v>
       </c>
-      <c r="AO5" s="295" t="s">
+      <c r="AO5" s="268" t="s">
         <v>82</v>
       </c>
-      <c r="AP5" s="295" t="s">
+      <c r="AP5" s="268" t="s">
         <v>83</v>
       </c>
-      <c r="AQ5" s="295" t="s">
+      <c r="AQ5" s="268" t="s">
         <v>84</v>
       </c>
-      <c r="AR5" s="296" t="s">
+      <c r="AR5" s="269" t="s">
         <v>5</v>
       </c>
-      <c r="AS5" s="296" t="s">
+      <c r="AS5" s="269" t="s">
         <v>6</v>
       </c>
       <c r="AT5" s="178">
@@ -4239,46 +4239,46 @@
         <f t="shared" si="1"/>
         <v>46112</v>
       </c>
-      <c r="BY5" s="290" t="s">
+      <c r="BY5" s="270" t="s">
         <v>85</v>
       </c>
-      <c r="BZ5" s="290" t="s">
+      <c r="BZ5" s="270" t="s">
         <v>86</v>
       </c>
-      <c r="CA5" s="290" t="s">
+      <c r="CA5" s="270" t="s">
         <v>87</v>
       </c>
-      <c r="CB5" s="290" t="s">
+      <c r="CB5" s="270" t="s">
         <v>88</v>
       </c>
-      <c r="CC5" s="290" t="s">
+      <c r="CC5" s="270" t="s">
         <v>89</v>
       </c>
-      <c r="CD5" s="290" t="s">
+      <c r="CD5" s="270" t="s">
         <v>90</v>
       </c>
-      <c r="CE5" s="290" t="s">
+      <c r="CE5" s="270" t="s">
         <v>91</v>
       </c>
-      <c r="CF5" s="288" t="s">
+      <c r="CF5" s="284" t="s">
         <v>19</v>
       </c>
-      <c r="CG5" s="288"/>
-      <c r="CH5" s="288"/>
-      <c r="CI5" s="288"/>
-      <c r="CJ5" s="288"/>
-      <c r="CK5" s="288"/>
-      <c r="CL5" s="288"/>
-      <c r="CM5" s="288"/>
-      <c r="CN5" s="288"/>
-      <c r="CO5" s="288"/>
-      <c r="CP5" s="288"/>
-      <c r="CQ5" s="266" t="s">
+      <c r="CG5" s="284"/>
+      <c r="CH5" s="284"/>
+      <c r="CI5" s="284"/>
+      <c r="CJ5" s="284"/>
+      <c r="CK5" s="284"/>
+      <c r="CL5" s="284"/>
+      <c r="CM5" s="284"/>
+      <c r="CN5" s="284"/>
+      <c r="CO5" s="284"/>
+      <c r="CP5" s="284"/>
+      <c r="CQ5" s="288" t="s">
         <v>59</v>
       </c>
-      <c r="CR5" s="267"/>
-      <c r="CS5" s="268"/>
-      <c r="CT5" s="273" t="s">
+      <c r="CR5" s="289"/>
+      <c r="CS5" s="290"/>
+      <c r="CT5" s="295" t="s">
         <v>60</v>
       </c>
       <c r="CU5" s="247" t="s">
@@ -4301,107 +4301,107 @@
       <c r="DF5" s="245" t="s">
         <v>127</v>
       </c>
-      <c r="DG5" s="269" t="s">
+      <c r="DG5" s="291" t="s">
         <v>117</v>
       </c>
-      <c r="DH5" s="274" t="s">
+      <c r="DH5" s="296" t="s">
         <v>112</v>
       </c>
-      <c r="DI5" s="271" t="s">
+      <c r="DI5" s="293" t="s">
         <v>81</v>
       </c>
-      <c r="DJ5" s="272"/>
-      <c r="DK5" s="275" t="s">
+      <c r="DJ5" s="294"/>
+      <c r="DK5" s="281" t="s">
         <v>61</v>
       </c>
-      <c r="DL5" s="292" t="s">
+      <c r="DL5" s="285" t="s">
         <v>8</v>
       </c>
-      <c r="DM5" s="276" t="s">
+      <c r="DM5" s="282" t="s">
         <v>71</v>
       </c>
-      <c r="DN5" s="276"/>
-      <c r="DO5" s="276"/>
-      <c r="DP5" s="276"/>
-      <c r="DQ5" s="276"/>
-      <c r="DR5" s="276"/>
-      <c r="DS5" s="277" t="s">
+      <c r="DN5" s="282"/>
+      <c r="DO5" s="282"/>
+      <c r="DP5" s="282"/>
+      <c r="DQ5" s="282"/>
+      <c r="DR5" s="282"/>
+      <c r="DS5" s="297" t="s">
         <v>12</v>
       </c>
-      <c r="DT5" s="276" t="s">
+      <c r="DT5" s="282" t="s">
         <v>125</v>
       </c>
-      <c r="DU5" s="293" t="s">
+      <c r="DU5" s="263" t="s">
         <v>13</v>
       </c>
-      <c r="DV5" s="264" t="s">
+      <c r="DV5" s="286" t="s">
         <v>64</v>
       </c>
-      <c r="DW5" s="265"/>
-      <c r="DX5" s="264"/>
-      <c r="DY5" s="285" t="s">
+      <c r="DW5" s="287"/>
+      <c r="DX5" s="286"/>
+      <c r="DY5" s="279" t="s">
         <v>63</v>
       </c>
-      <c r="DZ5" s="285"/>
-      <c r="EA5" s="285"/>
-      <c r="EB5" s="285"/>
-      <c r="EC5" s="286" t="s">
+      <c r="DZ5" s="279"/>
+      <c r="EA5" s="279"/>
+      <c r="EB5" s="279"/>
+      <c r="EC5" s="280" t="s">
         <v>128</v>
       </c>
-      <c r="ED5" s="276" t="s">
+      <c r="ED5" s="282" t="s">
         <v>7</v>
       </c>
-      <c r="EE5" s="262" t="s">
+      <c r="EE5" s="283" t="s">
         <v>65</v>
       </c>
-      <c r="EF5" s="262"/>
-      <c r="EG5" s="262" t="s">
+      <c r="EF5" s="283"/>
+      <c r="EG5" s="283" t="s">
         <v>66</v>
       </c>
-      <c r="EH5" s="262" t="s">
+      <c r="EH5" s="283" t="s">
         <v>67</v>
       </c>
-      <c r="EI5" s="262" t="s">
+      <c r="EI5" s="283" t="s">
         <v>72</v>
       </c>
-      <c r="EJ5" s="263" t="s">
+      <c r="EJ5" s="300" t="s">
         <v>78</v>
       </c>
-      <c r="EK5" s="263" t="s">
+      <c r="EK5" s="300" t="s">
         <v>80</v>
       </c>
-      <c r="EL5" s="263" t="s">
+      <c r="EL5" s="300" t="s">
         <v>79</v>
       </c>
-      <c r="EM5" s="280" t="s">
+      <c r="EM5" s="274" t="s">
         <v>124</v>
       </c>
-      <c r="EN5" s="260" t="s">
+      <c r="EN5" s="298" t="s">
         <v>118</v>
       </c>
-      <c r="EO5" s="282" t="s">
+      <c r="EO5" s="276" t="s">
         <v>130</v>
       </c>
-      <c r="EP5" s="284" t="s">
+      <c r="EP5" s="278" t="s">
         <v>122</v>
       </c>
-      <c r="EQ5" s="284" t="s">
+      <c r="EQ5" s="278" t="s">
         <v>121</v>
       </c>
-      <c r="ER5" s="278" t="s">
+      <c r="ER5" s="272" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:148" s="205" customFormat="1" ht="148.5" customHeight="1">
-      <c r="A6" s="287"/>
-      <c r="B6" s="293"/>
-      <c r="C6" s="287"/>
-      <c r="D6" s="297"/>
-      <c r="E6" s="299"/>
-      <c r="F6" s="287"/>
-      <c r="G6" s="287"/>
-      <c r="H6" s="287"/>
-      <c r="I6" s="294"/>
+      <c r="A6" s="262"/>
+      <c r="B6" s="263"/>
+      <c r="C6" s="262"/>
+      <c r="D6" s="264"/>
+      <c r="E6" s="266"/>
+      <c r="F6" s="262"/>
+      <c r="G6" s="262"/>
+      <c r="H6" s="262"/>
+      <c r="I6" s="267"/>
       <c r="J6" s="184" t="str">
         <f t="shared" ref="J6:AN6" si="2">IF(WEEKDAY(J5)=1,"CN",WEEKDAY(J5))</f>
         <v>CN</v>
@@ -4526,11 +4526,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AO6" s="295"/>
-      <c r="AP6" s="295"/>
-      <c r="AQ6" s="295"/>
-      <c r="AR6" s="296"/>
-      <c r="AS6" s="296"/>
+      <c r="AO6" s="268"/>
+      <c r="AP6" s="268"/>
+      <c r="AQ6" s="268"/>
+      <c r="AR6" s="269"/>
+      <c r="AS6" s="269"/>
       <c r="AT6" s="186" t="str">
         <f>+J6</f>
         <v>CN</v>
@@ -4655,13 +4655,13 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="BY6" s="291"/>
-      <c r="BZ6" s="291"/>
-      <c r="CA6" s="291"/>
-      <c r="CB6" s="291"/>
-      <c r="CC6" s="291"/>
-      <c r="CD6" s="291"/>
-      <c r="CE6" s="291"/>
+      <c r="BY6" s="271"/>
+      <c r="BZ6" s="271"/>
+      <c r="CA6" s="271"/>
+      <c r="CB6" s="271"/>
+      <c r="CC6" s="271"/>
+      <c r="CD6" s="271"/>
+      <c r="CE6" s="271"/>
       <c r="CF6" s="188" t="s">
         <v>92</v>
       </c>
@@ -4704,7 +4704,7 @@
       <c r="CS6" s="180" t="s">
         <v>58</v>
       </c>
-      <c r="CT6" s="273"/>
+      <c r="CT6" s="295"/>
       <c r="CU6" s="188" t="s">
         <v>103</v>
       </c>
@@ -4741,16 +4741,16 @@
       <c r="DF6" s="246" t="s">
         <v>129</v>
       </c>
-      <c r="DG6" s="270"/>
-      <c r="DH6" s="274"/>
+      <c r="DG6" s="292"/>
+      <c r="DH6" s="296"/>
       <c r="DI6" s="152" t="s">
         <v>14</v>
       </c>
       <c r="DJ6" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="DK6" s="275"/>
-      <c r="DL6" s="292"/>
+      <c r="DK6" s="281"/>
+      <c r="DL6" s="285"/>
       <c r="DM6" s="180" t="s">
         <v>9</v>
       </c>
@@ -4769,9 +4769,9 @@
       <c r="DR6" s="180" t="s">
         <v>115</v>
       </c>
-      <c r="DS6" s="277"/>
-      <c r="DT6" s="276"/>
-      <c r="DU6" s="293"/>
+      <c r="DS6" s="297"/>
+      <c r="DT6" s="282"/>
+      <c r="DU6" s="263"/>
       <c r="DV6" s="203">
         <v>0.17499999999999999</v>
       </c>
@@ -4793,170 +4793,170 @@
       <c r="EB6" s="152" t="s">
         <v>62</v>
       </c>
-      <c r="EC6" s="275"/>
-      <c r="ED6" s="276"/>
+      <c r="EC6" s="281"/>
+      <c r="ED6" s="282"/>
       <c r="EE6" s="182" t="s">
         <v>73</v>
       </c>
       <c r="EF6" s="182" t="s">
         <v>74</v>
       </c>
-      <c r="EG6" s="262"/>
-      <c r="EH6" s="262"/>
-      <c r="EI6" s="262"/>
-      <c r="EJ6" s="263"/>
-      <c r="EK6" s="263"/>
-      <c r="EL6" s="263"/>
-      <c r="EM6" s="281"/>
-      <c r="EN6" s="261"/>
-      <c r="EO6" s="283"/>
-      <c r="EP6" s="284"/>
-      <c r="EQ6" s="284"/>
-      <c r="ER6" s="278"/>
+      <c r="EG6" s="283"/>
+      <c r="EH6" s="283"/>
+      <c r="EI6" s="283"/>
+      <c r="EJ6" s="300"/>
+      <c r="EK6" s="300"/>
+      <c r="EL6" s="300"/>
+      <c r="EM6" s="275"/>
+      <c r="EN6" s="299"/>
+      <c r="EO6" s="277"/>
+      <c r="EP6" s="278"/>
+      <c r="EQ6" s="278"/>
+      <c r="ER6" s="272"/>
     </row>
     <row r="7" spans="1:148" s="106" customFormat="1" ht="87.75" customHeight="1">
-      <c r="A7" s="279"/>
-      <c r="B7" s="279"/>
-      <c r="C7" s="279"/>
-      <c r="D7" s="279"/>
-      <c r="E7" s="279"/>
-      <c r="F7" s="279"/>
-      <c r="G7" s="279"/>
-      <c r="H7" s="279"/>
-      <c r="I7" s="279"/>
-      <c r="J7" s="279"/>
-      <c r="K7" s="279"/>
-      <c r="L7" s="279"/>
-      <c r="M7" s="279"/>
-      <c r="N7" s="279"/>
-      <c r="O7" s="279"/>
-      <c r="P7" s="279"/>
-      <c r="Q7" s="279"/>
-      <c r="R7" s="279"/>
-      <c r="S7" s="279"/>
-      <c r="T7" s="279"/>
-      <c r="U7" s="279"/>
-      <c r="V7" s="279"/>
-      <c r="W7" s="279"/>
-      <c r="X7" s="279"/>
-      <c r="Y7" s="279"/>
-      <c r="Z7" s="279"/>
-      <c r="AA7" s="279"/>
-      <c r="AB7" s="279"/>
-      <c r="AC7" s="279"/>
-      <c r="AD7" s="279"/>
-      <c r="AE7" s="279"/>
-      <c r="AF7" s="279"/>
-      <c r="AG7" s="279"/>
-      <c r="AH7" s="279"/>
-      <c r="AI7" s="279"/>
-      <c r="AJ7" s="279"/>
-      <c r="AK7" s="279"/>
-      <c r="AL7" s="279"/>
-      <c r="AM7" s="279"/>
-      <c r="AN7" s="279"/>
-      <c r="AO7" s="279"/>
-      <c r="AP7" s="279"/>
-      <c r="AQ7" s="279"/>
-      <c r="AR7" s="279"/>
-      <c r="AS7" s="279"/>
-      <c r="AT7" s="279"/>
-      <c r="AU7" s="279"/>
-      <c r="AV7" s="279"/>
-      <c r="AW7" s="279"/>
-      <c r="AX7" s="279"/>
-      <c r="AY7" s="279"/>
-      <c r="AZ7" s="279"/>
-      <c r="BA7" s="279"/>
-      <c r="BB7" s="279"/>
-      <c r="BC7" s="279"/>
-      <c r="BD7" s="279"/>
-      <c r="BE7" s="279"/>
-      <c r="BF7" s="279"/>
-      <c r="BG7" s="279"/>
-      <c r="BH7" s="279"/>
-      <c r="BI7" s="279"/>
-      <c r="BJ7" s="279"/>
-      <c r="BK7" s="279"/>
-      <c r="BL7" s="279"/>
-      <c r="BM7" s="279"/>
-      <c r="BN7" s="279"/>
-      <c r="BO7" s="279"/>
-      <c r="BP7" s="279"/>
-      <c r="BQ7" s="279"/>
-      <c r="BR7" s="279"/>
-      <c r="BS7" s="279"/>
-      <c r="BT7" s="279"/>
-      <c r="BU7" s="279"/>
-      <c r="BV7" s="279"/>
-      <c r="BW7" s="279"/>
-      <c r="BX7" s="279"/>
-      <c r="BY7" s="279"/>
-      <c r="BZ7" s="279"/>
-      <c r="CA7" s="279"/>
-      <c r="CB7" s="279"/>
-      <c r="CC7" s="279"/>
-      <c r="CD7" s="279"/>
-      <c r="CE7" s="279"/>
-      <c r="CF7" s="279"/>
-      <c r="CG7" s="279"/>
-      <c r="CH7" s="279"/>
-      <c r="CI7" s="279"/>
-      <c r="CJ7" s="279"/>
-      <c r="CK7" s="279"/>
-      <c r="CL7" s="279"/>
-      <c r="CM7" s="279"/>
-      <c r="CN7" s="279"/>
-      <c r="CO7" s="279"/>
-      <c r="CP7" s="279"/>
-      <c r="CQ7" s="279"/>
-      <c r="CR7" s="279"/>
-      <c r="CS7" s="279"/>
-      <c r="CT7" s="279"/>
-      <c r="CU7" s="279"/>
-      <c r="CV7" s="279"/>
-      <c r="CW7" s="279"/>
-      <c r="CX7" s="279"/>
-      <c r="CY7" s="279"/>
-      <c r="CZ7" s="279"/>
-      <c r="DA7" s="279"/>
-      <c r="DB7" s="279"/>
-      <c r="DC7" s="279"/>
-      <c r="DD7" s="279"/>
-      <c r="DE7" s="279"/>
-      <c r="DF7" s="279"/>
-      <c r="DG7" s="279"/>
-      <c r="DH7" s="279"/>
-      <c r="DI7" s="279"/>
-      <c r="DJ7" s="279"/>
-      <c r="DK7" s="279"/>
-      <c r="DL7" s="279"/>
-      <c r="DM7" s="279"/>
-      <c r="DN7" s="279"/>
-      <c r="DO7" s="279"/>
-      <c r="DP7" s="279"/>
-      <c r="DQ7" s="279"/>
-      <c r="DR7" s="279"/>
-      <c r="DS7" s="279"/>
-      <c r="DT7" s="279"/>
-      <c r="DU7" s="279"/>
-      <c r="DV7" s="279"/>
-      <c r="DW7" s="279"/>
-      <c r="DX7" s="279"/>
-      <c r="DY7" s="279"/>
-      <c r="DZ7" s="279"/>
-      <c r="EA7" s="279"/>
-      <c r="EB7" s="279"/>
-      <c r="EC7" s="279"/>
-      <c r="ED7" s="279"/>
-      <c r="EE7" s="279"/>
-      <c r="EF7" s="279"/>
-      <c r="EG7" s="279"/>
-      <c r="EH7" s="279"/>
-      <c r="EI7" s="279"/>
-      <c r="EJ7" s="279"/>
-      <c r="EK7" s="279"/>
-      <c r="EL7" s="279"/>
+      <c r="A7" s="273"/>
+      <c r="B7" s="273"/>
+      <c r="C7" s="273"/>
+      <c r="D7" s="273"/>
+      <c r="E7" s="273"/>
+      <c r="F7" s="273"/>
+      <c r="G7" s="273"/>
+      <c r="H7" s="273"/>
+      <c r="I7" s="273"/>
+      <c r="J7" s="273"/>
+      <c r="K7" s="273"/>
+      <c r="L7" s="273"/>
+      <c r="M7" s="273"/>
+      <c r="N7" s="273"/>
+      <c r="O7" s="273"/>
+      <c r="P7" s="273"/>
+      <c r="Q7" s="273"/>
+      <c r="R7" s="273"/>
+      <c r="S7" s="273"/>
+      <c r="T7" s="273"/>
+      <c r="U7" s="273"/>
+      <c r="V7" s="273"/>
+      <c r="W7" s="273"/>
+      <c r="X7" s="273"/>
+      <c r="Y7" s="273"/>
+      <c r="Z7" s="273"/>
+      <c r="AA7" s="273"/>
+      <c r="AB7" s="273"/>
+      <c r="AC7" s="273"/>
+      <c r="AD7" s="273"/>
+      <c r="AE7" s="273"/>
+      <c r="AF7" s="273"/>
+      <c r="AG7" s="273"/>
+      <c r="AH7" s="273"/>
+      <c r="AI7" s="273"/>
+      <c r="AJ7" s="273"/>
+      <c r="AK7" s="273"/>
+      <c r="AL7" s="273"/>
+      <c r="AM7" s="273"/>
+      <c r="AN7" s="273"/>
+      <c r="AO7" s="273"/>
+      <c r="AP7" s="273"/>
+      <c r="AQ7" s="273"/>
+      <c r="AR7" s="273"/>
+      <c r="AS7" s="273"/>
+      <c r="AT7" s="273"/>
+      <c r="AU7" s="273"/>
+      <c r="AV7" s="273"/>
+      <c r="AW7" s="273"/>
+      <c r="AX7" s="273"/>
+      <c r="AY7" s="273"/>
+      <c r="AZ7" s="273"/>
+      <c r="BA7" s="273"/>
+      <c r="BB7" s="273"/>
+      <c r="BC7" s="273"/>
+      <c r="BD7" s="273"/>
+      <c r="BE7" s="273"/>
+      <c r="BF7" s="273"/>
+      <c r="BG7" s="273"/>
+      <c r="BH7" s="273"/>
+      <c r="BI7" s="273"/>
+      <c r="BJ7" s="273"/>
+      <c r="BK7" s="273"/>
+      <c r="BL7" s="273"/>
+      <c r="BM7" s="273"/>
+      <c r="BN7" s="273"/>
+      <c r="BO7" s="273"/>
+      <c r="BP7" s="273"/>
+      <c r="BQ7" s="273"/>
+      <c r="BR7" s="273"/>
+      <c r="BS7" s="273"/>
+      <c r="BT7" s="273"/>
+      <c r="BU7" s="273"/>
+      <c r="BV7" s="273"/>
+      <c r="BW7" s="273"/>
+      <c r="BX7" s="273"/>
+      <c r="BY7" s="273"/>
+      <c r="BZ7" s="273"/>
+      <c r="CA7" s="273"/>
+      <c r="CB7" s="273"/>
+      <c r="CC7" s="273"/>
+      <c r="CD7" s="273"/>
+      <c r="CE7" s="273"/>
+      <c r="CF7" s="273"/>
+      <c r="CG7" s="273"/>
+      <c r="CH7" s="273"/>
+      <c r="CI7" s="273"/>
+      <c r="CJ7" s="273"/>
+      <c r="CK7" s="273"/>
+      <c r="CL7" s="273"/>
+      <c r="CM7" s="273"/>
+      <c r="CN7" s="273"/>
+      <c r="CO7" s="273"/>
+      <c r="CP7" s="273"/>
+      <c r="CQ7" s="273"/>
+      <c r="CR7" s="273"/>
+      <c r="CS7" s="273"/>
+      <c r="CT7" s="273"/>
+      <c r="CU7" s="273"/>
+      <c r="CV7" s="273"/>
+      <c r="CW7" s="273"/>
+      <c r="CX7" s="273"/>
+      <c r="CY7" s="273"/>
+      <c r="CZ7" s="273"/>
+      <c r="DA7" s="273"/>
+      <c r="DB7" s="273"/>
+      <c r="DC7" s="273"/>
+      <c r="DD7" s="273"/>
+      <c r="DE7" s="273"/>
+      <c r="DF7" s="273"/>
+      <c r="DG7" s="273"/>
+      <c r="DH7" s="273"/>
+      <c r="DI7" s="273"/>
+      <c r="DJ7" s="273"/>
+      <c r="DK7" s="273"/>
+      <c r="DL7" s="273"/>
+      <c r="DM7" s="273"/>
+      <c r="DN7" s="273"/>
+      <c r="DO7" s="273"/>
+      <c r="DP7" s="273"/>
+      <c r="DQ7" s="273"/>
+      <c r="DR7" s="273"/>
+      <c r="DS7" s="273"/>
+      <c r="DT7" s="273"/>
+      <c r="DU7" s="273"/>
+      <c r="DV7" s="273"/>
+      <c r="DW7" s="273"/>
+      <c r="DX7" s="273"/>
+      <c r="DY7" s="273"/>
+      <c r="DZ7" s="273"/>
+      <c r="EA7" s="273"/>
+      <c r="EB7" s="273"/>
+      <c r="EC7" s="273"/>
+      <c r="ED7" s="273"/>
+      <c r="EE7" s="273"/>
+      <c r="EF7" s="273"/>
+      <c r="EG7" s="273"/>
+      <c r="EH7" s="273"/>
+      <c r="EI7" s="273"/>
+      <c r="EJ7" s="273"/>
+      <c r="EK7" s="273"/>
+      <c r="EL7" s="273"/>
       <c r="EM7" s="238"/>
       <c r="EN7" s="238"/>
       <c r="EO7" s="238"/>
@@ -5114,39 +5114,39 @@
         <v>0</v>
       </c>
       <c r="BP8" s="155">
-        <f t="shared" ref="BP8" si="31">+IF(AF8="N","0.5N",IF(AF8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BP8:BQ8" si="31">+IF(AF8="N","0.5N",IF(AF8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BQ8" s="155">
-        <f t="shared" ref="BQ8" si="32">+IF(AG8="N","0.5N",IF(AG8="Đ","0.5Đ",0))</f>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="BR8" s="155">
-        <f t="shared" ref="BR8" si="33">+IF(AH8="N","0.5N",IF(AH8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BR8" si="32">+IF(AH8="N","0.5N",IF(AH8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BS8" s="155">
-        <f t="shared" ref="BS8" si="34">+IF(AI8="N","0.5N",IF(AI8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BS8" si="33">+IF(AI8="N","0.5N",IF(AI8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BT8" s="155">
-        <f t="shared" ref="BT8" si="35">+IF(AJ8="N","0.5N",IF(AJ8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BT8" si="34">+IF(AJ8="N","0.5N",IF(AJ8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BU8" s="155">
-        <f t="shared" ref="BU8" si="36">+IF(AK8="N","0.5N",IF(AK8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BU8" si="35">+IF(AK8="N","0.5N",IF(AK8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BV8" s="155">
-        <f t="shared" ref="BV8" si="37">+IF(AL8="N","0.5N",IF(AL8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BV8" si="36">+IF(AL8="N","0.5N",IF(AL8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BW8" s="155">
-        <f t="shared" ref="BW8" si="38">+IF(AM8="N","0.5N",IF(AM8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BW8" si="37">+IF(AM8="N","0.5N",IF(AM8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BX8" s="155">
-        <f t="shared" ref="BX8" si="39">+IF(AN8="N","0.5N",IF(AN8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BX8" si="38">+IF(AN8="N","0.5N",IF(AN8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BY8" s="167">
@@ -5154,19 +5154,19 @@
         <v>0</v>
       </c>
       <c r="BZ8" s="167">
-        <f t="shared" ref="BZ8" si="40">COUNTIF(AT8:BX8,"1Đ")+(COUNTIF(AT8:BX8,"2Đ")*2)+(COUNTIF(AT8:BX8,"0.5Đ")/2)</f>
+        <f t="shared" ref="BZ8" si="39">COUNTIF(AT8:BX8,"1Đ")+(COUNTIF(AT8:BX8,"2Đ")*2)+(COUNTIF(AT8:BX8,"0.5Đ")/2)</f>
         <v>0</v>
       </c>
       <c r="CA8" s="167">
-        <f t="shared" ref="CA8" si="41">COUNTIF(AT8:BX8,"1N")+(COUNTIF(AT8:BX8,"2N")*2)+(COUNTIF(AT8:BX8,"0.5N")/2)</f>
+        <f t="shared" ref="CA8" si="40">COUNTIF(AT8:BX8,"1N")+(COUNTIF(AT8:BX8,"2N")*2)+(COUNTIF(AT8:BX8,"0.5N")/2)</f>
         <v>0</v>
       </c>
       <c r="CB8" s="167">
-        <f t="shared" ref="CB8" si="42">COUNTIF(AT8:BX8,"1LN")</f>
+        <f>COUNTIF(AT8:BX8,"1LN")+COUNTIF(AT8:BX8,"0.5LN")*0.5</f>
         <v>0</v>
       </c>
       <c r="CC8" s="167">
-        <f t="shared" ref="CC8" si="43">COUNTIF(AT8:BX8,"1LĐ")</f>
+        <f t="shared" ref="CC8" si="41">COUNTIF(AT8:BX8,"1LĐ")</f>
         <v>0</v>
       </c>
       <c r="CD8" s="163">
@@ -5174,48 +5174,48 @@
         <v>0</v>
       </c>
       <c r="CE8" s="170">
-        <f t="shared" ref="CE8" si="44">COUNTIF(AT8:BX8,"CNĐ")+(COUNTIF(AT8:BX8,"CNĐ/2")/2)</f>
+        <f t="shared" ref="CE8" si="42">COUNTIF(AT8:BX8,"CNĐ")+(COUNTIF(AT8:BX8,"CNĐ/2")/2)</f>
         <v>0</v>
       </c>
       <c r="CF8" s="171">
-        <f t="shared" ref="CF8" si="45">+AO8</f>
+        <f t="shared" ref="CF8" si="43">+AO8</f>
         <v>0</v>
       </c>
       <c r="CG8" s="171">
-        <f t="shared" ref="CG8" si="46">+AP8*8*0.3125</f>
+        <f t="shared" ref="CG8" si="44">+AP8*8*0.3125</f>
         <v>0</v>
       </c>
       <c r="CH8" s="171">
-        <f t="shared" ref="CH8" si="47">+AR8+AS8</f>
+        <f t="shared" ref="CH8" si="45">+AR8+AS8</f>
         <v>0</v>
       </c>
       <c r="CI8" s="171">
-        <f t="shared" ref="CI8" si="48">+CA8</f>
+        <f t="shared" ref="CI8" si="46">+CA8</f>
         <v>0</v>
       </c>
       <c r="CJ8" s="171">
-        <f t="shared" ref="CJ8" si="49">+AP8*8*0.6875</f>
+        <f t="shared" ref="CJ8" si="47">+AP8*8*0.6875</f>
         <v>0</v>
       </c>
       <c r="CK8" s="171">
-        <f t="shared" ref="CK8" si="50">+BZ8</f>
+        <f t="shared" ref="CK8" si="48">+BZ8</f>
         <v>0</v>
       </c>
       <c r="CL8" s="171"/>
       <c r="CM8" s="171">
-        <f t="shared" ref="CM8" si="51">+CE8</f>
+        <f t="shared" ref="CM8" si="49">+CE8</f>
         <v>0</v>
       </c>
       <c r="CN8" s="171">
-        <f t="shared" ref="CN8" si="52">+CD8</f>
+        <f t="shared" ref="CN8" si="50">+CD8</f>
         <v>0</v>
       </c>
       <c r="CO8" s="169">
-        <f t="shared" ref="CO8" si="53">+CB8</f>
+        <f t="shared" ref="CO8" si="51">+CB8</f>
         <v>0</v>
       </c>
       <c r="CP8" s="159">
-        <f t="shared" ref="CP8" si="54">+CC8</f>
+        <f t="shared" ref="CP8" si="52">+CC8</f>
         <v>0</v>
       </c>
       <c r="CQ8" s="159">
@@ -5224,104 +5224,104 @@
       </c>
       <c r="CR8" s="156"/>
       <c r="CS8" s="159">
-        <f t="shared" ref="CS8" si="55">IF($G$4&lt;20000000000,0,IF($G$4&lt;=30000000000,2000000,IF($G$4&lt;=50000000000,2300000,IF($G$4&lt;=50000000000,2000000,IF($G$4&lt;=70000000000,3000000,IF($G$4&gt;70000000000,3500000,0))))))</f>
+        <f t="shared" ref="CS8" si="53">IF($G$4&lt;20000000000,0,IF($G$4&lt;=30000000000,2000000,IF($G$4&lt;=50000000000,2300000,IF($G$4&lt;=50000000000,2000000,IF($G$4&lt;=70000000000,3000000,IF($G$4&gt;70000000000,3500000,0))))))</f>
         <v>0</v>
       </c>
       <c r="CT8" s="157">
-        <f t="shared" ref="CT8" si="56">+I8+CQ8+CR8+CS8</f>
+        <f t="shared" ref="CT8" si="54">+I8+CQ8+CR8+CS8</f>
         <v>0</v>
       </c>
       <c r="CU8" s="158">
-        <f t="shared" ref="CU8" si="57">+I8/26*(CF8+(CG8/8)+CH8)</f>
+        <f t="shared" ref="CU8" si="55">+I8/26*(CF8+(CG8/8)+CH8)</f>
         <v>0</v>
       </c>
       <c r="CV8" s="158">
-        <f t="shared" ref="CV8" si="58">+(I8/26/8)*150%*CI8</f>
+        <f t="shared" ref="CV8" si="56">+(I8/26/8)*150%*CI8</f>
         <v>0</v>
       </c>
       <c r="CW8" s="158">
-        <f t="shared" ref="CW8" si="59">+(I8/26/8)*130%*CJ8</f>
+        <f t="shared" ref="CW8" si="57">+(I8/26/8)*130%*CJ8</f>
         <v>0</v>
       </c>
       <c r="CX8" s="158">
-        <f t="shared" ref="CX8" si="60">+(I8/26/8)*200%*CK8</f>
+        <f t="shared" ref="CX8" si="58">+(I8/26/8)*200%*CK8</f>
         <v>0</v>
       </c>
       <c r="CY8" s="158">
-        <f t="shared" ref="CY8" si="61">+(I8/26/8)*210%*CL8</f>
+        <f t="shared" ref="CY8" si="59">+(I8/26/8)*210%*CL8</f>
         <v>0</v>
       </c>
       <c r="CZ8" s="158">
-        <f t="shared" ref="CZ8" si="62">+(I8/26/8)*270%*CM8</f>
+        <f t="shared" ref="CZ8" si="60">+(I8/26/8)*270%*CM8</f>
         <v>0</v>
       </c>
       <c r="DA8" s="158">
-        <f t="shared" ref="DA8" si="63">+(I8/26/8)*200%*CN8</f>
+        <f t="shared" ref="DA8" si="61">+(I8/26/8)*200%*CN8</f>
         <v>0</v>
       </c>
       <c r="DB8" s="158">
-        <f t="shared" ref="DB8" si="64">+(I8/3.25)*300%*CO8</f>
+        <f>+(I8/26)*300%*CO8</f>
         <v>0</v>
       </c>
       <c r="DC8" s="158">
-        <f t="shared" ref="DC8" si="65">+(I8/26/8)*390%*CP8</f>
+        <f t="shared" ref="DC8" si="62">+(I8/26/8)*390%*CP8</f>
         <v>0</v>
       </c>
       <c r="DD8" s="159">
-        <f t="shared" ref="DD8" si="66">+CS8/26*(CF8+(CG8+CJ8)/8)</f>
+        <f t="shared" ref="DD8" si="63">+CS8/26*(CF8+(CG8+CJ8)/8)</f>
         <v>0</v>
       </c>
       <c r="DE8" s="211">
-        <f t="shared" ref="DE8" si="67">IF(OR(H8="CV",H8="KTT",H8="QL",H8="QĐ",H8="TL",H8="PGĐ"),2000000,IF(OR(H8="NV",H8="KT", H8="TK"),1500000,IF(OR(H8="CN",H8="LX"),1000000,0)))/26*(CF8+(CG8+CJ8)/8)</f>
+        <f t="shared" ref="DE8" si="64">IF(OR(H8="CV",H8="KTT",H8="QL",H8="QĐ",H8="TL",H8="PGĐ"),2000000,IF(OR(H8="NV",H8="KT", H8="TK"),1500000,IF(OR(H8="CN",H8="LX"),1000000,0)))/26*(CF8+(CG8+CJ8)/8)</f>
         <v>0</v>
       </c>
       <c r="DF8" s="211">
-        <f t="shared" ref="DF8" si="68">+DD8+DE8</f>
+        <f t="shared" ref="DF8" si="65">+DD8+DE8</f>
         <v>0</v>
       </c>
       <c r="DG8" s="254"/>
       <c r="DH8" s="158">
-        <f t="shared" ref="DH8" si="69">+CU8+CV8+CW8+CX8+CY8+CZ8+DA8+DB8+DC8+DF8+DG8</f>
+        <f t="shared" ref="DH8" si="66">+CU8+CV8+CW8+CX8+CY8+CZ8+DA8+DB8+DC8+DF8+DG8</f>
         <v>0</v>
       </c>
       <c r="DI8" s="164">
-        <f t="shared" ref="DI8" si="70">+CQ8/26*AQ8</f>
+        <f t="shared" ref="DI8" si="67">+CQ8/26*AQ8</f>
         <v>0</v>
       </c>
       <c r="DJ8" s="164">
-        <f t="shared" ref="DJ8" si="71">+CR8/26*AQ8</f>
+        <f t="shared" ref="DJ8" si="68">+CR8/26*AQ8</f>
         <v>0</v>
       </c>
       <c r="DK8" s="164">
-        <f t="shared" ref="DK8" si="72">+DH8+DI8+DJ8</f>
+        <f t="shared" ref="DK8" si="69">+DH8+DI8+DJ8</f>
         <v>0</v>
       </c>
       <c r="DL8" s="172">
-        <f t="shared" ref="DL8" si="73">I8</f>
+        <f t="shared" ref="DL8" si="70">I8</f>
         <v>0</v>
       </c>
       <c r="DM8" s="159">
-        <f t="shared" ref="DM8" si="74">DL8*8%</f>
+        <f t="shared" ref="DM8" si="71">DL8*8%</f>
         <v>0</v>
       </c>
       <c r="DN8" s="159">
-        <f t="shared" ref="DN8" si="75">DL8*1.5%</f>
+        <f t="shared" ref="DN8" si="72">DL8*1.5%</f>
         <v>0</v>
       </c>
       <c r="DO8" s="159">
-        <f t="shared" ref="DO8" si="76">DL8*1%</f>
+        <f t="shared" ref="DO8" si="73">DL8*1%</f>
         <v>0</v>
       </c>
       <c r="DP8" s="159">
-        <f t="shared" ref="DP8" si="77">EI8</f>
+        <f t="shared" ref="DP8" si="74">EI8</f>
         <v>0</v>
       </c>
       <c r="DQ8" s="159">
-        <f t="shared" ref="DQ8" si="78">+SUM(DM8:DP8)</f>
+        <f t="shared" ref="DQ8" si="75">+SUM(DM8:DP8)</f>
         <v>0</v>
       </c>
       <c r="DR8" s="159">
-        <f t="shared" ref="DR8" si="79">SUM(DM8:DO8)</f>
+        <f t="shared" ref="DR8" si="76">SUM(DM8:DO8)</f>
         <v>0</v>
       </c>
       <c r="DS8" s="160">
@@ -5358,7 +5358,7 @@
         <v>0</v>
       </c>
       <c r="EB8" s="173">
-        <f t="shared" ref="EB8" si="80">DY8+DZ8+EA8</f>
+        <f t="shared" ref="EB8" si="77">DY8+DZ8+EA8</f>
         <v>0</v>
       </c>
       <c r="EC8" s="164">
@@ -5385,7 +5385,7 @@
         <v>-775000</v>
       </c>
       <c r="EI8" s="172">
-        <f t="shared" ref="EI8" si="81">+IF(EH8&lt;0,0,EH8)</f>
+        <f t="shared" ref="EI8" si="78">+IF(EH8&lt;0,0,EH8)</f>
         <v>0</v>
       </c>
       <c r="EJ8" s="165" t="b">
@@ -27077,38 +27077,22 @@
   </sheetData>
   <autoFilter ref="A6:ER8" xr:uid="{00000000-0001-0000-0900-000000000000}"/>
   <mergeCells count="64">
-    <mergeCell ref="AO1:AS1"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="S4:U4"/>
-    <mergeCell ref="W4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AD4"/>
-    <mergeCell ref="AG4:AI4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="BG4:BI4"/>
-    <mergeCell ref="AT4:AU4"/>
-    <mergeCell ref="AO5:AO6"/>
-    <mergeCell ref="AP5:AP6"/>
-    <mergeCell ref="AQ5:AQ6"/>
-    <mergeCell ref="AR5:AR6"/>
-    <mergeCell ref="AS5:AS6"/>
-    <mergeCell ref="BJ4:BK4"/>
-    <mergeCell ref="BL4:BN4"/>
-    <mergeCell ref="BQ4:BS4"/>
-    <mergeCell ref="BC4:BE4"/>
-    <mergeCell ref="CD5:CD6"/>
-    <mergeCell ref="BY5:BY6"/>
-    <mergeCell ref="BZ5:BZ6"/>
-    <mergeCell ref="CA5:CA6"/>
-    <mergeCell ref="CB5:CB6"/>
-    <mergeCell ref="CC5:CC6"/>
+    <mergeCell ref="EN5:EN6"/>
+    <mergeCell ref="EI5:EI6"/>
+    <mergeCell ref="EJ5:EJ6"/>
+    <mergeCell ref="EK5:EK6"/>
+    <mergeCell ref="EL5:EL6"/>
+    <mergeCell ref="EH5:EH6"/>
+    <mergeCell ref="DV5:DX5"/>
+    <mergeCell ref="CQ5:CS5"/>
+    <mergeCell ref="DG5:DG6"/>
+    <mergeCell ref="DI5:DJ5"/>
+    <mergeCell ref="CT5:CT6"/>
+    <mergeCell ref="DH5:DH6"/>
+    <mergeCell ref="DK5:DK6"/>
+    <mergeCell ref="DM5:DR5"/>
+    <mergeCell ref="DS5:DS6"/>
+    <mergeCell ref="DU5:DU6"/>
     <mergeCell ref="ER5:ER6"/>
     <mergeCell ref="A7:EL7"/>
     <mergeCell ref="EM5:EM6"/>
@@ -27125,22 +27109,38 @@
     <mergeCell ref="DL5:DL6"/>
     <mergeCell ref="EG5:EG6"/>
     <mergeCell ref="EQ5:EQ6"/>
-    <mergeCell ref="EH5:EH6"/>
-    <mergeCell ref="DV5:DX5"/>
-    <mergeCell ref="CQ5:CS5"/>
-    <mergeCell ref="DG5:DG6"/>
-    <mergeCell ref="DI5:DJ5"/>
-    <mergeCell ref="CT5:CT6"/>
-    <mergeCell ref="DH5:DH6"/>
-    <mergeCell ref="DK5:DK6"/>
-    <mergeCell ref="DM5:DR5"/>
-    <mergeCell ref="DS5:DS6"/>
-    <mergeCell ref="DU5:DU6"/>
-    <mergeCell ref="EN5:EN6"/>
-    <mergeCell ref="EI5:EI6"/>
-    <mergeCell ref="EJ5:EJ6"/>
-    <mergeCell ref="EK5:EK6"/>
-    <mergeCell ref="EL5:EL6"/>
+    <mergeCell ref="BJ4:BK4"/>
+    <mergeCell ref="BL4:BN4"/>
+    <mergeCell ref="BQ4:BS4"/>
+    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="CD5:CD6"/>
+    <mergeCell ref="BY5:BY6"/>
+    <mergeCell ref="BZ5:BZ6"/>
+    <mergeCell ref="CA5:CA6"/>
+    <mergeCell ref="CB5:CB6"/>
+    <mergeCell ref="CC5:CC6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="BG4:BI4"/>
+    <mergeCell ref="AT4:AU4"/>
+    <mergeCell ref="AO5:AO6"/>
+    <mergeCell ref="AP5:AP6"/>
+    <mergeCell ref="AQ5:AQ6"/>
+    <mergeCell ref="AR5:AR6"/>
+    <mergeCell ref="AS5:AS6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="AO1:AS1"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="S4:U4"/>
+    <mergeCell ref="W4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="AG4:AI4"/>
   </mergeCells>
   <conditionalFormatting sqref="A5 A8:B8">
     <cfRule type="duplicateValues" dxfId="20" priority="20879"/>
@@ -27797,11 +27797,11 @@
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
       <c r="H8" s="20"/>
-      <c r="I8" s="301">
+      <c r="I8" s="307">
         <v>2026</v>
       </c>
-      <c r="J8" s="302"/>
-      <c r="K8" s="302"/>
+      <c r="J8" s="308"/>
+      <c r="K8" s="308"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="21" t="s">
@@ -27826,13 +27826,13 @@
     <row r="9" spans="1:29" ht="15.75" customHeight="1" thickBot="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="303" t="s">
+      <c r="C9" s="309" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="304"/>
-      <c r="E9" s="304"/>
-      <c r="F9" s="304"/>
-      <c r="G9" s="304"/>
+      <c r="D9" s="310"/>
+      <c r="E9" s="310"/>
+      <c r="F9" s="310"/>
+      <c r="G9" s="310"/>
       <c r="H9" s="20"/>
       <c r="I9" s="24"/>
       <c r="J9" s="24"/>
@@ -27928,19 +27928,19 @@
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
-      <c r="J12" s="305" t="s">
+      <c r="J12" s="311" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="304"/>
-      <c r="L12" s="304"/>
-      <c r="M12" s="304"/>
-      <c r="N12" s="304"/>
-      <c r="O12" s="304"/>
-      <c r="P12" s="306">
+      <c r="K12" s="310"/>
+      <c r="L12" s="310"/>
+      <c r="M12" s="310"/>
+      <c r="N12" s="310"/>
+      <c r="O12" s="310"/>
+      <c r="P12" s="312">
         <f>I8</f>
         <v>2026</v>
       </c>
-      <c r="Q12" s="304"/>
+      <c r="Q12" s="310"/>
       <c r="R12" s="33"/>
       <c r="S12" s="34"/>
       <c r="T12" s="34"/>
@@ -28204,38 +28204,38 @@
     </row>
     <row r="21" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A21" s="39"/>
-      <c r="B21" s="307" t="s">
+      <c r="B21" s="306" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="308"/>
-      <c r="D21" s="308"/>
-      <c r="E21" s="308"/>
-      <c r="F21" s="308"/>
-      <c r="G21" s="308"/>
-      <c r="H21" s="308"/>
-      <c r="I21" s="308"/>
+      <c r="C21" s="302"/>
+      <c r="D21" s="302"/>
+      <c r="E21" s="302"/>
+      <c r="F21" s="302"/>
+      <c r="G21" s="302"/>
+      <c r="H21" s="302"/>
+      <c r="I21" s="302"/>
       <c r="J21" s="40"/>
-      <c r="K21" s="309" t="s">
+      <c r="K21" s="303" t="s">
         <v>37</v>
       </c>
-      <c r="L21" s="308"/>
-      <c r="M21" s="308"/>
-      <c r="N21" s="308"/>
-      <c r="O21" s="308"/>
-      <c r="P21" s="308"/>
-      <c r="Q21" s="308"/>
-      <c r="R21" s="308"/>
+      <c r="L21" s="302"/>
+      <c r="M21" s="302"/>
+      <c r="N21" s="302"/>
+      <c r="O21" s="302"/>
+      <c r="P21" s="302"/>
+      <c r="Q21" s="302"/>
+      <c r="R21" s="302"/>
       <c r="S21" s="40"/>
-      <c r="T21" s="310" t="s">
+      <c r="T21" s="301" t="s">
         <v>38</v>
       </c>
-      <c r="U21" s="308"/>
-      <c r="V21" s="308"/>
-      <c r="W21" s="308"/>
-      <c r="X21" s="308"/>
-      <c r="Y21" s="308"/>
-      <c r="Z21" s="308"/>
-      <c r="AA21" s="308"/>
+      <c r="U21" s="302"/>
+      <c r="V21" s="302"/>
+      <c r="W21" s="302"/>
+      <c r="X21" s="302"/>
+      <c r="Y21" s="302"/>
+      <c r="Z21" s="302"/>
+      <c r="AA21" s="302"/>
       <c r="AB21" s="41"/>
       <c r="AC21" s="42"/>
     </row>
@@ -29135,38 +29135,38 @@
     </row>
     <row r="35" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="311" t="s">
+      <c r="B35" s="304" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="308"/>
-      <c r="D35" s="308"/>
-      <c r="E35" s="308"/>
-      <c r="F35" s="308"/>
-      <c r="G35" s="308"/>
-      <c r="H35" s="308"/>
-      <c r="I35" s="308"/>
+      <c r="C35" s="302"/>
+      <c r="D35" s="302"/>
+      <c r="E35" s="302"/>
+      <c r="F35" s="302"/>
+      <c r="G35" s="302"/>
+      <c r="H35" s="302"/>
+      <c r="I35" s="302"/>
       <c r="J35" s="40"/>
-      <c r="K35" s="312" t="s">
+      <c r="K35" s="305" t="s">
         <v>48</v>
       </c>
-      <c r="L35" s="308"/>
-      <c r="M35" s="308"/>
-      <c r="N35" s="308"/>
-      <c r="O35" s="308"/>
-      <c r="P35" s="308"/>
-      <c r="Q35" s="308"/>
-      <c r="R35" s="308"/>
+      <c r="L35" s="302"/>
+      <c r="M35" s="302"/>
+      <c r="N35" s="302"/>
+      <c r="O35" s="302"/>
+      <c r="P35" s="302"/>
+      <c r="Q35" s="302"/>
+      <c r="R35" s="302"/>
       <c r="S35" s="40"/>
-      <c r="T35" s="309" t="s">
+      <c r="T35" s="303" t="s">
         <v>49</v>
       </c>
-      <c r="U35" s="308"/>
-      <c r="V35" s="308"/>
-      <c r="W35" s="308"/>
-      <c r="X35" s="308"/>
-      <c r="Y35" s="308"/>
-      <c r="Z35" s="308"/>
-      <c r="AA35" s="308"/>
+      <c r="U35" s="302"/>
+      <c r="V35" s="302"/>
+      <c r="W35" s="302"/>
+      <c r="X35" s="302"/>
+      <c r="Y35" s="302"/>
+      <c r="Z35" s="302"/>
+      <c r="AA35" s="302"/>
       <c r="AB35" s="70"/>
       <c r="AC35" s="40"/>
     </row>
@@ -30055,38 +30055,38 @@
     </row>
     <row r="49" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A49" s="69"/>
-      <c r="B49" s="309" t="s">
+      <c r="B49" s="303" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="308"/>
-      <c r="D49" s="308"/>
-      <c r="E49" s="308"/>
-      <c r="F49" s="308"/>
-      <c r="G49" s="308"/>
-      <c r="H49" s="308"/>
-      <c r="I49" s="308"/>
+      <c r="C49" s="302"/>
+      <c r="D49" s="302"/>
+      <c r="E49" s="302"/>
+      <c r="F49" s="302"/>
+      <c r="G49" s="302"/>
+      <c r="H49" s="302"/>
+      <c r="I49" s="302"/>
       <c r="J49" s="40"/>
-      <c r="K49" s="311" t="s">
+      <c r="K49" s="304" t="s">
         <v>51</v>
       </c>
-      <c r="L49" s="308"/>
-      <c r="M49" s="308"/>
-      <c r="N49" s="308"/>
-      <c r="O49" s="308"/>
-      <c r="P49" s="308"/>
-      <c r="Q49" s="308"/>
-      <c r="R49" s="308"/>
+      <c r="L49" s="302"/>
+      <c r="M49" s="302"/>
+      <c r="N49" s="302"/>
+      <c r="O49" s="302"/>
+      <c r="P49" s="302"/>
+      <c r="Q49" s="302"/>
+      <c r="R49" s="302"/>
       <c r="S49" s="40"/>
-      <c r="T49" s="307" t="s">
+      <c r="T49" s="306" t="s">
         <v>52</v>
       </c>
-      <c r="U49" s="308"/>
-      <c r="V49" s="308"/>
-      <c r="W49" s="308"/>
-      <c r="X49" s="308"/>
-      <c r="Y49" s="308"/>
-      <c r="Z49" s="308"/>
-      <c r="AA49" s="308"/>
+      <c r="U49" s="302"/>
+      <c r="V49" s="302"/>
+      <c r="W49" s="302"/>
+      <c r="X49" s="302"/>
+      <c r="Y49" s="302"/>
+      <c r="Z49" s="302"/>
+      <c r="AA49" s="302"/>
       <c r="AB49" s="70"/>
       <c r="AC49" s="40"/>
     </row>
@@ -30975,38 +30975,38 @@
     </row>
     <row r="63" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A63" s="69"/>
-      <c r="B63" s="310" t="s">
+      <c r="B63" s="301" t="s">
         <v>53</v>
       </c>
-      <c r="C63" s="308"/>
-      <c r="D63" s="308"/>
-      <c r="E63" s="308"/>
-      <c r="F63" s="308"/>
-      <c r="G63" s="308"/>
-      <c r="H63" s="308"/>
-      <c r="I63" s="308"/>
+      <c r="C63" s="302"/>
+      <c r="D63" s="302"/>
+      <c r="E63" s="302"/>
+      <c r="F63" s="302"/>
+      <c r="G63" s="302"/>
+      <c r="H63" s="302"/>
+      <c r="I63" s="302"/>
       <c r="J63" s="40"/>
-      <c r="K63" s="309" t="s">
+      <c r="K63" s="303" t="s">
         <v>54</v>
       </c>
-      <c r="L63" s="308"/>
-      <c r="M63" s="308"/>
-      <c r="N63" s="308"/>
-      <c r="O63" s="308"/>
-      <c r="P63" s="308"/>
-      <c r="Q63" s="308"/>
-      <c r="R63" s="308"/>
+      <c r="L63" s="302"/>
+      <c r="M63" s="302"/>
+      <c r="N63" s="302"/>
+      <c r="O63" s="302"/>
+      <c r="P63" s="302"/>
+      <c r="Q63" s="302"/>
+      <c r="R63" s="302"/>
       <c r="S63" s="40"/>
-      <c r="T63" s="311" t="s">
+      <c r="T63" s="304" t="s">
         <v>55</v>
       </c>
-      <c r="U63" s="308"/>
-      <c r="V63" s="308"/>
-      <c r="W63" s="308"/>
-      <c r="X63" s="308"/>
-      <c r="Y63" s="308"/>
-      <c r="Z63" s="308"/>
-      <c r="AA63" s="308"/>
+      <c r="U63" s="302"/>
+      <c r="V63" s="302"/>
+      <c r="W63" s="302"/>
+      <c r="X63" s="302"/>
+      <c r="Y63" s="302"/>
+      <c r="Z63" s="302"/>
+      <c r="AA63" s="302"/>
       <c r="AB63" s="70"/>
       <c r="AC63" s="40"/>
     </row>
@@ -60541,6 +60541,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="J12:O12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="K21:R21"/>
     <mergeCell ref="B63:I63"/>
     <mergeCell ref="K63:R63"/>
     <mergeCell ref="T63:AA63"/>
@@ -60551,12 +60557,6 @@
     <mergeCell ref="B49:I49"/>
     <mergeCell ref="K49:R49"/>
     <mergeCell ref="T49:AA49"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="J12:O12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="K21:R21"/>
   </mergeCells>
   <conditionalFormatting sqref="C51:I55">
     <cfRule type="expression" dxfId="2" priority="3">

</xml_diff>

<commit_message>
- fix cách tính điểm kpi , tính từng bước 1 nó mới không sai
</commit_message>
<xml_diff>
--- a/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
+++ b/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonzai/dev/odoo 19/odoo/my_custom_addons/dl_salary_kpi/static/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F823649D-7A95-C24F-896C-7B74BD7D0E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{663DD088-5A8E-1B4F-8E8A-045185F17206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
           <rPr>
             <b/>
             <sz val="12"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -92,7 +92,7 @@
         <r>
           <rPr>
             <sz val="9"/>
-            <color indexed="81"/>
+            <color rgb="FF000000"/>
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
@@ -552,7 +552,7 @@
     <numFmt numFmtId="174" formatCode="\TGeneral"/>
     <numFmt numFmtId="175" formatCode="_-* #,##0.0\ _₫_-;\-* #,##0.0\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
   </numFmts>
-  <fonts count="84">
+  <fonts count="86">
     <font>
       <sz val="10"/>
       <name val="Encysoft Times"/>
@@ -1085,6 +1085,19 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="25">
@@ -2408,82 +2421,16 @@
     <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="66" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="67" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="67" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2519,33 +2466,83 @@
     <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="66" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="67" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="7" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2560,6 +2557,22 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="32">
@@ -2820,7 +2833,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4095750" y="266700"/>
+          <a:off x="4870450" y="266700"/>
           <a:ext cx="914400" cy="38100"/>
           <a:chOff x="4888800" y="3780000"/>
           <a:chExt cx="914400" cy="0"/>
@@ -3261,86 +3274,86 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:ER165"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="20" outlineLevelCol="2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="20" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="17.796875" style="95" customWidth="1"/>
-    <col min="2" max="2" width="30.19921875" style="95" customWidth="1"/>
-    <col min="3" max="3" width="45.796875" style="94" customWidth="1"/>
-    <col min="4" max="4" width="24.3984375" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="5" width="29.19921875" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="6" max="6" width="15.3984375" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="7" max="7" width="31.796875" style="220" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="8" max="8" width="13.796875" style="95" customWidth="1" collapsed="1"/>
-    <col min="9" max="9" width="25.19921875" style="101" customWidth="1"/>
-    <col min="10" max="40" width="11.796875" style="1" customWidth="1" outlineLevel="1"/>
-    <col min="41" max="43" width="15.796875" style="92" customWidth="1" outlineLevel="1"/>
-    <col min="44" max="44" width="14.3984375" style="1" customWidth="1" outlineLevel="1"/>
-    <col min="45" max="45" width="14.59765625" style="228" customWidth="1" outlineLevel="1"/>
+    <col min="1" max="1" width="17.83203125" style="95" customWidth="1"/>
+    <col min="2" max="2" width="30.1640625" style="95" customWidth="1"/>
+    <col min="3" max="3" width="45.83203125" style="94" customWidth="1"/>
+    <col min="4" max="4" width="24.33203125" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="29.1640625" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="15.33203125" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="31.83203125" style="220" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="13.83203125" style="95" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="25.1640625" style="101" customWidth="1"/>
+    <col min="10" max="40" width="11.83203125" style="1" customWidth="1" outlineLevel="1"/>
+    <col min="41" max="43" width="15.83203125" style="92" customWidth="1" outlineLevel="1"/>
+    <col min="44" max="44" width="14.33203125" style="1" customWidth="1" outlineLevel="1"/>
+    <col min="45" max="45" width="14.6640625" style="228" customWidth="1" outlineLevel="1"/>
     <col min="46" max="54" width="13" style="1" customWidth="1" outlineLevel="1"/>
     <col min="55" max="55" width="13" style="102" customWidth="1" outlineLevel="1"/>
     <col min="56" max="59" width="13" style="1" customWidth="1" outlineLevel="1"/>
-    <col min="60" max="60" width="15.796875" style="1" customWidth="1" outlineLevel="1"/>
+    <col min="60" max="60" width="15.83203125" style="1" customWidth="1" outlineLevel="1"/>
     <col min="61" max="66" width="13" style="1" customWidth="1" outlineLevel="1"/>
-    <col min="67" max="67" width="15.19921875" style="1" customWidth="1" outlineLevel="1"/>
+    <col min="67" max="67" width="15.1640625" style="1" customWidth="1" outlineLevel="1"/>
     <col min="68" max="73" width="13" style="1" customWidth="1" outlineLevel="1"/>
     <col min="74" max="74" width="15" style="1" customWidth="1" outlineLevel="1"/>
     <col min="75" max="76" width="13" style="1" customWidth="1" outlineLevel="1"/>
-    <col min="77" max="83" width="15.59765625" style="136" customWidth="1" outlineLevel="1"/>
-    <col min="84" max="84" width="17.59765625" style="147" customWidth="1"/>
-    <col min="85" max="85" width="16.59765625" style="136" customWidth="1"/>
+    <col min="77" max="83" width="15.6640625" style="136" customWidth="1" outlineLevel="1"/>
+    <col min="84" max="84" width="17.6640625" style="147" customWidth="1"/>
+    <col min="85" max="85" width="16.6640625" style="136" customWidth="1"/>
     <col min="86" max="86" width="14" style="147" customWidth="1"/>
-    <col min="87" max="87" width="15.796875" style="147" customWidth="1"/>
-    <col min="88" max="88" width="16.796875" style="136" customWidth="1"/>
+    <col min="87" max="87" width="15.83203125" style="147" customWidth="1"/>
+    <col min="88" max="88" width="16.83203125" style="136" customWidth="1"/>
     <col min="89" max="93" width="14" style="136" customWidth="1"/>
     <col min="94" max="94" width="14" style="136" customWidth="1" outlineLevel="1"/>
-    <col min="95" max="95" width="26.19921875" style="1" customWidth="1" outlineLevel="1"/>
-    <col min="96" max="96" width="26.19921875" style="102" customWidth="1" outlineLevel="1"/>
-    <col min="97" max="97" width="26.19921875" style="225" customWidth="1" outlineLevel="1"/>
-    <col min="98" max="98" width="24.19921875" style="102" customWidth="1" outlineLevel="1"/>
+    <col min="95" max="95" width="26.1640625" style="1" customWidth="1" outlineLevel="1"/>
+    <col min="96" max="96" width="26.1640625" style="102" customWidth="1" outlineLevel="1"/>
+    <col min="97" max="97" width="26.1640625" style="225" customWidth="1" outlineLevel="1"/>
+    <col min="98" max="98" width="24.1640625" style="102" customWidth="1" outlineLevel="1"/>
     <col min="99" max="99" width="26" style="136" customWidth="1"/>
-    <col min="100" max="100" width="21.796875" style="136" customWidth="1"/>
-    <col min="101" max="101" width="21.19921875" style="136" customWidth="1"/>
-    <col min="102" max="102" width="18.59765625" style="136" customWidth="1"/>
-    <col min="103" max="103" width="16.19921875" style="136" customWidth="1"/>
-    <col min="104" max="104" width="18.59765625" style="136" customWidth="1"/>
-    <col min="105" max="105" width="20.796875" style="136" customWidth="1"/>
-    <col min="106" max="107" width="16.3984375" style="136" customWidth="1"/>
-    <col min="108" max="108" width="23.3984375" style="136" customWidth="1"/>
-    <col min="109" max="110" width="27.796875" style="210" customWidth="1"/>
-    <col min="111" max="111" width="27.796875" style="255" customWidth="1"/>
-    <col min="112" max="112" width="25.19921875" style="136" customWidth="1"/>
-    <col min="113" max="113" width="22.59765625" style="102" customWidth="1"/>
-    <col min="114" max="114" width="24.796875" style="102" customWidth="1"/>
-    <col min="115" max="115" width="27.59765625" style="102" customWidth="1"/>
-    <col min="116" max="116" width="33.796875" style="102" customWidth="1"/>
-    <col min="117" max="119" width="25.796875" style="102" customWidth="1"/>
-    <col min="120" max="120" width="20.796875" style="143" customWidth="1"/>
-    <col min="121" max="121" width="22.19921875" style="143" customWidth="1"/>
-    <col min="122" max="122" width="22.796875" style="143" customWidth="1"/>
-    <col min="123" max="123" width="31.796875" style="102" customWidth="1"/>
-    <col min="124" max="124" width="26.59765625" style="102" customWidth="1"/>
-    <col min="125" max="125" width="24.796875" style="102" customWidth="1" outlineLevel="2"/>
-    <col min="126" max="126" width="27.3984375" style="102" customWidth="1" outlineLevel="2"/>
-    <col min="127" max="127" width="27.3984375" style="99" customWidth="1" outlineLevel="2"/>
-    <col min="128" max="128" width="27.3984375" style="102" customWidth="1" outlineLevel="2"/>
-    <col min="129" max="129" width="23.59765625" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="130" max="131" width="22.19921875" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="132" max="132" width="28.19921875" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="133" max="133" width="27.796875" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="134" max="134" width="28.796875" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="135" max="135" width="29.19921875" style="102" customWidth="1" outlineLevel="2"/>
-    <col min="136" max="136" width="21.796875" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="137" max="137" width="25.3984375" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="138" max="138" width="24.19921875" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="139" max="139" width="21.19921875" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="100" max="100" width="21.83203125" style="136" customWidth="1"/>
+    <col min="101" max="101" width="21.1640625" style="136" customWidth="1"/>
+    <col min="102" max="102" width="18.6640625" style="136" customWidth="1"/>
+    <col min="103" max="103" width="16.1640625" style="136" customWidth="1"/>
+    <col min="104" max="104" width="18.6640625" style="136" customWidth="1"/>
+    <col min="105" max="105" width="20.83203125" style="136" customWidth="1"/>
+    <col min="106" max="107" width="16.33203125" style="136" customWidth="1"/>
+    <col min="108" max="108" width="23.33203125" style="136" customWidth="1"/>
+    <col min="109" max="110" width="27.83203125" style="210" customWidth="1"/>
+    <col min="111" max="111" width="27.83203125" style="255" customWidth="1"/>
+    <col min="112" max="112" width="25.1640625" style="136" customWidth="1"/>
+    <col min="113" max="113" width="22.6640625" style="102" customWidth="1"/>
+    <col min="114" max="114" width="24.83203125" style="102" customWidth="1"/>
+    <col min="115" max="115" width="27.6640625" style="102" customWidth="1"/>
+    <col min="116" max="116" width="33.83203125" style="102" customWidth="1"/>
+    <col min="117" max="119" width="25.83203125" style="102" customWidth="1"/>
+    <col min="120" max="120" width="20.83203125" style="143" customWidth="1"/>
+    <col min="121" max="121" width="22.1640625" style="143" customWidth="1"/>
+    <col min="122" max="122" width="22.83203125" style="143" customWidth="1"/>
+    <col min="123" max="123" width="31.83203125" style="102" customWidth="1"/>
+    <col min="124" max="124" width="26.6640625" style="102" customWidth="1"/>
+    <col min="125" max="125" width="24.83203125" style="102" customWidth="1" outlineLevel="2"/>
+    <col min="126" max="126" width="27.33203125" style="102" customWidth="1" outlineLevel="2"/>
+    <col min="127" max="127" width="27.33203125" style="99" customWidth="1" outlineLevel="2"/>
+    <col min="128" max="128" width="27.33203125" style="102" customWidth="1" outlineLevel="2"/>
+    <col min="129" max="129" width="23.6640625" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="130" max="131" width="22.1640625" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="132" max="132" width="28.1640625" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="133" max="133" width="27.83203125" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="134" max="134" width="28.83203125" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="135" max="135" width="29.1640625" style="102" customWidth="1" outlineLevel="2"/>
+    <col min="136" max="136" width="21.83203125" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="137" max="137" width="25.33203125" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="138" max="138" width="24.1640625" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="139" max="139" width="21.1640625" style="94" customWidth="1" outlineLevel="2"/>
     <col min="140" max="140" width="25" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="141" max="141" width="29.19921875" style="95" customWidth="1" outlineLevel="2"/>
-    <col min="142" max="145" width="31.59765625" style="95" customWidth="1" outlineLevel="2"/>
-    <col min="146" max="146" width="36.3984375" style="95" customWidth="1"/>
-    <col min="147" max="147" width="35.796875" style="95" customWidth="1"/>
-    <col min="148" max="148" width="41.796875" style="242" customWidth="1"/>
-    <col min="149" max="150" width="9.19921875" style="94" customWidth="1"/>
-    <col min="151" max="16384" width="9.19921875" style="94"/>
+    <col min="141" max="141" width="29.1640625" style="95" customWidth="1" outlineLevel="2"/>
+    <col min="142" max="145" width="31.6640625" style="95" customWidth="1" outlineLevel="2"/>
+    <col min="146" max="146" width="36.33203125" style="95" customWidth="1"/>
+    <col min="147" max="147" width="35.83203125" style="95" customWidth="1"/>
+    <col min="148" max="148" width="41.83203125" style="242" customWidth="1"/>
+    <col min="149" max="150" width="9.1640625" style="94" customWidth="1"/>
+    <col min="151" max="16384" width="9.1640625" style="94"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:148" s="127" customFormat="1" ht="37.5" customHeight="1">
@@ -3384,11 +3397,11 @@
       <c r="AL1" s="212"/>
       <c r="AM1" s="212"/>
       <c r="AN1" s="212"/>
-      <c r="AO1" s="260"/>
-      <c r="AP1" s="260"/>
-      <c r="AQ1" s="260"/>
-      <c r="AR1" s="260"/>
-      <c r="AS1" s="260"/>
+      <c r="AO1" s="300"/>
+      <c r="AP1" s="300"/>
+      <c r="AQ1" s="300"/>
+      <c r="AR1" s="300"/>
+      <c r="AS1" s="300"/>
       <c r="AT1" s="120"/>
       <c r="AU1" s="120"/>
       <c r="AV1" s="120"/>
@@ -3790,10 +3803,10 @@
       <c r="G4" s="232"/>
       <c r="H4" s="108"/>
       <c r="I4" s="256"/>
-      <c r="J4" s="261" t="s">
+      <c r="J4" s="293" t="s">
         <v>68</v>
       </c>
-      <c r="K4" s="261"/>
+      <c r="K4" s="293"/>
       <c r="L4" s="258">
         <v>3</v>
       </c>
@@ -3807,23 +3820,23 @@
       </c>
       <c r="Q4" s="259"/>
       <c r="R4" s="109"/>
-      <c r="S4" s="261"/>
-      <c r="T4" s="261"/>
-      <c r="U4" s="261"/>
+      <c r="S4" s="293"/>
+      <c r="T4" s="293"/>
+      <c r="U4" s="293"/>
       <c r="V4" s="109"/>
-      <c r="W4" s="261"/>
-      <c r="X4" s="261"/>
-      <c r="Y4" s="261"/>
-      <c r="Z4" s="261"/>
-      <c r="AA4" s="261"/>
-      <c r="AB4" s="261"/>
-      <c r="AC4" s="261"/>
-      <c r="AD4" s="261"/>
+      <c r="W4" s="293"/>
+      <c r="X4" s="293"/>
+      <c r="Y4" s="293"/>
+      <c r="Z4" s="293"/>
+      <c r="AA4" s="293"/>
+      <c r="AB4" s="293"/>
+      <c r="AC4" s="293"/>
+      <c r="AD4" s="293"/>
       <c r="AE4" s="109"/>
       <c r="AF4" s="110"/>
-      <c r="AG4" s="261"/>
-      <c r="AH4" s="261"/>
-      <c r="AI4" s="261"/>
+      <c r="AG4" s="293"/>
+      <c r="AH4" s="293"/>
+      <c r="AI4" s="293"/>
       <c r="AJ4" s="109"/>
       <c r="AK4" s="109"/>
       <c r="AL4" s="109"/>
@@ -3834,10 +3847,10 @@
       <c r="AQ4" s="113"/>
       <c r="AR4" s="221"/>
       <c r="AS4" s="227"/>
-      <c r="AT4" s="261" t="s">
+      <c r="AT4" s="293" t="s">
         <v>68</v>
       </c>
-      <c r="AU4" s="261"/>
+      <c r="AU4" s="293"/>
       <c r="AV4" s="258">
         <f>L4</f>
         <v>3</v>
@@ -3853,23 +3866,23 @@
       </c>
       <c r="BA4" s="259"/>
       <c r="BB4" s="109"/>
-      <c r="BC4" s="261"/>
-      <c r="BD4" s="261"/>
-      <c r="BE4" s="261"/>
+      <c r="BC4" s="293"/>
+      <c r="BD4" s="293"/>
+      <c r="BE4" s="293"/>
       <c r="BF4" s="109"/>
-      <c r="BG4" s="261"/>
-      <c r="BH4" s="261"/>
-      <c r="BI4" s="261"/>
-      <c r="BJ4" s="261"/>
-      <c r="BK4" s="261"/>
-      <c r="BL4" s="261"/>
-      <c r="BM4" s="261"/>
-      <c r="BN4" s="261"/>
+      <c r="BG4" s="293"/>
+      <c r="BH4" s="293"/>
+      <c r="BI4" s="293"/>
+      <c r="BJ4" s="293"/>
+      <c r="BK4" s="293"/>
+      <c r="BL4" s="293"/>
+      <c r="BM4" s="293"/>
+      <c r="BN4" s="293"/>
       <c r="BO4" s="109"/>
       <c r="BP4" s="110"/>
-      <c r="BQ4" s="261"/>
-      <c r="BR4" s="261"/>
-      <c r="BS4" s="261"/>
+      <c r="BQ4" s="293"/>
+      <c r="BR4" s="293"/>
+      <c r="BS4" s="293"/>
       <c r="BT4" s="114"/>
       <c r="BU4" s="114" t="str">
         <f>IF(WEEKDAY(BU5,1)=1,"CN","")</f>
@@ -3949,31 +3962,31 @@
       <c r="ER4" s="237"/>
     </row>
     <row r="5" spans="1:148" s="183" customFormat="1" ht="92.25" customHeight="1">
-      <c r="A5" s="262" t="s">
+      <c r="A5" s="288" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="263" t="s">
+      <c r="B5" s="278" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="262" t="s">
+      <c r="C5" s="288" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="264" t="s">
+      <c r="D5" s="297" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="265" t="s">
+      <c r="E5" s="298" t="s">
         <v>120</v>
       </c>
-      <c r="F5" s="262" t="s">
+      <c r="F5" s="288" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="262" t="s">
+      <c r="G5" s="288" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="262" t="s">
+      <c r="H5" s="288" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="267" t="s">
+      <c r="I5" s="294" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="174">
@@ -4100,19 +4113,19 @@
         <f t="shared" si="0"/>
         <v>46112</v>
       </c>
-      <c r="AO5" s="268" t="s">
+      <c r="AO5" s="295" t="s">
         <v>82</v>
       </c>
-      <c r="AP5" s="268" t="s">
+      <c r="AP5" s="295" t="s">
         <v>83</v>
       </c>
-      <c r="AQ5" s="268" t="s">
+      <c r="AQ5" s="295" t="s">
         <v>84</v>
       </c>
-      <c r="AR5" s="269" t="s">
+      <c r="AR5" s="296" t="s">
         <v>5</v>
       </c>
-      <c r="AS5" s="269" t="s">
+      <c r="AS5" s="296" t="s">
         <v>6</v>
       </c>
       <c r="AT5" s="178">
@@ -4239,46 +4252,46 @@
         <f t="shared" si="1"/>
         <v>46112</v>
       </c>
-      <c r="BY5" s="270" t="s">
+      <c r="BY5" s="290" t="s">
         <v>85</v>
       </c>
-      <c r="BZ5" s="270" t="s">
+      <c r="BZ5" s="290" t="s">
         <v>86</v>
       </c>
-      <c r="CA5" s="270" t="s">
+      <c r="CA5" s="290" t="s">
         <v>87</v>
       </c>
-      <c r="CB5" s="270" t="s">
+      <c r="CB5" s="290" t="s">
         <v>88</v>
       </c>
-      <c r="CC5" s="270" t="s">
+      <c r="CC5" s="290" t="s">
         <v>89</v>
       </c>
-      <c r="CD5" s="270" t="s">
+      <c r="CD5" s="290" t="s">
         <v>90</v>
       </c>
-      <c r="CE5" s="270" t="s">
+      <c r="CE5" s="290" t="s">
         <v>91</v>
       </c>
-      <c r="CF5" s="284" t="s">
+      <c r="CF5" s="289" t="s">
         <v>19</v>
       </c>
-      <c r="CG5" s="284"/>
-      <c r="CH5" s="284"/>
-      <c r="CI5" s="284"/>
-      <c r="CJ5" s="284"/>
-      <c r="CK5" s="284"/>
-      <c r="CL5" s="284"/>
-      <c r="CM5" s="284"/>
-      <c r="CN5" s="284"/>
-      <c r="CO5" s="284"/>
-      <c r="CP5" s="284"/>
-      <c r="CQ5" s="288" t="s">
+      <c r="CG5" s="289"/>
+      <c r="CH5" s="289"/>
+      <c r="CI5" s="289"/>
+      <c r="CJ5" s="289"/>
+      <c r="CK5" s="289"/>
+      <c r="CL5" s="289"/>
+      <c r="CM5" s="289"/>
+      <c r="CN5" s="289"/>
+      <c r="CO5" s="289"/>
+      <c r="CP5" s="289"/>
+      <c r="CQ5" s="266" t="s">
         <v>59</v>
       </c>
-      <c r="CR5" s="289"/>
-      <c r="CS5" s="290"/>
-      <c r="CT5" s="295" t="s">
+      <c r="CR5" s="267"/>
+      <c r="CS5" s="268"/>
+      <c r="CT5" s="273" t="s">
         <v>60</v>
       </c>
       <c r="CU5" s="247" t="s">
@@ -4301,107 +4314,107 @@
       <c r="DF5" s="245" t="s">
         <v>127</v>
       </c>
-      <c r="DG5" s="291" t="s">
+      <c r="DG5" s="269" t="s">
         <v>117</v>
       </c>
-      <c r="DH5" s="296" t="s">
+      <c r="DH5" s="274" t="s">
         <v>112</v>
       </c>
-      <c r="DI5" s="293" t="s">
+      <c r="DI5" s="271" t="s">
         <v>81</v>
       </c>
-      <c r="DJ5" s="294"/>
-      <c r="DK5" s="281" t="s">
+      <c r="DJ5" s="272"/>
+      <c r="DK5" s="275" t="s">
         <v>61</v>
       </c>
-      <c r="DL5" s="285" t="s">
+      <c r="DL5" s="292" t="s">
         <v>8</v>
       </c>
-      <c r="DM5" s="282" t="s">
+      <c r="DM5" s="276" t="s">
         <v>71</v>
       </c>
-      <c r="DN5" s="282"/>
-      <c r="DO5" s="282"/>
-      <c r="DP5" s="282"/>
-      <c r="DQ5" s="282"/>
-      <c r="DR5" s="282"/>
-      <c r="DS5" s="297" t="s">
+      <c r="DN5" s="276"/>
+      <c r="DO5" s="276"/>
+      <c r="DP5" s="276"/>
+      <c r="DQ5" s="276"/>
+      <c r="DR5" s="276"/>
+      <c r="DS5" s="277" t="s">
         <v>12</v>
       </c>
-      <c r="DT5" s="282" t="s">
+      <c r="DT5" s="276" t="s">
         <v>125</v>
       </c>
-      <c r="DU5" s="263" t="s">
+      <c r="DU5" s="278" t="s">
         <v>13</v>
       </c>
-      <c r="DV5" s="286" t="s">
+      <c r="DV5" s="264" t="s">
         <v>64</v>
       </c>
-      <c r="DW5" s="287"/>
-      <c r="DX5" s="286"/>
-      <c r="DY5" s="279" t="s">
+      <c r="DW5" s="265"/>
+      <c r="DX5" s="264"/>
+      <c r="DY5" s="286" t="s">
         <v>63</v>
       </c>
-      <c r="DZ5" s="279"/>
-      <c r="EA5" s="279"/>
-      <c r="EB5" s="279"/>
-      <c r="EC5" s="280" t="s">
+      <c r="DZ5" s="286"/>
+      <c r="EA5" s="286"/>
+      <c r="EB5" s="286"/>
+      <c r="EC5" s="287" t="s">
         <v>128</v>
       </c>
-      <c r="ED5" s="282" t="s">
+      <c r="ED5" s="276" t="s">
         <v>7</v>
       </c>
-      <c r="EE5" s="283" t="s">
+      <c r="EE5" s="262" t="s">
         <v>65</v>
       </c>
-      <c r="EF5" s="283"/>
-      <c r="EG5" s="283" t="s">
+      <c r="EF5" s="262"/>
+      <c r="EG5" s="262" t="s">
         <v>66</v>
       </c>
-      <c r="EH5" s="283" t="s">
+      <c r="EH5" s="262" t="s">
         <v>67</v>
       </c>
-      <c r="EI5" s="283" t="s">
+      <c r="EI5" s="262" t="s">
         <v>72</v>
       </c>
-      <c r="EJ5" s="300" t="s">
+      <c r="EJ5" s="263" t="s">
         <v>78</v>
       </c>
-      <c r="EK5" s="300" t="s">
+      <c r="EK5" s="263" t="s">
         <v>80</v>
       </c>
-      <c r="EL5" s="300" t="s">
+      <c r="EL5" s="263" t="s">
         <v>79</v>
       </c>
-      <c r="EM5" s="274" t="s">
+      <c r="EM5" s="281" t="s">
         <v>124</v>
       </c>
-      <c r="EN5" s="298" t="s">
+      <c r="EN5" s="260" t="s">
         <v>118</v>
       </c>
-      <c r="EO5" s="276" t="s">
+      <c r="EO5" s="283" t="s">
         <v>130</v>
       </c>
-      <c r="EP5" s="278" t="s">
+      <c r="EP5" s="285" t="s">
         <v>122</v>
       </c>
-      <c r="EQ5" s="278" t="s">
+      <c r="EQ5" s="285" t="s">
         <v>121</v>
       </c>
-      <c r="ER5" s="272" t="s">
+      <c r="ER5" s="279" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:148" s="205" customFormat="1" ht="148.5" customHeight="1">
-      <c r="A6" s="262"/>
-      <c r="B6" s="263"/>
-      <c r="C6" s="262"/>
-      <c r="D6" s="264"/>
-      <c r="E6" s="266"/>
-      <c r="F6" s="262"/>
-      <c r="G6" s="262"/>
-      <c r="H6" s="262"/>
-      <c r="I6" s="267"/>
+      <c r="A6" s="288"/>
+      <c r="B6" s="278"/>
+      <c r="C6" s="288"/>
+      <c r="D6" s="297"/>
+      <c r="E6" s="299"/>
+      <c r="F6" s="288"/>
+      <c r="G6" s="288"/>
+      <c r="H6" s="288"/>
+      <c r="I6" s="294"/>
       <c r="J6" s="184" t="str">
         <f t="shared" ref="J6:AN6" si="2">IF(WEEKDAY(J5)=1,"CN",WEEKDAY(J5))</f>
         <v>CN</v>
@@ -4526,11 +4539,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AO6" s="268"/>
-      <c r="AP6" s="268"/>
-      <c r="AQ6" s="268"/>
-      <c r="AR6" s="269"/>
-      <c r="AS6" s="269"/>
+      <c r="AO6" s="295"/>
+      <c r="AP6" s="295"/>
+      <c r="AQ6" s="295"/>
+      <c r="AR6" s="296"/>
+      <c r="AS6" s="296"/>
       <c r="AT6" s="186" t="str">
         <f>+J6</f>
         <v>CN</v>
@@ -4655,13 +4668,13 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="BY6" s="271"/>
-      <c r="BZ6" s="271"/>
-      <c r="CA6" s="271"/>
-      <c r="CB6" s="271"/>
-      <c r="CC6" s="271"/>
-      <c r="CD6" s="271"/>
-      <c r="CE6" s="271"/>
+      <c r="BY6" s="291"/>
+      <c r="BZ6" s="291"/>
+      <c r="CA6" s="291"/>
+      <c r="CB6" s="291"/>
+      <c r="CC6" s="291"/>
+      <c r="CD6" s="291"/>
+      <c r="CE6" s="291"/>
       <c r="CF6" s="188" t="s">
         <v>92</v>
       </c>
@@ -4704,7 +4717,7 @@
       <c r="CS6" s="180" t="s">
         <v>58</v>
       </c>
-      <c r="CT6" s="295"/>
+      <c r="CT6" s="273"/>
       <c r="CU6" s="188" t="s">
         <v>103</v>
       </c>
@@ -4741,16 +4754,16 @@
       <c r="DF6" s="246" t="s">
         <v>129</v>
       </c>
-      <c r="DG6" s="292"/>
-      <c r="DH6" s="296"/>
+      <c r="DG6" s="270"/>
+      <c r="DH6" s="274"/>
       <c r="DI6" s="152" t="s">
         <v>14</v>
       </c>
       <c r="DJ6" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="DK6" s="281"/>
-      <c r="DL6" s="285"/>
+      <c r="DK6" s="275"/>
+      <c r="DL6" s="292"/>
       <c r="DM6" s="180" t="s">
         <v>9</v>
       </c>
@@ -4769,9 +4782,9 @@
       <c r="DR6" s="180" t="s">
         <v>115</v>
       </c>
-      <c r="DS6" s="297"/>
-      <c r="DT6" s="282"/>
-      <c r="DU6" s="263"/>
+      <c r="DS6" s="277"/>
+      <c r="DT6" s="276"/>
+      <c r="DU6" s="278"/>
       <c r="DV6" s="203">
         <v>0.17499999999999999</v>
       </c>
@@ -4793,170 +4806,170 @@
       <c r="EB6" s="152" t="s">
         <v>62</v>
       </c>
-      <c r="EC6" s="281"/>
-      <c r="ED6" s="282"/>
+      <c r="EC6" s="275"/>
+      <c r="ED6" s="276"/>
       <c r="EE6" s="182" t="s">
         <v>73</v>
       </c>
       <c r="EF6" s="182" t="s">
         <v>74</v>
       </c>
-      <c r="EG6" s="283"/>
-      <c r="EH6" s="283"/>
-      <c r="EI6" s="283"/>
-      <c r="EJ6" s="300"/>
-      <c r="EK6" s="300"/>
-      <c r="EL6" s="300"/>
-      <c r="EM6" s="275"/>
-      <c r="EN6" s="299"/>
-      <c r="EO6" s="277"/>
-      <c r="EP6" s="278"/>
-      <c r="EQ6" s="278"/>
-      <c r="ER6" s="272"/>
+      <c r="EG6" s="262"/>
+      <c r="EH6" s="262"/>
+      <c r="EI6" s="262"/>
+      <c r="EJ6" s="263"/>
+      <c r="EK6" s="263"/>
+      <c r="EL6" s="263"/>
+      <c r="EM6" s="282"/>
+      <c r="EN6" s="261"/>
+      <c r="EO6" s="284"/>
+      <c r="EP6" s="285"/>
+      <c r="EQ6" s="285"/>
+      <c r="ER6" s="279"/>
     </row>
     <row r="7" spans="1:148" s="106" customFormat="1" ht="87.75" customHeight="1">
-      <c r="A7" s="273"/>
-      <c r="B7" s="273"/>
-      <c r="C7" s="273"/>
-      <c r="D7" s="273"/>
-      <c r="E7" s="273"/>
-      <c r="F7" s="273"/>
-      <c r="G7" s="273"/>
-      <c r="H7" s="273"/>
-      <c r="I7" s="273"/>
-      <c r="J7" s="273"/>
-      <c r="K7" s="273"/>
-      <c r="L7" s="273"/>
-      <c r="M7" s="273"/>
-      <c r="N7" s="273"/>
-      <c r="O7" s="273"/>
-      <c r="P7" s="273"/>
-      <c r="Q7" s="273"/>
-      <c r="R7" s="273"/>
-      <c r="S7" s="273"/>
-      <c r="T7" s="273"/>
-      <c r="U7" s="273"/>
-      <c r="V7" s="273"/>
-      <c r="W7" s="273"/>
-      <c r="X7" s="273"/>
-      <c r="Y7" s="273"/>
-      <c r="Z7" s="273"/>
-      <c r="AA7" s="273"/>
-      <c r="AB7" s="273"/>
-      <c r="AC7" s="273"/>
-      <c r="AD7" s="273"/>
-      <c r="AE7" s="273"/>
-      <c r="AF7" s="273"/>
-      <c r="AG7" s="273"/>
-      <c r="AH7" s="273"/>
-      <c r="AI7" s="273"/>
-      <c r="AJ7" s="273"/>
-      <c r="AK7" s="273"/>
-      <c r="AL7" s="273"/>
-      <c r="AM7" s="273"/>
-      <c r="AN7" s="273"/>
-      <c r="AO7" s="273"/>
-      <c r="AP7" s="273"/>
-      <c r="AQ7" s="273"/>
-      <c r="AR7" s="273"/>
-      <c r="AS7" s="273"/>
-      <c r="AT7" s="273"/>
-      <c r="AU7" s="273"/>
-      <c r="AV7" s="273"/>
-      <c r="AW7" s="273"/>
-      <c r="AX7" s="273"/>
-      <c r="AY7" s="273"/>
-      <c r="AZ7" s="273"/>
-      <c r="BA7" s="273"/>
-      <c r="BB7" s="273"/>
-      <c r="BC7" s="273"/>
-      <c r="BD7" s="273"/>
-      <c r="BE7" s="273"/>
-      <c r="BF7" s="273"/>
-      <c r="BG7" s="273"/>
-      <c r="BH7" s="273"/>
-      <c r="BI7" s="273"/>
-      <c r="BJ7" s="273"/>
-      <c r="BK7" s="273"/>
-      <c r="BL7" s="273"/>
-      <c r="BM7" s="273"/>
-      <c r="BN7" s="273"/>
-      <c r="BO7" s="273"/>
-      <c r="BP7" s="273"/>
-      <c r="BQ7" s="273"/>
-      <c r="BR7" s="273"/>
-      <c r="BS7" s="273"/>
-      <c r="BT7" s="273"/>
-      <c r="BU7" s="273"/>
-      <c r="BV7" s="273"/>
-      <c r="BW7" s="273"/>
-      <c r="BX7" s="273"/>
-      <c r="BY7" s="273"/>
-      <c r="BZ7" s="273"/>
-      <c r="CA7" s="273"/>
-      <c r="CB7" s="273"/>
-      <c r="CC7" s="273"/>
-      <c r="CD7" s="273"/>
-      <c r="CE7" s="273"/>
-      <c r="CF7" s="273"/>
-      <c r="CG7" s="273"/>
-      <c r="CH7" s="273"/>
-      <c r="CI7" s="273"/>
-      <c r="CJ7" s="273"/>
-      <c r="CK7" s="273"/>
-      <c r="CL7" s="273"/>
-      <c r="CM7" s="273"/>
-      <c r="CN7" s="273"/>
-      <c r="CO7" s="273"/>
-      <c r="CP7" s="273"/>
-      <c r="CQ7" s="273"/>
-      <c r="CR7" s="273"/>
-      <c r="CS7" s="273"/>
-      <c r="CT7" s="273"/>
-      <c r="CU7" s="273"/>
-      <c r="CV7" s="273"/>
-      <c r="CW7" s="273"/>
-      <c r="CX7" s="273"/>
-      <c r="CY7" s="273"/>
-      <c r="CZ7" s="273"/>
-      <c r="DA7" s="273"/>
-      <c r="DB7" s="273"/>
-      <c r="DC7" s="273"/>
-      <c r="DD7" s="273"/>
-      <c r="DE7" s="273"/>
-      <c r="DF7" s="273"/>
-      <c r="DG7" s="273"/>
-      <c r="DH7" s="273"/>
-      <c r="DI7" s="273"/>
-      <c r="DJ7" s="273"/>
-      <c r="DK7" s="273"/>
-      <c r="DL7" s="273"/>
-      <c r="DM7" s="273"/>
-      <c r="DN7" s="273"/>
-      <c r="DO7" s="273"/>
-      <c r="DP7" s="273"/>
-      <c r="DQ7" s="273"/>
-      <c r="DR7" s="273"/>
-      <c r="DS7" s="273"/>
-      <c r="DT7" s="273"/>
-      <c r="DU7" s="273"/>
-      <c r="DV7" s="273"/>
-      <c r="DW7" s="273"/>
-      <c r="DX7" s="273"/>
-      <c r="DY7" s="273"/>
-      <c r="DZ7" s="273"/>
-      <c r="EA7" s="273"/>
-      <c r="EB7" s="273"/>
-      <c r="EC7" s="273"/>
-      <c r="ED7" s="273"/>
-      <c r="EE7" s="273"/>
-      <c r="EF7" s="273"/>
-      <c r="EG7" s="273"/>
-      <c r="EH7" s="273"/>
-      <c r="EI7" s="273"/>
-      <c r="EJ7" s="273"/>
-      <c r="EK7" s="273"/>
-      <c r="EL7" s="273"/>
+      <c r="A7" s="280"/>
+      <c r="B7" s="280"/>
+      <c r="C7" s="280"/>
+      <c r="D7" s="280"/>
+      <c r="E7" s="280"/>
+      <c r="F7" s="280"/>
+      <c r="G7" s="280"/>
+      <c r="H7" s="280"/>
+      <c r="I7" s="280"/>
+      <c r="J7" s="280"/>
+      <c r="K7" s="280"/>
+      <c r="L7" s="280"/>
+      <c r="M7" s="280"/>
+      <c r="N7" s="280"/>
+      <c r="O7" s="280"/>
+      <c r="P7" s="280"/>
+      <c r="Q7" s="280"/>
+      <c r="R7" s="280"/>
+      <c r="S7" s="280"/>
+      <c r="T7" s="280"/>
+      <c r="U7" s="280"/>
+      <c r="V7" s="280"/>
+      <c r="W7" s="280"/>
+      <c r="X7" s="280"/>
+      <c r="Y7" s="280"/>
+      <c r="Z7" s="280"/>
+      <c r="AA7" s="280"/>
+      <c r="AB7" s="280"/>
+      <c r="AC7" s="280"/>
+      <c r="AD7" s="280"/>
+      <c r="AE7" s="280"/>
+      <c r="AF7" s="280"/>
+      <c r="AG7" s="280"/>
+      <c r="AH7" s="280"/>
+      <c r="AI7" s="280"/>
+      <c r="AJ7" s="280"/>
+      <c r="AK7" s="280"/>
+      <c r="AL7" s="280"/>
+      <c r="AM7" s="280"/>
+      <c r="AN7" s="280"/>
+      <c r="AO7" s="280"/>
+      <c r="AP7" s="280"/>
+      <c r="AQ7" s="280"/>
+      <c r="AR7" s="280"/>
+      <c r="AS7" s="280"/>
+      <c r="AT7" s="280"/>
+      <c r="AU7" s="280"/>
+      <c r="AV7" s="280"/>
+      <c r="AW7" s="280"/>
+      <c r="AX7" s="280"/>
+      <c r="AY7" s="280"/>
+      <c r="AZ7" s="280"/>
+      <c r="BA7" s="280"/>
+      <c r="BB7" s="280"/>
+      <c r="BC7" s="280"/>
+      <c r="BD7" s="280"/>
+      <c r="BE7" s="280"/>
+      <c r="BF7" s="280"/>
+      <c r="BG7" s="280"/>
+      <c r="BH7" s="280"/>
+      <c r="BI7" s="280"/>
+      <c r="BJ7" s="280"/>
+      <c r="BK7" s="280"/>
+      <c r="BL7" s="280"/>
+      <c r="BM7" s="280"/>
+      <c r="BN7" s="280"/>
+      <c r="BO7" s="280"/>
+      <c r="BP7" s="280"/>
+      <c r="BQ7" s="280"/>
+      <c r="BR7" s="280"/>
+      <c r="BS7" s="280"/>
+      <c r="BT7" s="280"/>
+      <c r="BU7" s="280"/>
+      <c r="BV7" s="280"/>
+      <c r="BW7" s="280"/>
+      <c r="BX7" s="280"/>
+      <c r="BY7" s="280"/>
+      <c r="BZ7" s="280"/>
+      <c r="CA7" s="280"/>
+      <c r="CB7" s="280"/>
+      <c r="CC7" s="280"/>
+      <c r="CD7" s="280"/>
+      <c r="CE7" s="280"/>
+      <c r="CF7" s="280"/>
+      <c r="CG7" s="280"/>
+      <c r="CH7" s="280"/>
+      <c r="CI7" s="280"/>
+      <c r="CJ7" s="280"/>
+      <c r="CK7" s="280"/>
+      <c r="CL7" s="280"/>
+      <c r="CM7" s="280"/>
+      <c r="CN7" s="280"/>
+      <c r="CO7" s="280"/>
+      <c r="CP7" s="280"/>
+      <c r="CQ7" s="280"/>
+      <c r="CR7" s="280"/>
+      <c r="CS7" s="280"/>
+      <c r="CT7" s="280"/>
+      <c r="CU7" s="280"/>
+      <c r="CV7" s="280"/>
+      <c r="CW7" s="280"/>
+      <c r="CX7" s="280"/>
+      <c r="CY7" s="280"/>
+      <c r="CZ7" s="280"/>
+      <c r="DA7" s="280"/>
+      <c r="DB7" s="280"/>
+      <c r="DC7" s="280"/>
+      <c r="DD7" s="280"/>
+      <c r="DE7" s="280"/>
+      <c r="DF7" s="280"/>
+      <c r="DG7" s="280"/>
+      <c r="DH7" s="280"/>
+      <c r="DI7" s="280"/>
+      <c r="DJ7" s="280"/>
+      <c r="DK7" s="280"/>
+      <c r="DL7" s="280"/>
+      <c r="DM7" s="280"/>
+      <c r="DN7" s="280"/>
+      <c r="DO7" s="280"/>
+      <c r="DP7" s="280"/>
+      <c r="DQ7" s="280"/>
+      <c r="DR7" s="280"/>
+      <c r="DS7" s="280"/>
+      <c r="DT7" s="280"/>
+      <c r="DU7" s="280"/>
+      <c r="DV7" s="280"/>
+      <c r="DW7" s="280"/>
+      <c r="DX7" s="280"/>
+      <c r="DY7" s="280"/>
+      <c r="DZ7" s="280"/>
+      <c r="EA7" s="280"/>
+      <c r="EB7" s="280"/>
+      <c r="EC7" s="280"/>
+      <c r="ED7" s="280"/>
+      <c r="EE7" s="280"/>
+      <c r="EF7" s="280"/>
+      <c r="EG7" s="280"/>
+      <c r="EH7" s="280"/>
+      <c r="EI7" s="280"/>
+      <c r="EJ7" s="280"/>
+      <c r="EK7" s="280"/>
+      <c r="EL7" s="280"/>
       <c r="EM7" s="238"/>
       <c r="EN7" s="238"/>
       <c r="EO7" s="238"/>
@@ -5219,7 +5232,7 @@
         <v>0</v>
       </c>
       <c r="CQ8" s="159">
-        <f>+IF(F8="x",500000,0)</f>
+        <f>+IF(F8="Nữ",500000,0)</f>
         <v>0</v>
       </c>
       <c r="CR8" s="156"/>
@@ -5388,12 +5401,12 @@
         <f t="shared" ref="EI8" si="78">+IF(EH8&lt;0,0,EH8)</f>
         <v>0</v>
       </c>
-      <c r="EJ8" s="165" t="b">
-        <f>+IF(AQ8&gt;0,I8/26)</f>
+      <c r="EJ8" s="165">
+        <f>+IF(AQ8&gt;0,I8/26,0)</f>
         <v>0</v>
       </c>
-      <c r="EK8" s="165" t="b">
-        <f>+IF(AQ8&gt;0,ED8*6%)</f>
+      <c r="EK8" s="165">
+        <f>+IF(AQ8&gt;0,ED8*6%,0)</f>
         <v>0</v>
       </c>
       <c r="EL8" s="165">
@@ -27077,22 +27090,38 @@
   </sheetData>
   <autoFilter ref="A6:ER8" xr:uid="{00000000-0001-0000-0900-000000000000}"/>
   <mergeCells count="64">
-    <mergeCell ref="EN5:EN6"/>
-    <mergeCell ref="EI5:EI6"/>
-    <mergeCell ref="EJ5:EJ6"/>
-    <mergeCell ref="EK5:EK6"/>
-    <mergeCell ref="EL5:EL6"/>
-    <mergeCell ref="EH5:EH6"/>
-    <mergeCell ref="DV5:DX5"/>
-    <mergeCell ref="CQ5:CS5"/>
-    <mergeCell ref="DG5:DG6"/>
-    <mergeCell ref="DI5:DJ5"/>
-    <mergeCell ref="CT5:CT6"/>
-    <mergeCell ref="DH5:DH6"/>
-    <mergeCell ref="DK5:DK6"/>
-    <mergeCell ref="DM5:DR5"/>
-    <mergeCell ref="DS5:DS6"/>
-    <mergeCell ref="DU5:DU6"/>
+    <mergeCell ref="AO1:AS1"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="S4:U4"/>
+    <mergeCell ref="W4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="AG4:AI4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="BG4:BI4"/>
+    <mergeCell ref="AT4:AU4"/>
+    <mergeCell ref="AO5:AO6"/>
+    <mergeCell ref="AP5:AP6"/>
+    <mergeCell ref="AQ5:AQ6"/>
+    <mergeCell ref="AR5:AR6"/>
+    <mergeCell ref="AS5:AS6"/>
+    <mergeCell ref="BJ4:BK4"/>
+    <mergeCell ref="BL4:BN4"/>
+    <mergeCell ref="BQ4:BS4"/>
+    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="CD5:CD6"/>
+    <mergeCell ref="BY5:BY6"/>
+    <mergeCell ref="BZ5:BZ6"/>
+    <mergeCell ref="CA5:CA6"/>
+    <mergeCell ref="CB5:CB6"/>
+    <mergeCell ref="CC5:CC6"/>
     <mergeCell ref="ER5:ER6"/>
     <mergeCell ref="A7:EL7"/>
     <mergeCell ref="EM5:EM6"/>
@@ -27109,38 +27138,22 @@
     <mergeCell ref="DL5:DL6"/>
     <mergeCell ref="EG5:EG6"/>
     <mergeCell ref="EQ5:EQ6"/>
-    <mergeCell ref="BJ4:BK4"/>
-    <mergeCell ref="BL4:BN4"/>
-    <mergeCell ref="BQ4:BS4"/>
-    <mergeCell ref="BC4:BE4"/>
-    <mergeCell ref="CD5:CD6"/>
-    <mergeCell ref="BY5:BY6"/>
-    <mergeCell ref="BZ5:BZ6"/>
-    <mergeCell ref="CA5:CA6"/>
-    <mergeCell ref="CB5:CB6"/>
-    <mergeCell ref="CC5:CC6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="BG4:BI4"/>
-    <mergeCell ref="AT4:AU4"/>
-    <mergeCell ref="AO5:AO6"/>
-    <mergeCell ref="AP5:AP6"/>
-    <mergeCell ref="AQ5:AQ6"/>
-    <mergeCell ref="AR5:AR6"/>
-    <mergeCell ref="AS5:AS6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="AO1:AS1"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="S4:U4"/>
-    <mergeCell ref="W4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AD4"/>
-    <mergeCell ref="AG4:AI4"/>
+    <mergeCell ref="EH5:EH6"/>
+    <mergeCell ref="DV5:DX5"/>
+    <mergeCell ref="CQ5:CS5"/>
+    <mergeCell ref="DG5:DG6"/>
+    <mergeCell ref="DI5:DJ5"/>
+    <mergeCell ref="CT5:CT6"/>
+    <mergeCell ref="DH5:DH6"/>
+    <mergeCell ref="DK5:DK6"/>
+    <mergeCell ref="DM5:DR5"/>
+    <mergeCell ref="DS5:DS6"/>
+    <mergeCell ref="DU5:DU6"/>
+    <mergeCell ref="EN5:EN6"/>
+    <mergeCell ref="EI5:EI6"/>
+    <mergeCell ref="EJ5:EJ6"/>
+    <mergeCell ref="EK5:EK6"/>
+    <mergeCell ref="EL5:EL6"/>
   </mergeCells>
   <conditionalFormatting sqref="A5 A8:B8">
     <cfRule type="duplicateValues" dxfId="20" priority="20879"/>
@@ -27214,20 +27227,20 @@
     <tabColor rgb="FFFF00FF"/>
   </sheetPr>
   <dimension ref="A1:AC1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.796875" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.83203125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="4.796875" style="9" customWidth="1"/>
-    <col min="2" max="2" width="3.796875" style="9" customWidth="1"/>
-    <col min="3" max="10" width="6.3984375" style="9" customWidth="1"/>
-    <col min="11" max="11" width="3.796875" style="9" customWidth="1"/>
-    <col min="12" max="17" width="6.3984375" style="9" customWidth="1"/>
-    <col min="18" max="18" width="4.19921875" style="9" customWidth="1"/>
-    <col min="19" max="19" width="6.3984375" style="9" customWidth="1"/>
-    <col min="20" max="20" width="3.796875" style="9" customWidth="1"/>
-    <col min="21" max="27" width="6.3984375" style="9" customWidth="1"/>
-    <col min="28" max="28" width="4.796875" style="9" customWidth="1"/>
-    <col min="29" max="29" width="10.19921875" style="9" customWidth="1"/>
-    <col min="30" max="16384" width="12.796875" style="9"/>
+    <col min="1" max="1" width="4.83203125" style="9" customWidth="1"/>
+    <col min="2" max="2" width="3.83203125" style="9" customWidth="1"/>
+    <col min="3" max="10" width="6.33203125" style="9" customWidth="1"/>
+    <col min="11" max="11" width="3.83203125" style="9" customWidth="1"/>
+    <col min="12" max="17" width="6.33203125" style="9" customWidth="1"/>
+    <col min="18" max="18" width="4.1640625" style="9" customWidth="1"/>
+    <col min="19" max="19" width="6.33203125" style="9" customWidth="1"/>
+    <col min="20" max="20" width="3.83203125" style="9" customWidth="1"/>
+    <col min="21" max="27" width="6.33203125" style="9" customWidth="1"/>
+    <col min="28" max="28" width="4.83203125" style="9" customWidth="1"/>
+    <col min="29" max="29" width="10.1640625" style="9" customWidth="1"/>
+    <col min="30" max="16384" width="12.83203125" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="12.75" hidden="1" customHeight="1">
@@ -27797,11 +27810,11 @@
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
       <c r="H8" s="20"/>
-      <c r="I8" s="307">
+      <c r="I8" s="301">
         <v>2026</v>
       </c>
-      <c r="J8" s="308"/>
-      <c r="K8" s="308"/>
+      <c r="J8" s="302"/>
+      <c r="K8" s="302"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="21" t="s">
@@ -27826,13 +27839,13 @@
     <row r="9" spans="1:29" ht="15.75" customHeight="1" thickBot="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="309" t="s">
+      <c r="C9" s="303" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="310"/>
-      <c r="E9" s="310"/>
-      <c r="F9" s="310"/>
-      <c r="G9" s="310"/>
+      <c r="D9" s="304"/>
+      <c r="E9" s="304"/>
+      <c r="F9" s="304"/>
+      <c r="G9" s="304"/>
       <c r="H9" s="20"/>
       <c r="I9" s="24"/>
       <c r="J9" s="24"/>
@@ -27928,19 +27941,19 @@
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
-      <c r="J12" s="311" t="s">
+      <c r="J12" s="305" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="310"/>
-      <c r="L12" s="310"/>
-      <c r="M12" s="310"/>
-      <c r="N12" s="310"/>
-      <c r="O12" s="310"/>
-      <c r="P12" s="312">
+      <c r="K12" s="304"/>
+      <c r="L12" s="304"/>
+      <c r="M12" s="304"/>
+      <c r="N12" s="304"/>
+      <c r="O12" s="304"/>
+      <c r="P12" s="306">
         <f>I8</f>
         <v>2026</v>
       </c>
-      <c r="Q12" s="310"/>
+      <c r="Q12" s="304"/>
       <c r="R12" s="33"/>
       <c r="S12" s="34"/>
       <c r="T12" s="34"/>
@@ -28204,38 +28217,38 @@
     </row>
     <row r="21" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A21" s="39"/>
-      <c r="B21" s="306" t="s">
+      <c r="B21" s="307" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="302"/>
-      <c r="D21" s="302"/>
-      <c r="E21" s="302"/>
-      <c r="F21" s="302"/>
-      <c r="G21" s="302"/>
-      <c r="H21" s="302"/>
-      <c r="I21" s="302"/>
+      <c r="C21" s="308"/>
+      <c r="D21" s="308"/>
+      <c r="E21" s="308"/>
+      <c r="F21" s="308"/>
+      <c r="G21" s="308"/>
+      <c r="H21" s="308"/>
+      <c r="I21" s="308"/>
       <c r="J21" s="40"/>
-      <c r="K21" s="303" t="s">
+      <c r="K21" s="309" t="s">
         <v>37</v>
       </c>
-      <c r="L21" s="302"/>
-      <c r="M21" s="302"/>
-      <c r="N21" s="302"/>
-      <c r="O21" s="302"/>
-      <c r="P21" s="302"/>
-      <c r="Q21" s="302"/>
-      <c r="R21" s="302"/>
+      <c r="L21" s="308"/>
+      <c r="M21" s="308"/>
+      <c r="N21" s="308"/>
+      <c r="O21" s="308"/>
+      <c r="P21" s="308"/>
+      <c r="Q21" s="308"/>
+      <c r="R21" s="308"/>
       <c r="S21" s="40"/>
-      <c r="T21" s="301" t="s">
+      <c r="T21" s="310" t="s">
         <v>38</v>
       </c>
-      <c r="U21" s="302"/>
-      <c r="V21" s="302"/>
-      <c r="W21" s="302"/>
-      <c r="X21" s="302"/>
-      <c r="Y21" s="302"/>
-      <c r="Z21" s="302"/>
-      <c r="AA21" s="302"/>
+      <c r="U21" s="308"/>
+      <c r="V21" s="308"/>
+      <c r="W21" s="308"/>
+      <c r="X21" s="308"/>
+      <c r="Y21" s="308"/>
+      <c r="Z21" s="308"/>
+      <c r="AA21" s="308"/>
       <c r="AB21" s="41"/>
       <c r="AC21" s="42"/>
     </row>
@@ -29135,38 +29148,38 @@
     </row>
     <row r="35" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="304" t="s">
+      <c r="B35" s="311" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="302"/>
-      <c r="D35" s="302"/>
-      <c r="E35" s="302"/>
-      <c r="F35" s="302"/>
-      <c r="G35" s="302"/>
-      <c r="H35" s="302"/>
-      <c r="I35" s="302"/>
+      <c r="C35" s="308"/>
+      <c r="D35" s="308"/>
+      <c r="E35" s="308"/>
+      <c r="F35" s="308"/>
+      <c r="G35" s="308"/>
+      <c r="H35" s="308"/>
+      <c r="I35" s="308"/>
       <c r="J35" s="40"/>
-      <c r="K35" s="305" t="s">
+      <c r="K35" s="312" t="s">
         <v>48</v>
       </c>
-      <c r="L35" s="302"/>
-      <c r="M35" s="302"/>
-      <c r="N35" s="302"/>
-      <c r="O35" s="302"/>
-      <c r="P35" s="302"/>
-      <c r="Q35" s="302"/>
-      <c r="R35" s="302"/>
+      <c r="L35" s="308"/>
+      <c r="M35" s="308"/>
+      <c r="N35" s="308"/>
+      <c r="O35" s="308"/>
+      <c r="P35" s="308"/>
+      <c r="Q35" s="308"/>
+      <c r="R35" s="308"/>
       <c r="S35" s="40"/>
-      <c r="T35" s="303" t="s">
+      <c r="T35" s="309" t="s">
         <v>49</v>
       </c>
-      <c r="U35" s="302"/>
-      <c r="V35" s="302"/>
-      <c r="W35" s="302"/>
-      <c r="X35" s="302"/>
-      <c r="Y35" s="302"/>
-      <c r="Z35" s="302"/>
-      <c r="AA35" s="302"/>
+      <c r="U35" s="308"/>
+      <c r="V35" s="308"/>
+      <c r="W35" s="308"/>
+      <c r="X35" s="308"/>
+      <c r="Y35" s="308"/>
+      <c r="Z35" s="308"/>
+      <c r="AA35" s="308"/>
       <c r="AB35" s="70"/>
       <c r="AC35" s="40"/>
     </row>
@@ -30055,38 +30068,38 @@
     </row>
     <row r="49" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A49" s="69"/>
-      <c r="B49" s="303" t="s">
+      <c r="B49" s="309" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="302"/>
-      <c r="D49" s="302"/>
-      <c r="E49" s="302"/>
-      <c r="F49" s="302"/>
-      <c r="G49" s="302"/>
-      <c r="H49" s="302"/>
-      <c r="I49" s="302"/>
+      <c r="C49" s="308"/>
+      <c r="D49" s="308"/>
+      <c r="E49" s="308"/>
+      <c r="F49" s="308"/>
+      <c r="G49" s="308"/>
+      <c r="H49" s="308"/>
+      <c r="I49" s="308"/>
       <c r="J49" s="40"/>
-      <c r="K49" s="304" t="s">
+      <c r="K49" s="311" t="s">
         <v>51</v>
       </c>
-      <c r="L49" s="302"/>
-      <c r="M49" s="302"/>
-      <c r="N49" s="302"/>
-      <c r="O49" s="302"/>
-      <c r="P49" s="302"/>
-      <c r="Q49" s="302"/>
-      <c r="R49" s="302"/>
+      <c r="L49" s="308"/>
+      <c r="M49" s="308"/>
+      <c r="N49" s="308"/>
+      <c r="O49" s="308"/>
+      <c r="P49" s="308"/>
+      <c r="Q49" s="308"/>
+      <c r="R49" s="308"/>
       <c r="S49" s="40"/>
-      <c r="T49" s="306" t="s">
+      <c r="T49" s="307" t="s">
         <v>52</v>
       </c>
-      <c r="U49" s="302"/>
-      <c r="V49" s="302"/>
-      <c r="W49" s="302"/>
-      <c r="X49" s="302"/>
-      <c r="Y49" s="302"/>
-      <c r="Z49" s="302"/>
-      <c r="AA49" s="302"/>
+      <c r="U49" s="308"/>
+      <c r="V49" s="308"/>
+      <c r="W49" s="308"/>
+      <c r="X49" s="308"/>
+      <c r="Y49" s="308"/>
+      <c r="Z49" s="308"/>
+      <c r="AA49" s="308"/>
       <c r="AB49" s="70"/>
       <c r="AC49" s="40"/>
     </row>
@@ -30975,38 +30988,38 @@
     </row>
     <row r="63" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A63" s="69"/>
-      <c r="B63" s="301" t="s">
+      <c r="B63" s="310" t="s">
         <v>53</v>
       </c>
-      <c r="C63" s="302"/>
-      <c r="D63" s="302"/>
-      <c r="E63" s="302"/>
-      <c r="F63" s="302"/>
-      <c r="G63" s="302"/>
-      <c r="H63" s="302"/>
-      <c r="I63" s="302"/>
+      <c r="C63" s="308"/>
+      <c r="D63" s="308"/>
+      <c r="E63" s="308"/>
+      <c r="F63" s="308"/>
+      <c r="G63" s="308"/>
+      <c r="H63" s="308"/>
+      <c r="I63" s="308"/>
       <c r="J63" s="40"/>
-      <c r="K63" s="303" t="s">
+      <c r="K63" s="309" t="s">
         <v>54</v>
       </c>
-      <c r="L63" s="302"/>
-      <c r="M63" s="302"/>
-      <c r="N63" s="302"/>
-      <c r="O63" s="302"/>
-      <c r="P63" s="302"/>
-      <c r="Q63" s="302"/>
-      <c r="R63" s="302"/>
+      <c r="L63" s="308"/>
+      <c r="M63" s="308"/>
+      <c r="N63" s="308"/>
+      <c r="O63" s="308"/>
+      <c r="P63" s="308"/>
+      <c r="Q63" s="308"/>
+      <c r="R63" s="308"/>
       <c r="S63" s="40"/>
-      <c r="T63" s="304" t="s">
+      <c r="T63" s="311" t="s">
         <v>55</v>
       </c>
-      <c r="U63" s="302"/>
-      <c r="V63" s="302"/>
-      <c r="W63" s="302"/>
-      <c r="X63" s="302"/>
-      <c r="Y63" s="302"/>
-      <c r="Z63" s="302"/>
-      <c r="AA63" s="302"/>
+      <c r="U63" s="308"/>
+      <c r="V63" s="308"/>
+      <c r="W63" s="308"/>
+      <c r="X63" s="308"/>
+      <c r="Y63" s="308"/>
+      <c r="Z63" s="308"/>
+      <c r="AA63" s="308"/>
       <c r="AB63" s="70"/>
       <c r="AC63" s="40"/>
     </row>
@@ -60541,12 +60554,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="J12:O12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="K21:R21"/>
     <mergeCell ref="B63:I63"/>
     <mergeCell ref="K63:R63"/>
     <mergeCell ref="T63:AA63"/>
@@ -60557,6 +60564,12 @@
     <mergeCell ref="B49:I49"/>
     <mergeCell ref="K49:R49"/>
     <mergeCell ref="T49:AA49"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="J12:O12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="K21:R21"/>
   </mergeCells>
   <conditionalFormatting sqref="C51:I55">
     <cfRule type="expression" dxfId="2" priority="3">

</xml_diff>

<commit_message>
chỉnh lại công thức tính phép lễ. nếu đi làm 13 công + phép lễ thì được hưởng 1 ngày phép
</commit_message>
<xml_diff>
--- a/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
+++ b/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonzai/dev/odoo 19/odoo/my_custom_addons/dl_salary_kpi/static/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{663DD088-5A8E-1B4F-8E8A-045185F17206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{727446F4-B647-DE4F-833B-DDB1CC986A9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="17820" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kangatang" sheetId="43" state="veryHidden" r:id="rId1"/>
@@ -2421,16 +2421,82 @@
     <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2466,83 +2532,33 @@
     <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="66" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="67" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="67" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="7" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2557,22 +2573,6 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="32">
@@ -3397,11 +3397,11 @@
       <c r="AL1" s="212"/>
       <c r="AM1" s="212"/>
       <c r="AN1" s="212"/>
-      <c r="AO1" s="300"/>
-      <c r="AP1" s="300"/>
-      <c r="AQ1" s="300"/>
-      <c r="AR1" s="300"/>
-      <c r="AS1" s="300"/>
+      <c r="AO1" s="260"/>
+      <c r="AP1" s="260"/>
+      <c r="AQ1" s="260"/>
+      <c r="AR1" s="260"/>
+      <c r="AS1" s="260"/>
       <c r="AT1" s="120"/>
       <c r="AU1" s="120"/>
       <c r="AV1" s="120"/>
@@ -3803,10 +3803,10 @@
       <c r="G4" s="232"/>
       <c r="H4" s="108"/>
       <c r="I4" s="256"/>
-      <c r="J4" s="293" t="s">
+      <c r="J4" s="261" t="s">
         <v>68</v>
       </c>
-      <c r="K4" s="293"/>
+      <c r="K4" s="261"/>
       <c r="L4" s="258">
         <v>3</v>
       </c>
@@ -3820,23 +3820,23 @@
       </c>
       <c r="Q4" s="259"/>
       <c r="R4" s="109"/>
-      <c r="S4" s="293"/>
-      <c r="T4" s="293"/>
-      <c r="U4" s="293"/>
+      <c r="S4" s="261"/>
+      <c r="T4" s="261"/>
+      <c r="U4" s="261"/>
       <c r="V4" s="109"/>
-      <c r="W4" s="293"/>
-      <c r="X4" s="293"/>
-      <c r="Y4" s="293"/>
-      <c r="Z4" s="293"/>
-      <c r="AA4" s="293"/>
-      <c r="AB4" s="293"/>
-      <c r="AC4" s="293"/>
-      <c r="AD4" s="293"/>
+      <c r="W4" s="261"/>
+      <c r="X4" s="261"/>
+      <c r="Y4" s="261"/>
+      <c r="Z4" s="261"/>
+      <c r="AA4" s="261"/>
+      <c r="AB4" s="261"/>
+      <c r="AC4" s="261"/>
+      <c r="AD4" s="261"/>
       <c r="AE4" s="109"/>
       <c r="AF4" s="110"/>
-      <c r="AG4" s="293"/>
-      <c r="AH4" s="293"/>
-      <c r="AI4" s="293"/>
+      <c r="AG4" s="261"/>
+      <c r="AH4" s="261"/>
+      <c r="AI4" s="261"/>
       <c r="AJ4" s="109"/>
       <c r="AK4" s="109"/>
       <c r="AL4" s="109"/>
@@ -3847,10 +3847,10 @@
       <c r="AQ4" s="113"/>
       <c r="AR4" s="221"/>
       <c r="AS4" s="227"/>
-      <c r="AT4" s="293" t="s">
+      <c r="AT4" s="261" t="s">
         <v>68</v>
       </c>
-      <c r="AU4" s="293"/>
+      <c r="AU4" s="261"/>
       <c r="AV4" s="258">
         <f>L4</f>
         <v>3</v>
@@ -3866,23 +3866,23 @@
       </c>
       <c r="BA4" s="259"/>
       <c r="BB4" s="109"/>
-      <c r="BC4" s="293"/>
-      <c r="BD4" s="293"/>
-      <c r="BE4" s="293"/>
+      <c r="BC4" s="261"/>
+      <c r="BD4" s="261"/>
+      <c r="BE4" s="261"/>
       <c r="BF4" s="109"/>
-      <c r="BG4" s="293"/>
-      <c r="BH4" s="293"/>
-      <c r="BI4" s="293"/>
-      <c r="BJ4" s="293"/>
-      <c r="BK4" s="293"/>
-      <c r="BL4" s="293"/>
-      <c r="BM4" s="293"/>
-      <c r="BN4" s="293"/>
+      <c r="BG4" s="261"/>
+      <c r="BH4" s="261"/>
+      <c r="BI4" s="261"/>
+      <c r="BJ4" s="261"/>
+      <c r="BK4" s="261"/>
+      <c r="BL4" s="261"/>
+      <c r="BM4" s="261"/>
+      <c r="BN4" s="261"/>
       <c r="BO4" s="109"/>
       <c r="BP4" s="110"/>
-      <c r="BQ4" s="293"/>
-      <c r="BR4" s="293"/>
-      <c r="BS4" s="293"/>
+      <c r="BQ4" s="261"/>
+      <c r="BR4" s="261"/>
+      <c r="BS4" s="261"/>
       <c r="BT4" s="114"/>
       <c r="BU4" s="114" t="str">
         <f>IF(WEEKDAY(BU5,1)=1,"CN","")</f>
@@ -3962,31 +3962,31 @@
       <c r="ER4" s="237"/>
     </row>
     <row r="5" spans="1:148" s="183" customFormat="1" ht="92.25" customHeight="1">
-      <c r="A5" s="288" t="s">
+      <c r="A5" s="262" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="278" t="s">
+      <c r="B5" s="263" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="288" t="s">
+      <c r="C5" s="262" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="297" t="s">
+      <c r="D5" s="264" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="298" t="s">
+      <c r="E5" s="265" t="s">
         <v>120</v>
       </c>
-      <c r="F5" s="288" t="s">
+      <c r="F5" s="262" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="288" t="s">
+      <c r="G5" s="262" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="288" t="s">
+      <c r="H5" s="262" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="294" t="s">
+      <c r="I5" s="267" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="174">
@@ -4113,19 +4113,19 @@
         <f t="shared" si="0"/>
         <v>46112</v>
       </c>
-      <c r="AO5" s="295" t="s">
+      <c r="AO5" s="268" t="s">
         <v>82</v>
       </c>
-      <c r="AP5" s="295" t="s">
+      <c r="AP5" s="268" t="s">
         <v>83</v>
       </c>
-      <c r="AQ5" s="295" t="s">
+      <c r="AQ5" s="268" t="s">
         <v>84</v>
       </c>
-      <c r="AR5" s="296" t="s">
+      <c r="AR5" s="269" t="s">
         <v>5</v>
       </c>
-      <c r="AS5" s="296" t="s">
+      <c r="AS5" s="269" t="s">
         <v>6</v>
       </c>
       <c r="AT5" s="178">
@@ -4252,46 +4252,46 @@
         <f t="shared" si="1"/>
         <v>46112</v>
       </c>
-      <c r="BY5" s="290" t="s">
+      <c r="BY5" s="270" t="s">
         <v>85</v>
       </c>
-      <c r="BZ5" s="290" t="s">
+      <c r="BZ5" s="270" t="s">
         <v>86</v>
       </c>
-      <c r="CA5" s="290" t="s">
+      <c r="CA5" s="270" t="s">
         <v>87</v>
       </c>
-      <c r="CB5" s="290" t="s">
+      <c r="CB5" s="270" t="s">
         <v>88</v>
       </c>
-      <c r="CC5" s="290" t="s">
+      <c r="CC5" s="270" t="s">
         <v>89</v>
       </c>
-      <c r="CD5" s="290" t="s">
+      <c r="CD5" s="270" t="s">
         <v>90</v>
       </c>
-      <c r="CE5" s="290" t="s">
+      <c r="CE5" s="270" t="s">
         <v>91</v>
       </c>
-      <c r="CF5" s="289" t="s">
+      <c r="CF5" s="284" t="s">
         <v>19</v>
       </c>
-      <c r="CG5" s="289"/>
-      <c r="CH5" s="289"/>
-      <c r="CI5" s="289"/>
-      <c r="CJ5" s="289"/>
-      <c r="CK5" s="289"/>
-      <c r="CL5" s="289"/>
-      <c r="CM5" s="289"/>
-      <c r="CN5" s="289"/>
-      <c r="CO5" s="289"/>
-      <c r="CP5" s="289"/>
-      <c r="CQ5" s="266" t="s">
+      <c r="CG5" s="284"/>
+      <c r="CH5" s="284"/>
+      <c r="CI5" s="284"/>
+      <c r="CJ5" s="284"/>
+      <c r="CK5" s="284"/>
+      <c r="CL5" s="284"/>
+      <c r="CM5" s="284"/>
+      <c r="CN5" s="284"/>
+      <c r="CO5" s="284"/>
+      <c r="CP5" s="284"/>
+      <c r="CQ5" s="288" t="s">
         <v>59</v>
       </c>
-      <c r="CR5" s="267"/>
-      <c r="CS5" s="268"/>
-      <c r="CT5" s="273" t="s">
+      <c r="CR5" s="289"/>
+      <c r="CS5" s="290"/>
+      <c r="CT5" s="295" t="s">
         <v>60</v>
       </c>
       <c r="CU5" s="247" t="s">
@@ -4314,107 +4314,107 @@
       <c r="DF5" s="245" t="s">
         <v>127</v>
       </c>
-      <c r="DG5" s="269" t="s">
+      <c r="DG5" s="291" t="s">
         <v>117</v>
       </c>
-      <c r="DH5" s="274" t="s">
+      <c r="DH5" s="296" t="s">
         <v>112</v>
       </c>
-      <c r="DI5" s="271" t="s">
+      <c r="DI5" s="293" t="s">
         <v>81</v>
       </c>
-      <c r="DJ5" s="272"/>
-      <c r="DK5" s="275" t="s">
+      <c r="DJ5" s="294"/>
+      <c r="DK5" s="281" t="s">
         <v>61</v>
       </c>
-      <c r="DL5" s="292" t="s">
+      <c r="DL5" s="285" t="s">
         <v>8</v>
       </c>
-      <c r="DM5" s="276" t="s">
+      <c r="DM5" s="282" t="s">
         <v>71</v>
       </c>
-      <c r="DN5" s="276"/>
-      <c r="DO5" s="276"/>
-      <c r="DP5" s="276"/>
-      <c r="DQ5" s="276"/>
-      <c r="DR5" s="276"/>
-      <c r="DS5" s="277" t="s">
+      <c r="DN5" s="282"/>
+      <c r="DO5" s="282"/>
+      <c r="DP5" s="282"/>
+      <c r="DQ5" s="282"/>
+      <c r="DR5" s="282"/>
+      <c r="DS5" s="297" t="s">
         <v>12</v>
       </c>
-      <c r="DT5" s="276" t="s">
+      <c r="DT5" s="282" t="s">
         <v>125</v>
       </c>
-      <c r="DU5" s="278" t="s">
+      <c r="DU5" s="263" t="s">
         <v>13</v>
       </c>
-      <c r="DV5" s="264" t="s">
+      <c r="DV5" s="286" t="s">
         <v>64</v>
       </c>
-      <c r="DW5" s="265"/>
-      <c r="DX5" s="264"/>
-      <c r="DY5" s="286" t="s">
+      <c r="DW5" s="287"/>
+      <c r="DX5" s="286"/>
+      <c r="DY5" s="279" t="s">
         <v>63</v>
       </c>
-      <c r="DZ5" s="286"/>
-      <c r="EA5" s="286"/>
-      <c r="EB5" s="286"/>
-      <c r="EC5" s="287" t="s">
+      <c r="DZ5" s="279"/>
+      <c r="EA5" s="279"/>
+      <c r="EB5" s="279"/>
+      <c r="EC5" s="280" t="s">
         <v>128</v>
       </c>
-      <c r="ED5" s="276" t="s">
+      <c r="ED5" s="282" t="s">
         <v>7</v>
       </c>
-      <c r="EE5" s="262" t="s">
+      <c r="EE5" s="283" t="s">
         <v>65</v>
       </c>
-      <c r="EF5" s="262"/>
-      <c r="EG5" s="262" t="s">
+      <c r="EF5" s="283"/>
+      <c r="EG5" s="283" t="s">
         <v>66</v>
       </c>
-      <c r="EH5" s="262" t="s">
+      <c r="EH5" s="283" t="s">
         <v>67</v>
       </c>
-      <c r="EI5" s="262" t="s">
+      <c r="EI5" s="283" t="s">
         <v>72</v>
       </c>
-      <c r="EJ5" s="263" t="s">
+      <c r="EJ5" s="300" t="s">
         <v>78</v>
       </c>
-      <c r="EK5" s="263" t="s">
+      <c r="EK5" s="300" t="s">
         <v>80</v>
       </c>
-      <c r="EL5" s="263" t="s">
+      <c r="EL5" s="300" t="s">
         <v>79</v>
       </c>
-      <c r="EM5" s="281" t="s">
+      <c r="EM5" s="274" t="s">
         <v>124</v>
       </c>
-      <c r="EN5" s="260" t="s">
+      <c r="EN5" s="298" t="s">
         <v>118</v>
       </c>
-      <c r="EO5" s="283" t="s">
+      <c r="EO5" s="276" t="s">
         <v>130</v>
       </c>
-      <c r="EP5" s="285" t="s">
+      <c r="EP5" s="278" t="s">
         <v>122</v>
       </c>
-      <c r="EQ5" s="285" t="s">
+      <c r="EQ5" s="278" t="s">
         <v>121</v>
       </c>
-      <c r="ER5" s="279" t="s">
+      <c r="ER5" s="272" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:148" s="205" customFormat="1" ht="148.5" customHeight="1">
-      <c r="A6" s="288"/>
-      <c r="B6" s="278"/>
-      <c r="C6" s="288"/>
-      <c r="D6" s="297"/>
-      <c r="E6" s="299"/>
-      <c r="F6" s="288"/>
-      <c r="G6" s="288"/>
-      <c r="H6" s="288"/>
-      <c r="I6" s="294"/>
+      <c r="A6" s="262"/>
+      <c r="B6" s="263"/>
+      <c r="C6" s="262"/>
+      <c r="D6" s="264"/>
+      <c r="E6" s="266"/>
+      <c r="F6" s="262"/>
+      <c r="G6" s="262"/>
+      <c r="H6" s="262"/>
+      <c r="I6" s="267"/>
       <c r="J6" s="184" t="str">
         <f t="shared" ref="J6:AN6" si="2">IF(WEEKDAY(J5)=1,"CN",WEEKDAY(J5))</f>
         <v>CN</v>
@@ -4539,11 +4539,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AO6" s="295"/>
-      <c r="AP6" s="295"/>
-      <c r="AQ6" s="295"/>
-      <c r="AR6" s="296"/>
-      <c r="AS6" s="296"/>
+      <c r="AO6" s="268"/>
+      <c r="AP6" s="268"/>
+      <c r="AQ6" s="268"/>
+      <c r="AR6" s="269"/>
+      <c r="AS6" s="269"/>
       <c r="AT6" s="186" t="str">
         <f>+J6</f>
         <v>CN</v>
@@ -4668,13 +4668,13 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="BY6" s="291"/>
-      <c r="BZ6" s="291"/>
-      <c r="CA6" s="291"/>
-      <c r="CB6" s="291"/>
-      <c r="CC6" s="291"/>
-      <c r="CD6" s="291"/>
-      <c r="CE6" s="291"/>
+      <c r="BY6" s="271"/>
+      <c r="BZ6" s="271"/>
+      <c r="CA6" s="271"/>
+      <c r="CB6" s="271"/>
+      <c r="CC6" s="271"/>
+      <c r="CD6" s="271"/>
+      <c r="CE6" s="271"/>
       <c r="CF6" s="188" t="s">
         <v>92</v>
       </c>
@@ -4717,7 +4717,7 @@
       <c r="CS6" s="180" t="s">
         <v>58</v>
       </c>
-      <c r="CT6" s="273"/>
+      <c r="CT6" s="295"/>
       <c r="CU6" s="188" t="s">
         <v>103</v>
       </c>
@@ -4754,16 +4754,16 @@
       <c r="DF6" s="246" t="s">
         <v>129</v>
       </c>
-      <c r="DG6" s="270"/>
-      <c r="DH6" s="274"/>
+      <c r="DG6" s="292"/>
+      <c r="DH6" s="296"/>
       <c r="DI6" s="152" t="s">
         <v>14</v>
       </c>
       <c r="DJ6" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="DK6" s="275"/>
-      <c r="DL6" s="292"/>
+      <c r="DK6" s="281"/>
+      <c r="DL6" s="285"/>
       <c r="DM6" s="180" t="s">
         <v>9</v>
       </c>
@@ -4782,9 +4782,9 @@
       <c r="DR6" s="180" t="s">
         <v>115</v>
       </c>
-      <c r="DS6" s="277"/>
-      <c r="DT6" s="276"/>
-      <c r="DU6" s="278"/>
+      <c r="DS6" s="297"/>
+      <c r="DT6" s="282"/>
+      <c r="DU6" s="263"/>
       <c r="DV6" s="203">
         <v>0.17499999999999999</v>
       </c>
@@ -4806,170 +4806,170 @@
       <c r="EB6" s="152" t="s">
         <v>62</v>
       </c>
-      <c r="EC6" s="275"/>
-      <c r="ED6" s="276"/>
+      <c r="EC6" s="281"/>
+      <c r="ED6" s="282"/>
       <c r="EE6" s="182" t="s">
         <v>73</v>
       </c>
       <c r="EF6" s="182" t="s">
         <v>74</v>
       </c>
-      <c r="EG6" s="262"/>
-      <c r="EH6" s="262"/>
-      <c r="EI6" s="262"/>
-      <c r="EJ6" s="263"/>
-      <c r="EK6" s="263"/>
-      <c r="EL6" s="263"/>
-      <c r="EM6" s="282"/>
-      <c r="EN6" s="261"/>
-      <c r="EO6" s="284"/>
-      <c r="EP6" s="285"/>
-      <c r="EQ6" s="285"/>
-      <c r="ER6" s="279"/>
+      <c r="EG6" s="283"/>
+      <c r="EH6" s="283"/>
+      <c r="EI6" s="283"/>
+      <c r="EJ6" s="300"/>
+      <c r="EK6" s="300"/>
+      <c r="EL6" s="300"/>
+      <c r="EM6" s="275"/>
+      <c r="EN6" s="299"/>
+      <c r="EO6" s="277"/>
+      <c r="EP6" s="278"/>
+      <c r="EQ6" s="278"/>
+      <c r="ER6" s="272"/>
     </row>
     <row r="7" spans="1:148" s="106" customFormat="1" ht="87.75" customHeight="1">
-      <c r="A7" s="280"/>
-      <c r="B7" s="280"/>
-      <c r="C7" s="280"/>
-      <c r="D7" s="280"/>
-      <c r="E7" s="280"/>
-      <c r="F7" s="280"/>
-      <c r="G7" s="280"/>
-      <c r="H7" s="280"/>
-      <c r="I7" s="280"/>
-      <c r="J7" s="280"/>
-      <c r="K7" s="280"/>
-      <c r="L7" s="280"/>
-      <c r="M7" s="280"/>
-      <c r="N7" s="280"/>
-      <c r="O7" s="280"/>
-      <c r="P7" s="280"/>
-      <c r="Q7" s="280"/>
-      <c r="R7" s="280"/>
-      <c r="S7" s="280"/>
-      <c r="T7" s="280"/>
-      <c r="U7" s="280"/>
-      <c r="V7" s="280"/>
-      <c r="W7" s="280"/>
-      <c r="X7" s="280"/>
-      <c r="Y7" s="280"/>
-      <c r="Z7" s="280"/>
-      <c r="AA7" s="280"/>
-      <c r="AB7" s="280"/>
-      <c r="AC7" s="280"/>
-      <c r="AD7" s="280"/>
-      <c r="AE7" s="280"/>
-      <c r="AF7" s="280"/>
-      <c r="AG7" s="280"/>
-      <c r="AH7" s="280"/>
-      <c r="AI7" s="280"/>
-      <c r="AJ7" s="280"/>
-      <c r="AK7" s="280"/>
-      <c r="AL7" s="280"/>
-      <c r="AM7" s="280"/>
-      <c r="AN7" s="280"/>
-      <c r="AO7" s="280"/>
-      <c r="AP7" s="280"/>
-      <c r="AQ7" s="280"/>
-      <c r="AR7" s="280"/>
-      <c r="AS7" s="280"/>
-      <c r="AT7" s="280"/>
-      <c r="AU7" s="280"/>
-      <c r="AV7" s="280"/>
-      <c r="AW7" s="280"/>
-      <c r="AX7" s="280"/>
-      <c r="AY7" s="280"/>
-      <c r="AZ7" s="280"/>
-      <c r="BA7" s="280"/>
-      <c r="BB7" s="280"/>
-      <c r="BC7" s="280"/>
-      <c r="BD7" s="280"/>
-      <c r="BE7" s="280"/>
-      <c r="BF7" s="280"/>
-      <c r="BG7" s="280"/>
-      <c r="BH7" s="280"/>
-      <c r="BI7" s="280"/>
-      <c r="BJ7" s="280"/>
-      <c r="BK7" s="280"/>
-      <c r="BL7" s="280"/>
-      <c r="BM7" s="280"/>
-      <c r="BN7" s="280"/>
-      <c r="BO7" s="280"/>
-      <c r="BP7" s="280"/>
-      <c r="BQ7" s="280"/>
-      <c r="BR7" s="280"/>
-      <c r="BS7" s="280"/>
-      <c r="BT7" s="280"/>
-      <c r="BU7" s="280"/>
-      <c r="BV7" s="280"/>
-      <c r="BW7" s="280"/>
-      <c r="BX7" s="280"/>
-      <c r="BY7" s="280"/>
-      <c r="BZ7" s="280"/>
-      <c r="CA7" s="280"/>
-      <c r="CB7" s="280"/>
-      <c r="CC7" s="280"/>
-      <c r="CD7" s="280"/>
-      <c r="CE7" s="280"/>
-      <c r="CF7" s="280"/>
-      <c r="CG7" s="280"/>
-      <c r="CH7" s="280"/>
-      <c r="CI7" s="280"/>
-      <c r="CJ7" s="280"/>
-      <c r="CK7" s="280"/>
-      <c r="CL7" s="280"/>
-      <c r="CM7" s="280"/>
-      <c r="CN7" s="280"/>
-      <c r="CO7" s="280"/>
-      <c r="CP7" s="280"/>
-      <c r="CQ7" s="280"/>
-      <c r="CR7" s="280"/>
-      <c r="CS7" s="280"/>
-      <c r="CT7" s="280"/>
-      <c r="CU7" s="280"/>
-      <c r="CV7" s="280"/>
-      <c r="CW7" s="280"/>
-      <c r="CX7" s="280"/>
-      <c r="CY7" s="280"/>
-      <c r="CZ7" s="280"/>
-      <c r="DA7" s="280"/>
-      <c r="DB7" s="280"/>
-      <c r="DC7" s="280"/>
-      <c r="DD7" s="280"/>
-      <c r="DE7" s="280"/>
-      <c r="DF7" s="280"/>
-      <c r="DG7" s="280"/>
-      <c r="DH7" s="280"/>
-      <c r="DI7" s="280"/>
-      <c r="DJ7" s="280"/>
-      <c r="DK7" s="280"/>
-      <c r="DL7" s="280"/>
-      <c r="DM7" s="280"/>
-      <c r="DN7" s="280"/>
-      <c r="DO7" s="280"/>
-      <c r="DP7" s="280"/>
-      <c r="DQ7" s="280"/>
-      <c r="DR7" s="280"/>
-      <c r="DS7" s="280"/>
-      <c r="DT7" s="280"/>
-      <c r="DU7" s="280"/>
-      <c r="DV7" s="280"/>
-      <c r="DW7" s="280"/>
-      <c r="DX7" s="280"/>
-      <c r="DY7" s="280"/>
-      <c r="DZ7" s="280"/>
-      <c r="EA7" s="280"/>
-      <c r="EB7" s="280"/>
-      <c r="EC7" s="280"/>
-      <c r="ED7" s="280"/>
-      <c r="EE7" s="280"/>
-      <c r="EF7" s="280"/>
-      <c r="EG7" s="280"/>
-      <c r="EH7" s="280"/>
-      <c r="EI7" s="280"/>
-      <c r="EJ7" s="280"/>
-      <c r="EK7" s="280"/>
-      <c r="EL7" s="280"/>
+      <c r="A7" s="273"/>
+      <c r="B7" s="273"/>
+      <c r="C7" s="273"/>
+      <c r="D7" s="273"/>
+      <c r="E7" s="273"/>
+      <c r="F7" s="273"/>
+      <c r="G7" s="273"/>
+      <c r="H7" s="273"/>
+      <c r="I7" s="273"/>
+      <c r="J7" s="273"/>
+      <c r="K7" s="273"/>
+      <c r="L7" s="273"/>
+      <c r="M7" s="273"/>
+      <c r="N7" s="273"/>
+      <c r="O7" s="273"/>
+      <c r="P7" s="273"/>
+      <c r="Q7" s="273"/>
+      <c r="R7" s="273"/>
+      <c r="S7" s="273"/>
+      <c r="T7" s="273"/>
+      <c r="U7" s="273"/>
+      <c r="V7" s="273"/>
+      <c r="W7" s="273"/>
+      <c r="X7" s="273"/>
+      <c r="Y7" s="273"/>
+      <c r="Z7" s="273"/>
+      <c r="AA7" s="273"/>
+      <c r="AB7" s="273"/>
+      <c r="AC7" s="273"/>
+      <c r="AD7" s="273"/>
+      <c r="AE7" s="273"/>
+      <c r="AF7" s="273"/>
+      <c r="AG7" s="273"/>
+      <c r="AH7" s="273"/>
+      <c r="AI7" s="273"/>
+      <c r="AJ7" s="273"/>
+      <c r="AK7" s="273"/>
+      <c r="AL7" s="273"/>
+      <c r="AM7" s="273"/>
+      <c r="AN7" s="273"/>
+      <c r="AO7" s="273"/>
+      <c r="AP7" s="273"/>
+      <c r="AQ7" s="273"/>
+      <c r="AR7" s="273"/>
+      <c r="AS7" s="273"/>
+      <c r="AT7" s="273"/>
+      <c r="AU7" s="273"/>
+      <c r="AV7" s="273"/>
+      <c r="AW7" s="273"/>
+      <c r="AX7" s="273"/>
+      <c r="AY7" s="273"/>
+      <c r="AZ7" s="273"/>
+      <c r="BA7" s="273"/>
+      <c r="BB7" s="273"/>
+      <c r="BC7" s="273"/>
+      <c r="BD7" s="273"/>
+      <c r="BE7" s="273"/>
+      <c r="BF7" s="273"/>
+      <c r="BG7" s="273"/>
+      <c r="BH7" s="273"/>
+      <c r="BI7" s="273"/>
+      <c r="BJ7" s="273"/>
+      <c r="BK7" s="273"/>
+      <c r="BL7" s="273"/>
+      <c r="BM7" s="273"/>
+      <c r="BN7" s="273"/>
+      <c r="BO7" s="273"/>
+      <c r="BP7" s="273"/>
+      <c r="BQ7" s="273"/>
+      <c r="BR7" s="273"/>
+      <c r="BS7" s="273"/>
+      <c r="BT7" s="273"/>
+      <c r="BU7" s="273"/>
+      <c r="BV7" s="273"/>
+      <c r="BW7" s="273"/>
+      <c r="BX7" s="273"/>
+      <c r="BY7" s="273"/>
+      <c r="BZ7" s="273"/>
+      <c r="CA7" s="273"/>
+      <c r="CB7" s="273"/>
+      <c r="CC7" s="273"/>
+      <c r="CD7" s="273"/>
+      <c r="CE7" s="273"/>
+      <c r="CF7" s="273"/>
+      <c r="CG7" s="273"/>
+      <c r="CH7" s="273"/>
+      <c r="CI7" s="273"/>
+      <c r="CJ7" s="273"/>
+      <c r="CK7" s="273"/>
+      <c r="CL7" s="273"/>
+      <c r="CM7" s="273"/>
+      <c r="CN7" s="273"/>
+      <c r="CO7" s="273"/>
+      <c r="CP7" s="273"/>
+      <c r="CQ7" s="273"/>
+      <c r="CR7" s="273"/>
+      <c r="CS7" s="273"/>
+      <c r="CT7" s="273"/>
+      <c r="CU7" s="273"/>
+      <c r="CV7" s="273"/>
+      <c r="CW7" s="273"/>
+      <c r="CX7" s="273"/>
+      <c r="CY7" s="273"/>
+      <c r="CZ7" s="273"/>
+      <c r="DA7" s="273"/>
+      <c r="DB7" s="273"/>
+      <c r="DC7" s="273"/>
+      <c r="DD7" s="273"/>
+      <c r="DE7" s="273"/>
+      <c r="DF7" s="273"/>
+      <c r="DG7" s="273"/>
+      <c r="DH7" s="273"/>
+      <c r="DI7" s="273"/>
+      <c r="DJ7" s="273"/>
+      <c r="DK7" s="273"/>
+      <c r="DL7" s="273"/>
+      <c r="DM7" s="273"/>
+      <c r="DN7" s="273"/>
+      <c r="DO7" s="273"/>
+      <c r="DP7" s="273"/>
+      <c r="DQ7" s="273"/>
+      <c r="DR7" s="273"/>
+      <c r="DS7" s="273"/>
+      <c r="DT7" s="273"/>
+      <c r="DU7" s="273"/>
+      <c r="DV7" s="273"/>
+      <c r="DW7" s="273"/>
+      <c r="DX7" s="273"/>
+      <c r="DY7" s="273"/>
+      <c r="DZ7" s="273"/>
+      <c r="EA7" s="273"/>
+      <c r="EB7" s="273"/>
+      <c r="EC7" s="273"/>
+      <c r="ED7" s="273"/>
+      <c r="EE7" s="273"/>
+      <c r="EF7" s="273"/>
+      <c r="EG7" s="273"/>
+      <c r="EH7" s="273"/>
+      <c r="EI7" s="273"/>
+      <c r="EJ7" s="273"/>
+      <c r="EK7" s="273"/>
+      <c r="EL7" s="273"/>
       <c r="EM7" s="238"/>
       <c r="EN7" s="238"/>
       <c r="EO7" s="238"/>
@@ -5023,143 +5023,143 @@
         <v>0</v>
       </c>
       <c r="AP8" s="167">
-        <f t="shared" ref="AP8" si="5">COUNTIF(J8:AN8,"Đ")</f>
+        <f>COUNTIF(J8:AN8,"Đ")+(COUNTIF(J8:AN8,"Đ/2")/2)</f>
         <v>0</v>
       </c>
       <c r="AQ8" s="167">
-        <f t="shared" ref="AQ8" si="6">AO8+AP8</f>
+        <f t="shared" ref="AQ8" si="5">AO8+AP8</f>
         <v>0</v>
       </c>
       <c r="AR8" s="159">
-        <f t="shared" ref="AR8" si="7">COUNTIF(J8:AN8,"PL")</f>
+        <f t="shared" ref="AR8" si="6">COUNTIF(J8:AN8,"PL")</f>
         <v>0</v>
       </c>
       <c r="AS8" s="156">
-        <f t="shared" ref="AS8" si="8">IF(AQ8&gt;=20,1,0)</f>
+        <f>IF(AQ8 + AR8&gt;=13,1,0)</f>
         <v>0</v>
       </c>
       <c r="AT8" s="155">
-        <f t="shared" ref="AT8" si="9">+IF(J8="N","0.5N",IF(J8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="AT8" si="7">+IF(J8="N","0.5N",IF(J8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="AU8" s="155">
-        <f t="shared" ref="AU8" si="10">+IF(K8="N","0.5N",IF(K8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="AU8" si="8">+IF(K8="N","0.5N",IF(K8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="AV8" s="155">
-        <f t="shared" ref="AV8" si="11">+IF(L8="N","0.5N",IF(L8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="AV8" si="9">+IF(L8="N","0.5N",IF(L8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="AW8" s="155">
-        <f t="shared" ref="AW8" si="12">+IF(M8="N","0.5N",IF(M8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="AW8" si="10">+IF(M8="N","0.5N",IF(M8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="AX8" s="155">
-        <f t="shared" ref="AX8" si="13">+IF(N8="N","0.5N",IF(N8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="AX8" si="11">+IF(N8="N","0.5N",IF(N8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="AY8" s="155">
-        <f t="shared" ref="AY8" si="14">+IF(O8="N","0.5N",IF(O8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="AY8" si="12">+IF(O8="N","0.5N",IF(O8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="AZ8" s="155">
-        <f t="shared" ref="AZ8" si="15">+IF(P8="N","0.5N",IF(P8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="AZ8" si="13">+IF(P8="N","0.5N",IF(P8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BA8" s="155">
-        <f t="shared" ref="BA8" si="16">+IF(Q8="N","0.5N",IF(Q8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BA8" si="14">+IF(Q8="N","0.5N",IF(Q8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BB8" s="155">
-        <f t="shared" ref="BB8" si="17">+IF(R8="N","0.5N",IF(R8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BB8" si="15">+IF(R8="N","0.5N",IF(R8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BC8" s="155">
-        <f t="shared" ref="BC8" si="18">+IF(S8="N","0.5N",IF(S8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BC8" si="16">+IF(S8="N","0.5N",IF(S8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BD8" s="155">
-        <f t="shared" ref="BD8" si="19">+IF(T8="N","0.5N",IF(T8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BD8" si="17">+IF(T8="N","0.5N",IF(T8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BE8" s="155">
-        <f t="shared" ref="BE8" si="20">+IF(U8="N","0.5N",IF(U8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BE8" si="18">+IF(U8="N","0.5N",IF(U8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BF8" s="155">
-        <f t="shared" ref="BF8" si="21">+IF(V8="N","0.5N",IF(V8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BF8" si="19">+IF(V8="N","0.5N",IF(V8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BG8" s="155">
-        <f t="shared" ref="BG8" si="22">+IF(W8="N","0.5N",IF(W8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BG8" si="20">+IF(W8="N","0.5N",IF(W8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BH8" s="155">
-        <f t="shared" ref="BH8" si="23">+IF(X8="N","0.5N",IF(X8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BH8" si="21">+IF(X8="N","0.5N",IF(X8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BI8" s="155">
-        <f t="shared" ref="BI8" si="24">+IF(Y8="N","0.5N",IF(Y8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BI8" si="22">+IF(Y8="N","0.5N",IF(Y8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BJ8" s="155">
-        <f t="shared" ref="BJ8" si="25">+IF(Z8="N","0.5N",IF(Z8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BJ8" si="23">+IF(Z8="N","0.5N",IF(Z8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BK8" s="155">
-        <f t="shared" ref="BK8" si="26">+IF(AA8="N","0.5N",IF(AA8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BK8" si="24">+IF(AA8="N","0.5N",IF(AA8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BL8" s="155">
-        <f t="shared" ref="BL8" si="27">+IF(AB8="N","0.5N",IF(AB8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BL8" si="25">+IF(AB8="N","0.5N",IF(AB8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BM8" s="155">
-        <f t="shared" ref="BM8" si="28">+IF(AC8="N","0.5N",IF(AC8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BM8" si="26">+IF(AC8="N","0.5N",IF(AC8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BN8" s="155">
-        <f t="shared" ref="BN8" si="29">+IF(AD8="N","0.5N",IF(AD8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BN8" si="27">+IF(AD8="N","0.5N",IF(AD8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BO8" s="155">
-        <f t="shared" ref="BO8" si="30">+IF(AE8="N","0.5N",IF(AE8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BO8" si="28">+IF(AE8="N","0.5N",IF(AE8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BP8" s="155">
-        <f t="shared" ref="BP8:BQ8" si="31">+IF(AF8="N","0.5N",IF(AF8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BP8:BQ8" si="29">+IF(AF8="N","0.5N",IF(AF8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BQ8" s="155">
-        <f t="shared" si="31"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BR8" s="155">
-        <f t="shared" ref="BR8" si="32">+IF(AH8="N","0.5N",IF(AH8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BR8" si="30">+IF(AH8="N","0.5N",IF(AH8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BS8" s="155">
-        <f t="shared" ref="BS8" si="33">+IF(AI8="N","0.5N",IF(AI8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BS8" si="31">+IF(AI8="N","0.5N",IF(AI8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BT8" s="155">
-        <f t="shared" ref="BT8" si="34">+IF(AJ8="N","0.5N",IF(AJ8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BT8" si="32">+IF(AJ8="N","0.5N",IF(AJ8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BU8" s="155">
-        <f t="shared" ref="BU8" si="35">+IF(AK8="N","0.5N",IF(AK8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BU8" si="33">+IF(AK8="N","0.5N",IF(AK8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BV8" s="155">
-        <f t="shared" ref="BV8" si="36">+IF(AL8="N","0.5N",IF(AL8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BV8" si="34">+IF(AL8="N","0.5N",IF(AL8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BW8" s="155">
-        <f t="shared" ref="BW8" si="37">+IF(AM8="N","0.5N",IF(AM8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BW8" si="35">+IF(AM8="N","0.5N",IF(AM8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BX8" s="155">
-        <f t="shared" ref="BX8" si="38">+IF(AN8="N","0.5N",IF(AN8="Đ","0.5Đ",0))</f>
+        <f t="shared" ref="BX8" si="36">+IF(AN8="N","0.5N",IF(AN8="Đ","0.5Đ",0))</f>
         <v>0</v>
       </c>
       <c r="BY8" s="167">
@@ -5167,11 +5167,11 @@
         <v>0</v>
       </c>
       <c r="BZ8" s="167">
-        <f t="shared" ref="BZ8" si="39">COUNTIF(AT8:BX8,"1Đ")+(COUNTIF(AT8:BX8,"2Đ")*2)+(COUNTIF(AT8:BX8,"0.5Đ")/2)</f>
+        <f t="shared" ref="BZ8" si="37">COUNTIF(AT8:BX8,"1Đ")+(COUNTIF(AT8:BX8,"2Đ")*2)+(COUNTIF(AT8:BX8,"0.5Đ")/2)</f>
         <v>0</v>
       </c>
       <c r="CA8" s="167">
-        <f t="shared" ref="CA8" si="40">COUNTIF(AT8:BX8,"1N")+(COUNTIF(AT8:BX8,"2N")*2)+(COUNTIF(AT8:BX8,"0.5N")/2)</f>
+        <f t="shared" ref="CA8" si="38">COUNTIF(AT8:BX8,"1N")+(COUNTIF(AT8:BX8,"2N")*2)+(COUNTIF(AT8:BX8,"0.5N")/2)</f>
         <v>0</v>
       </c>
       <c r="CB8" s="167">
@@ -5179,7 +5179,7 @@
         <v>0</v>
       </c>
       <c r="CC8" s="167">
-        <f t="shared" ref="CC8" si="41">COUNTIF(AT8:BX8,"1LĐ")</f>
+        <f t="shared" ref="CC8" si="39">COUNTIF(AT8:BX8,"1LĐ")</f>
         <v>0</v>
       </c>
       <c r="CD8" s="163">
@@ -5187,48 +5187,48 @@
         <v>0</v>
       </c>
       <c r="CE8" s="170">
-        <f t="shared" ref="CE8" si="42">COUNTIF(AT8:BX8,"CNĐ")+(COUNTIF(AT8:BX8,"CNĐ/2")/2)</f>
+        <f t="shared" ref="CE8" si="40">COUNTIF(AT8:BX8,"CNĐ")+(COUNTIF(AT8:BX8,"CNĐ/2")/2)</f>
         <v>0</v>
       </c>
       <c r="CF8" s="171">
-        <f t="shared" ref="CF8" si="43">+AO8</f>
+        <f t="shared" ref="CF8" si="41">+AO8</f>
         <v>0</v>
       </c>
       <c r="CG8" s="171">
-        <f t="shared" ref="CG8" si="44">+AP8*8*0.3125</f>
+        <f t="shared" ref="CG8" si="42">+AP8*8*0.3125</f>
         <v>0</v>
       </c>
       <c r="CH8" s="171">
-        <f t="shared" ref="CH8" si="45">+AR8+AS8</f>
+        <f t="shared" ref="CH8" si="43">+AR8+AS8</f>
         <v>0</v>
       </c>
       <c r="CI8" s="171">
-        <f t="shared" ref="CI8" si="46">+CA8</f>
+        <f t="shared" ref="CI8" si="44">+CA8</f>
         <v>0</v>
       </c>
       <c r="CJ8" s="171">
-        <f t="shared" ref="CJ8" si="47">+AP8*8*0.6875</f>
+        <f t="shared" ref="CJ8" si="45">+AP8*8*0.6875</f>
         <v>0</v>
       </c>
       <c r="CK8" s="171">
-        <f t="shared" ref="CK8" si="48">+BZ8</f>
+        <f t="shared" ref="CK8" si="46">+BZ8</f>
         <v>0</v>
       </c>
       <c r="CL8" s="171"/>
       <c r="CM8" s="171">
-        <f t="shared" ref="CM8" si="49">+CE8</f>
+        <f t="shared" ref="CM8" si="47">+CE8</f>
         <v>0</v>
       </c>
       <c r="CN8" s="171">
-        <f t="shared" ref="CN8" si="50">+CD8</f>
+        <f t="shared" ref="CN8" si="48">+CD8</f>
         <v>0</v>
       </c>
       <c r="CO8" s="169">
-        <f t="shared" ref="CO8" si="51">+CB8</f>
+        <f t="shared" ref="CO8" si="49">+CB8</f>
         <v>0</v>
       </c>
       <c r="CP8" s="159">
-        <f t="shared" ref="CP8" si="52">+CC8</f>
+        <f t="shared" ref="CP8" si="50">+CC8</f>
         <v>0</v>
       </c>
       <c r="CQ8" s="159">
@@ -5237,39 +5237,39 @@
       </c>
       <c r="CR8" s="156"/>
       <c r="CS8" s="159">
-        <f t="shared" ref="CS8" si="53">IF($G$4&lt;20000000000,0,IF($G$4&lt;=30000000000,2000000,IF($G$4&lt;=50000000000,2300000,IF($G$4&lt;=50000000000,2000000,IF($G$4&lt;=70000000000,3000000,IF($G$4&gt;70000000000,3500000,0))))))</f>
+        <f t="shared" ref="CS8" si="51">IF($G$4&lt;20000000000,0,IF($G$4&lt;=30000000000,2000000,IF($G$4&lt;=50000000000,2300000,IF($G$4&lt;=50000000000,2000000,IF($G$4&lt;=70000000000,3000000,IF($G$4&gt;70000000000,3500000,0))))))</f>
         <v>0</v>
       </c>
       <c r="CT8" s="157">
-        <f t="shared" ref="CT8" si="54">+I8+CQ8+CR8+CS8</f>
+        <f t="shared" ref="CT8" si="52">+I8+CQ8+CR8+CS8</f>
         <v>0</v>
       </c>
       <c r="CU8" s="158">
-        <f t="shared" ref="CU8" si="55">+I8/26*(CF8+(CG8/8)+CH8)</f>
+        <f t="shared" ref="CU8" si="53">+I8/26*(CF8+(CG8/8)+CH8)</f>
         <v>0</v>
       </c>
       <c r="CV8" s="158">
-        <f t="shared" ref="CV8" si="56">+(I8/26/8)*150%*CI8</f>
+        <f t="shared" ref="CV8" si="54">+(I8/26/8)*150%*CI8</f>
         <v>0</v>
       </c>
       <c r="CW8" s="158">
-        <f t="shared" ref="CW8" si="57">+(I8/26/8)*130%*CJ8</f>
+        <f t="shared" ref="CW8" si="55">+(I8/26/8)*130%*CJ8</f>
         <v>0</v>
       </c>
       <c r="CX8" s="158">
-        <f t="shared" ref="CX8" si="58">+(I8/26/8)*200%*CK8</f>
+        <f t="shared" ref="CX8" si="56">+(I8/26/8)*200%*CK8</f>
         <v>0</v>
       </c>
       <c r="CY8" s="158">
-        <f t="shared" ref="CY8" si="59">+(I8/26/8)*210%*CL8</f>
+        <f t="shared" ref="CY8" si="57">+(I8/26/8)*210%*CL8</f>
         <v>0</v>
       </c>
       <c r="CZ8" s="158">
-        <f t="shared" ref="CZ8" si="60">+(I8/26/8)*270%*CM8</f>
+        <f t="shared" ref="CZ8" si="58">+(I8/26/8)*270%*CM8</f>
         <v>0</v>
       </c>
       <c r="DA8" s="158">
-        <f t="shared" ref="DA8" si="61">+(I8/26/8)*200%*CN8</f>
+        <f t="shared" ref="DA8" si="59">+(I8/26/8)*200%*CN8</f>
         <v>0</v>
       </c>
       <c r="DB8" s="158">
@@ -5277,64 +5277,64 @@
         <v>0</v>
       </c>
       <c r="DC8" s="158">
-        <f t="shared" ref="DC8" si="62">+(I8/26/8)*390%*CP8</f>
+        <f t="shared" ref="DC8" si="60">+(I8/26/8)*390%*CP8</f>
         <v>0</v>
       </c>
       <c r="DD8" s="159">
-        <f t="shared" ref="DD8" si="63">+CS8/26*(CF8+(CG8+CJ8)/8)</f>
+        <f t="shared" ref="DD8" si="61">+CS8/26*(CF8+(CG8+CJ8)/8)</f>
         <v>0</v>
       </c>
       <c r="DE8" s="211">
-        <f t="shared" ref="DE8" si="64">IF(OR(H8="CV",H8="KTT",H8="QL",H8="QĐ",H8="TL",H8="PGĐ"),2000000,IF(OR(H8="NV",H8="KT", H8="TK"),1500000,IF(OR(H8="CN",H8="LX"),1000000,0)))/26*(CF8+(CG8+CJ8)/8)</f>
+        <f t="shared" ref="DE8" si="62">IF(OR(H8="CV",H8="KTT",H8="QL",H8="QĐ",H8="TL",H8="PGĐ"),2000000,IF(OR(H8="NV",H8="KT", H8="TK"),1500000,IF(OR(H8="CN",H8="LX"),1000000,0)))/26*(CF8+(CG8+CJ8)/8)</f>
         <v>0</v>
       </c>
       <c r="DF8" s="211">
-        <f t="shared" ref="DF8" si="65">+DD8+DE8</f>
+        <f t="shared" ref="DF8" si="63">+DD8+DE8</f>
         <v>0</v>
       </c>
       <c r="DG8" s="254"/>
       <c r="DH8" s="158">
-        <f t="shared" ref="DH8" si="66">+CU8+CV8+CW8+CX8+CY8+CZ8+DA8+DB8+DC8+DF8+DG8</f>
+        <f t="shared" ref="DH8" si="64">+CU8+CV8+CW8+CX8+CY8+CZ8+DA8+DB8+DC8+DF8+DG8</f>
         <v>0</v>
       </c>
       <c r="DI8" s="164">
-        <f t="shared" ref="DI8" si="67">+CQ8/26*AQ8</f>
+        <f t="shared" ref="DI8" si="65">+CQ8/26*AQ8</f>
         <v>0</v>
       </c>
       <c r="DJ8" s="164">
-        <f t="shared" ref="DJ8" si="68">+CR8/26*AQ8</f>
+        <f t="shared" ref="DJ8" si="66">+CR8/26*AQ8</f>
         <v>0</v>
       </c>
       <c r="DK8" s="164">
-        <f t="shared" ref="DK8" si="69">+DH8+DI8+DJ8</f>
+        <f t="shared" ref="DK8" si="67">+DH8+DI8+DJ8</f>
         <v>0</v>
       </c>
       <c r="DL8" s="172">
-        <f t="shared" ref="DL8" si="70">I8</f>
+        <f t="shared" ref="DL8" si="68">I8</f>
         <v>0</v>
       </c>
       <c r="DM8" s="159">
-        <f t="shared" ref="DM8" si="71">DL8*8%</f>
+        <f t="shared" ref="DM8" si="69">DL8*8%</f>
         <v>0</v>
       </c>
       <c r="DN8" s="159">
-        <f t="shared" ref="DN8" si="72">DL8*1.5%</f>
+        <f t="shared" ref="DN8" si="70">DL8*1.5%</f>
         <v>0</v>
       </c>
       <c r="DO8" s="159">
-        <f t="shared" ref="DO8" si="73">DL8*1%</f>
+        <f t="shared" ref="DO8" si="71">DL8*1%</f>
         <v>0</v>
       </c>
       <c r="DP8" s="159">
-        <f t="shared" ref="DP8" si="74">EI8</f>
+        <f t="shared" ref="DP8" si="72">EI8</f>
         <v>0</v>
       </c>
       <c r="DQ8" s="159">
-        <f t="shared" ref="DQ8" si="75">+SUM(DM8:DP8)</f>
+        <f t="shared" ref="DQ8" si="73">+SUM(DM8:DP8)</f>
         <v>0</v>
       </c>
       <c r="DR8" s="159">
-        <f t="shared" ref="DR8" si="76">SUM(DM8:DO8)</f>
+        <f t="shared" ref="DR8" si="74">SUM(DM8:DO8)</f>
         <v>0</v>
       </c>
       <c r="DS8" s="160">
@@ -5371,7 +5371,7 @@
         <v>0</v>
       </c>
       <c r="EB8" s="173">
-        <f t="shared" ref="EB8" si="77">DY8+DZ8+EA8</f>
+        <f t="shared" ref="EB8" si="75">DY8+DZ8+EA8</f>
         <v>0</v>
       </c>
       <c r="EC8" s="164">
@@ -5398,7 +5398,7 @@
         <v>-775000</v>
       </c>
       <c r="EI8" s="172">
-        <f t="shared" ref="EI8" si="78">+IF(EH8&lt;0,0,EH8)</f>
+        <f t="shared" ref="EI8" si="76">+IF(EH8&lt;0,0,EH8)</f>
         <v>0</v>
       </c>
       <c r="EJ8" s="165">
@@ -27090,38 +27090,22 @@
   </sheetData>
   <autoFilter ref="A6:ER8" xr:uid="{00000000-0001-0000-0900-000000000000}"/>
   <mergeCells count="64">
-    <mergeCell ref="AO1:AS1"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="S4:U4"/>
-    <mergeCell ref="W4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AD4"/>
-    <mergeCell ref="AG4:AI4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="BG4:BI4"/>
-    <mergeCell ref="AT4:AU4"/>
-    <mergeCell ref="AO5:AO6"/>
-    <mergeCell ref="AP5:AP6"/>
-    <mergeCell ref="AQ5:AQ6"/>
-    <mergeCell ref="AR5:AR6"/>
-    <mergeCell ref="AS5:AS6"/>
-    <mergeCell ref="BJ4:BK4"/>
-    <mergeCell ref="BL4:BN4"/>
-    <mergeCell ref="BQ4:BS4"/>
-    <mergeCell ref="BC4:BE4"/>
-    <mergeCell ref="CD5:CD6"/>
-    <mergeCell ref="BY5:BY6"/>
-    <mergeCell ref="BZ5:BZ6"/>
-    <mergeCell ref="CA5:CA6"/>
-    <mergeCell ref="CB5:CB6"/>
-    <mergeCell ref="CC5:CC6"/>
+    <mergeCell ref="EN5:EN6"/>
+    <mergeCell ref="EI5:EI6"/>
+    <mergeCell ref="EJ5:EJ6"/>
+    <mergeCell ref="EK5:EK6"/>
+    <mergeCell ref="EL5:EL6"/>
+    <mergeCell ref="EH5:EH6"/>
+    <mergeCell ref="DV5:DX5"/>
+    <mergeCell ref="CQ5:CS5"/>
+    <mergeCell ref="DG5:DG6"/>
+    <mergeCell ref="DI5:DJ5"/>
+    <mergeCell ref="CT5:CT6"/>
+    <mergeCell ref="DH5:DH6"/>
+    <mergeCell ref="DK5:DK6"/>
+    <mergeCell ref="DM5:DR5"/>
+    <mergeCell ref="DS5:DS6"/>
+    <mergeCell ref="DU5:DU6"/>
     <mergeCell ref="ER5:ER6"/>
     <mergeCell ref="A7:EL7"/>
     <mergeCell ref="EM5:EM6"/>
@@ -27138,22 +27122,38 @@
     <mergeCell ref="DL5:DL6"/>
     <mergeCell ref="EG5:EG6"/>
     <mergeCell ref="EQ5:EQ6"/>
-    <mergeCell ref="EH5:EH6"/>
-    <mergeCell ref="DV5:DX5"/>
-    <mergeCell ref="CQ5:CS5"/>
-    <mergeCell ref="DG5:DG6"/>
-    <mergeCell ref="DI5:DJ5"/>
-    <mergeCell ref="CT5:CT6"/>
-    <mergeCell ref="DH5:DH6"/>
-    <mergeCell ref="DK5:DK6"/>
-    <mergeCell ref="DM5:DR5"/>
-    <mergeCell ref="DS5:DS6"/>
-    <mergeCell ref="DU5:DU6"/>
-    <mergeCell ref="EN5:EN6"/>
-    <mergeCell ref="EI5:EI6"/>
-    <mergeCell ref="EJ5:EJ6"/>
-    <mergeCell ref="EK5:EK6"/>
-    <mergeCell ref="EL5:EL6"/>
+    <mergeCell ref="BJ4:BK4"/>
+    <mergeCell ref="BL4:BN4"/>
+    <mergeCell ref="BQ4:BS4"/>
+    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="CD5:CD6"/>
+    <mergeCell ref="BY5:BY6"/>
+    <mergeCell ref="BZ5:BZ6"/>
+    <mergeCell ref="CA5:CA6"/>
+    <mergeCell ref="CB5:CB6"/>
+    <mergeCell ref="CC5:CC6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="BG4:BI4"/>
+    <mergeCell ref="AT4:AU4"/>
+    <mergeCell ref="AO5:AO6"/>
+    <mergeCell ref="AP5:AP6"/>
+    <mergeCell ref="AQ5:AQ6"/>
+    <mergeCell ref="AR5:AR6"/>
+    <mergeCell ref="AS5:AS6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="AO1:AS1"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="S4:U4"/>
+    <mergeCell ref="W4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="AG4:AI4"/>
   </mergeCells>
   <conditionalFormatting sqref="A5 A8:B8">
     <cfRule type="duplicateValues" dxfId="20" priority="20879"/>
@@ -27810,11 +27810,11 @@
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
       <c r="H8" s="20"/>
-      <c r="I8" s="301">
+      <c r="I8" s="307">
         <v>2026</v>
       </c>
-      <c r="J8" s="302"/>
-      <c r="K8" s="302"/>
+      <c r="J8" s="308"/>
+      <c r="K8" s="308"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="21" t="s">
@@ -27839,13 +27839,13 @@
     <row r="9" spans="1:29" ht="15.75" customHeight="1" thickBot="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="303" t="s">
+      <c r="C9" s="309" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="304"/>
-      <c r="E9" s="304"/>
-      <c r="F9" s="304"/>
-      <c r="G9" s="304"/>
+      <c r="D9" s="310"/>
+      <c r="E9" s="310"/>
+      <c r="F9" s="310"/>
+      <c r="G9" s="310"/>
       <c r="H9" s="20"/>
       <c r="I9" s="24"/>
       <c r="J9" s="24"/>
@@ -27941,19 +27941,19 @@
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
-      <c r="J12" s="305" t="s">
+      <c r="J12" s="311" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="304"/>
-      <c r="L12" s="304"/>
-      <c r="M12" s="304"/>
-      <c r="N12" s="304"/>
-      <c r="O12" s="304"/>
-      <c r="P12" s="306">
+      <c r="K12" s="310"/>
+      <c r="L12" s="310"/>
+      <c r="M12" s="310"/>
+      <c r="N12" s="310"/>
+      <c r="O12" s="310"/>
+      <c r="P12" s="312">
         <f>I8</f>
         <v>2026</v>
       </c>
-      <c r="Q12" s="304"/>
+      <c r="Q12" s="310"/>
       <c r="R12" s="33"/>
       <c r="S12" s="34"/>
       <c r="T12" s="34"/>
@@ -28217,38 +28217,38 @@
     </row>
     <row r="21" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A21" s="39"/>
-      <c r="B21" s="307" t="s">
+      <c r="B21" s="306" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="308"/>
-      <c r="D21" s="308"/>
-      <c r="E21" s="308"/>
-      <c r="F21" s="308"/>
-      <c r="G21" s="308"/>
-      <c r="H21" s="308"/>
-      <c r="I21" s="308"/>
+      <c r="C21" s="302"/>
+      <c r="D21" s="302"/>
+      <c r="E21" s="302"/>
+      <c r="F21" s="302"/>
+      <c r="G21" s="302"/>
+      <c r="H21" s="302"/>
+      <c r="I21" s="302"/>
       <c r="J21" s="40"/>
-      <c r="K21" s="309" t="s">
+      <c r="K21" s="303" t="s">
         <v>37</v>
       </c>
-      <c r="L21" s="308"/>
-      <c r="M21" s="308"/>
-      <c r="N21" s="308"/>
-      <c r="O21" s="308"/>
-      <c r="P21" s="308"/>
-      <c r="Q21" s="308"/>
-      <c r="R21" s="308"/>
+      <c r="L21" s="302"/>
+      <c r="M21" s="302"/>
+      <c r="N21" s="302"/>
+      <c r="O21" s="302"/>
+      <c r="P21" s="302"/>
+      <c r="Q21" s="302"/>
+      <c r="R21" s="302"/>
       <c r="S21" s="40"/>
-      <c r="T21" s="310" t="s">
+      <c r="T21" s="301" t="s">
         <v>38</v>
       </c>
-      <c r="U21" s="308"/>
-      <c r="V21" s="308"/>
-      <c r="W21" s="308"/>
-      <c r="X21" s="308"/>
-      <c r="Y21" s="308"/>
-      <c r="Z21" s="308"/>
-      <c r="AA21" s="308"/>
+      <c r="U21" s="302"/>
+      <c r="V21" s="302"/>
+      <c r="W21" s="302"/>
+      <c r="X21" s="302"/>
+      <c r="Y21" s="302"/>
+      <c r="Z21" s="302"/>
+      <c r="AA21" s="302"/>
       <c r="AB21" s="41"/>
       <c r="AC21" s="42"/>
     </row>
@@ -29148,38 +29148,38 @@
     </row>
     <row r="35" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="311" t="s">
+      <c r="B35" s="304" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="308"/>
-      <c r="D35" s="308"/>
-      <c r="E35" s="308"/>
-      <c r="F35" s="308"/>
-      <c r="G35" s="308"/>
-      <c r="H35" s="308"/>
-      <c r="I35" s="308"/>
+      <c r="C35" s="302"/>
+      <c r="D35" s="302"/>
+      <c r="E35" s="302"/>
+      <c r="F35" s="302"/>
+      <c r="G35" s="302"/>
+      <c r="H35" s="302"/>
+      <c r="I35" s="302"/>
       <c r="J35" s="40"/>
-      <c r="K35" s="312" t="s">
+      <c r="K35" s="305" t="s">
         <v>48</v>
       </c>
-      <c r="L35" s="308"/>
-      <c r="M35" s="308"/>
-      <c r="N35" s="308"/>
-      <c r="O35" s="308"/>
-      <c r="P35" s="308"/>
-      <c r="Q35" s="308"/>
-      <c r="R35" s="308"/>
+      <c r="L35" s="302"/>
+      <c r="M35" s="302"/>
+      <c r="N35" s="302"/>
+      <c r="O35" s="302"/>
+      <c r="P35" s="302"/>
+      <c r="Q35" s="302"/>
+      <c r="R35" s="302"/>
       <c r="S35" s="40"/>
-      <c r="T35" s="309" t="s">
+      <c r="T35" s="303" t="s">
         <v>49</v>
       </c>
-      <c r="U35" s="308"/>
-      <c r="V35" s="308"/>
-      <c r="W35" s="308"/>
-      <c r="X35" s="308"/>
-      <c r="Y35" s="308"/>
-      <c r="Z35" s="308"/>
-      <c r="AA35" s="308"/>
+      <c r="U35" s="302"/>
+      <c r="V35" s="302"/>
+      <c r="W35" s="302"/>
+      <c r="X35" s="302"/>
+      <c r="Y35" s="302"/>
+      <c r="Z35" s="302"/>
+      <c r="AA35" s="302"/>
       <c r="AB35" s="70"/>
       <c r="AC35" s="40"/>
     </row>
@@ -30068,38 +30068,38 @@
     </row>
     <row r="49" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A49" s="69"/>
-      <c r="B49" s="309" t="s">
+      <c r="B49" s="303" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="308"/>
-      <c r="D49" s="308"/>
-      <c r="E49" s="308"/>
-      <c r="F49" s="308"/>
-      <c r="G49" s="308"/>
-      <c r="H49" s="308"/>
-      <c r="I49" s="308"/>
+      <c r="C49" s="302"/>
+      <c r="D49" s="302"/>
+      <c r="E49" s="302"/>
+      <c r="F49" s="302"/>
+      <c r="G49" s="302"/>
+      <c r="H49" s="302"/>
+      <c r="I49" s="302"/>
       <c r="J49" s="40"/>
-      <c r="K49" s="311" t="s">
+      <c r="K49" s="304" t="s">
         <v>51</v>
       </c>
-      <c r="L49" s="308"/>
-      <c r="M49" s="308"/>
-      <c r="N49" s="308"/>
-      <c r="O49" s="308"/>
-      <c r="P49" s="308"/>
-      <c r="Q49" s="308"/>
-      <c r="R49" s="308"/>
+      <c r="L49" s="302"/>
+      <c r="M49" s="302"/>
+      <c r="N49" s="302"/>
+      <c r="O49" s="302"/>
+      <c r="P49" s="302"/>
+      <c r="Q49" s="302"/>
+      <c r="R49" s="302"/>
       <c r="S49" s="40"/>
-      <c r="T49" s="307" t="s">
+      <c r="T49" s="306" t="s">
         <v>52</v>
       </c>
-      <c r="U49" s="308"/>
-      <c r="V49" s="308"/>
-      <c r="W49" s="308"/>
-      <c r="X49" s="308"/>
-      <c r="Y49" s="308"/>
-      <c r="Z49" s="308"/>
-      <c r="AA49" s="308"/>
+      <c r="U49" s="302"/>
+      <c r="V49" s="302"/>
+      <c r="W49" s="302"/>
+      <c r="X49" s="302"/>
+      <c r="Y49" s="302"/>
+      <c r="Z49" s="302"/>
+      <c r="AA49" s="302"/>
       <c r="AB49" s="70"/>
       <c r="AC49" s="40"/>
     </row>
@@ -30988,38 +30988,38 @@
     </row>
     <row r="63" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A63" s="69"/>
-      <c r="B63" s="310" t="s">
+      <c r="B63" s="301" t="s">
         <v>53</v>
       </c>
-      <c r="C63" s="308"/>
-      <c r="D63" s="308"/>
-      <c r="E63" s="308"/>
-      <c r="F63" s="308"/>
-      <c r="G63" s="308"/>
-      <c r="H63" s="308"/>
-      <c r="I63" s="308"/>
+      <c r="C63" s="302"/>
+      <c r="D63" s="302"/>
+      <c r="E63" s="302"/>
+      <c r="F63" s="302"/>
+      <c r="G63" s="302"/>
+      <c r="H63" s="302"/>
+      <c r="I63" s="302"/>
       <c r="J63" s="40"/>
-      <c r="K63" s="309" t="s">
+      <c r="K63" s="303" t="s">
         <v>54</v>
       </c>
-      <c r="L63" s="308"/>
-      <c r="M63" s="308"/>
-      <c r="N63" s="308"/>
-      <c r="O63" s="308"/>
-      <c r="P63" s="308"/>
-      <c r="Q63" s="308"/>
-      <c r="R63" s="308"/>
+      <c r="L63" s="302"/>
+      <c r="M63" s="302"/>
+      <c r="N63" s="302"/>
+      <c r="O63" s="302"/>
+      <c r="P63" s="302"/>
+      <c r="Q63" s="302"/>
+      <c r="R63" s="302"/>
       <c r="S63" s="40"/>
-      <c r="T63" s="311" t="s">
+      <c r="T63" s="304" t="s">
         <v>55</v>
       </c>
-      <c r="U63" s="308"/>
-      <c r="V63" s="308"/>
-      <c r="W63" s="308"/>
-      <c r="X63" s="308"/>
-      <c r="Y63" s="308"/>
-      <c r="Z63" s="308"/>
-      <c r="AA63" s="308"/>
+      <c r="U63" s="302"/>
+      <c r="V63" s="302"/>
+      <c r="W63" s="302"/>
+      <c r="X63" s="302"/>
+      <c r="Y63" s="302"/>
+      <c r="Z63" s="302"/>
+      <c r="AA63" s="302"/>
       <c r="AB63" s="70"/>
       <c r="AC63" s="40"/>
     </row>
@@ -60554,6 +60554,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="J12:O12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="K21:R21"/>
     <mergeCell ref="B63:I63"/>
     <mergeCell ref="K63:R63"/>
     <mergeCell ref="T63:AA63"/>
@@ -60564,12 +60570,6 @@
     <mergeCell ref="B49:I49"/>
     <mergeCell ref="K49:R49"/>
     <mergeCell ref="T49:AA49"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="J12:O12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="K21:R21"/>
   </mergeCells>
   <conditionalFormatting sqref="C51:I55">
     <cfRule type="expression" dxfId="2" priority="3">

</xml_diff>

<commit_message>
hot fix những công thức support cho các công ty nhỏ
</commit_message>
<xml_diff>
--- a/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
+++ b/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonzai/dev/odoo 19/odoo/my_custom_addons/dl_salary_kpi/static/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{727446F4-B647-DE4F-833B-DDB1CC986A9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87EFFE75-9BC6-A84B-8B84-DE1CD0F87995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="17820" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kangatang" sheetId="43" state="veryHidden" r:id="rId1"/>
@@ -1100,7 +1100,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="25">
+  <fills count="27">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1241,6 +1241,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1764,7 +1776,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="313">
+  <cellXfs count="315">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="169" fontId="12" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2421,82 +2433,16 @@
     <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="66" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="67" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="67" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2532,33 +2478,83 @@
     <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="66" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="67" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="7" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2573,6 +2569,28 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="78" fillId="25" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="78" fillId="26" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="32">
@@ -2833,7 +2851,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4870450" y="266700"/>
+          <a:off x="4095750" y="266700"/>
           <a:ext cx="914400" cy="38100"/>
           <a:chOff x="4888800" y="3780000"/>
           <a:chExt cx="914400" cy="0"/>
@@ -3274,86 +3292,86 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:ER165"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="20" outlineLevelCol="2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="20" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="17.83203125" style="95" customWidth="1"/>
-    <col min="2" max="2" width="30.1640625" style="95" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" style="94" customWidth="1"/>
-    <col min="4" max="4" width="24.33203125" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="5" width="29.1640625" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="6" max="6" width="15.33203125" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="7" max="7" width="31.83203125" style="220" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="8" max="8" width="13.83203125" style="95" customWidth="1" collapsed="1"/>
-    <col min="9" max="9" width="25.1640625" style="101" customWidth="1"/>
-    <col min="10" max="40" width="11.83203125" style="1" customWidth="1" outlineLevel="1"/>
-    <col min="41" max="43" width="15.83203125" style="92" customWidth="1" outlineLevel="1"/>
-    <col min="44" max="44" width="14.33203125" style="1" customWidth="1" outlineLevel="1"/>
-    <col min="45" max="45" width="14.6640625" style="228" customWidth="1" outlineLevel="1"/>
+    <col min="1" max="1" width="17.796875" style="95" customWidth="1"/>
+    <col min="2" max="2" width="30.19921875" style="95" customWidth="1"/>
+    <col min="3" max="3" width="45.796875" style="94" customWidth="1"/>
+    <col min="4" max="4" width="24.3984375" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="29.19921875" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="15.3984375" style="100" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="31.796875" style="220" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="13.796875" style="95" customWidth="1" collapsed="1"/>
+    <col min="9" max="9" width="25.19921875" style="101" customWidth="1"/>
+    <col min="10" max="40" width="11.796875" style="1" customWidth="1" outlineLevel="1"/>
+    <col min="41" max="43" width="15.796875" style="92" customWidth="1" outlineLevel="1"/>
+    <col min="44" max="44" width="14.3984375" style="1" customWidth="1" outlineLevel="1"/>
+    <col min="45" max="45" width="14.59765625" style="228" customWidth="1" outlineLevel="1"/>
     <col min="46" max="54" width="13" style="1" customWidth="1" outlineLevel="1"/>
     <col min="55" max="55" width="13" style="102" customWidth="1" outlineLevel="1"/>
     <col min="56" max="59" width="13" style="1" customWidth="1" outlineLevel="1"/>
-    <col min="60" max="60" width="15.83203125" style="1" customWidth="1" outlineLevel="1"/>
+    <col min="60" max="60" width="15.796875" style="1" customWidth="1" outlineLevel="1"/>
     <col min="61" max="66" width="13" style="1" customWidth="1" outlineLevel="1"/>
-    <col min="67" max="67" width="15.1640625" style="1" customWidth="1" outlineLevel="1"/>
+    <col min="67" max="67" width="15.19921875" style="1" customWidth="1" outlineLevel="1"/>
     <col min="68" max="73" width="13" style="1" customWidth="1" outlineLevel="1"/>
     <col min="74" max="74" width="15" style="1" customWidth="1" outlineLevel="1"/>
     <col min="75" max="76" width="13" style="1" customWidth="1" outlineLevel="1"/>
-    <col min="77" max="83" width="15.6640625" style="136" customWidth="1" outlineLevel="1"/>
-    <col min="84" max="84" width="17.6640625" style="147" customWidth="1"/>
-    <col min="85" max="85" width="16.6640625" style="136" customWidth="1"/>
+    <col min="77" max="83" width="15.59765625" style="136" customWidth="1" outlineLevel="1"/>
+    <col min="84" max="84" width="17.59765625" style="147" customWidth="1"/>
+    <col min="85" max="85" width="16.59765625" style="136" customWidth="1"/>
     <col min="86" max="86" width="14" style="147" customWidth="1"/>
-    <col min="87" max="87" width="15.83203125" style="147" customWidth="1"/>
-    <col min="88" max="88" width="16.83203125" style="136" customWidth="1"/>
+    <col min="87" max="87" width="15.796875" style="147" customWidth="1"/>
+    <col min="88" max="88" width="16.796875" style="136" customWidth="1"/>
     <col min="89" max="93" width="14" style="136" customWidth="1"/>
     <col min="94" max="94" width="14" style="136" customWidth="1" outlineLevel="1"/>
-    <col min="95" max="95" width="26.1640625" style="1" customWidth="1" outlineLevel="1"/>
-    <col min="96" max="96" width="26.1640625" style="102" customWidth="1" outlineLevel="1"/>
-    <col min="97" max="97" width="26.1640625" style="225" customWidth="1" outlineLevel="1"/>
-    <col min="98" max="98" width="24.1640625" style="102" customWidth="1" outlineLevel="1"/>
+    <col min="95" max="95" width="26.19921875" style="1" customWidth="1" outlineLevel="1"/>
+    <col min="96" max="96" width="26.19921875" style="102" customWidth="1" outlineLevel="1"/>
+    <col min="97" max="97" width="26.19921875" style="225" customWidth="1" outlineLevel="1"/>
+    <col min="98" max="98" width="24.19921875" style="102" customWidth="1" outlineLevel="1"/>
     <col min="99" max="99" width="26" style="136" customWidth="1"/>
-    <col min="100" max="100" width="21.83203125" style="136" customWidth="1"/>
-    <col min="101" max="101" width="21.1640625" style="136" customWidth="1"/>
-    <col min="102" max="102" width="18.6640625" style="136" customWidth="1"/>
-    <col min="103" max="103" width="16.1640625" style="136" customWidth="1"/>
-    <col min="104" max="104" width="18.6640625" style="136" customWidth="1"/>
-    <col min="105" max="105" width="20.83203125" style="136" customWidth="1"/>
-    <col min="106" max="107" width="16.33203125" style="136" customWidth="1"/>
-    <col min="108" max="108" width="23.33203125" style="136" customWidth="1"/>
-    <col min="109" max="110" width="27.83203125" style="210" customWidth="1"/>
-    <col min="111" max="111" width="27.83203125" style="255" customWidth="1"/>
-    <col min="112" max="112" width="25.1640625" style="136" customWidth="1"/>
-    <col min="113" max="113" width="22.6640625" style="102" customWidth="1"/>
-    <col min="114" max="114" width="24.83203125" style="102" customWidth="1"/>
-    <col min="115" max="115" width="27.6640625" style="102" customWidth="1"/>
-    <col min="116" max="116" width="33.83203125" style="102" customWidth="1"/>
-    <col min="117" max="119" width="25.83203125" style="102" customWidth="1"/>
-    <col min="120" max="120" width="20.83203125" style="143" customWidth="1"/>
-    <col min="121" max="121" width="22.1640625" style="143" customWidth="1"/>
-    <col min="122" max="122" width="22.83203125" style="143" customWidth="1"/>
-    <col min="123" max="123" width="31.83203125" style="102" customWidth="1"/>
-    <col min="124" max="124" width="26.6640625" style="102" customWidth="1"/>
-    <col min="125" max="125" width="24.83203125" style="102" customWidth="1" outlineLevel="2"/>
-    <col min="126" max="126" width="27.33203125" style="102" customWidth="1" outlineLevel="2"/>
-    <col min="127" max="127" width="27.33203125" style="99" customWidth="1" outlineLevel="2"/>
-    <col min="128" max="128" width="27.33203125" style="102" customWidth="1" outlineLevel="2"/>
-    <col min="129" max="129" width="23.6640625" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="130" max="131" width="22.1640625" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="132" max="132" width="28.1640625" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="133" max="133" width="27.83203125" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="134" max="134" width="28.83203125" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="135" max="135" width="29.1640625" style="102" customWidth="1" outlineLevel="2"/>
-    <col min="136" max="136" width="21.83203125" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="137" max="137" width="25.33203125" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="138" max="138" width="24.1640625" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="139" max="139" width="21.1640625" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="100" max="100" width="21.796875" style="136" customWidth="1"/>
+    <col min="101" max="101" width="21.19921875" style="136" customWidth="1"/>
+    <col min="102" max="102" width="18.59765625" style="136" customWidth="1"/>
+    <col min="103" max="103" width="16.19921875" style="136" customWidth="1"/>
+    <col min="104" max="104" width="18.59765625" style="136" customWidth="1"/>
+    <col min="105" max="105" width="20.796875" style="136" customWidth="1"/>
+    <col min="106" max="107" width="16.3984375" style="136" customWidth="1"/>
+    <col min="108" max="108" width="23.3984375" style="136" customWidth="1"/>
+    <col min="109" max="110" width="27.796875" style="210" customWidth="1"/>
+    <col min="111" max="111" width="27.796875" style="255" customWidth="1"/>
+    <col min="112" max="112" width="25.19921875" style="136" customWidth="1"/>
+    <col min="113" max="113" width="22.59765625" style="102" customWidth="1"/>
+    <col min="114" max="114" width="24.796875" style="102" customWidth="1"/>
+    <col min="115" max="115" width="27.59765625" style="102" customWidth="1"/>
+    <col min="116" max="116" width="33.796875" style="102" customWidth="1"/>
+    <col min="117" max="119" width="25.796875" style="102" customWidth="1"/>
+    <col min="120" max="120" width="20.796875" style="143" customWidth="1"/>
+    <col min="121" max="121" width="22.19921875" style="143" customWidth="1"/>
+    <col min="122" max="122" width="22.796875" style="143" customWidth="1"/>
+    <col min="123" max="123" width="31.796875" style="102" customWidth="1"/>
+    <col min="124" max="124" width="26.59765625" style="102" customWidth="1"/>
+    <col min="125" max="125" width="24.796875" style="102" customWidth="1" outlineLevel="2"/>
+    <col min="126" max="126" width="27.3984375" style="102" customWidth="1" outlineLevel="2"/>
+    <col min="127" max="127" width="27.3984375" style="99" customWidth="1" outlineLevel="2"/>
+    <col min="128" max="128" width="27.3984375" style="102" customWidth="1" outlineLevel="2"/>
+    <col min="129" max="129" width="23.59765625" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="130" max="131" width="22.19921875" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="132" max="132" width="28.19921875" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="133" max="133" width="27.796875" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="134" max="134" width="28.796875" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="135" max="135" width="29.19921875" style="102" customWidth="1" outlineLevel="2"/>
+    <col min="136" max="136" width="21.796875" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="137" max="137" width="25.3984375" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="138" max="138" width="24.19921875" style="94" customWidth="1" outlineLevel="2"/>
+    <col min="139" max="139" width="21.19921875" style="94" customWidth="1" outlineLevel="2"/>
     <col min="140" max="140" width="25" style="94" customWidth="1" outlineLevel="2"/>
-    <col min="141" max="141" width="29.1640625" style="95" customWidth="1" outlineLevel="2"/>
-    <col min="142" max="145" width="31.6640625" style="95" customWidth="1" outlineLevel="2"/>
-    <col min="146" max="146" width="36.33203125" style="95" customWidth="1"/>
-    <col min="147" max="147" width="35.83203125" style="95" customWidth="1"/>
-    <col min="148" max="148" width="41.83203125" style="242" customWidth="1"/>
-    <col min="149" max="150" width="9.1640625" style="94" customWidth="1"/>
-    <col min="151" max="16384" width="9.1640625" style="94"/>
+    <col min="141" max="141" width="29.19921875" style="95" customWidth="1" outlineLevel="2"/>
+    <col min="142" max="145" width="31.59765625" style="95" customWidth="1" outlineLevel="2"/>
+    <col min="146" max="146" width="36.3984375" style="95" customWidth="1"/>
+    <col min="147" max="147" width="35.796875" style="95" customWidth="1"/>
+    <col min="148" max="148" width="41.796875" style="242" customWidth="1"/>
+    <col min="149" max="150" width="9.19921875" style="94" customWidth="1"/>
+    <col min="151" max="16384" width="9.19921875" style="94"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:148" s="127" customFormat="1" ht="37.5" customHeight="1">
@@ -3397,11 +3415,11 @@
       <c r="AL1" s="212"/>
       <c r="AM1" s="212"/>
       <c r="AN1" s="212"/>
-      <c r="AO1" s="260"/>
-      <c r="AP1" s="260"/>
-      <c r="AQ1" s="260"/>
-      <c r="AR1" s="260"/>
-      <c r="AS1" s="260"/>
+      <c r="AO1" s="300"/>
+      <c r="AP1" s="300"/>
+      <c r="AQ1" s="300"/>
+      <c r="AR1" s="300"/>
+      <c r="AS1" s="300"/>
       <c r="AT1" s="120"/>
       <c r="AU1" s="120"/>
       <c r="AV1" s="120"/>
@@ -3803,10 +3821,10 @@
       <c r="G4" s="232"/>
       <c r="H4" s="108"/>
       <c r="I4" s="256"/>
-      <c r="J4" s="261" t="s">
+      <c r="J4" s="293" t="s">
         <v>68</v>
       </c>
-      <c r="K4" s="261"/>
+      <c r="K4" s="293"/>
       <c r="L4" s="258">
         <v>3</v>
       </c>
@@ -3820,23 +3838,23 @@
       </c>
       <c r="Q4" s="259"/>
       <c r="R4" s="109"/>
-      <c r="S4" s="261"/>
-      <c r="T4" s="261"/>
-      <c r="U4" s="261"/>
+      <c r="S4" s="293"/>
+      <c r="T4" s="293"/>
+      <c r="U4" s="293"/>
       <c r="V4" s="109"/>
-      <c r="W4" s="261"/>
-      <c r="X4" s="261"/>
-      <c r="Y4" s="261"/>
-      <c r="Z4" s="261"/>
-      <c r="AA4" s="261"/>
-      <c r="AB4" s="261"/>
-      <c r="AC4" s="261"/>
-      <c r="AD4" s="261"/>
+      <c r="W4" s="293"/>
+      <c r="X4" s="293"/>
+      <c r="Y4" s="293"/>
+      <c r="Z4" s="293"/>
+      <c r="AA4" s="293"/>
+      <c r="AB4" s="293"/>
+      <c r="AC4" s="293"/>
+      <c r="AD4" s="293"/>
       <c r="AE4" s="109"/>
       <c r="AF4" s="110"/>
-      <c r="AG4" s="261"/>
-      <c r="AH4" s="261"/>
-      <c r="AI4" s="261"/>
+      <c r="AG4" s="293"/>
+      <c r="AH4" s="293"/>
+      <c r="AI4" s="293"/>
       <c r="AJ4" s="109"/>
       <c r="AK4" s="109"/>
       <c r="AL4" s="109"/>
@@ -3847,10 +3865,10 @@
       <c r="AQ4" s="113"/>
       <c r="AR4" s="221"/>
       <c r="AS4" s="227"/>
-      <c r="AT4" s="261" t="s">
+      <c r="AT4" s="293" t="s">
         <v>68</v>
       </c>
-      <c r="AU4" s="261"/>
+      <c r="AU4" s="293"/>
       <c r="AV4" s="258">
         <f>L4</f>
         <v>3</v>
@@ -3866,23 +3884,23 @@
       </c>
       <c r="BA4" s="259"/>
       <c r="BB4" s="109"/>
-      <c r="BC4" s="261"/>
-      <c r="BD4" s="261"/>
-      <c r="BE4" s="261"/>
+      <c r="BC4" s="293"/>
+      <c r="BD4" s="293"/>
+      <c r="BE4" s="293"/>
       <c r="BF4" s="109"/>
-      <c r="BG4" s="261"/>
-      <c r="BH4" s="261"/>
-      <c r="BI4" s="261"/>
-      <c r="BJ4" s="261"/>
-      <c r="BK4" s="261"/>
-      <c r="BL4" s="261"/>
-      <c r="BM4" s="261"/>
-      <c r="BN4" s="261"/>
+      <c r="BG4" s="293"/>
+      <c r="BH4" s="293"/>
+      <c r="BI4" s="293"/>
+      <c r="BJ4" s="293"/>
+      <c r="BK4" s="293"/>
+      <c r="BL4" s="293"/>
+      <c r="BM4" s="293"/>
+      <c r="BN4" s="293"/>
       <c r="BO4" s="109"/>
       <c r="BP4" s="110"/>
-      <c r="BQ4" s="261"/>
-      <c r="BR4" s="261"/>
-      <c r="BS4" s="261"/>
+      <c r="BQ4" s="293"/>
+      <c r="BR4" s="293"/>
+      <c r="BS4" s="293"/>
       <c r="BT4" s="114"/>
       <c r="BU4" s="114" t="str">
         <f>IF(WEEKDAY(BU5,1)=1,"CN","")</f>
@@ -3962,31 +3980,31 @@
       <c r="ER4" s="237"/>
     </row>
     <row r="5" spans="1:148" s="183" customFormat="1" ht="92.25" customHeight="1">
-      <c r="A5" s="262" t="s">
+      <c r="A5" s="288" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="263" t="s">
+      <c r="B5" s="278" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="262" t="s">
+      <c r="C5" s="288" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="264" t="s">
+      <c r="D5" s="297" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="265" t="s">
+      <c r="E5" s="298" t="s">
         <v>120</v>
       </c>
-      <c r="F5" s="262" t="s">
+      <c r="F5" s="288" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="262" t="s">
+      <c r="G5" s="288" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="262" t="s">
+      <c r="H5" s="288" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="267" t="s">
+      <c r="I5" s="294" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="174">
@@ -4113,19 +4131,19 @@
         <f t="shared" si="0"/>
         <v>46112</v>
       </c>
-      <c r="AO5" s="268" t="s">
+      <c r="AO5" s="295" t="s">
         <v>82</v>
       </c>
-      <c r="AP5" s="268" t="s">
+      <c r="AP5" s="295" t="s">
         <v>83</v>
       </c>
-      <c r="AQ5" s="268" t="s">
+      <c r="AQ5" s="295" t="s">
         <v>84</v>
       </c>
-      <c r="AR5" s="269" t="s">
+      <c r="AR5" s="296" t="s">
         <v>5</v>
       </c>
-      <c r="AS5" s="269" t="s">
+      <c r="AS5" s="296" t="s">
         <v>6</v>
       </c>
       <c r="AT5" s="178">
@@ -4252,46 +4270,46 @@
         <f t="shared" si="1"/>
         <v>46112</v>
       </c>
-      <c r="BY5" s="270" t="s">
+      <c r="BY5" s="290" t="s">
         <v>85</v>
       </c>
-      <c r="BZ5" s="270" t="s">
+      <c r="BZ5" s="290" t="s">
         <v>86</v>
       </c>
-      <c r="CA5" s="270" t="s">
+      <c r="CA5" s="290" t="s">
         <v>87</v>
       </c>
-      <c r="CB5" s="270" t="s">
+      <c r="CB5" s="290" t="s">
         <v>88</v>
       </c>
-      <c r="CC5" s="270" t="s">
+      <c r="CC5" s="290" t="s">
         <v>89</v>
       </c>
-      <c r="CD5" s="270" t="s">
+      <c r="CD5" s="290" t="s">
         <v>90</v>
       </c>
-      <c r="CE5" s="270" t="s">
+      <c r="CE5" s="290" t="s">
         <v>91</v>
       </c>
-      <c r="CF5" s="284" t="s">
+      <c r="CF5" s="289" t="s">
         <v>19</v>
       </c>
-      <c r="CG5" s="284"/>
-      <c r="CH5" s="284"/>
-      <c r="CI5" s="284"/>
-      <c r="CJ5" s="284"/>
-      <c r="CK5" s="284"/>
-      <c r="CL5" s="284"/>
-      <c r="CM5" s="284"/>
-      <c r="CN5" s="284"/>
-      <c r="CO5" s="284"/>
-      <c r="CP5" s="284"/>
-      <c r="CQ5" s="288" t="s">
+      <c r="CG5" s="289"/>
+      <c r="CH5" s="289"/>
+      <c r="CI5" s="289"/>
+      <c r="CJ5" s="289"/>
+      <c r="CK5" s="289"/>
+      <c r="CL5" s="289"/>
+      <c r="CM5" s="289"/>
+      <c r="CN5" s="289"/>
+      <c r="CO5" s="289"/>
+      <c r="CP5" s="289"/>
+      <c r="CQ5" s="266" t="s">
         <v>59</v>
       </c>
-      <c r="CR5" s="289"/>
-      <c r="CS5" s="290"/>
-      <c r="CT5" s="295" t="s">
+      <c r="CR5" s="267"/>
+      <c r="CS5" s="268"/>
+      <c r="CT5" s="273" t="s">
         <v>60</v>
       </c>
       <c r="CU5" s="247" t="s">
@@ -4314,107 +4332,107 @@
       <c r="DF5" s="245" t="s">
         <v>127</v>
       </c>
-      <c r="DG5" s="291" t="s">
+      <c r="DG5" s="269" t="s">
         <v>117</v>
       </c>
-      <c r="DH5" s="296" t="s">
+      <c r="DH5" s="274" t="s">
         <v>112</v>
       </c>
-      <c r="DI5" s="293" t="s">
+      <c r="DI5" s="271" t="s">
         <v>81</v>
       </c>
-      <c r="DJ5" s="294"/>
-      <c r="DK5" s="281" t="s">
+      <c r="DJ5" s="272"/>
+      <c r="DK5" s="275" t="s">
         <v>61</v>
       </c>
-      <c r="DL5" s="285" t="s">
+      <c r="DL5" s="292" t="s">
         <v>8</v>
       </c>
-      <c r="DM5" s="282" t="s">
+      <c r="DM5" s="276" t="s">
         <v>71</v>
       </c>
-      <c r="DN5" s="282"/>
-      <c r="DO5" s="282"/>
-      <c r="DP5" s="282"/>
-      <c r="DQ5" s="282"/>
-      <c r="DR5" s="282"/>
-      <c r="DS5" s="297" t="s">
+      <c r="DN5" s="276"/>
+      <c r="DO5" s="276"/>
+      <c r="DP5" s="276"/>
+      <c r="DQ5" s="276"/>
+      <c r="DR5" s="276"/>
+      <c r="DS5" s="277" t="s">
         <v>12</v>
       </c>
-      <c r="DT5" s="282" t="s">
+      <c r="DT5" s="276" t="s">
         <v>125</v>
       </c>
-      <c r="DU5" s="263" t="s">
+      <c r="DU5" s="278" t="s">
         <v>13</v>
       </c>
-      <c r="DV5" s="286" t="s">
+      <c r="DV5" s="264" t="s">
         <v>64</v>
       </c>
-      <c r="DW5" s="287"/>
-      <c r="DX5" s="286"/>
-      <c r="DY5" s="279" t="s">
+      <c r="DW5" s="265"/>
+      <c r="DX5" s="264"/>
+      <c r="DY5" s="286" t="s">
         <v>63</v>
       </c>
-      <c r="DZ5" s="279"/>
-      <c r="EA5" s="279"/>
-      <c r="EB5" s="279"/>
-      <c r="EC5" s="280" t="s">
+      <c r="DZ5" s="286"/>
+      <c r="EA5" s="286"/>
+      <c r="EB5" s="286"/>
+      <c r="EC5" s="287" t="s">
         <v>128</v>
       </c>
-      <c r="ED5" s="282" t="s">
+      <c r="ED5" s="276" t="s">
         <v>7</v>
       </c>
-      <c r="EE5" s="283" t="s">
+      <c r="EE5" s="262" t="s">
         <v>65</v>
       </c>
-      <c r="EF5" s="283"/>
-      <c r="EG5" s="283" t="s">
+      <c r="EF5" s="262"/>
+      <c r="EG5" s="262" t="s">
         <v>66</v>
       </c>
-      <c r="EH5" s="283" t="s">
+      <c r="EH5" s="262" t="s">
         <v>67</v>
       </c>
-      <c r="EI5" s="283" t="s">
+      <c r="EI5" s="262" t="s">
         <v>72</v>
       </c>
-      <c r="EJ5" s="300" t="s">
+      <c r="EJ5" s="263" t="s">
         <v>78</v>
       </c>
-      <c r="EK5" s="300" t="s">
+      <c r="EK5" s="263" t="s">
         <v>80</v>
       </c>
-      <c r="EL5" s="300" t="s">
+      <c r="EL5" s="263" t="s">
         <v>79</v>
       </c>
-      <c r="EM5" s="274" t="s">
+      <c r="EM5" s="281" t="s">
         <v>124</v>
       </c>
-      <c r="EN5" s="298" t="s">
+      <c r="EN5" s="260" t="s">
         <v>118</v>
       </c>
-      <c r="EO5" s="276" t="s">
+      <c r="EO5" s="283" t="s">
         <v>130</v>
       </c>
-      <c r="EP5" s="278" t="s">
+      <c r="EP5" s="285" t="s">
         <v>122</v>
       </c>
-      <c r="EQ5" s="278" t="s">
+      <c r="EQ5" s="285" t="s">
         <v>121</v>
       </c>
-      <c r="ER5" s="272" t="s">
+      <c r="ER5" s="279" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:148" s="205" customFormat="1" ht="148.5" customHeight="1">
-      <c r="A6" s="262"/>
-      <c r="B6" s="263"/>
-      <c r="C6" s="262"/>
-      <c r="D6" s="264"/>
-      <c r="E6" s="266"/>
-      <c r="F6" s="262"/>
-      <c r="G6" s="262"/>
-      <c r="H6" s="262"/>
-      <c r="I6" s="267"/>
+      <c r="A6" s="288"/>
+      <c r="B6" s="278"/>
+      <c r="C6" s="288"/>
+      <c r="D6" s="297"/>
+      <c r="E6" s="299"/>
+      <c r="F6" s="288"/>
+      <c r="G6" s="288"/>
+      <c r="H6" s="288"/>
+      <c r="I6" s="294"/>
       <c r="J6" s="184" t="str">
         <f t="shared" ref="J6:AN6" si="2">IF(WEEKDAY(J5)=1,"CN",WEEKDAY(J5))</f>
         <v>CN</v>
@@ -4539,11 +4557,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AO6" s="268"/>
-      <c r="AP6" s="268"/>
-      <c r="AQ6" s="268"/>
-      <c r="AR6" s="269"/>
-      <c r="AS6" s="269"/>
+      <c r="AO6" s="295"/>
+      <c r="AP6" s="295"/>
+      <c r="AQ6" s="295"/>
+      <c r="AR6" s="296"/>
+      <c r="AS6" s="296"/>
       <c r="AT6" s="186" t="str">
         <f>+J6</f>
         <v>CN</v>
@@ -4668,13 +4686,13 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="BY6" s="271"/>
-      <c r="BZ6" s="271"/>
-      <c r="CA6" s="271"/>
-      <c r="CB6" s="271"/>
-      <c r="CC6" s="271"/>
-      <c r="CD6" s="271"/>
-      <c r="CE6" s="271"/>
+      <c r="BY6" s="291"/>
+      <c r="BZ6" s="291"/>
+      <c r="CA6" s="291"/>
+      <c r="CB6" s="291"/>
+      <c r="CC6" s="291"/>
+      <c r="CD6" s="291"/>
+      <c r="CE6" s="291"/>
       <c r="CF6" s="188" t="s">
         <v>92</v>
       </c>
@@ -4717,7 +4735,7 @@
       <c r="CS6" s="180" t="s">
         <v>58</v>
       </c>
-      <c r="CT6" s="295"/>
+      <c r="CT6" s="273"/>
       <c r="CU6" s="188" t="s">
         <v>103</v>
       </c>
@@ -4754,16 +4772,16 @@
       <c r="DF6" s="246" t="s">
         <v>129</v>
       </c>
-      <c r="DG6" s="292"/>
-      <c r="DH6" s="296"/>
+      <c r="DG6" s="270"/>
+      <c r="DH6" s="274"/>
       <c r="DI6" s="152" t="s">
         <v>14</v>
       </c>
       <c r="DJ6" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="DK6" s="281"/>
-      <c r="DL6" s="285"/>
+      <c r="DK6" s="275"/>
+      <c r="DL6" s="292"/>
       <c r="DM6" s="180" t="s">
         <v>9</v>
       </c>
@@ -4782,9 +4800,9 @@
       <c r="DR6" s="180" t="s">
         <v>115</v>
       </c>
-      <c r="DS6" s="297"/>
-      <c r="DT6" s="282"/>
-      <c r="DU6" s="263"/>
+      <c r="DS6" s="277"/>
+      <c r="DT6" s="276"/>
+      <c r="DU6" s="278"/>
       <c r="DV6" s="203">
         <v>0.17499999999999999</v>
       </c>
@@ -4806,170 +4824,170 @@
       <c r="EB6" s="152" t="s">
         <v>62</v>
       </c>
-      <c r="EC6" s="281"/>
-      <c r="ED6" s="282"/>
+      <c r="EC6" s="275"/>
+      <c r="ED6" s="276"/>
       <c r="EE6" s="182" t="s">
         <v>73</v>
       </c>
       <c r="EF6" s="182" t="s">
         <v>74</v>
       </c>
-      <c r="EG6" s="283"/>
-      <c r="EH6" s="283"/>
-      <c r="EI6" s="283"/>
-      <c r="EJ6" s="300"/>
-      <c r="EK6" s="300"/>
-      <c r="EL6" s="300"/>
-      <c r="EM6" s="275"/>
-      <c r="EN6" s="299"/>
-      <c r="EO6" s="277"/>
-      <c r="EP6" s="278"/>
-      <c r="EQ6" s="278"/>
-      <c r="ER6" s="272"/>
+      <c r="EG6" s="262"/>
+      <c r="EH6" s="262"/>
+      <c r="EI6" s="262"/>
+      <c r="EJ6" s="263"/>
+      <c r="EK6" s="263"/>
+      <c r="EL6" s="263"/>
+      <c r="EM6" s="282"/>
+      <c r="EN6" s="261"/>
+      <c r="EO6" s="284"/>
+      <c r="EP6" s="285"/>
+      <c r="EQ6" s="285"/>
+      <c r="ER6" s="279"/>
     </row>
     <row r="7" spans="1:148" s="106" customFormat="1" ht="87.75" customHeight="1">
-      <c r="A7" s="273"/>
-      <c r="B7" s="273"/>
-      <c r="C7" s="273"/>
-      <c r="D7" s="273"/>
-      <c r="E7" s="273"/>
-      <c r="F7" s="273"/>
-      <c r="G7" s="273"/>
-      <c r="H7" s="273"/>
-      <c r="I7" s="273"/>
-      <c r="J7" s="273"/>
-      <c r="K7" s="273"/>
-      <c r="L7" s="273"/>
-      <c r="M7" s="273"/>
-      <c r="N7" s="273"/>
-      <c r="O7" s="273"/>
-      <c r="P7" s="273"/>
-      <c r="Q7" s="273"/>
-      <c r="R7" s="273"/>
-      <c r="S7" s="273"/>
-      <c r="T7" s="273"/>
-      <c r="U7" s="273"/>
-      <c r="V7" s="273"/>
-      <c r="W7" s="273"/>
-      <c r="X7" s="273"/>
-      <c r="Y7" s="273"/>
-      <c r="Z7" s="273"/>
-      <c r="AA7" s="273"/>
-      <c r="AB7" s="273"/>
-      <c r="AC7" s="273"/>
-      <c r="AD7" s="273"/>
-      <c r="AE7" s="273"/>
-      <c r="AF7" s="273"/>
-      <c r="AG7" s="273"/>
-      <c r="AH7" s="273"/>
-      <c r="AI7" s="273"/>
-      <c r="AJ7" s="273"/>
-      <c r="AK7" s="273"/>
-      <c r="AL7" s="273"/>
-      <c r="AM7" s="273"/>
-      <c r="AN7" s="273"/>
-      <c r="AO7" s="273"/>
-      <c r="AP7" s="273"/>
-      <c r="AQ7" s="273"/>
-      <c r="AR7" s="273"/>
-      <c r="AS7" s="273"/>
-      <c r="AT7" s="273"/>
-      <c r="AU7" s="273"/>
-      <c r="AV7" s="273"/>
-      <c r="AW7" s="273"/>
-      <c r="AX7" s="273"/>
-      <c r="AY7" s="273"/>
-      <c r="AZ7" s="273"/>
-      <c r="BA7" s="273"/>
-      <c r="BB7" s="273"/>
-      <c r="BC7" s="273"/>
-      <c r="BD7" s="273"/>
-      <c r="BE7" s="273"/>
-      <c r="BF7" s="273"/>
-      <c r="BG7" s="273"/>
-      <c r="BH7" s="273"/>
-      <c r="BI7" s="273"/>
-      <c r="BJ7" s="273"/>
-      <c r="BK7" s="273"/>
-      <c r="BL7" s="273"/>
-      <c r="BM7" s="273"/>
-      <c r="BN7" s="273"/>
-      <c r="BO7" s="273"/>
-      <c r="BP7" s="273"/>
-      <c r="BQ7" s="273"/>
-      <c r="BR7" s="273"/>
-      <c r="BS7" s="273"/>
-      <c r="BT7" s="273"/>
-      <c r="BU7" s="273"/>
-      <c r="BV7" s="273"/>
-      <c r="BW7" s="273"/>
-      <c r="BX7" s="273"/>
-      <c r="BY7" s="273"/>
-      <c r="BZ7" s="273"/>
-      <c r="CA7" s="273"/>
-      <c r="CB7" s="273"/>
-      <c r="CC7" s="273"/>
-      <c r="CD7" s="273"/>
-      <c r="CE7" s="273"/>
-      <c r="CF7" s="273"/>
-      <c r="CG7" s="273"/>
-      <c r="CH7" s="273"/>
-      <c r="CI7" s="273"/>
-      <c r="CJ7" s="273"/>
-      <c r="CK7" s="273"/>
-      <c r="CL7" s="273"/>
-      <c r="CM7" s="273"/>
-      <c r="CN7" s="273"/>
-      <c r="CO7" s="273"/>
-      <c r="CP7" s="273"/>
-      <c r="CQ7" s="273"/>
-      <c r="CR7" s="273"/>
-      <c r="CS7" s="273"/>
-      <c r="CT7" s="273"/>
-      <c r="CU7" s="273"/>
-      <c r="CV7" s="273"/>
-      <c r="CW7" s="273"/>
-      <c r="CX7" s="273"/>
-      <c r="CY7" s="273"/>
-      <c r="CZ7" s="273"/>
-      <c r="DA7" s="273"/>
-      <c r="DB7" s="273"/>
-      <c r="DC7" s="273"/>
-      <c r="DD7" s="273"/>
-      <c r="DE7" s="273"/>
-      <c r="DF7" s="273"/>
-      <c r="DG7" s="273"/>
-      <c r="DH7" s="273"/>
-      <c r="DI7" s="273"/>
-      <c r="DJ7" s="273"/>
-      <c r="DK7" s="273"/>
-      <c r="DL7" s="273"/>
-      <c r="DM7" s="273"/>
-      <c r="DN7" s="273"/>
-      <c r="DO7" s="273"/>
-      <c r="DP7" s="273"/>
-      <c r="DQ7" s="273"/>
-      <c r="DR7" s="273"/>
-      <c r="DS7" s="273"/>
-      <c r="DT7" s="273"/>
-      <c r="DU7" s="273"/>
-      <c r="DV7" s="273"/>
-      <c r="DW7" s="273"/>
-      <c r="DX7" s="273"/>
-      <c r="DY7" s="273"/>
-      <c r="DZ7" s="273"/>
-      <c r="EA7" s="273"/>
-      <c r="EB7" s="273"/>
-      <c r="EC7" s="273"/>
-      <c r="ED7" s="273"/>
-      <c r="EE7" s="273"/>
-      <c r="EF7" s="273"/>
-      <c r="EG7" s="273"/>
-      <c r="EH7" s="273"/>
-      <c r="EI7" s="273"/>
-      <c r="EJ7" s="273"/>
-      <c r="EK7" s="273"/>
-      <c r="EL7" s="273"/>
+      <c r="A7" s="280"/>
+      <c r="B7" s="280"/>
+      <c r="C7" s="280"/>
+      <c r="D7" s="280"/>
+      <c r="E7" s="280"/>
+      <c r="F7" s="280"/>
+      <c r="G7" s="280"/>
+      <c r="H7" s="280"/>
+      <c r="I7" s="280"/>
+      <c r="J7" s="280"/>
+      <c r="K7" s="280"/>
+      <c r="L7" s="280"/>
+      <c r="M7" s="280"/>
+      <c r="N7" s="280"/>
+      <c r="O7" s="280"/>
+      <c r="P7" s="280"/>
+      <c r="Q7" s="280"/>
+      <c r="R7" s="280"/>
+      <c r="S7" s="280"/>
+      <c r="T7" s="280"/>
+      <c r="U7" s="280"/>
+      <c r="V7" s="280"/>
+      <c r="W7" s="280"/>
+      <c r="X7" s="280"/>
+      <c r="Y7" s="280"/>
+      <c r="Z7" s="280"/>
+      <c r="AA7" s="280"/>
+      <c r="AB7" s="280"/>
+      <c r="AC7" s="280"/>
+      <c r="AD7" s="280"/>
+      <c r="AE7" s="280"/>
+      <c r="AF7" s="280"/>
+      <c r="AG7" s="280"/>
+      <c r="AH7" s="280"/>
+      <c r="AI7" s="280"/>
+      <c r="AJ7" s="280"/>
+      <c r="AK7" s="280"/>
+      <c r="AL7" s="280"/>
+      <c r="AM7" s="280"/>
+      <c r="AN7" s="280"/>
+      <c r="AO7" s="280"/>
+      <c r="AP7" s="280"/>
+      <c r="AQ7" s="280"/>
+      <c r="AR7" s="280"/>
+      <c r="AS7" s="280"/>
+      <c r="AT7" s="280"/>
+      <c r="AU7" s="280"/>
+      <c r="AV7" s="280"/>
+      <c r="AW7" s="280"/>
+      <c r="AX7" s="280"/>
+      <c r="AY7" s="280"/>
+      <c r="AZ7" s="280"/>
+      <c r="BA7" s="280"/>
+      <c r="BB7" s="280"/>
+      <c r="BC7" s="280"/>
+      <c r="BD7" s="280"/>
+      <c r="BE7" s="280"/>
+      <c r="BF7" s="280"/>
+      <c r="BG7" s="280"/>
+      <c r="BH7" s="280"/>
+      <c r="BI7" s="280"/>
+      <c r="BJ7" s="280"/>
+      <c r="BK7" s="280"/>
+      <c r="BL7" s="280"/>
+      <c r="BM7" s="280"/>
+      <c r="BN7" s="280"/>
+      <c r="BO7" s="280"/>
+      <c r="BP7" s="280"/>
+      <c r="BQ7" s="280"/>
+      <c r="BR7" s="280"/>
+      <c r="BS7" s="280"/>
+      <c r="BT7" s="280"/>
+      <c r="BU7" s="280"/>
+      <c r="BV7" s="280"/>
+      <c r="BW7" s="280"/>
+      <c r="BX7" s="280"/>
+      <c r="BY7" s="280"/>
+      <c r="BZ7" s="280"/>
+      <c r="CA7" s="280"/>
+      <c r="CB7" s="280"/>
+      <c r="CC7" s="280"/>
+      <c r="CD7" s="280"/>
+      <c r="CE7" s="280"/>
+      <c r="CF7" s="280"/>
+      <c r="CG7" s="280"/>
+      <c r="CH7" s="280"/>
+      <c r="CI7" s="280"/>
+      <c r="CJ7" s="280"/>
+      <c r="CK7" s="280"/>
+      <c r="CL7" s="280"/>
+      <c r="CM7" s="280"/>
+      <c r="CN7" s="280"/>
+      <c r="CO7" s="280"/>
+      <c r="CP7" s="280"/>
+      <c r="CQ7" s="280"/>
+      <c r="CR7" s="280"/>
+      <c r="CS7" s="280"/>
+      <c r="CT7" s="280"/>
+      <c r="CU7" s="280"/>
+      <c r="CV7" s="280"/>
+      <c r="CW7" s="280"/>
+      <c r="CX7" s="280"/>
+      <c r="CY7" s="280"/>
+      <c r="CZ7" s="280"/>
+      <c r="DA7" s="280"/>
+      <c r="DB7" s="280"/>
+      <c r="DC7" s="280"/>
+      <c r="DD7" s="280"/>
+      <c r="DE7" s="280"/>
+      <c r="DF7" s="280"/>
+      <c r="DG7" s="280"/>
+      <c r="DH7" s="280"/>
+      <c r="DI7" s="280"/>
+      <c r="DJ7" s="280"/>
+      <c r="DK7" s="280"/>
+      <c r="DL7" s="280"/>
+      <c r="DM7" s="280"/>
+      <c r="DN7" s="280"/>
+      <c r="DO7" s="280"/>
+      <c r="DP7" s="280"/>
+      <c r="DQ7" s="280"/>
+      <c r="DR7" s="280"/>
+      <c r="DS7" s="280"/>
+      <c r="DT7" s="280"/>
+      <c r="DU7" s="280"/>
+      <c r="DV7" s="280"/>
+      <c r="DW7" s="280"/>
+      <c r="DX7" s="280"/>
+      <c r="DY7" s="280"/>
+      <c r="DZ7" s="280"/>
+      <c r="EA7" s="280"/>
+      <c r="EB7" s="280"/>
+      <c r="EC7" s="280"/>
+      <c r="ED7" s="280"/>
+      <c r="EE7" s="280"/>
+      <c r="EF7" s="280"/>
+      <c r="EG7" s="280"/>
+      <c r="EH7" s="280"/>
+      <c r="EI7" s="280"/>
+      <c r="EJ7" s="280"/>
+      <c r="EK7" s="280"/>
+      <c r="EL7" s="280"/>
       <c r="EM7" s="238"/>
       <c r="EN7" s="238"/>
       <c r="EO7" s="238"/>
@@ -5236,40 +5254,37 @@
         <v>0</v>
       </c>
       <c r="CR8" s="156"/>
-      <c r="CS8" s="159">
-        <f t="shared" ref="CS8" si="51">IF($G$4&lt;20000000000,0,IF($G$4&lt;=30000000000,2000000,IF($G$4&lt;=50000000000,2300000,IF($G$4&lt;=50000000000,2000000,IF($G$4&lt;=70000000000,3000000,IF($G$4&gt;70000000000,3500000,0))))))</f>
+      <c r="CS8" s="314"/>
+      <c r="CT8" s="157">
+        <f t="shared" ref="CT8" si="51">+I8+CQ8+CR8+CS8</f>
         <v>0</v>
       </c>
-      <c r="CT8" s="157">
-        <f t="shared" ref="CT8" si="52">+I8+CQ8+CR8+CS8</f>
+      <c r="CU8" s="158">
+        <f t="shared" ref="CU8" si="52">+I8/26*(CF8+(CG8/8)+CH8)</f>
         <v>0</v>
       </c>
-      <c r="CU8" s="158">
-        <f t="shared" ref="CU8" si="53">+I8/26*(CF8+(CG8/8)+CH8)</f>
+      <c r="CV8" s="158">
+        <f t="shared" ref="CV8" si="53">+(I8/26/8)*150%*CI8</f>
         <v>0</v>
       </c>
-      <c r="CV8" s="158">
-        <f t="shared" ref="CV8" si="54">+(I8/26/8)*150%*CI8</f>
+      <c r="CW8" s="158">
+        <f t="shared" ref="CW8" si="54">+(I8/26/8)*130%*CJ8</f>
         <v>0</v>
       </c>
-      <c r="CW8" s="158">
-        <f t="shared" ref="CW8" si="55">+(I8/26/8)*130%*CJ8</f>
+      <c r="CX8" s="158">
+        <f t="shared" ref="CX8" si="55">+(I8/26/8)*200%*CK8</f>
         <v>0</v>
       </c>
-      <c r="CX8" s="158">
-        <f t="shared" ref="CX8" si="56">+(I8/26/8)*200%*CK8</f>
+      <c r="CY8" s="158">
+        <f t="shared" ref="CY8" si="56">+(I8/26/8)*210%*CL8</f>
         <v>0</v>
       </c>
-      <c r="CY8" s="158">
-        <f t="shared" ref="CY8" si="57">+(I8/26/8)*210%*CL8</f>
+      <c r="CZ8" s="158">
+        <f t="shared" ref="CZ8" si="57">+(I8/26/8)*270%*CM8</f>
         <v>0</v>
       </c>
-      <c r="CZ8" s="158">
-        <f t="shared" ref="CZ8" si="58">+(I8/26/8)*270%*CM8</f>
-        <v>0</v>
-      </c>
       <c r="DA8" s="158">
-        <f t="shared" ref="DA8" si="59">+(I8/26/8)*200%*CN8</f>
+        <f t="shared" ref="DA8" si="58">+(I8/26/8)*200%*CN8</f>
         <v>0</v>
       </c>
       <c r="DB8" s="158">
@@ -5277,64 +5292,61 @@
         <v>0</v>
       </c>
       <c r="DC8" s="158">
-        <f t="shared" ref="DC8" si="60">+(I8/26/8)*390%*CP8</f>
+        <f t="shared" ref="DC8" si="59">+(I8/26/8)*390%*CP8</f>
         <v>0</v>
       </c>
       <c r="DD8" s="159">
-        <f t="shared" ref="DD8" si="61">+CS8/26*(CF8+(CG8+CJ8)/8)</f>
+        <f t="shared" ref="DD8" si="60">+CS8/26*(CF8+(CG8+CJ8)/8)</f>
         <v>0</v>
       </c>
-      <c r="DE8" s="211">
-        <f t="shared" ref="DE8" si="62">IF(OR(H8="CV",H8="KTT",H8="QL",H8="QĐ",H8="TL",H8="PGĐ"),2000000,IF(OR(H8="NV",H8="KT", H8="TK"),1500000,IF(OR(H8="CN",H8="LX"),1000000,0)))/26*(CF8+(CG8+CJ8)/8)</f>
-        <v>0</v>
-      </c>
+      <c r="DE8" s="313"/>
       <c r="DF8" s="211">
-        <f t="shared" ref="DF8" si="63">+DD8+DE8</f>
+        <f t="shared" ref="DF8" si="61">+DD8+DE8</f>
         <v>0</v>
       </c>
       <c r="DG8" s="254"/>
       <c r="DH8" s="158">
-        <f t="shared" ref="DH8" si="64">+CU8+CV8+CW8+CX8+CY8+CZ8+DA8+DB8+DC8+DF8+DG8</f>
+        <f t="shared" ref="DH8" si="62">+CU8+CV8+CW8+CX8+CY8+CZ8+DA8+DB8+DC8+DF8+DG8</f>
         <v>0</v>
       </c>
       <c r="DI8" s="164">
-        <f t="shared" ref="DI8" si="65">+CQ8/26*AQ8</f>
+        <f t="shared" ref="DI8" si="63">+CQ8/26*AQ8</f>
         <v>0</v>
       </c>
       <c r="DJ8" s="164">
-        <f t="shared" ref="DJ8" si="66">+CR8/26*AQ8</f>
+        <f t="shared" ref="DJ8" si="64">+CR8/26*AQ8</f>
         <v>0</v>
       </c>
       <c r="DK8" s="164">
-        <f t="shared" ref="DK8" si="67">+DH8+DI8+DJ8</f>
+        <f t="shared" ref="DK8" si="65">+DH8+DI8+DJ8</f>
         <v>0</v>
       </c>
       <c r="DL8" s="172">
-        <f t="shared" ref="DL8" si="68">I8</f>
+        <f t="shared" ref="DL8" si="66">I8</f>
         <v>0</v>
       </c>
       <c r="DM8" s="159">
-        <f t="shared" ref="DM8" si="69">DL8*8%</f>
+        <f t="shared" ref="DM8" si="67">DL8*8%</f>
         <v>0</v>
       </c>
       <c r="DN8" s="159">
-        <f t="shared" ref="DN8" si="70">DL8*1.5%</f>
+        <f t="shared" ref="DN8" si="68">DL8*1.5%</f>
         <v>0</v>
       </c>
       <c r="DO8" s="159">
-        <f t="shared" ref="DO8" si="71">DL8*1%</f>
+        <f t="shared" ref="DO8" si="69">DL8*1%</f>
         <v>0</v>
       </c>
       <c r="DP8" s="159">
-        <f t="shared" ref="DP8" si="72">EI8</f>
+        <f t="shared" ref="DP8" si="70">EI8</f>
         <v>0</v>
       </c>
       <c r="DQ8" s="159">
-        <f t="shared" ref="DQ8" si="73">+SUM(DM8:DP8)</f>
+        <f t="shared" ref="DQ8" si="71">+SUM(DM8:DP8)</f>
         <v>0</v>
       </c>
       <c r="DR8" s="159">
-        <f t="shared" ref="DR8" si="74">SUM(DM8:DO8)</f>
+        <f t="shared" ref="DR8" si="72">SUM(DM8:DO8)</f>
         <v>0</v>
       </c>
       <c r="DS8" s="160">
@@ -5371,7 +5383,7 @@
         <v>0</v>
       </c>
       <c r="EB8" s="173">
-        <f t="shared" ref="EB8" si="75">DY8+DZ8+EA8</f>
+        <f t="shared" ref="EB8" si="73">DY8+DZ8+EA8</f>
         <v>0</v>
       </c>
       <c r="EC8" s="164">
@@ -5398,7 +5410,7 @@
         <v>-775000</v>
       </c>
       <c r="EI8" s="172">
-        <f t="shared" ref="EI8" si="76">+IF(EH8&lt;0,0,EH8)</f>
+        <f t="shared" ref="EI8" si="74">+IF(EH8&lt;0,0,EH8)</f>
         <v>0</v>
       </c>
       <c r="EJ8" s="165">
@@ -27090,22 +27102,38 @@
   </sheetData>
   <autoFilter ref="A6:ER8" xr:uid="{00000000-0001-0000-0900-000000000000}"/>
   <mergeCells count="64">
-    <mergeCell ref="EN5:EN6"/>
-    <mergeCell ref="EI5:EI6"/>
-    <mergeCell ref="EJ5:EJ6"/>
-    <mergeCell ref="EK5:EK6"/>
-    <mergeCell ref="EL5:EL6"/>
-    <mergeCell ref="EH5:EH6"/>
-    <mergeCell ref="DV5:DX5"/>
-    <mergeCell ref="CQ5:CS5"/>
-    <mergeCell ref="DG5:DG6"/>
-    <mergeCell ref="DI5:DJ5"/>
-    <mergeCell ref="CT5:CT6"/>
-    <mergeCell ref="DH5:DH6"/>
-    <mergeCell ref="DK5:DK6"/>
-    <mergeCell ref="DM5:DR5"/>
-    <mergeCell ref="DS5:DS6"/>
-    <mergeCell ref="DU5:DU6"/>
+    <mergeCell ref="AO1:AS1"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="S4:U4"/>
+    <mergeCell ref="W4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="AG4:AI4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="BG4:BI4"/>
+    <mergeCell ref="AT4:AU4"/>
+    <mergeCell ref="AO5:AO6"/>
+    <mergeCell ref="AP5:AP6"/>
+    <mergeCell ref="AQ5:AQ6"/>
+    <mergeCell ref="AR5:AR6"/>
+    <mergeCell ref="AS5:AS6"/>
+    <mergeCell ref="BJ4:BK4"/>
+    <mergeCell ref="BL4:BN4"/>
+    <mergeCell ref="BQ4:BS4"/>
+    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="CD5:CD6"/>
+    <mergeCell ref="BY5:BY6"/>
+    <mergeCell ref="BZ5:BZ6"/>
+    <mergeCell ref="CA5:CA6"/>
+    <mergeCell ref="CB5:CB6"/>
+    <mergeCell ref="CC5:CC6"/>
     <mergeCell ref="ER5:ER6"/>
     <mergeCell ref="A7:EL7"/>
     <mergeCell ref="EM5:EM6"/>
@@ -27122,38 +27150,22 @@
     <mergeCell ref="DL5:DL6"/>
     <mergeCell ref="EG5:EG6"/>
     <mergeCell ref="EQ5:EQ6"/>
-    <mergeCell ref="BJ4:BK4"/>
-    <mergeCell ref="BL4:BN4"/>
-    <mergeCell ref="BQ4:BS4"/>
-    <mergeCell ref="BC4:BE4"/>
-    <mergeCell ref="CD5:CD6"/>
-    <mergeCell ref="BY5:BY6"/>
-    <mergeCell ref="BZ5:BZ6"/>
-    <mergeCell ref="CA5:CA6"/>
-    <mergeCell ref="CB5:CB6"/>
-    <mergeCell ref="CC5:CC6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="BG4:BI4"/>
-    <mergeCell ref="AT4:AU4"/>
-    <mergeCell ref="AO5:AO6"/>
-    <mergeCell ref="AP5:AP6"/>
-    <mergeCell ref="AQ5:AQ6"/>
-    <mergeCell ref="AR5:AR6"/>
-    <mergeCell ref="AS5:AS6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="AO1:AS1"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="S4:U4"/>
-    <mergeCell ref="W4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AD4"/>
-    <mergeCell ref="AG4:AI4"/>
+    <mergeCell ref="EH5:EH6"/>
+    <mergeCell ref="DV5:DX5"/>
+    <mergeCell ref="CQ5:CS5"/>
+    <mergeCell ref="DG5:DG6"/>
+    <mergeCell ref="DI5:DJ5"/>
+    <mergeCell ref="CT5:CT6"/>
+    <mergeCell ref="DH5:DH6"/>
+    <mergeCell ref="DK5:DK6"/>
+    <mergeCell ref="DM5:DR5"/>
+    <mergeCell ref="DS5:DS6"/>
+    <mergeCell ref="DU5:DU6"/>
+    <mergeCell ref="EN5:EN6"/>
+    <mergeCell ref="EI5:EI6"/>
+    <mergeCell ref="EJ5:EJ6"/>
+    <mergeCell ref="EK5:EK6"/>
+    <mergeCell ref="EL5:EL6"/>
   </mergeCells>
   <conditionalFormatting sqref="A5 A8:B8">
     <cfRule type="duplicateValues" dxfId="20" priority="20879"/>
@@ -27227,20 +27239,20 @@
     <tabColor rgb="FFFF00FF"/>
   </sheetPr>
   <dimension ref="A1:AC1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.83203125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.796875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="4.83203125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="3.83203125" style="9" customWidth="1"/>
-    <col min="3" max="10" width="6.33203125" style="9" customWidth="1"/>
-    <col min="11" max="11" width="3.83203125" style="9" customWidth="1"/>
-    <col min="12" max="17" width="6.33203125" style="9" customWidth="1"/>
-    <col min="18" max="18" width="4.1640625" style="9" customWidth="1"/>
-    <col min="19" max="19" width="6.33203125" style="9" customWidth="1"/>
-    <col min="20" max="20" width="3.83203125" style="9" customWidth="1"/>
-    <col min="21" max="27" width="6.33203125" style="9" customWidth="1"/>
-    <col min="28" max="28" width="4.83203125" style="9" customWidth="1"/>
-    <col min="29" max="29" width="10.1640625" style="9" customWidth="1"/>
-    <col min="30" max="16384" width="12.83203125" style="9"/>
+    <col min="1" max="1" width="4.796875" style="9" customWidth="1"/>
+    <col min="2" max="2" width="3.796875" style="9" customWidth="1"/>
+    <col min="3" max="10" width="6.3984375" style="9" customWidth="1"/>
+    <col min="11" max="11" width="3.796875" style="9" customWidth="1"/>
+    <col min="12" max="17" width="6.3984375" style="9" customWidth="1"/>
+    <col min="18" max="18" width="4.19921875" style="9" customWidth="1"/>
+    <col min="19" max="19" width="6.3984375" style="9" customWidth="1"/>
+    <col min="20" max="20" width="3.796875" style="9" customWidth="1"/>
+    <col min="21" max="27" width="6.3984375" style="9" customWidth="1"/>
+    <col min="28" max="28" width="4.796875" style="9" customWidth="1"/>
+    <col min="29" max="29" width="10.19921875" style="9" customWidth="1"/>
+    <col min="30" max="16384" width="12.796875" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="12.75" hidden="1" customHeight="1">
@@ -27810,11 +27822,11 @@
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
       <c r="H8" s="20"/>
-      <c r="I8" s="307">
+      <c r="I8" s="301">
         <v>2026</v>
       </c>
-      <c r="J8" s="308"/>
-      <c r="K8" s="308"/>
+      <c r="J8" s="302"/>
+      <c r="K8" s="302"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="21" t="s">
@@ -27839,13 +27851,13 @@
     <row r="9" spans="1:29" ht="15.75" customHeight="1" thickBot="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="309" t="s">
+      <c r="C9" s="303" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="310"/>
-      <c r="E9" s="310"/>
-      <c r="F9" s="310"/>
-      <c r="G9" s="310"/>
+      <c r="D9" s="304"/>
+      <c r="E9" s="304"/>
+      <c r="F9" s="304"/>
+      <c r="G9" s="304"/>
       <c r="H9" s="20"/>
       <c r="I9" s="24"/>
       <c r="J9" s="24"/>
@@ -27941,19 +27953,19 @@
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
-      <c r="J12" s="311" t="s">
+      <c r="J12" s="305" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="310"/>
-      <c r="L12" s="310"/>
-      <c r="M12" s="310"/>
-      <c r="N12" s="310"/>
-      <c r="O12" s="310"/>
-      <c r="P12" s="312">
+      <c r="K12" s="304"/>
+      <c r="L12" s="304"/>
+      <c r="M12" s="304"/>
+      <c r="N12" s="304"/>
+      <c r="O12" s="304"/>
+      <c r="P12" s="306">
         <f>I8</f>
         <v>2026</v>
       </c>
-      <c r="Q12" s="310"/>
+      <c r="Q12" s="304"/>
       <c r="R12" s="33"/>
       <c r="S12" s="34"/>
       <c r="T12" s="34"/>
@@ -28217,38 +28229,38 @@
     </row>
     <row r="21" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A21" s="39"/>
-      <c r="B21" s="306" t="s">
+      <c r="B21" s="307" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="302"/>
-      <c r="D21" s="302"/>
-      <c r="E21" s="302"/>
-      <c r="F21" s="302"/>
-      <c r="G21" s="302"/>
-      <c r="H21" s="302"/>
-      <c r="I21" s="302"/>
+      <c r="C21" s="308"/>
+      <c r="D21" s="308"/>
+      <c r="E21" s="308"/>
+      <c r="F21" s="308"/>
+      <c r="G21" s="308"/>
+      <c r="H21" s="308"/>
+      <c r="I21" s="308"/>
       <c r="J21" s="40"/>
-      <c r="K21" s="303" t="s">
+      <c r="K21" s="309" t="s">
         <v>37</v>
       </c>
-      <c r="L21" s="302"/>
-      <c r="M21" s="302"/>
-      <c r="N21" s="302"/>
-      <c r="O21" s="302"/>
-      <c r="P21" s="302"/>
-      <c r="Q21" s="302"/>
-      <c r="R21" s="302"/>
+      <c r="L21" s="308"/>
+      <c r="M21" s="308"/>
+      <c r="N21" s="308"/>
+      <c r="O21" s="308"/>
+      <c r="P21" s="308"/>
+      <c r="Q21" s="308"/>
+      <c r="R21" s="308"/>
       <c r="S21" s="40"/>
-      <c r="T21" s="301" t="s">
+      <c r="T21" s="310" t="s">
         <v>38</v>
       </c>
-      <c r="U21" s="302"/>
-      <c r="V21" s="302"/>
-      <c r="W21" s="302"/>
-      <c r="X21" s="302"/>
-      <c r="Y21" s="302"/>
-      <c r="Z21" s="302"/>
-      <c r="AA21" s="302"/>
+      <c r="U21" s="308"/>
+      <c r="V21" s="308"/>
+      <c r="W21" s="308"/>
+      <c r="X21" s="308"/>
+      <c r="Y21" s="308"/>
+      <c r="Z21" s="308"/>
+      <c r="AA21" s="308"/>
       <c r="AB21" s="41"/>
       <c r="AC21" s="42"/>
     </row>
@@ -29148,38 +29160,38 @@
     </row>
     <row r="35" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="304" t="s">
+      <c r="B35" s="311" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="302"/>
-      <c r="D35" s="302"/>
-      <c r="E35" s="302"/>
-      <c r="F35" s="302"/>
-      <c r="G35" s="302"/>
-      <c r="H35" s="302"/>
-      <c r="I35" s="302"/>
+      <c r="C35" s="308"/>
+      <c r="D35" s="308"/>
+      <c r="E35" s="308"/>
+      <c r="F35" s="308"/>
+      <c r="G35" s="308"/>
+      <c r="H35" s="308"/>
+      <c r="I35" s="308"/>
       <c r="J35" s="40"/>
-      <c r="K35" s="305" t="s">
+      <c r="K35" s="312" t="s">
         <v>48</v>
       </c>
-      <c r="L35" s="302"/>
-      <c r="M35" s="302"/>
-      <c r="N35" s="302"/>
-      <c r="O35" s="302"/>
-      <c r="P35" s="302"/>
-      <c r="Q35" s="302"/>
-      <c r="R35" s="302"/>
+      <c r="L35" s="308"/>
+      <c r="M35" s="308"/>
+      <c r="N35" s="308"/>
+      <c r="O35" s="308"/>
+      <c r="P35" s="308"/>
+      <c r="Q35" s="308"/>
+      <c r="R35" s="308"/>
       <c r="S35" s="40"/>
-      <c r="T35" s="303" t="s">
+      <c r="T35" s="309" t="s">
         <v>49</v>
       </c>
-      <c r="U35" s="302"/>
-      <c r="V35" s="302"/>
-      <c r="W35" s="302"/>
-      <c r="X35" s="302"/>
-      <c r="Y35" s="302"/>
-      <c r="Z35" s="302"/>
-      <c r="AA35" s="302"/>
+      <c r="U35" s="308"/>
+      <c r="V35" s="308"/>
+      <c r="W35" s="308"/>
+      <c r="X35" s="308"/>
+      <c r="Y35" s="308"/>
+      <c r="Z35" s="308"/>
+      <c r="AA35" s="308"/>
       <c r="AB35" s="70"/>
       <c r="AC35" s="40"/>
     </row>
@@ -30068,38 +30080,38 @@
     </row>
     <row r="49" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A49" s="69"/>
-      <c r="B49" s="303" t="s">
+      <c r="B49" s="309" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="302"/>
-      <c r="D49" s="302"/>
-      <c r="E49" s="302"/>
-      <c r="F49" s="302"/>
-      <c r="G49" s="302"/>
-      <c r="H49" s="302"/>
-      <c r="I49" s="302"/>
+      <c r="C49" s="308"/>
+      <c r="D49" s="308"/>
+      <c r="E49" s="308"/>
+      <c r="F49" s="308"/>
+      <c r="G49" s="308"/>
+      <c r="H49" s="308"/>
+      <c r="I49" s="308"/>
       <c r="J49" s="40"/>
-      <c r="K49" s="304" t="s">
+      <c r="K49" s="311" t="s">
         <v>51</v>
       </c>
-      <c r="L49" s="302"/>
-      <c r="M49" s="302"/>
-      <c r="N49" s="302"/>
-      <c r="O49" s="302"/>
-      <c r="P49" s="302"/>
-      <c r="Q49" s="302"/>
-      <c r="R49" s="302"/>
+      <c r="L49" s="308"/>
+      <c r="M49" s="308"/>
+      <c r="N49" s="308"/>
+      <c r="O49" s="308"/>
+      <c r="P49" s="308"/>
+      <c r="Q49" s="308"/>
+      <c r="R49" s="308"/>
       <c r="S49" s="40"/>
-      <c r="T49" s="306" t="s">
+      <c r="T49" s="307" t="s">
         <v>52</v>
       </c>
-      <c r="U49" s="302"/>
-      <c r="V49" s="302"/>
-      <c r="W49" s="302"/>
-      <c r="X49" s="302"/>
-      <c r="Y49" s="302"/>
-      <c r="Z49" s="302"/>
-      <c r="AA49" s="302"/>
+      <c r="U49" s="308"/>
+      <c r="V49" s="308"/>
+      <c r="W49" s="308"/>
+      <c r="X49" s="308"/>
+      <c r="Y49" s="308"/>
+      <c r="Z49" s="308"/>
+      <c r="AA49" s="308"/>
       <c r="AB49" s="70"/>
       <c r="AC49" s="40"/>
     </row>
@@ -30988,38 +31000,38 @@
     </row>
     <row r="63" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A63" s="69"/>
-      <c r="B63" s="301" t="s">
+      <c r="B63" s="310" t="s">
         <v>53</v>
       </c>
-      <c r="C63" s="302"/>
-      <c r="D63" s="302"/>
-      <c r="E63" s="302"/>
-      <c r="F63" s="302"/>
-      <c r="G63" s="302"/>
-      <c r="H63" s="302"/>
-      <c r="I63" s="302"/>
+      <c r="C63" s="308"/>
+      <c r="D63" s="308"/>
+      <c r="E63" s="308"/>
+      <c r="F63" s="308"/>
+      <c r="G63" s="308"/>
+      <c r="H63" s="308"/>
+      <c r="I63" s="308"/>
       <c r="J63" s="40"/>
-      <c r="K63" s="303" t="s">
+      <c r="K63" s="309" t="s">
         <v>54</v>
       </c>
-      <c r="L63" s="302"/>
-      <c r="M63" s="302"/>
-      <c r="N63" s="302"/>
-      <c r="O63" s="302"/>
-      <c r="P63" s="302"/>
-      <c r="Q63" s="302"/>
-      <c r="R63" s="302"/>
+      <c r="L63" s="308"/>
+      <c r="M63" s="308"/>
+      <c r="N63" s="308"/>
+      <c r="O63" s="308"/>
+      <c r="P63" s="308"/>
+      <c r="Q63" s="308"/>
+      <c r="R63" s="308"/>
       <c r="S63" s="40"/>
-      <c r="T63" s="304" t="s">
+      <c r="T63" s="311" t="s">
         <v>55</v>
       </c>
-      <c r="U63" s="302"/>
-      <c r="V63" s="302"/>
-      <c r="W63" s="302"/>
-      <c r="X63" s="302"/>
-      <c r="Y63" s="302"/>
-      <c r="Z63" s="302"/>
-      <c r="AA63" s="302"/>
+      <c r="U63" s="308"/>
+      <c r="V63" s="308"/>
+      <c r="W63" s="308"/>
+      <c r="X63" s="308"/>
+      <c r="Y63" s="308"/>
+      <c r="Z63" s="308"/>
+      <c r="AA63" s="308"/>
       <c r="AB63" s="70"/>
       <c r="AC63" s="40"/>
     </row>
@@ -60554,12 +60566,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="J12:O12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="K21:R21"/>
     <mergeCell ref="B63:I63"/>
     <mergeCell ref="K63:R63"/>
     <mergeCell ref="T63:AA63"/>
@@ -60570,6 +60576,12 @@
     <mergeCell ref="B49:I49"/>
     <mergeCell ref="K49:R49"/>
     <mergeCell ref="T49:AA49"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="J12:O12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="K21:R21"/>
   </mergeCells>
   <conditionalFormatting sqref="C51:I55">
     <cfRule type="expression" dxfId="2" priority="3">

</xml_diff>

<commit_message>
sử lý trưởng hợp truy thu bảo hiểm . có 2 trường hợp truy thu vào chi phí doanh nghiệp và truy thu vào chi phí người lao động.
</commit_message>
<xml_diff>
--- a/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
+++ b/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonzai/dev/odoo 19/odoo/my_custom_addons/dl_salary_kpi/static/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87EFFE75-9BC6-A84B-8B84-DE1CD0F87995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20A8277D-3347-5D4C-B21E-0616A791625C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="480" windowWidth="38400" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kangatang" sheetId="43" state="veryHidden" r:id="rId1"/>
@@ -75,6 +75,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>ADMIN</author>
+    <author>sonzai</author>
   </authors>
   <commentList>
     <comment ref="DK5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0900-000001000000}">
@@ -125,12 +126,65 @@
         </r>
       </text>
     </comment>
+    <comment ref="ES5" authorId="1" shapeId="0" xr:uid="{875C98E4-B4B6-8648-88B7-D03E21863E5B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>sonzai:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">0: không cần truy thu
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">1: Truy thu vào doanh nghiệp
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>2:: Truy thu vào người lao động</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="132">
   <si>
     <t>STT</t>
   </si>
@@ -524,13 +578,16 @@
     <t>In</t>
   </si>
   <si>
-    <t>8/3</t>
-  </si>
-  <si>
     <t>Thưởng doanh thu/Thưởng năng suất</t>
   </si>
   <si>
     <t>LƯƠNG CHI TIỀN MẶT</t>
+  </si>
+  <si>
+    <t>Truy thu BHYT</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -552,7 +609,7 @@
     <numFmt numFmtId="174" formatCode="\TGeneral"/>
     <numFmt numFmtId="175" formatCode="_-* #,##0.0\ _₫_-;\-* #,##0.0\ _₫_-;_-* &quot;-&quot;??\ _₫_-;_-@_-"/>
   </numFmts>
-  <fonts count="86">
+  <fonts count="88">
     <font>
       <sz val="10"/>
       <name val="Encysoft Times"/>
@@ -1095,6 +1152,19 @@
     </font>
     <font>
       <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
       <family val="2"/>
@@ -1776,7 +1846,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="315">
+  <cellXfs count="317">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="169" fontId="12" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2433,16 +2503,88 @@
     <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="78" fillId="25" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="78" fillId="26" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="55" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="81" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2478,83 +2620,33 @@
     <xf numFmtId="169" fontId="55" fillId="12" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="55" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="66" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="67" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="67" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="55" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="77" fillId="6" borderId="1" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="77" fillId="13" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="68" fillId="2" borderId="34" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="55" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="77" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="7" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2570,27 +2662,11 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="78" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="78" fillId="25" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="78" fillId="26" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="32">
@@ -2981,6 +3057,10 @@
 </externalLink>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -3291,7 +3371,7 @@
     <tabColor rgb="FFFF0000"/>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:ER165"/>
+  <dimension ref="A1:ES165"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="20" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="17.796875" style="95" customWidth="1"/>
@@ -3370,11 +3450,12 @@
     <col min="146" max="146" width="36.3984375" style="95" customWidth="1"/>
     <col min="147" max="147" width="35.796875" style="95" customWidth="1"/>
     <col min="148" max="148" width="41.796875" style="242" customWidth="1"/>
-    <col min="149" max="150" width="9.19921875" style="94" customWidth="1"/>
+    <col min="149" max="149" width="23.59765625" style="94" customWidth="1"/>
+    <col min="150" max="150" width="9.19921875" style="94" customWidth="1"/>
     <col min="151" max="16384" width="9.19921875" style="94"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:148" s="127" customFormat="1" ht="37.5" customHeight="1">
+    <row r="1" spans="1:149" s="127" customFormat="1" ht="37.5" customHeight="1">
       <c r="A1" s="151"/>
       <c r="B1" s="151"/>
       <c r="C1" s="118"/>
@@ -3415,11 +3496,11 @@
       <c r="AL1" s="212"/>
       <c r="AM1" s="212"/>
       <c r="AN1" s="212"/>
-      <c r="AO1" s="300"/>
-      <c r="AP1" s="300"/>
-      <c r="AQ1" s="300"/>
-      <c r="AR1" s="300"/>
-      <c r="AS1" s="300"/>
+      <c r="AO1" s="262"/>
+      <c r="AP1" s="262"/>
+      <c r="AQ1" s="262"/>
+      <c r="AR1" s="262"/>
+      <c r="AS1" s="262"/>
       <c r="AT1" s="120"/>
       <c r="AU1" s="120"/>
       <c r="AV1" s="120"/>
@@ -3518,7 +3599,7 @@
       <c r="EQ1" s="233"/>
       <c r="ER1" s="234"/>
     </row>
-    <row r="2" spans="1:148" s="127" customFormat="1" ht="37.5" customHeight="1">
+    <row r="2" spans="1:149" s="127" customFormat="1" ht="37.5" customHeight="1">
       <c r="A2" s="148"/>
       <c r="B2" s="148"/>
       <c r="C2" s="128"/>
@@ -3662,7 +3743,7 @@
       <c r="EQ2" s="233"/>
       <c r="ER2" s="234"/>
     </row>
-    <row r="3" spans="1:148" s="127" customFormat="1" ht="37.5" customHeight="1">
+    <row r="3" spans="1:149" s="127" customFormat="1" ht="37.5" customHeight="1">
       <c r="A3" s="148" t="s">
         <v>123</v>
       </c>
@@ -3809,7 +3890,7 @@
       <c r="EQ3" s="233"/>
       <c r="ER3" s="234"/>
     </row>
-    <row r="4" spans="1:148" s="105" customFormat="1" ht="63" customHeight="1">
+    <row r="4" spans="1:149" s="105" customFormat="1" ht="63" customHeight="1">
       <c r="A4" s="206"/>
       <c r="B4" s="206"/>
       <c r="C4" s="107"/>
@@ -3821,10 +3902,10 @@
       <c r="G4" s="232"/>
       <c r="H4" s="108"/>
       <c r="I4" s="256"/>
-      <c r="J4" s="293" t="s">
+      <c r="J4" s="263" t="s">
         <v>68</v>
       </c>
-      <c r="K4" s="293"/>
+      <c r="K4" s="263"/>
       <c r="L4" s="258">
         <v>3</v>
       </c>
@@ -3838,23 +3919,23 @@
       </c>
       <c r="Q4" s="259"/>
       <c r="R4" s="109"/>
-      <c r="S4" s="293"/>
-      <c r="T4" s="293"/>
-      <c r="U4" s="293"/>
+      <c r="S4" s="263"/>
+      <c r="T4" s="263"/>
+      <c r="U4" s="263"/>
       <c r="V4" s="109"/>
-      <c r="W4" s="293"/>
-      <c r="X4" s="293"/>
-      <c r="Y4" s="293"/>
-      <c r="Z4" s="293"/>
-      <c r="AA4" s="293"/>
-      <c r="AB4" s="293"/>
-      <c r="AC4" s="293"/>
-      <c r="AD4" s="293"/>
+      <c r="W4" s="263"/>
+      <c r="X4" s="263"/>
+      <c r="Y4" s="263"/>
+      <c r="Z4" s="263"/>
+      <c r="AA4" s="263"/>
+      <c r="AB4" s="263"/>
+      <c r="AC4" s="263"/>
+      <c r="AD4" s="263"/>
       <c r="AE4" s="109"/>
       <c r="AF4" s="110"/>
-      <c r="AG4" s="293"/>
-      <c r="AH4" s="293"/>
-      <c r="AI4" s="293"/>
+      <c r="AG4" s="263"/>
+      <c r="AH4" s="263"/>
+      <c r="AI4" s="263"/>
       <c r="AJ4" s="109"/>
       <c r="AK4" s="109"/>
       <c r="AL4" s="109"/>
@@ -3865,10 +3946,10 @@
       <c r="AQ4" s="113"/>
       <c r="AR4" s="221"/>
       <c r="AS4" s="227"/>
-      <c r="AT4" s="293" t="s">
+      <c r="AT4" s="263" t="s">
         <v>68</v>
       </c>
-      <c r="AU4" s="293"/>
+      <c r="AU4" s="263"/>
       <c r="AV4" s="258">
         <f>L4</f>
         <v>3</v>
@@ -3884,23 +3965,23 @@
       </c>
       <c r="BA4" s="259"/>
       <c r="BB4" s="109"/>
-      <c r="BC4" s="293"/>
-      <c r="BD4" s="293"/>
-      <c r="BE4" s="293"/>
+      <c r="BC4" s="263"/>
+      <c r="BD4" s="263"/>
+      <c r="BE4" s="263"/>
       <c r="BF4" s="109"/>
-      <c r="BG4" s="293"/>
-      <c r="BH4" s="293"/>
-      <c r="BI4" s="293"/>
-      <c r="BJ4" s="293"/>
-      <c r="BK4" s="293"/>
-      <c r="BL4" s="293"/>
-      <c r="BM4" s="293"/>
-      <c r="BN4" s="293"/>
+      <c r="BG4" s="263"/>
+      <c r="BH4" s="263"/>
+      <c r="BI4" s="263"/>
+      <c r="BJ4" s="263"/>
+      <c r="BK4" s="263"/>
+      <c r="BL4" s="263"/>
+      <c r="BM4" s="263"/>
+      <c r="BN4" s="263"/>
       <c r="BO4" s="109"/>
       <c r="BP4" s="110"/>
-      <c r="BQ4" s="293"/>
-      <c r="BR4" s="293"/>
-      <c r="BS4" s="293"/>
+      <c r="BQ4" s="263"/>
+      <c r="BR4" s="263"/>
+      <c r="BS4" s="263"/>
       <c r="BT4" s="114"/>
       <c r="BU4" s="114" t="str">
         <f>IF(WEEKDAY(BU5,1)=1,"CN","")</f>
@@ -3979,32 +4060,32 @@
       <c r="EQ4" s="236"/>
       <c r="ER4" s="237"/>
     </row>
-    <row r="5" spans="1:148" s="183" customFormat="1" ht="92.25" customHeight="1">
-      <c r="A5" s="288" t="s">
+    <row r="5" spans="1:149" s="183" customFormat="1" ht="92.25" customHeight="1">
+      <c r="A5" s="264" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="278" t="s">
+      <c r="B5" s="265" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="288" t="s">
+      <c r="C5" s="264" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="297" t="s">
+      <c r="D5" s="266" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="298" t="s">
+      <c r="E5" s="267" t="s">
         <v>120</v>
       </c>
-      <c r="F5" s="288" t="s">
+      <c r="F5" s="264" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="288" t="s">
+      <c r="G5" s="264" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="288" t="s">
+      <c r="H5" s="264" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="294" t="s">
+      <c r="I5" s="269" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="174">
@@ -4131,19 +4212,19 @@
         <f t="shared" si="0"/>
         <v>46112</v>
       </c>
-      <c r="AO5" s="295" t="s">
+      <c r="AO5" s="270" t="s">
         <v>82</v>
       </c>
-      <c r="AP5" s="295" t="s">
+      <c r="AP5" s="270" t="s">
         <v>83</v>
       </c>
-      <c r="AQ5" s="295" t="s">
+      <c r="AQ5" s="270" t="s">
         <v>84</v>
       </c>
-      <c r="AR5" s="296" t="s">
+      <c r="AR5" s="271" t="s">
         <v>5</v>
       </c>
-      <c r="AS5" s="296" t="s">
+      <c r="AS5" s="271" t="s">
         <v>6</v>
       </c>
       <c r="AT5" s="178">
@@ -4270,46 +4351,46 @@
         <f t="shared" si="1"/>
         <v>46112</v>
       </c>
-      <c r="BY5" s="290" t="s">
+      <c r="BY5" s="272" t="s">
         <v>85</v>
       </c>
-      <c r="BZ5" s="290" t="s">
+      <c r="BZ5" s="272" t="s">
         <v>86</v>
       </c>
-      <c r="CA5" s="290" t="s">
+      <c r="CA5" s="272" t="s">
         <v>87</v>
       </c>
-      <c r="CB5" s="290" t="s">
+      <c r="CB5" s="272" t="s">
         <v>88</v>
       </c>
-      <c r="CC5" s="290" t="s">
+      <c r="CC5" s="272" t="s">
         <v>89</v>
       </c>
-      <c r="CD5" s="290" t="s">
+      <c r="CD5" s="272" t="s">
         <v>90</v>
       </c>
-      <c r="CE5" s="290" t="s">
+      <c r="CE5" s="272" t="s">
         <v>91</v>
       </c>
-      <c r="CF5" s="289" t="s">
+      <c r="CF5" s="286" t="s">
         <v>19</v>
       </c>
-      <c r="CG5" s="289"/>
-      <c r="CH5" s="289"/>
-      <c r="CI5" s="289"/>
-      <c r="CJ5" s="289"/>
-      <c r="CK5" s="289"/>
-      <c r="CL5" s="289"/>
-      <c r="CM5" s="289"/>
-      <c r="CN5" s="289"/>
-      <c r="CO5" s="289"/>
-      <c r="CP5" s="289"/>
-      <c r="CQ5" s="266" t="s">
+      <c r="CG5" s="286"/>
+      <c r="CH5" s="286"/>
+      <c r="CI5" s="286"/>
+      <c r="CJ5" s="286"/>
+      <c r="CK5" s="286"/>
+      <c r="CL5" s="286"/>
+      <c r="CM5" s="286"/>
+      <c r="CN5" s="286"/>
+      <c r="CO5" s="286"/>
+      <c r="CP5" s="286"/>
+      <c r="CQ5" s="290" t="s">
         <v>59</v>
       </c>
-      <c r="CR5" s="267"/>
-      <c r="CS5" s="268"/>
-      <c r="CT5" s="273" t="s">
+      <c r="CR5" s="291"/>
+      <c r="CS5" s="292"/>
+      <c r="CT5" s="297" t="s">
         <v>60</v>
       </c>
       <c r="CU5" s="247" t="s">
@@ -4332,107 +4413,110 @@
       <c r="DF5" s="245" t="s">
         <v>127</v>
       </c>
-      <c r="DG5" s="269" t="s">
+      <c r="DG5" s="293" t="s">
         <v>117</v>
       </c>
-      <c r="DH5" s="274" t="s">
+      <c r="DH5" s="298" t="s">
         <v>112</v>
       </c>
-      <c r="DI5" s="271" t="s">
+      <c r="DI5" s="295" t="s">
         <v>81</v>
       </c>
-      <c r="DJ5" s="272"/>
-      <c r="DK5" s="275" t="s">
+      <c r="DJ5" s="296"/>
+      <c r="DK5" s="283" t="s">
         <v>61</v>
       </c>
-      <c r="DL5" s="292" t="s">
+      <c r="DL5" s="287" t="s">
         <v>8</v>
       </c>
-      <c r="DM5" s="276" t="s">
+      <c r="DM5" s="284" t="s">
         <v>71</v>
       </c>
-      <c r="DN5" s="276"/>
-      <c r="DO5" s="276"/>
-      <c r="DP5" s="276"/>
-      <c r="DQ5" s="276"/>
-      <c r="DR5" s="276"/>
-      <c r="DS5" s="277" t="s">
+      <c r="DN5" s="284"/>
+      <c r="DO5" s="284"/>
+      <c r="DP5" s="284"/>
+      <c r="DQ5" s="284"/>
+      <c r="DR5" s="284"/>
+      <c r="DS5" s="299" t="s">
         <v>12</v>
       </c>
-      <c r="DT5" s="276" t="s">
+      <c r="DT5" s="284" t="s">
         <v>125</v>
       </c>
-      <c r="DU5" s="278" t="s">
+      <c r="DU5" s="265" t="s">
         <v>13</v>
       </c>
-      <c r="DV5" s="264" t="s">
+      <c r="DV5" s="288" t="s">
         <v>64</v>
       </c>
-      <c r="DW5" s="265"/>
-      <c r="DX5" s="264"/>
-      <c r="DY5" s="286" t="s">
+      <c r="DW5" s="289"/>
+      <c r="DX5" s="288"/>
+      <c r="DY5" s="281" t="s">
         <v>63</v>
       </c>
-      <c r="DZ5" s="286"/>
-      <c r="EA5" s="286"/>
-      <c r="EB5" s="286"/>
-      <c r="EC5" s="287" t="s">
-        <v>128</v>
-      </c>
-      <c r="ED5" s="276" t="s">
+      <c r="DZ5" s="281"/>
+      <c r="EA5" s="281"/>
+      <c r="EB5" s="281"/>
+      <c r="EC5" s="282" t="s">
+        <v>131</v>
+      </c>
+      <c r="ED5" s="284" t="s">
         <v>7</v>
       </c>
-      <c r="EE5" s="262" t="s">
+      <c r="EE5" s="285" t="s">
         <v>65</v>
       </c>
-      <c r="EF5" s="262"/>
-      <c r="EG5" s="262" t="s">
+      <c r="EF5" s="285"/>
+      <c r="EG5" s="285" t="s">
         <v>66</v>
       </c>
-      <c r="EH5" s="262" t="s">
+      <c r="EH5" s="285" t="s">
         <v>67</v>
       </c>
-      <c r="EI5" s="262" t="s">
+      <c r="EI5" s="285" t="s">
         <v>72</v>
       </c>
-      <c r="EJ5" s="263" t="s">
+      <c r="EJ5" s="302" t="s">
         <v>78</v>
       </c>
-      <c r="EK5" s="263" t="s">
+      <c r="EK5" s="302" t="s">
         <v>80</v>
       </c>
-      <c r="EL5" s="263" t="s">
+      <c r="EL5" s="302" t="s">
         <v>79</v>
       </c>
-      <c r="EM5" s="281" t="s">
+      <c r="EM5" s="276" t="s">
         <v>124</v>
       </c>
-      <c r="EN5" s="260" t="s">
+      <c r="EN5" s="300" t="s">
         <v>118</v>
       </c>
-      <c r="EO5" s="283" t="s">
+      <c r="EO5" s="278" t="s">
+        <v>129</v>
+      </c>
+      <c r="EP5" s="280" t="s">
+        <v>122</v>
+      </c>
+      <c r="EQ5" s="280" t="s">
+        <v>121</v>
+      </c>
+      <c r="ER5" s="274" t="s">
+        <v>119</v>
+      </c>
+      <c r="ES5" s="316" t="s">
         <v>130</v>
       </c>
-      <c r="EP5" s="285" t="s">
-        <v>122</v>
-      </c>
-      <c r="EQ5" s="285" t="s">
-        <v>121</v>
-      </c>
-      <c r="ER5" s="279" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="6" spans="1:148" s="205" customFormat="1" ht="148.5" customHeight="1">
-      <c r="A6" s="288"/>
-      <c r="B6" s="278"/>
-      <c r="C6" s="288"/>
-      <c r="D6" s="297"/>
-      <c r="E6" s="299"/>
-      <c r="F6" s="288"/>
-      <c r="G6" s="288"/>
-      <c r="H6" s="288"/>
-      <c r="I6" s="294"/>
+    </row>
+    <row r="6" spans="1:149" s="205" customFormat="1" ht="148.5" customHeight="1">
+      <c r="A6" s="264"/>
+      <c r="B6" s="265"/>
+      <c r="C6" s="264"/>
+      <c r="D6" s="266"/>
+      <c r="E6" s="268"/>
+      <c r="F6" s="264"/>
+      <c r="G6" s="264"/>
+      <c r="H6" s="264"/>
+      <c r="I6" s="269"/>
       <c r="J6" s="184" t="str">
         <f t="shared" ref="J6:AN6" si="2">IF(WEEKDAY(J5)=1,"CN",WEEKDAY(J5))</f>
         <v>CN</v>
@@ -4557,11 +4641,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AO6" s="295"/>
-      <c r="AP6" s="295"/>
-      <c r="AQ6" s="295"/>
-      <c r="AR6" s="296"/>
-      <c r="AS6" s="296"/>
+      <c r="AO6" s="270"/>
+      <c r="AP6" s="270"/>
+      <c r="AQ6" s="270"/>
+      <c r="AR6" s="271"/>
+      <c r="AS6" s="271"/>
       <c r="AT6" s="186" t="str">
         <f>+J6</f>
         <v>CN</v>
@@ -4686,13 +4770,13 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="BY6" s="291"/>
-      <c r="BZ6" s="291"/>
-      <c r="CA6" s="291"/>
-      <c r="CB6" s="291"/>
-      <c r="CC6" s="291"/>
-      <c r="CD6" s="291"/>
-      <c r="CE6" s="291"/>
+      <c r="BY6" s="273"/>
+      <c r="BZ6" s="273"/>
+      <c r="CA6" s="273"/>
+      <c r="CB6" s="273"/>
+      <c r="CC6" s="273"/>
+      <c r="CD6" s="273"/>
+      <c r="CE6" s="273"/>
       <c r="CF6" s="188" t="s">
         <v>92</v>
       </c>
@@ -4735,7 +4819,7 @@
       <c r="CS6" s="180" t="s">
         <v>58</v>
       </c>
-      <c r="CT6" s="273"/>
+      <c r="CT6" s="297"/>
       <c r="CU6" s="188" t="s">
         <v>103</v>
       </c>
@@ -4770,18 +4854,18 @@
         <v>116</v>
       </c>
       <c r="DF6" s="246" t="s">
-        <v>129</v>
-      </c>
-      <c r="DG6" s="270"/>
-      <c r="DH6" s="274"/>
+        <v>128</v>
+      </c>
+      <c r="DG6" s="294"/>
+      <c r="DH6" s="298"/>
       <c r="DI6" s="152" t="s">
         <v>14</v>
       </c>
       <c r="DJ6" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="DK6" s="275"/>
-      <c r="DL6" s="292"/>
+      <c r="DK6" s="283"/>
+      <c r="DL6" s="287"/>
       <c r="DM6" s="180" t="s">
         <v>9</v>
       </c>
@@ -4800,9 +4884,9 @@
       <c r="DR6" s="180" t="s">
         <v>115</v>
       </c>
-      <c r="DS6" s="277"/>
-      <c r="DT6" s="276"/>
-      <c r="DU6" s="278"/>
+      <c r="DS6" s="299"/>
+      <c r="DT6" s="284"/>
+      <c r="DU6" s="265"/>
       <c r="DV6" s="203">
         <v>0.17499999999999999</v>
       </c>
@@ -4824,178 +4908,180 @@
       <c r="EB6" s="152" t="s">
         <v>62</v>
       </c>
-      <c r="EC6" s="275"/>
-      <c r="ED6" s="276"/>
+      <c r="EC6" s="283"/>
+      <c r="ED6" s="284"/>
       <c r="EE6" s="182" t="s">
         <v>73</v>
       </c>
       <c r="EF6" s="182" t="s">
         <v>74</v>
       </c>
-      <c r="EG6" s="262"/>
-      <c r="EH6" s="262"/>
-      <c r="EI6" s="262"/>
-      <c r="EJ6" s="263"/>
-      <c r="EK6" s="263"/>
-      <c r="EL6" s="263"/>
-      <c r="EM6" s="282"/>
-      <c r="EN6" s="261"/>
-      <c r="EO6" s="284"/>
-      <c r="EP6" s="285"/>
-      <c r="EQ6" s="285"/>
-      <c r="ER6" s="279"/>
-    </row>
-    <row r="7" spans="1:148" s="106" customFormat="1" ht="87.75" customHeight="1">
-      <c r="A7" s="280"/>
-      <c r="B7" s="280"/>
-      <c r="C7" s="280"/>
-      <c r="D7" s="280"/>
-      <c r="E7" s="280"/>
-      <c r="F7" s="280"/>
-      <c r="G7" s="280"/>
-      <c r="H7" s="280"/>
-      <c r="I7" s="280"/>
-      <c r="J7" s="280"/>
-      <c r="K7" s="280"/>
-      <c r="L7" s="280"/>
-      <c r="M7" s="280"/>
-      <c r="N7" s="280"/>
-      <c r="O7" s="280"/>
-      <c r="P7" s="280"/>
-      <c r="Q7" s="280"/>
-      <c r="R7" s="280"/>
-      <c r="S7" s="280"/>
-      <c r="T7" s="280"/>
-      <c r="U7" s="280"/>
-      <c r="V7" s="280"/>
-      <c r="W7" s="280"/>
-      <c r="X7" s="280"/>
-      <c r="Y7" s="280"/>
-      <c r="Z7" s="280"/>
-      <c r="AA7" s="280"/>
-      <c r="AB7" s="280"/>
-      <c r="AC7" s="280"/>
-      <c r="AD7" s="280"/>
-      <c r="AE7" s="280"/>
-      <c r="AF7" s="280"/>
-      <c r="AG7" s="280"/>
-      <c r="AH7" s="280"/>
-      <c r="AI7" s="280"/>
-      <c r="AJ7" s="280"/>
-      <c r="AK7" s="280"/>
-      <c r="AL7" s="280"/>
-      <c r="AM7" s="280"/>
-      <c r="AN7" s="280"/>
-      <c r="AO7" s="280"/>
-      <c r="AP7" s="280"/>
-      <c r="AQ7" s="280"/>
-      <c r="AR7" s="280"/>
-      <c r="AS7" s="280"/>
-      <c r="AT7" s="280"/>
-      <c r="AU7" s="280"/>
-      <c r="AV7" s="280"/>
-      <c r="AW7" s="280"/>
-      <c r="AX7" s="280"/>
-      <c r="AY7" s="280"/>
-      <c r="AZ7" s="280"/>
-      <c r="BA7" s="280"/>
-      <c r="BB7" s="280"/>
-      <c r="BC7" s="280"/>
-      <c r="BD7" s="280"/>
-      <c r="BE7" s="280"/>
-      <c r="BF7" s="280"/>
-      <c r="BG7" s="280"/>
-      <c r="BH7" s="280"/>
-      <c r="BI7" s="280"/>
-      <c r="BJ7" s="280"/>
-      <c r="BK7" s="280"/>
-      <c r="BL7" s="280"/>
-      <c r="BM7" s="280"/>
-      <c r="BN7" s="280"/>
-      <c r="BO7" s="280"/>
-      <c r="BP7" s="280"/>
-      <c r="BQ7" s="280"/>
-      <c r="BR7" s="280"/>
-      <c r="BS7" s="280"/>
-      <c r="BT7" s="280"/>
-      <c r="BU7" s="280"/>
-      <c r="BV7" s="280"/>
-      <c r="BW7" s="280"/>
-      <c r="BX7" s="280"/>
-      <c r="BY7" s="280"/>
-      <c r="BZ7" s="280"/>
-      <c r="CA7" s="280"/>
-      <c r="CB7" s="280"/>
-      <c r="CC7" s="280"/>
-      <c r="CD7" s="280"/>
-      <c r="CE7" s="280"/>
-      <c r="CF7" s="280"/>
-      <c r="CG7" s="280"/>
-      <c r="CH7" s="280"/>
-      <c r="CI7" s="280"/>
-      <c r="CJ7" s="280"/>
-      <c r="CK7" s="280"/>
-      <c r="CL7" s="280"/>
-      <c r="CM7" s="280"/>
-      <c r="CN7" s="280"/>
-      <c r="CO7" s="280"/>
-      <c r="CP7" s="280"/>
-      <c r="CQ7" s="280"/>
-      <c r="CR7" s="280"/>
-      <c r="CS7" s="280"/>
-      <c r="CT7" s="280"/>
-      <c r="CU7" s="280"/>
-      <c r="CV7" s="280"/>
-      <c r="CW7" s="280"/>
-      <c r="CX7" s="280"/>
-      <c r="CY7" s="280"/>
-      <c r="CZ7" s="280"/>
-      <c r="DA7" s="280"/>
-      <c r="DB7" s="280"/>
-      <c r="DC7" s="280"/>
-      <c r="DD7" s="280"/>
-      <c r="DE7" s="280"/>
-      <c r="DF7" s="280"/>
-      <c r="DG7" s="280"/>
-      <c r="DH7" s="280"/>
-      <c r="DI7" s="280"/>
-      <c r="DJ7" s="280"/>
-      <c r="DK7" s="280"/>
-      <c r="DL7" s="280"/>
-      <c r="DM7" s="280"/>
-      <c r="DN7" s="280"/>
-      <c r="DO7" s="280"/>
-      <c r="DP7" s="280"/>
-      <c r="DQ7" s="280"/>
-      <c r="DR7" s="280"/>
-      <c r="DS7" s="280"/>
-      <c r="DT7" s="280"/>
-      <c r="DU7" s="280"/>
-      <c r="DV7" s="280"/>
-      <c r="DW7" s="280"/>
-      <c r="DX7" s="280"/>
-      <c r="DY7" s="280"/>
-      <c r="DZ7" s="280"/>
-      <c r="EA7" s="280"/>
-      <c r="EB7" s="280"/>
-      <c r="EC7" s="280"/>
-      <c r="ED7" s="280"/>
-      <c r="EE7" s="280"/>
-      <c r="EF7" s="280"/>
-      <c r="EG7" s="280"/>
-      <c r="EH7" s="280"/>
-      <c r="EI7" s="280"/>
-      <c r="EJ7" s="280"/>
-      <c r="EK7" s="280"/>
-      <c r="EL7" s="280"/>
+      <c r="EG6" s="285"/>
+      <c r="EH6" s="285"/>
+      <c r="EI6" s="285"/>
+      <c r="EJ6" s="302"/>
+      <c r="EK6" s="302"/>
+      <c r="EL6" s="302"/>
+      <c r="EM6" s="277"/>
+      <c r="EN6" s="301"/>
+      <c r="EO6" s="279"/>
+      <c r="EP6" s="280"/>
+      <c r="EQ6" s="280"/>
+      <c r="ER6" s="274"/>
+      <c r="ES6" s="316"/>
+    </row>
+    <row r="7" spans="1:149" s="106" customFormat="1" ht="87.75" customHeight="1">
+      <c r="A7" s="275"/>
+      <c r="B7" s="275"/>
+      <c r="C7" s="275"/>
+      <c r="D7" s="275"/>
+      <c r="E7" s="275"/>
+      <c r="F7" s="275"/>
+      <c r="G7" s="275"/>
+      <c r="H7" s="275"/>
+      <c r="I7" s="275"/>
+      <c r="J7" s="275"/>
+      <c r="K7" s="275"/>
+      <c r="L7" s="275"/>
+      <c r="M7" s="275"/>
+      <c r="N7" s="275"/>
+      <c r="O7" s="275"/>
+      <c r="P7" s="275"/>
+      <c r="Q7" s="275"/>
+      <c r="R7" s="275"/>
+      <c r="S7" s="275"/>
+      <c r="T7" s="275"/>
+      <c r="U7" s="275"/>
+      <c r="V7" s="275"/>
+      <c r="W7" s="275"/>
+      <c r="X7" s="275"/>
+      <c r="Y7" s="275"/>
+      <c r="Z7" s="275"/>
+      <c r="AA7" s="275"/>
+      <c r="AB7" s="275"/>
+      <c r="AC7" s="275"/>
+      <c r="AD7" s="275"/>
+      <c r="AE7" s="275"/>
+      <c r="AF7" s="275"/>
+      <c r="AG7" s="275"/>
+      <c r="AH7" s="275"/>
+      <c r="AI7" s="275"/>
+      <c r="AJ7" s="275"/>
+      <c r="AK7" s="275"/>
+      <c r="AL7" s="275"/>
+      <c r="AM7" s="275"/>
+      <c r="AN7" s="275"/>
+      <c r="AO7" s="275"/>
+      <c r="AP7" s="275"/>
+      <c r="AQ7" s="275"/>
+      <c r="AR7" s="275"/>
+      <c r="AS7" s="275"/>
+      <c r="AT7" s="275"/>
+      <c r="AU7" s="275"/>
+      <c r="AV7" s="275"/>
+      <c r="AW7" s="275"/>
+      <c r="AX7" s="275"/>
+      <c r="AY7" s="275"/>
+      <c r="AZ7" s="275"/>
+      <c r="BA7" s="275"/>
+      <c r="BB7" s="275"/>
+      <c r="BC7" s="275"/>
+      <c r="BD7" s="275"/>
+      <c r="BE7" s="275"/>
+      <c r="BF7" s="275"/>
+      <c r="BG7" s="275"/>
+      <c r="BH7" s="275"/>
+      <c r="BI7" s="275"/>
+      <c r="BJ7" s="275"/>
+      <c r="BK7" s="275"/>
+      <c r="BL7" s="275"/>
+      <c r="BM7" s="275"/>
+      <c r="BN7" s="275"/>
+      <c r="BO7" s="275"/>
+      <c r="BP7" s="275"/>
+      <c r="BQ7" s="275"/>
+      <c r="BR7" s="275"/>
+      <c r="BS7" s="275"/>
+      <c r="BT7" s="275"/>
+      <c r="BU7" s="275"/>
+      <c r="BV7" s="275"/>
+      <c r="BW7" s="275"/>
+      <c r="BX7" s="275"/>
+      <c r="BY7" s="275"/>
+      <c r="BZ7" s="275"/>
+      <c r="CA7" s="275"/>
+      <c r="CB7" s="275"/>
+      <c r="CC7" s="275"/>
+      <c r="CD7" s="275"/>
+      <c r="CE7" s="275"/>
+      <c r="CF7" s="275"/>
+      <c r="CG7" s="275"/>
+      <c r="CH7" s="275"/>
+      <c r="CI7" s="275"/>
+      <c r="CJ7" s="275"/>
+      <c r="CK7" s="275"/>
+      <c r="CL7" s="275"/>
+      <c r="CM7" s="275"/>
+      <c r="CN7" s="275"/>
+      <c r="CO7" s="275"/>
+      <c r="CP7" s="275"/>
+      <c r="CQ7" s="275"/>
+      <c r="CR7" s="275"/>
+      <c r="CS7" s="275"/>
+      <c r="CT7" s="275"/>
+      <c r="CU7" s="275"/>
+      <c r="CV7" s="275"/>
+      <c r="CW7" s="275"/>
+      <c r="CX7" s="275"/>
+      <c r="CY7" s="275"/>
+      <c r="CZ7" s="275"/>
+      <c r="DA7" s="275"/>
+      <c r="DB7" s="275"/>
+      <c r="DC7" s="275"/>
+      <c r="DD7" s="275"/>
+      <c r="DE7" s="275"/>
+      <c r="DF7" s="275"/>
+      <c r="DG7" s="275"/>
+      <c r="DH7" s="275"/>
+      <c r="DI7" s="275"/>
+      <c r="DJ7" s="275"/>
+      <c r="DK7" s="275"/>
+      <c r="DL7" s="275"/>
+      <c r="DM7" s="275"/>
+      <c r="DN7" s="275"/>
+      <c r="DO7" s="275"/>
+      <c r="DP7" s="275"/>
+      <c r="DQ7" s="275"/>
+      <c r="DR7" s="275"/>
+      <c r="DS7" s="275"/>
+      <c r="DT7" s="275"/>
+      <c r="DU7" s="275"/>
+      <c r="DV7" s="275"/>
+      <c r="DW7" s="275"/>
+      <c r="DX7" s="275"/>
+      <c r="DY7" s="275"/>
+      <c r="DZ7" s="275"/>
+      <c r="EA7" s="275"/>
+      <c r="EB7" s="275"/>
+      <c r="EC7" s="275"/>
+      <c r="ED7" s="275"/>
+      <c r="EE7" s="275"/>
+      <c r="EF7" s="275"/>
+      <c r="EG7" s="275"/>
+      <c r="EH7" s="275"/>
+      <c r="EI7" s="275"/>
+      <c r="EJ7" s="275"/>
+      <c r="EK7" s="275"/>
+      <c r="EL7" s="275"/>
       <c r="EM7" s="238"/>
       <c r="EN7" s="238"/>
       <c r="EO7" s="238"/>
       <c r="EP7" s="239"/>
       <c r="EQ7" s="239"/>
       <c r="ER7" s="239"/>
-    </row>
-    <row r="8" spans="1:148" s="168" customFormat="1" ht="84" customHeight="1">
+      <c r="ES7" s="239"/>
+    </row>
+    <row r="8" spans="1:149" s="168" customFormat="1" ht="84" customHeight="1">
       <c r="A8" s="150"/>
       <c r="B8" s="150"/>
       <c r="C8" s="162"/>
@@ -5254,7 +5340,7 @@
         <v>0</v>
       </c>
       <c r="CR8" s="156"/>
-      <c r="CS8" s="314"/>
+      <c r="CS8" s="261"/>
       <c r="CT8" s="157">
         <f t="shared" ref="CT8" si="51">+I8+CQ8+CR8+CS8</f>
         <v>0</v>
@@ -5299,7 +5385,7 @@
         <f t="shared" ref="DD8" si="60">+CS8/26*(CF8+(CG8+CJ8)/8)</f>
         <v>0</v>
       </c>
-      <c r="DE8" s="313"/>
+      <c r="DE8" s="260"/>
       <c r="DF8" s="211">
         <f t="shared" ref="DF8" si="61">+DD8+DE8</f>
         <v>0</v>
@@ -5330,23 +5416,23 @@
         <v>0</v>
       </c>
       <c r="DN8" s="159">
-        <f t="shared" ref="DN8" si="68">DL8*1.5%</f>
+        <f>IF(ES8=0,DL8*1.5%,IF(ES8=1,0,DL8*1.5%+DL8*3%))</f>
         <v>0</v>
       </c>
       <c r="DO8" s="159">
-        <f t="shared" ref="DO8" si="69">DL8*1%</f>
+        <f t="shared" ref="DO8" si="68">DL8*1%</f>
         <v>0</v>
       </c>
       <c r="DP8" s="159">
-        <f t="shared" ref="DP8" si="70">EI8</f>
+        <f t="shared" ref="DP8" si="69">EI8</f>
         <v>0</v>
       </c>
       <c r="DQ8" s="159">
-        <f t="shared" ref="DQ8" si="71">+SUM(DM8:DP8)</f>
+        <f t="shared" ref="DQ8" si="70">+SUM(DM8:DP8)</f>
         <v>0</v>
       </c>
       <c r="DR8" s="159">
-        <f t="shared" ref="DR8" si="72">SUM(DM8:DO8)</f>
+        <f t="shared" ref="DR8" si="71">SUM(DM8:DO8)</f>
         <v>0</v>
       </c>
       <c r="DS8" s="160">
@@ -5363,7 +5449,7 @@
         <v>0</v>
       </c>
       <c r="DW8" s="159">
-        <f>DL8*$DW$6</f>
+        <f>IF(ES8=0,DL8*1.5%,IF(ES8=1,DL8*1.5%+DL8*3%,0))</f>
         <v>0</v>
       </c>
       <c r="DX8" s="159">
@@ -5383,7 +5469,7 @@
         <v>0</v>
       </c>
       <c r="EB8" s="173">
-        <f t="shared" ref="EB8" si="73">DY8+DZ8+EA8</f>
+        <f t="shared" ref="EB8" si="72">DY8+DZ8+EA8</f>
         <v>0</v>
       </c>
       <c r="EC8" s="164">
@@ -5410,7 +5496,7 @@
         <v>-775000</v>
       </c>
       <c r="EI8" s="172">
-        <f t="shared" ref="EI8" si="74">+IF(EH8&lt;0,0,EH8)</f>
+        <f t="shared" ref="EI8" si="73">+IF(EH8&lt;0,0,EH8)</f>
         <v>0</v>
       </c>
       <c r="EJ8" s="165">
@@ -5431,8 +5517,11 @@
       <c r="EP8" s="150"/>
       <c r="EQ8" s="150"/>
       <c r="ER8" s="240"/>
-    </row>
-    <row r="9" spans="1:148" s="93" customFormat="1">
+      <c r="ES8" s="315">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:149" s="93" customFormat="1">
       <c r="A9" s="95"/>
       <c r="B9" s="95"/>
       <c r="D9" s="97"/>
@@ -5570,7 +5659,7 @@
       <c r="EQ9" s="98"/>
       <c r="ER9" s="241"/>
     </row>
-    <row r="10" spans="1:148" s="93" customFormat="1">
+    <row r="10" spans="1:149" s="93" customFormat="1">
       <c r="A10" s="95"/>
       <c r="B10" s="95"/>
       <c r="D10" s="97"/>
@@ -5708,7 +5797,7 @@
       <c r="EQ10" s="98"/>
       <c r="ER10" s="241"/>
     </row>
-    <row r="11" spans="1:148" s="93" customFormat="1">
+    <row r="11" spans="1:149" s="93" customFormat="1">
       <c r="A11" s="95"/>
       <c r="B11" s="95"/>
       <c r="D11" s="97"/>
@@ -5846,7 +5935,7 @@
       <c r="EQ11" s="98"/>
       <c r="ER11" s="241"/>
     </row>
-    <row r="12" spans="1:148" s="93" customFormat="1">
+    <row r="12" spans="1:149" s="93" customFormat="1">
       <c r="A12" s="95"/>
       <c r="B12" s="95"/>
       <c r="D12" s="97"/>
@@ -5984,7 +6073,7 @@
       <c r="EQ12" s="98"/>
       <c r="ER12" s="241"/>
     </row>
-    <row r="13" spans="1:148" s="93" customFormat="1">
+    <row r="13" spans="1:149" s="93" customFormat="1">
       <c r="A13" s="95"/>
       <c r="B13" s="95"/>
       <c r="D13" s="97"/>
@@ -6122,7 +6211,7 @@
       <c r="EQ13" s="98"/>
       <c r="ER13" s="241"/>
     </row>
-    <row r="14" spans="1:148" s="93" customFormat="1">
+    <row r="14" spans="1:149" s="93" customFormat="1">
       <c r="A14" s="95"/>
       <c r="B14" s="95"/>
       <c r="D14" s="97"/>
@@ -6260,7 +6349,7 @@
       <c r="EQ14" s="98"/>
       <c r="ER14" s="241"/>
     </row>
-    <row r="15" spans="1:148" s="93" customFormat="1">
+    <row r="15" spans="1:149" s="93" customFormat="1">
       <c r="A15" s="95"/>
       <c r="B15" s="95"/>
       <c r="D15" s="97"/>
@@ -6398,7 +6487,7 @@
       <c r="EQ15" s="98"/>
       <c r="ER15" s="241"/>
     </row>
-    <row r="16" spans="1:148" s="93" customFormat="1">
+    <row r="16" spans="1:149" s="93" customFormat="1">
       <c r="A16" s="95"/>
       <c r="B16" s="95"/>
       <c r="D16" s="97"/>
@@ -27101,39 +27190,24 @@
     </row>
   </sheetData>
   <autoFilter ref="A6:ER8" xr:uid="{00000000-0001-0000-0900-000000000000}"/>
-  <mergeCells count="64">
-    <mergeCell ref="AO1:AS1"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="S4:U4"/>
-    <mergeCell ref="W4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AD4"/>
-    <mergeCell ref="AG4:AI4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="BG4:BI4"/>
-    <mergeCell ref="AT4:AU4"/>
-    <mergeCell ref="AO5:AO6"/>
-    <mergeCell ref="AP5:AP6"/>
-    <mergeCell ref="AQ5:AQ6"/>
-    <mergeCell ref="AR5:AR6"/>
-    <mergeCell ref="AS5:AS6"/>
-    <mergeCell ref="BJ4:BK4"/>
-    <mergeCell ref="BL4:BN4"/>
-    <mergeCell ref="BQ4:BS4"/>
-    <mergeCell ref="BC4:BE4"/>
-    <mergeCell ref="CD5:CD6"/>
-    <mergeCell ref="BY5:BY6"/>
-    <mergeCell ref="BZ5:BZ6"/>
-    <mergeCell ref="CA5:CA6"/>
-    <mergeCell ref="CB5:CB6"/>
-    <mergeCell ref="CC5:CC6"/>
+  <mergeCells count="65">
+    <mergeCell ref="ES5:ES6"/>
+    <mergeCell ref="EN5:EN6"/>
+    <mergeCell ref="EI5:EI6"/>
+    <mergeCell ref="EJ5:EJ6"/>
+    <mergeCell ref="EK5:EK6"/>
+    <mergeCell ref="EL5:EL6"/>
+    <mergeCell ref="EH5:EH6"/>
+    <mergeCell ref="DV5:DX5"/>
+    <mergeCell ref="CQ5:CS5"/>
+    <mergeCell ref="DG5:DG6"/>
+    <mergeCell ref="DI5:DJ5"/>
+    <mergeCell ref="CT5:CT6"/>
+    <mergeCell ref="DH5:DH6"/>
+    <mergeCell ref="DK5:DK6"/>
+    <mergeCell ref="DM5:DR5"/>
+    <mergeCell ref="DS5:DS6"/>
+    <mergeCell ref="DU5:DU6"/>
     <mergeCell ref="ER5:ER6"/>
     <mergeCell ref="A7:EL7"/>
     <mergeCell ref="EM5:EM6"/>
@@ -27150,22 +27224,38 @@
     <mergeCell ref="DL5:DL6"/>
     <mergeCell ref="EG5:EG6"/>
     <mergeCell ref="EQ5:EQ6"/>
-    <mergeCell ref="EH5:EH6"/>
-    <mergeCell ref="DV5:DX5"/>
-    <mergeCell ref="CQ5:CS5"/>
-    <mergeCell ref="DG5:DG6"/>
-    <mergeCell ref="DI5:DJ5"/>
-    <mergeCell ref="CT5:CT6"/>
-    <mergeCell ref="DH5:DH6"/>
-    <mergeCell ref="DK5:DK6"/>
-    <mergeCell ref="DM5:DR5"/>
-    <mergeCell ref="DS5:DS6"/>
-    <mergeCell ref="DU5:DU6"/>
-    <mergeCell ref="EN5:EN6"/>
-    <mergeCell ref="EI5:EI6"/>
-    <mergeCell ref="EJ5:EJ6"/>
-    <mergeCell ref="EK5:EK6"/>
-    <mergeCell ref="EL5:EL6"/>
+    <mergeCell ref="BJ4:BK4"/>
+    <mergeCell ref="BL4:BN4"/>
+    <mergeCell ref="BQ4:BS4"/>
+    <mergeCell ref="BC4:BE4"/>
+    <mergeCell ref="CD5:CD6"/>
+    <mergeCell ref="BY5:BY6"/>
+    <mergeCell ref="BZ5:BZ6"/>
+    <mergeCell ref="CA5:CA6"/>
+    <mergeCell ref="CB5:CB6"/>
+    <mergeCell ref="CC5:CC6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="BG4:BI4"/>
+    <mergeCell ref="AT4:AU4"/>
+    <mergeCell ref="AO5:AO6"/>
+    <mergeCell ref="AP5:AP6"/>
+    <mergeCell ref="AQ5:AQ6"/>
+    <mergeCell ref="AR5:AR6"/>
+    <mergeCell ref="AS5:AS6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="AO1:AS1"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="S4:U4"/>
+    <mergeCell ref="W4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AD4"/>
+    <mergeCell ref="AG4:AI4"/>
   </mergeCells>
   <conditionalFormatting sqref="A5 A8:B8">
     <cfRule type="duplicateValues" dxfId="20" priority="20879"/>
@@ -27822,11 +27912,11 @@
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
       <c r="H8" s="20"/>
-      <c r="I8" s="301">
+      <c r="I8" s="309">
         <v>2026</v>
       </c>
-      <c r="J8" s="302"/>
-      <c r="K8" s="302"/>
+      <c r="J8" s="310"/>
+      <c r="K8" s="310"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="21" t="s">
@@ -27851,13 +27941,13 @@
     <row r="9" spans="1:29" ht="15.75" customHeight="1" thickBot="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="303" t="s">
+      <c r="C9" s="311" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="304"/>
-      <c r="E9" s="304"/>
-      <c r="F9" s="304"/>
-      <c r="G9" s="304"/>
+      <c r="D9" s="312"/>
+      <c r="E9" s="312"/>
+      <c r="F9" s="312"/>
+      <c r="G9" s="312"/>
       <c r="H9" s="20"/>
       <c r="I9" s="24"/>
       <c r="J9" s="24"/>
@@ -27953,19 +28043,19 @@
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
-      <c r="J12" s="305" t="s">
+      <c r="J12" s="313" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="304"/>
-      <c r="L12" s="304"/>
-      <c r="M12" s="304"/>
-      <c r="N12" s="304"/>
-      <c r="O12" s="304"/>
-      <c r="P12" s="306">
+      <c r="K12" s="312"/>
+      <c r="L12" s="312"/>
+      <c r="M12" s="312"/>
+      <c r="N12" s="312"/>
+      <c r="O12" s="312"/>
+      <c r="P12" s="314">
         <f>I8</f>
         <v>2026</v>
       </c>
-      <c r="Q12" s="304"/>
+      <c r="Q12" s="312"/>
       <c r="R12" s="33"/>
       <c r="S12" s="34"/>
       <c r="T12" s="34"/>
@@ -28229,38 +28319,38 @@
     </row>
     <row r="21" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A21" s="39"/>
-      <c r="B21" s="307" t="s">
+      <c r="B21" s="308" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="308"/>
-      <c r="D21" s="308"/>
-      <c r="E21" s="308"/>
-      <c r="F21" s="308"/>
-      <c r="G21" s="308"/>
-      <c r="H21" s="308"/>
-      <c r="I21" s="308"/>
+      <c r="C21" s="304"/>
+      <c r="D21" s="304"/>
+      <c r="E21" s="304"/>
+      <c r="F21" s="304"/>
+      <c r="G21" s="304"/>
+      <c r="H21" s="304"/>
+      <c r="I21" s="304"/>
       <c r="J21" s="40"/>
-      <c r="K21" s="309" t="s">
+      <c r="K21" s="305" t="s">
         <v>37</v>
       </c>
-      <c r="L21" s="308"/>
-      <c r="M21" s="308"/>
-      <c r="N21" s="308"/>
-      <c r="O21" s="308"/>
-      <c r="P21" s="308"/>
-      <c r="Q21" s="308"/>
-      <c r="R21" s="308"/>
+      <c r="L21" s="304"/>
+      <c r="M21" s="304"/>
+      <c r="N21" s="304"/>
+      <c r="O21" s="304"/>
+      <c r="P21" s="304"/>
+      <c r="Q21" s="304"/>
+      <c r="R21" s="304"/>
       <c r="S21" s="40"/>
-      <c r="T21" s="310" t="s">
+      <c r="T21" s="303" t="s">
         <v>38</v>
       </c>
-      <c r="U21" s="308"/>
-      <c r="V21" s="308"/>
-      <c r="W21" s="308"/>
-      <c r="X21" s="308"/>
-      <c r="Y21" s="308"/>
-      <c r="Z21" s="308"/>
-      <c r="AA21" s="308"/>
+      <c r="U21" s="304"/>
+      <c r="V21" s="304"/>
+      <c r="W21" s="304"/>
+      <c r="X21" s="304"/>
+      <c r="Y21" s="304"/>
+      <c r="Z21" s="304"/>
+      <c r="AA21" s="304"/>
       <c r="AB21" s="41"/>
       <c r="AC21" s="42"/>
     </row>
@@ -29160,38 +29250,38 @@
     </row>
     <row r="35" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="311" t="s">
+      <c r="B35" s="306" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="308"/>
-      <c r="D35" s="308"/>
-      <c r="E35" s="308"/>
-      <c r="F35" s="308"/>
-      <c r="G35" s="308"/>
-      <c r="H35" s="308"/>
-      <c r="I35" s="308"/>
+      <c r="C35" s="304"/>
+      <c r="D35" s="304"/>
+      <c r="E35" s="304"/>
+      <c r="F35" s="304"/>
+      <c r="G35" s="304"/>
+      <c r="H35" s="304"/>
+      <c r="I35" s="304"/>
       <c r="J35" s="40"/>
-      <c r="K35" s="312" t="s">
+      <c r="K35" s="307" t="s">
         <v>48</v>
       </c>
-      <c r="L35" s="308"/>
-      <c r="M35" s="308"/>
-      <c r="N35" s="308"/>
-      <c r="O35" s="308"/>
-      <c r="P35" s="308"/>
-      <c r="Q35" s="308"/>
-      <c r="R35" s="308"/>
+      <c r="L35" s="304"/>
+      <c r="M35" s="304"/>
+      <c r="N35" s="304"/>
+      <c r="O35" s="304"/>
+      <c r="P35" s="304"/>
+      <c r="Q35" s="304"/>
+      <c r="R35" s="304"/>
       <c r="S35" s="40"/>
-      <c r="T35" s="309" t="s">
+      <c r="T35" s="305" t="s">
         <v>49</v>
       </c>
-      <c r="U35" s="308"/>
-      <c r="V35" s="308"/>
-      <c r="W35" s="308"/>
-      <c r="X35" s="308"/>
-      <c r="Y35" s="308"/>
-      <c r="Z35" s="308"/>
-      <c r="AA35" s="308"/>
+      <c r="U35" s="304"/>
+      <c r="V35" s="304"/>
+      <c r="W35" s="304"/>
+      <c r="X35" s="304"/>
+      <c r="Y35" s="304"/>
+      <c r="Z35" s="304"/>
+      <c r="AA35" s="304"/>
       <c r="AB35" s="70"/>
       <c r="AC35" s="40"/>
     </row>
@@ -30080,38 +30170,38 @@
     </row>
     <row r="49" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A49" s="69"/>
-      <c r="B49" s="309" t="s">
+      <c r="B49" s="305" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="308"/>
-      <c r="D49" s="308"/>
-      <c r="E49" s="308"/>
-      <c r="F49" s="308"/>
-      <c r="G49" s="308"/>
-      <c r="H49" s="308"/>
-      <c r="I49" s="308"/>
+      <c r="C49" s="304"/>
+      <c r="D49" s="304"/>
+      <c r="E49" s="304"/>
+      <c r="F49" s="304"/>
+      <c r="G49" s="304"/>
+      <c r="H49" s="304"/>
+      <c r="I49" s="304"/>
       <c r="J49" s="40"/>
-      <c r="K49" s="311" t="s">
+      <c r="K49" s="306" t="s">
         <v>51</v>
       </c>
-      <c r="L49" s="308"/>
-      <c r="M49" s="308"/>
-      <c r="N49" s="308"/>
-      <c r="O49" s="308"/>
-      <c r="P49" s="308"/>
-      <c r="Q49" s="308"/>
-      <c r="R49" s="308"/>
+      <c r="L49" s="304"/>
+      <c r="M49" s="304"/>
+      <c r="N49" s="304"/>
+      <c r="O49" s="304"/>
+      <c r="P49" s="304"/>
+      <c r="Q49" s="304"/>
+      <c r="R49" s="304"/>
       <c r="S49" s="40"/>
-      <c r="T49" s="307" t="s">
+      <c r="T49" s="308" t="s">
         <v>52</v>
       </c>
-      <c r="U49" s="308"/>
-      <c r="V49" s="308"/>
-      <c r="W49" s="308"/>
-      <c r="X49" s="308"/>
-      <c r="Y49" s="308"/>
-      <c r="Z49" s="308"/>
-      <c r="AA49" s="308"/>
+      <c r="U49" s="304"/>
+      <c r="V49" s="304"/>
+      <c r="W49" s="304"/>
+      <c r="X49" s="304"/>
+      <c r="Y49" s="304"/>
+      <c r="Z49" s="304"/>
+      <c r="AA49" s="304"/>
       <c r="AB49" s="70"/>
       <c r="AC49" s="40"/>
     </row>
@@ -31000,38 +31090,38 @@
     </row>
     <row r="63" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A63" s="69"/>
-      <c r="B63" s="310" t="s">
+      <c r="B63" s="303" t="s">
         <v>53</v>
       </c>
-      <c r="C63" s="308"/>
-      <c r="D63" s="308"/>
-      <c r="E63" s="308"/>
-      <c r="F63" s="308"/>
-      <c r="G63" s="308"/>
-      <c r="H63" s="308"/>
-      <c r="I63" s="308"/>
+      <c r="C63" s="304"/>
+      <c r="D63" s="304"/>
+      <c r="E63" s="304"/>
+      <c r="F63" s="304"/>
+      <c r="G63" s="304"/>
+      <c r="H63" s="304"/>
+      <c r="I63" s="304"/>
       <c r="J63" s="40"/>
-      <c r="K63" s="309" t="s">
+      <c r="K63" s="305" t="s">
         <v>54</v>
       </c>
-      <c r="L63" s="308"/>
-      <c r="M63" s="308"/>
-      <c r="N63" s="308"/>
-      <c r="O63" s="308"/>
-      <c r="P63" s="308"/>
-      <c r="Q63" s="308"/>
-      <c r="R63" s="308"/>
+      <c r="L63" s="304"/>
+      <c r="M63" s="304"/>
+      <c r="N63" s="304"/>
+      <c r="O63" s="304"/>
+      <c r="P63" s="304"/>
+      <c r="Q63" s="304"/>
+      <c r="R63" s="304"/>
       <c r="S63" s="40"/>
-      <c r="T63" s="311" t="s">
+      <c r="T63" s="306" t="s">
         <v>55</v>
       </c>
-      <c r="U63" s="308"/>
-      <c r="V63" s="308"/>
-      <c r="W63" s="308"/>
-      <c r="X63" s="308"/>
-      <c r="Y63" s="308"/>
-      <c r="Z63" s="308"/>
-      <c r="AA63" s="308"/>
+      <c r="U63" s="304"/>
+      <c r="V63" s="304"/>
+      <c r="W63" s="304"/>
+      <c r="X63" s="304"/>
+      <c r="Y63" s="304"/>
+      <c r="Z63" s="304"/>
+      <c r="AA63" s="304"/>
       <c r="AB63" s="70"/>
       <c r="AC63" s="40"/>
     </row>
@@ -60566,6 +60656,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="J12:O12"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="K21:R21"/>
     <mergeCell ref="B63:I63"/>
     <mergeCell ref="K63:R63"/>
     <mergeCell ref="T63:AA63"/>
@@ -60576,12 +60672,6 @@
     <mergeCell ref="B49:I49"/>
     <mergeCell ref="K49:R49"/>
     <mergeCell ref="T49:AA49"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="J12:O12"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="K21:R21"/>
   </mergeCells>
   <conditionalFormatting sqref="C51:I55">
     <cfRule type="expression" dxfId="2" priority="3">

</xml_diff>

<commit_message>
thêm tính năng truy thu bhyt hoàn thành
</commit_message>
<xml_diff>
--- a/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
+++ b/my_custom_addons/dl_salary_kpi/static/src/templates/TEMPLATE_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonzai/dev/odoo 19/odoo/my_custom_addons/dl_salary_kpi/static/src/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20A8277D-3347-5D4C-B21E-0616A791625C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D7CC795-BE69-F74E-B757-2AA2BF8501CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="480" windowWidth="38400" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-33720" yWindow="500" windowWidth="33720" windowHeight="19980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kangatang" sheetId="43" state="veryHidden" r:id="rId1"/>
@@ -2509,6 +2509,9 @@
     <xf numFmtId="169" fontId="78" fillId="26" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="78" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="71" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2543,9 +2546,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="174" fontId="55" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="66" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2623,6 +2623,9 @@
     <xf numFmtId="169" fontId="14" fillId="18" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="55" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="55" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2630,6 +2633,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="81" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="55" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="16" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2661,12 +2667,6 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="32">
@@ -3055,10 +3055,6 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3496,11 +3492,11 @@
       <c r="AL1" s="212"/>
       <c r="AM1" s="212"/>
       <c r="AN1" s="212"/>
-      <c r="AO1" s="262"/>
-      <c r="AP1" s="262"/>
-      <c r="AQ1" s="262"/>
-      <c r="AR1" s="262"/>
-      <c r="AS1" s="262"/>
+      <c r="AO1" s="263"/>
+      <c r="AP1" s="263"/>
+      <c r="AQ1" s="263"/>
+      <c r="AR1" s="263"/>
+      <c r="AS1" s="263"/>
       <c r="AT1" s="120"/>
       <c r="AU1" s="120"/>
       <c r="AV1" s="120"/>
@@ -3902,10 +3898,10 @@
       <c r="G4" s="232"/>
       <c r="H4" s="108"/>
       <c r="I4" s="256"/>
-      <c r="J4" s="263" t="s">
+      <c r="J4" s="264" t="s">
         <v>68</v>
       </c>
-      <c r="K4" s="263"/>
+      <c r="K4" s="264"/>
       <c r="L4" s="258">
         <v>3</v>
       </c>
@@ -3919,23 +3915,23 @@
       </c>
       <c r="Q4" s="259"/>
       <c r="R4" s="109"/>
-      <c r="S4" s="263"/>
-      <c r="T4" s="263"/>
-      <c r="U4" s="263"/>
+      <c r="S4" s="264"/>
+      <c r="T4" s="264"/>
+      <c r="U4" s="264"/>
       <c r="V4" s="109"/>
-      <c r="W4" s="263"/>
-      <c r="X4" s="263"/>
-      <c r="Y4" s="263"/>
-      <c r="Z4" s="263"/>
-      <c r="AA4" s="263"/>
-      <c r="AB4" s="263"/>
-      <c r="AC4" s="263"/>
-      <c r="AD4" s="263"/>
+      <c r="W4" s="264"/>
+      <c r="X4" s="264"/>
+      <c r="Y4" s="264"/>
+      <c r="Z4" s="264"/>
+      <c r="AA4" s="264"/>
+      <c r="AB4" s="264"/>
+      <c r="AC4" s="264"/>
+      <c r="AD4" s="264"/>
       <c r="AE4" s="109"/>
       <c r="AF4" s="110"/>
-      <c r="AG4" s="263"/>
-      <c r="AH4" s="263"/>
-      <c r="AI4" s="263"/>
+      <c r="AG4" s="264"/>
+      <c r="AH4" s="264"/>
+      <c r="AI4" s="264"/>
       <c r="AJ4" s="109"/>
       <c r="AK4" s="109"/>
       <c r="AL4" s="109"/>
@@ -3946,10 +3942,10 @@
       <c r="AQ4" s="113"/>
       <c r="AR4" s="221"/>
       <c r="AS4" s="227"/>
-      <c r="AT4" s="263" t="s">
+      <c r="AT4" s="264" t="s">
         <v>68</v>
       </c>
-      <c r="AU4" s="263"/>
+      <c r="AU4" s="264"/>
       <c r="AV4" s="258">
         <f>L4</f>
         <v>3</v>
@@ -3965,23 +3961,23 @@
       </c>
       <c r="BA4" s="259"/>
       <c r="BB4" s="109"/>
-      <c r="BC4" s="263"/>
-      <c r="BD4" s="263"/>
-      <c r="BE4" s="263"/>
+      <c r="BC4" s="264"/>
+      <c r="BD4" s="264"/>
+      <c r="BE4" s="264"/>
       <c r="BF4" s="109"/>
-      <c r="BG4" s="263"/>
-      <c r="BH4" s="263"/>
-      <c r="BI4" s="263"/>
-      <c r="BJ4" s="263"/>
-      <c r="BK4" s="263"/>
-      <c r="BL4" s="263"/>
-      <c r="BM4" s="263"/>
-      <c r="BN4" s="263"/>
+      <c r="BG4" s="264"/>
+      <c r="BH4" s="264"/>
+      <c r="BI4" s="264"/>
+      <c r="BJ4" s="264"/>
+      <c r="BK4" s="264"/>
+      <c r="BL4" s="264"/>
+      <c r="BM4" s="264"/>
+      <c r="BN4" s="264"/>
       <c r="BO4" s="109"/>
       <c r="BP4" s="110"/>
-      <c r="BQ4" s="263"/>
-      <c r="BR4" s="263"/>
-      <c r="BS4" s="263"/>
+      <c r="BQ4" s="264"/>
+      <c r="BR4" s="264"/>
+      <c r="BS4" s="264"/>
       <c r="BT4" s="114"/>
       <c r="BU4" s="114" t="str">
         <f>IF(WEEKDAY(BU5,1)=1,"CN","")</f>
@@ -4061,31 +4057,31 @@
       <c r="ER4" s="237"/>
     </row>
     <row r="5" spans="1:149" s="183" customFormat="1" ht="92.25" customHeight="1">
-      <c r="A5" s="264" t="s">
+      <c r="A5" s="265" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="265" t="s">
+      <c r="B5" s="266" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="264" t="s">
+      <c r="C5" s="265" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="266" t="s">
+      <c r="D5" s="267" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="267" t="s">
+      <c r="E5" s="268" t="s">
         <v>120</v>
       </c>
-      <c r="F5" s="264" t="s">
+      <c r="F5" s="265" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="264" t="s">
+      <c r="G5" s="265" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="264" t="s">
+      <c r="H5" s="265" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="269" t="s">
+      <c r="I5" s="270" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="174">
@@ -4212,19 +4208,19 @@
         <f t="shared" si="0"/>
         <v>46112</v>
       </c>
-      <c r="AO5" s="270" t="s">
+      <c r="AO5" s="271" t="s">
         <v>82</v>
       </c>
-      <c r="AP5" s="270" t="s">
+      <c r="AP5" s="271" t="s">
         <v>83</v>
       </c>
-      <c r="AQ5" s="270" t="s">
+      <c r="AQ5" s="271" t="s">
         <v>84</v>
       </c>
-      <c r="AR5" s="271" t="s">
+      <c r="AR5" s="272" t="s">
         <v>5</v>
       </c>
-      <c r="AS5" s="271" t="s">
+      <c r="AS5" s="272" t="s">
         <v>6</v>
       </c>
       <c r="AT5" s="178">
@@ -4351,25 +4347,25 @@
         <f t="shared" si="1"/>
         <v>46112</v>
       </c>
-      <c r="BY5" s="272" t="s">
+      <c r="BY5" s="273" t="s">
         <v>85</v>
       </c>
-      <c r="BZ5" s="272" t="s">
+      <c r="BZ5" s="273" t="s">
         <v>86</v>
       </c>
-      <c r="CA5" s="272" t="s">
+      <c r="CA5" s="273" t="s">
         <v>87</v>
       </c>
-      <c r="CB5" s="272" t="s">
+      <c r="CB5" s="273" t="s">
         <v>88</v>
       </c>
-      <c r="CC5" s="272" t="s">
+      <c r="CC5" s="273" t="s">
         <v>89</v>
       </c>
-      <c r="CD5" s="272" t="s">
+      <c r="CD5" s="273" t="s">
         <v>90</v>
       </c>
-      <c r="CE5" s="272" t="s">
+      <c r="CE5" s="273" t="s">
         <v>91</v>
       </c>
       <c r="CF5" s="286" t="s">
@@ -4443,7 +4439,7 @@
       <c r="DT5" s="284" t="s">
         <v>125</v>
       </c>
-      <c r="DU5" s="265" t="s">
+      <c r="DU5" s="266" t="s">
         <v>13</v>
       </c>
       <c r="DV5" s="288" t="s">
@@ -4476,19 +4472,19 @@
       <c r="EI5" s="285" t="s">
         <v>72</v>
       </c>
-      <c r="EJ5" s="302" t="s">
+      <c r="EJ5" s="303" t="s">
         <v>78</v>
       </c>
-      <c r="EK5" s="302" t="s">
+      <c r="EK5" s="303" t="s">
         <v>80</v>
       </c>
-      <c r="EL5" s="302" t="s">
+      <c r="EL5" s="303" t="s">
         <v>79</v>
       </c>
       <c r="EM5" s="276" t="s">
         <v>124</v>
       </c>
-      <c r="EN5" s="300" t="s">
+      <c r="EN5" s="301" t="s">
         <v>118</v>
       </c>
       <c r="EO5" s="278" t="s">
@@ -4500,23 +4496,23 @@
       <c r="EQ5" s="280" t="s">
         <v>121</v>
       </c>
-      <c r="ER5" s="274" t="s">
+      <c r="ER5" s="304" t="s">
         <v>119</v>
       </c>
-      <c r="ES5" s="316" t="s">
+      <c r="ES5" s="300" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:149" s="205" customFormat="1" ht="148.5" customHeight="1">
-      <c r="A6" s="264"/>
-      <c r="B6" s="265"/>
-      <c r="C6" s="264"/>
-      <c r="D6" s="266"/>
-      <c r="E6" s="268"/>
-      <c r="F6" s="264"/>
-      <c r="G6" s="264"/>
-      <c r="H6" s="264"/>
-      <c r="I6" s="269"/>
+      <c r="A6" s="265"/>
+      <c r="B6" s="266"/>
+      <c r="C6" s="265"/>
+      <c r="D6" s="267"/>
+      <c r="E6" s="269"/>
+      <c r="F6" s="265"/>
+      <c r="G6" s="265"/>
+      <c r="H6" s="265"/>
+      <c r="I6" s="270"/>
       <c r="J6" s="184" t="str">
         <f t="shared" ref="J6:AN6" si="2">IF(WEEKDAY(J5)=1,"CN",WEEKDAY(J5))</f>
         <v>CN</v>
@@ -4641,11 +4637,11 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="AO6" s="270"/>
-      <c r="AP6" s="270"/>
-      <c r="AQ6" s="270"/>
-      <c r="AR6" s="271"/>
-      <c r="AS6" s="271"/>
+      <c r="AO6" s="271"/>
+      <c r="AP6" s="271"/>
+      <c r="AQ6" s="271"/>
+      <c r="AR6" s="272"/>
+      <c r="AS6" s="272"/>
       <c r="AT6" s="186" t="str">
         <f>+J6</f>
         <v>CN</v>
@@ -4770,13 +4766,13 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="BY6" s="273"/>
-      <c r="BZ6" s="273"/>
-      <c r="CA6" s="273"/>
-      <c r="CB6" s="273"/>
-      <c r="CC6" s="273"/>
-      <c r="CD6" s="273"/>
-      <c r="CE6" s="273"/>
+      <c r="BY6" s="274"/>
+      <c r="BZ6" s="274"/>
+      <c r="CA6" s="274"/>
+      <c r="CB6" s="274"/>
+      <c r="CC6" s="274"/>
+      <c r="CD6" s="274"/>
+      <c r="CE6" s="274"/>
       <c r="CF6" s="188" t="s">
         <v>92</v>
       </c>
@@ -4886,7 +4882,7 @@
       </c>
       <c r="DS6" s="299"/>
       <c r="DT6" s="284"/>
-      <c r="DU6" s="265"/>
+      <c r="DU6" s="266"/>
       <c r="DV6" s="203">
         <v>0.17499999999999999</v>
       </c>
@@ -4919,16 +4915,16 @@
       <c r="EG6" s="285"/>
       <c r="EH6" s="285"/>
       <c r="EI6" s="285"/>
-      <c r="EJ6" s="302"/>
-      <c r="EK6" s="302"/>
-      <c r="EL6" s="302"/>
+      <c r="EJ6" s="303"/>
+      <c r="EK6" s="303"/>
+      <c r="EL6" s="303"/>
       <c r="EM6" s="277"/>
-      <c r="EN6" s="301"/>
+      <c r="EN6" s="302"/>
       <c r="EO6" s="279"/>
       <c r="EP6" s="280"/>
       <c r="EQ6" s="280"/>
-      <c r="ER6" s="274"/>
-      <c r="ES6" s="316"/>
+      <c r="ER6" s="304"/>
+      <c r="ES6" s="300"/>
     </row>
     <row r="7" spans="1:149" s="106" customFormat="1" ht="87.75" customHeight="1">
       <c r="A7" s="275"/>
@@ -5412,7 +5408,7 @@
         <v>0</v>
       </c>
       <c r="DM8" s="159">
-        <f t="shared" ref="DM8" si="67">DL8*8%</f>
+        <f>IF(ES8 = 0,DL8*8%,0)</f>
         <v>0</v>
       </c>
       <c r="DN8" s="159">
@@ -5420,19 +5416,19 @@
         <v>0</v>
       </c>
       <c r="DO8" s="159">
-        <f t="shared" ref="DO8" si="68">DL8*1%</f>
+        <f>IF(ES8 = 0,DL8*1%,0)</f>
         <v>0</v>
       </c>
       <c r="DP8" s="159">
-        <f t="shared" ref="DP8" si="69">EI8</f>
+        <f t="shared" ref="DP8" si="67">EI8</f>
         <v>0</v>
       </c>
       <c r="DQ8" s="159">
-        <f t="shared" ref="DQ8" si="70">+SUM(DM8:DP8)</f>
+        <f t="shared" ref="DQ8" si="68">+SUM(DM8:DP8)</f>
         <v>0</v>
       </c>
       <c r="DR8" s="159">
-        <f t="shared" ref="DR8" si="71">SUM(DM8:DO8)</f>
+        <f t="shared" ref="DR8" si="69">SUM(DM8:DO8)</f>
         <v>0</v>
       </c>
       <c r="DS8" s="160">
@@ -5445,7 +5441,7 @@
         <v>0</v>
       </c>
       <c r="DV8" s="159">
-        <f>DL8*$DV$6</f>
+        <f>IF(ES8 = 0, DL8*$DV$6, 0)</f>
         <v>0</v>
       </c>
       <c r="DW8" s="159">
@@ -5453,7 +5449,7 @@
         <v>0</v>
       </c>
       <c r="DX8" s="159">
-        <f>DL8*$DX$6</f>
+        <f>IF(ES8 = 0, DL8*$DX$6, 0)</f>
         <v>0</v>
       </c>
       <c r="DY8" s="173">
@@ -5469,7 +5465,7 @@
         <v>0</v>
       </c>
       <c r="EB8" s="173">
-        <f t="shared" ref="EB8" si="72">DY8+DZ8+EA8</f>
+        <f t="shared" ref="EB8" si="70">DY8+DZ8+EA8</f>
         <v>0</v>
       </c>
       <c r="EC8" s="164">
@@ -5496,7 +5492,7 @@
         <v>-775000</v>
       </c>
       <c r="EI8" s="172">
-        <f t="shared" ref="EI8" si="73">+IF(EH8&lt;0,0,EH8)</f>
+        <f t="shared" ref="EI8" si="71">+IF(EH8&lt;0,0,EH8)</f>
         <v>0</v>
       </c>
       <c r="EJ8" s="165">
@@ -5517,7 +5513,7 @@
       <c r="EP8" s="150"/>
       <c r="EQ8" s="150"/>
       <c r="ER8" s="240"/>
-      <c r="ES8" s="315">
+      <c r="ES8" s="262">
         <v>0</v>
       </c>
     </row>
@@ -27197,6 +27193,8 @@
     <mergeCell ref="EJ5:EJ6"/>
     <mergeCell ref="EK5:EK6"/>
     <mergeCell ref="EL5:EL6"/>
+    <mergeCell ref="ER5:ER6"/>
+    <mergeCell ref="EQ5:EQ6"/>
     <mergeCell ref="EH5:EH6"/>
     <mergeCell ref="DV5:DX5"/>
     <mergeCell ref="CQ5:CS5"/>
@@ -27208,7 +27206,6 @@
     <mergeCell ref="DM5:DR5"/>
     <mergeCell ref="DS5:DS6"/>
     <mergeCell ref="DU5:DU6"/>
-    <mergeCell ref="ER5:ER6"/>
     <mergeCell ref="A7:EL7"/>
     <mergeCell ref="EM5:EM6"/>
     <mergeCell ref="EO5:EO6"/>
@@ -27223,7 +27220,8 @@
     <mergeCell ref="CE5:CE6"/>
     <mergeCell ref="DL5:DL6"/>
     <mergeCell ref="EG5:EG6"/>
-    <mergeCell ref="EQ5:EQ6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
     <mergeCell ref="BJ4:BK4"/>
     <mergeCell ref="BL4:BN4"/>
     <mergeCell ref="BQ4:BS4"/>
@@ -27234,8 +27232,6 @@
     <mergeCell ref="CA5:CA6"/>
     <mergeCell ref="CB5:CB6"/>
     <mergeCell ref="CC5:CC6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
     <mergeCell ref="I5:I6"/>
     <mergeCell ref="BG4:BI4"/>
     <mergeCell ref="AT4:AU4"/>
@@ -27912,11 +27908,11 @@
       <c r="F8" s="19"/>
       <c r="G8" s="19"/>
       <c r="H8" s="20"/>
-      <c r="I8" s="309">
+      <c r="I8" s="311">
         <v>2026</v>
       </c>
-      <c r="J8" s="310"/>
-      <c r="K8" s="310"/>
+      <c r="J8" s="312"/>
+      <c r="K8" s="312"/>
       <c r="L8" s="8"/>
       <c r="M8" s="8"/>
       <c r="N8" s="21" t="s">
@@ -27941,13 +27937,13 @@
     <row r="9" spans="1:29" ht="15.75" customHeight="1" thickBot="1">
       <c r="A9" s="23"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="311" t="s">
+      <c r="C9" s="313" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="312"/>
-      <c r="E9" s="312"/>
-      <c r="F9" s="312"/>
-      <c r="G9" s="312"/>
+      <c r="D9" s="314"/>
+      <c r="E9" s="314"/>
+      <c r="F9" s="314"/>
+      <c r="G9" s="314"/>
       <c r="H9" s="20"/>
       <c r="I9" s="24"/>
       <c r="J9" s="24"/>
@@ -28043,19 +28039,19 @@
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
-      <c r="J12" s="313" t="s">
+      <c r="J12" s="315" t="s">
         <v>35</v>
       </c>
-      <c r="K12" s="312"/>
-      <c r="L12" s="312"/>
-      <c r="M12" s="312"/>
-      <c r="N12" s="312"/>
-      <c r="O12" s="312"/>
-      <c r="P12" s="314">
+      <c r="K12" s="314"/>
+      <c r="L12" s="314"/>
+      <c r="M12" s="314"/>
+      <c r="N12" s="314"/>
+      <c r="O12" s="314"/>
+      <c r="P12" s="316">
         <f>I8</f>
         <v>2026</v>
       </c>
-      <c r="Q12" s="312"/>
+      <c r="Q12" s="314"/>
       <c r="R12" s="33"/>
       <c r="S12" s="34"/>
       <c r="T12" s="34"/>
@@ -28319,38 +28315,38 @@
     </row>
     <row r="21" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A21" s="39"/>
-      <c r="B21" s="308" t="s">
+      <c r="B21" s="310" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="304"/>
-      <c r="D21" s="304"/>
-      <c r="E21" s="304"/>
-      <c r="F21" s="304"/>
-      <c r="G21" s="304"/>
-      <c r="H21" s="304"/>
-      <c r="I21" s="304"/>
+      <c r="C21" s="306"/>
+      <c r="D21" s="306"/>
+      <c r="E21" s="306"/>
+      <c r="F21" s="306"/>
+      <c r="G21" s="306"/>
+      <c r="H21" s="306"/>
+      <c r="I21" s="306"/>
       <c r="J21" s="40"/>
-      <c r="K21" s="305" t="s">
+      <c r="K21" s="307" t="s">
         <v>37</v>
       </c>
-      <c r="L21" s="304"/>
-      <c r="M21" s="304"/>
-      <c r="N21" s="304"/>
-      <c r="O21" s="304"/>
-      <c r="P21" s="304"/>
-      <c r="Q21" s="304"/>
-      <c r="R21" s="304"/>
+      <c r="L21" s="306"/>
+      <c r="M21" s="306"/>
+      <c r="N21" s="306"/>
+      <c r="O21" s="306"/>
+      <c r="P21" s="306"/>
+      <c r="Q21" s="306"/>
+      <c r="R21" s="306"/>
       <c r="S21" s="40"/>
-      <c r="T21" s="303" t="s">
+      <c r="T21" s="305" t="s">
         <v>38</v>
       </c>
-      <c r="U21" s="304"/>
-      <c r="V21" s="304"/>
-      <c r="W21" s="304"/>
-      <c r="X21" s="304"/>
-      <c r="Y21" s="304"/>
-      <c r="Z21" s="304"/>
-      <c r="AA21" s="304"/>
+      <c r="U21" s="306"/>
+      <c r="V21" s="306"/>
+      <c r="W21" s="306"/>
+      <c r="X21" s="306"/>
+      <c r="Y21" s="306"/>
+      <c r="Z21" s="306"/>
+      <c r="AA21" s="306"/>
       <c r="AB21" s="41"/>
       <c r="AC21" s="42"/>
     </row>
@@ -29250,38 +29246,38 @@
     </row>
     <row r="35" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A35" s="69"/>
-      <c r="B35" s="306" t="s">
+      <c r="B35" s="308" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="304"/>
-      <c r="D35" s="304"/>
-      <c r="E35" s="304"/>
-      <c r="F35" s="304"/>
-      <c r="G35" s="304"/>
-      <c r="H35" s="304"/>
-      <c r="I35" s="304"/>
+      <c r="C35" s="306"/>
+      <c r="D35" s="306"/>
+      <c r="E35" s="306"/>
+      <c r="F35" s="306"/>
+      <c r="G35" s="306"/>
+      <c r="H35" s="306"/>
+      <c r="I35" s="306"/>
       <c r="J35" s="40"/>
-      <c r="K35" s="307" t="s">
+      <c r="K35" s="309" t="s">
         <v>48</v>
       </c>
-      <c r="L35" s="304"/>
-      <c r="M35" s="304"/>
-      <c r="N35" s="304"/>
-      <c r="O35" s="304"/>
-      <c r="P35" s="304"/>
-      <c r="Q35" s="304"/>
-      <c r="R35" s="304"/>
+      <c r="L35" s="306"/>
+      <c r="M35" s="306"/>
+      <c r="N35" s="306"/>
+      <c r="O35" s="306"/>
+      <c r="P35" s="306"/>
+      <c r="Q35" s="306"/>
+      <c r="R35" s="306"/>
       <c r="S35" s="40"/>
-      <c r="T35" s="305" t="s">
+      <c r="T35" s="307" t="s">
         <v>49</v>
       </c>
-      <c r="U35" s="304"/>
-      <c r="V35" s="304"/>
-      <c r="W35" s="304"/>
-      <c r="X35" s="304"/>
-      <c r="Y35" s="304"/>
-      <c r="Z35" s="304"/>
-      <c r="AA35" s="304"/>
+      <c r="U35" s="306"/>
+      <c r="V35" s="306"/>
+      <c r="W35" s="306"/>
+      <c r="X35" s="306"/>
+      <c r="Y35" s="306"/>
+      <c r="Z35" s="306"/>
+      <c r="AA35" s="306"/>
       <c r="AB35" s="70"/>
       <c r="AC35" s="40"/>
     </row>
@@ -30170,38 +30166,38 @@
     </row>
     <row r="49" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A49" s="69"/>
-      <c r="B49" s="305" t="s">
+      <c r="B49" s="307" t="s">
         <v>50</v>
       </c>
-      <c r="C49" s="304"/>
-      <c r="D49" s="304"/>
-      <c r="E49" s="304"/>
-      <c r="F49" s="304"/>
-      <c r="G49" s="304"/>
-      <c r="H49" s="304"/>
-      <c r="I49" s="304"/>
+      <c r="C49" s="306"/>
+      <c r="D49" s="306"/>
+      <c r="E49" s="306"/>
+      <c r="F49" s="306"/>
+      <c r="G49" s="306"/>
+      <c r="H49" s="306"/>
+      <c r="I49" s="306"/>
       <c r="J49" s="40"/>
-      <c r="K49" s="306" t="s">
+      <c r="K49" s="308" t="s">
         <v>51</v>
       </c>
-      <c r="L49" s="304"/>
-      <c r="M49" s="304"/>
-      <c r="N49" s="304"/>
-      <c r="O49" s="304"/>
-      <c r="P49" s="304"/>
-      <c r="Q49" s="304"/>
-      <c r="R49" s="304"/>
+      <c r="L49" s="306"/>
+      <c r="M49" s="306"/>
+      <c r="N49" s="306"/>
+      <c r="O49" s="306"/>
+      <c r="P49" s="306"/>
+      <c r="Q49" s="306"/>
+      <c r="R49" s="306"/>
       <c r="S49" s="40"/>
-      <c r="T49" s="308" t="s">
+      <c r="T49" s="310" t="s">
         <v>52</v>
       </c>
-      <c r="U49" s="304"/>
-      <c r="V49" s="304"/>
-      <c r="W49" s="304"/>
-      <c r="X49" s="304"/>
-      <c r="Y49" s="304"/>
-      <c r="Z49" s="304"/>
-      <c r="AA49" s="304"/>
+      <c r="U49" s="306"/>
+      <c r="V49" s="306"/>
+      <c r="W49" s="306"/>
+      <c r="X49" s="306"/>
+      <c r="Y49" s="306"/>
+      <c r="Z49" s="306"/>
+      <c r="AA49" s="306"/>
       <c r="AB49" s="70"/>
       <c r="AC49" s="40"/>
     </row>
@@ -31090,38 +31086,38 @@
     </row>
     <row r="63" spans="1:29" ht="18" customHeight="1" thickBot="1">
       <c r="A63" s="69"/>
-      <c r="B63" s="303" t="s">
+      <c r="B63" s="305" t="s">
         <v>53</v>
       </c>
-      <c r="C63" s="304"/>
-      <c r="D63" s="304"/>
-      <c r="E63" s="304"/>
-      <c r="F63" s="304"/>
-      <c r="G63" s="304"/>
-      <c r="H63" s="304"/>
-      <c r="I63" s="304"/>
+      <c r="C63" s="306"/>
+      <c r="D63" s="306"/>
+      <c r="E63" s="306"/>
+      <c r="F63" s="306"/>
+      <c r="G63" s="306"/>
+      <c r="H63" s="306"/>
+      <c r="I63" s="306"/>
       <c r="J63" s="40"/>
-      <c r="K63" s="305" t="s">
+      <c r="K63" s="307" t="s">
         <v>54</v>
       </c>
-      <c r="L63" s="304"/>
-      <c r="M63" s="304"/>
-      <c r="N63" s="304"/>
-      <c r="O63" s="304"/>
-      <c r="P63" s="304"/>
-      <c r="Q63" s="304"/>
-      <c r="R63" s="304"/>
+      <c r="L63" s="306"/>
+      <c r="M63" s="306"/>
+      <c r="N63" s="306"/>
+      <c r="O63" s="306"/>
+      <c r="P63" s="306"/>
+      <c r="Q63" s="306"/>
+      <c r="R63" s="306"/>
       <c r="S63" s="40"/>
-      <c r="T63" s="306" t="s">
+      <c r="T63" s="308" t="s">
         <v>55</v>
       </c>
-      <c r="U63" s="304"/>
-      <c r="V63" s="304"/>
-      <c r="W63" s="304"/>
-      <c r="X63" s="304"/>
-      <c r="Y63" s="304"/>
-      <c r="Z63" s="304"/>
-      <c r="AA63" s="304"/>
+      <c r="U63" s="306"/>
+      <c r="V63" s="306"/>
+      <c r="W63" s="306"/>
+      <c r="X63" s="306"/>
+      <c r="Y63" s="306"/>
+      <c r="Z63" s="306"/>
+      <c r="AA63" s="306"/>
       <c r="AB63" s="70"/>
       <c r="AC63" s="40"/>
     </row>

</xml_diff>